<commit_message>
Auto-deploy AR dashboard 2026-08-18 17:42
</commit_message>
<xml_diff>
--- a/AR Movement Report.xlsx
+++ b/AR Movement Report.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$123</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1055</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1059</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1320,7 +1320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1346,7 +1346,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data as of Tuesday, 18 August 2026 - 11:22  |  Source: PSI AR Monitoring Master.xlsx</t>
+          <t>Data as of Tuesday, 18 August 2026 - 17:42  |  Source: PSI AR Monitoring Master.xlsx</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="9" t="n">
-        <v>69718084636.44226</v>
+        <v>72452811302.08228</v>
       </c>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="10" t="n"/>
@@ -1394,7 +1394,7 @@
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="11" t="n"/>
       <c r="H7" s="13" t="n">
-        <v>12223583993.88358</v>
+        <v>14958310659.52359</v>
       </c>
       <c r="I7" s="10" t="n"/>
       <c r="J7" s="11" t="n"/>
@@ -1440,7 +1440,7 @@
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="19" t="n">
-        <v>30914968103.26546</v>
+        <v>33649694768.90546</v>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="10" t="n"/>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="26" t="n">
-        <v>23019402402.95342</v>
+        <v>25754129068.59342</v>
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="27" t="n">
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="B30" s="34" t="n">
-        <v>19336380190.49124</v>
+        <v>22071106856.13124</v>
       </c>
       <c r="C30" s="35" t="n">
         <v>3081528919.8</v>
@@ -2029,7 +2029,7 @@
         <v>22366266808.76546</v>
       </c>
       <c r="C41" s="49" t="n">
-        <v>8548701294.500001</v>
+        <v>11283427960.14</v>
       </c>
       <c r="D41" s="50">
         <f>SUM(B41:C41)</f>
@@ -2958,75 +2958,108 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="59" t="inlineStr">
+      <c r="A74" s="58" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="36" t="n">
+        <v>2734726665.64</v>
+      </c>
+      <c r="J74" s="37">
+        <f>SUM(B74:I74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="59" t="inlineStr">
         <is>
           <t>Total upcoming in October</t>
         </is>
       </c>
-      <c r="B74" s="40">
-        <f>SUM(B70:B73)</f>
+      <c r="B75" s="40">
+        <f>SUM(B70:B74)</f>
         <v/>
       </c>
-      <c r="C74" s="40">
-        <f>SUM(C70:C73)</f>
+      <c r="C75" s="40">
+        <f>SUM(C70:C74)</f>
         <v/>
       </c>
-      <c r="D74" s="40">
-        <f>SUM(D70:D73)</f>
+      <c r="D75" s="40">
+        <f>SUM(D70:D74)</f>
         <v/>
       </c>
-      <c r="E74" s="40">
-        <f>SUM(E70:E73)</f>
+      <c r="E75" s="40">
+        <f>SUM(E70:E74)</f>
         <v/>
       </c>
-      <c r="F74" s="40">
-        <f>SUM(F70:F73)</f>
+      <c r="F75" s="40">
+        <f>SUM(F70:F74)</f>
         <v/>
       </c>
-      <c r="G74" s="40">
-        <f>SUM(G70:G73)</f>
+      <c r="G75" s="40">
+        <f>SUM(G70:G74)</f>
         <v/>
       </c>
-      <c r="H74" s="40">
-        <f>SUM(H70:H73)</f>
+      <c r="H75" s="40">
+        <f>SUM(H70:H74)</f>
         <v/>
       </c>
-      <c r="I74" s="40">
-        <f>SUM(I70:I73)</f>
+      <c r="I75" s="40">
+        <f>SUM(I70:I74)</f>
         <v/>
       </c>
-      <c r="J74" s="40">
-        <f>SUM(J70:J73)</f>
+      <c r="J75" s="40">
+        <f>SUM(J70:J74)</f>
         <v/>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="60" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="60" t="inlineStr">
         <is>
           <t>Detail Sheets:</t>
         </is>
       </c>
-      <c r="B77" s="61" t="inlineStr">
+      <c r="B78" s="61" t="inlineStr">
         <is>
           <t>Daily Projection</t>
         </is>
       </c>
-      <c r="C77" s="61" t="inlineStr">
+      <c r="C78" s="61" t="inlineStr">
         <is>
           <t>Aging</t>
         </is>
       </c>
-      <c r="D77" s="61" t="inlineStr">
+      <c r="D78" s="61" t="inlineStr">
         <is>
           <t>Invoice vs Service</t>
         </is>
       </c>
-      <c r="E77" s="61" t="inlineStr">
+      <c r="E78" s="61" t="inlineStr">
         <is>
           <t>Service &amp; Billing</t>
         </is>
       </c>
-      <c r="F77" s="61" t="inlineStr">
+      <c r="F78" s="61" t="inlineStr">
         <is>
           <t>Raw Data</t>
         </is>
@@ -3062,11 +3095,11 @@
     <mergeCell ref="H6:J6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3400,7 +3433,7 @@
         <v>13809707763.51124</v>
       </c>
       <c r="D15" s="36" t="n">
-        <v>5526672426.98</v>
+        <v>8261399092.620001</v>
       </c>
       <c r="E15" s="36" t="n">
         <v>0</v>
@@ -3470,7 +3503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H123"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7468,24 +7501,160 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="39" t="inlineStr">
+      <c r="A123" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B123" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C123" s="76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
+        </is>
+      </c>
+      <c r="D123" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E123" s="77" t="n">
+        <v>1365520000</v>
+      </c>
+      <c r="F123" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G123" s="78" t="n">
+        <v>60</v>
+      </c>
+      <c r="H123" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B124" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C124" s="76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
+        </is>
+      </c>
+      <c r="D124" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E124" s="77" t="n">
+        <v>25780415.64</v>
+      </c>
+      <c r="F124" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G124" s="78" t="n">
+        <v>60</v>
+      </c>
+      <c r="H124" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B125" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C125" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
+        </is>
+      </c>
+      <c r="D125" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E125" s="77" t="n">
+        <v>1070726250</v>
+      </c>
+      <c r="F125" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G125" s="78" t="n">
+        <v>60</v>
+      </c>
+      <c r="H125" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B126" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C126" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
+        </is>
+      </c>
+      <c r="D126" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E126" s="77" t="n">
+        <v>272700000</v>
+      </c>
+      <c r="F126" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G126" s="78" t="n">
+        <v>60</v>
+      </c>
+      <c r="H126" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="39" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B123" s="79" t="n"/>
-      <c r="C123" s="79" t="n"/>
-      <c r="D123" s="79" t="n"/>
-      <c r="E123" s="80">
-        <f>SUM(E5:E122)</f>
+      <c r="B127" s="79" t="n"/>
+      <c r="C127" s="79" t="n"/>
+      <c r="D127" s="79" t="n"/>
+      <c r="E127" s="80">
+        <f>SUM(E5:E126)</f>
         <v/>
       </c>
-      <c r="F123" s="79" t="n"/>
-      <c r="G123" s="79" t="n"/>
-      <c r="H123" s="79" t="n"/>
+      <c r="F127" s="79" t="n"/>
+      <c r="G127" s="79" t="n"/>
+      <c r="H127" s="79" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H123"/>
+  <autoFilter ref="A4:H127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13595,25 +13764,25 @@
         <v>2735584761.64</v>
       </c>
       <c r="BQ33" s="86" t="n">
-        <v>0</v>
+        <v>2734726665.64</v>
       </c>
       <c r="BR33" s="36" t="n">
-        <v>2735584761.64</v>
+        <v>858095.9999995232</v>
       </c>
       <c r="BS33" s="85" t="n">
-        <v>0</v>
+        <v>2734726665.64</v>
       </c>
       <c r="BT33" s="86" t="n">
         <v>0</v>
       </c>
       <c r="BU33" s="36" t="n">
-        <v>0</v>
+        <v>2734726665.64</v>
       </c>
       <c r="BV33" s="40" t="n">
-        <v>54827133121.19</v>
+        <v>57561859786.83</v>
       </c>
       <c r="BW33" s="40" t="n">
-        <v>54827133121.19</v>
+        <v>57561859786.83</v>
       </c>
       <c r="BX33" s="40" t="n">
         <v>0</v>
@@ -15397,25 +15566,25 @@
         <v>12385574</v>
       </c>
       <c r="BQ42" s="90" t="n">
-        <v>0</v>
+        <v>12382742</v>
       </c>
       <c r="BR42" s="91" t="n">
-        <v>12385574</v>
+        <v>2832</v>
       </c>
       <c r="BS42" s="89" t="n">
-        <v>0</v>
+        <v>12382742</v>
       </c>
       <c r="BT42" s="90" t="n">
         <v>0</v>
       </c>
       <c r="BU42" s="91" t="n">
-        <v>0</v>
+        <v>12382742</v>
       </c>
       <c r="BV42" s="92" t="n">
-        <v>243124405.5</v>
+        <v>255507147.5</v>
       </c>
       <c r="BW42" s="92" t="n">
-        <v>243124405.5</v>
+        <v>255507147.5</v>
       </c>
       <c r="BX42" s="92" t="n">
         <v>0</v>
@@ -16156,20 +16325,20 @@
         </is>
       </c>
       <c r="B16" s="36" t="n">
-        <v>16097484417.24478</v>
+        <v>18832211082.88478</v>
       </c>
       <c r="C16" s="36" t="n">
         <v>11917212675.50339</v>
       </c>
       <c r="D16" s="97" t="n">
-        <v>4180271741.74139</v>
+        <v>6914998407.38139</v>
       </c>
       <c r="E16" s="98" t="n">
-        <v>0.7403152173725241</v>
+        <v>0.6328100626661982</v>
       </c>
       <c r="F16" s="99" t="inlineStr">
         <is>
-          <t>Partially uninvoiced</t>
+          <t>Many services uninvoiced</t>
         </is>
       </c>
     </row>
@@ -16183,13 +16352,13 @@
         <v>8853020012.243202</v>
       </c>
       <c r="C17" s="36" t="n">
-        <v>23019402402.95342</v>
+        <v>25754129068.59342</v>
       </c>
       <c r="D17" s="100" t="n">
-        <v>-14166382390.71022</v>
+        <v>-16901109056.35022</v>
       </c>
       <c r="E17" s="98" t="n">
-        <v>2.600175123417653</v>
+        <v>2.909078374721506</v>
       </c>
       <c r="F17" s="99" t="inlineStr">
         <is>
@@ -16276,7 +16445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1055"/>
+  <dimension ref="A1:Q1059"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -82167,29 +82336,41 @@
       </c>
       <c r="B1042" s="103" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C1042" s="103" t="n"/>
-      <c r="D1042" s="103" t="n"/>
-      <c r="E1042" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1042" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
+        </is>
+      </c>
+      <c r="D1042" s="104" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E1042" s="104" t="n">
+        <v>46312</v>
+      </c>
       <c r="F1042" s="103" t="n"/>
       <c r="G1042" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1042" s="103" t="inlineStr">
         <is>
-          <t>FIELD CORN</t>
+          <t>Rental CS</t>
         </is>
       </c>
       <c r="I1042" s="103" t="inlineStr">
         <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="J1042" s="103" t="n"/>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1042" s="103" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
       <c r="K1042" s="104" t="n">
         <v>46204</v>
       </c>
@@ -82197,16 +82378,22 @@
         <v>46234</v>
       </c>
       <c r="M1042" s="105" t="n">
-        <v>1034082</v>
+        <v>4000000</v>
       </c>
       <c r="N1042" s="105" t="n">
-        <v>4206172069.8522</v>
-      </c>
-      <c r="O1042" s="103" t="n"/>
-      <c r="P1042" s="103" t="n"/>
+        <v>1365520000</v>
+      </c>
+      <c r="O1042" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1042" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1042" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82218,29 +82405,41 @@
       </c>
       <c r="B1043" s="103" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C1043" s="103" t="n"/>
-      <c r="D1043" s="103" t="n"/>
-      <c r="E1043" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1043" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
+        </is>
+      </c>
+      <c r="D1043" s="104" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E1043" s="104" t="n">
+        <v>46312</v>
+      </c>
       <c r="F1043" s="103" t="n"/>
       <c r="G1043" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1043" s="103" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>Rental CS</t>
         </is>
       </c>
       <c r="I1043" s="103" t="inlineStr">
         <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="J1043" s="103" t="n"/>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1043" s="103" t="inlineStr">
+        <is>
+          <t>Handling</t>
+        </is>
+      </c>
       <c r="K1043" s="104" t="n">
         <v>46204</v>
       </c>
@@ -82248,16 +82447,22 @@
         <v>46234</v>
       </c>
       <c r="M1043" s="105" t="n">
-        <v>1816</v>
+        <v>607742</v>
       </c>
       <c r="N1043" s="105" t="n">
-        <v>9231791.4496</v>
-      </c>
-      <c r="O1043" s="103" t="n"/>
-      <c r="P1043" s="103" t="n"/>
+        <v>25780415.64</v>
+      </c>
+      <c r="O1043" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1043" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1043" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82269,26 +82474,34 @@
       </c>
       <c r="B1044" s="103" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C1044" s="103" t="n"/>
-      <c r="D1044" s="103" t="n"/>
-      <c r="E1044" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1044" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
+        </is>
+      </c>
+      <c r="D1044" s="104" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E1044" s="104" t="n">
+        <v>46312</v>
+      </c>
       <c r="F1044" s="103" t="n"/>
       <c r="G1044" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1044" s="103" t="inlineStr">
         <is>
-          <t>SWEET CORN</t>
+          <t>Rental CS</t>
         </is>
       </c>
       <c r="I1044" s="103" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1044" s="103" t="n"/>
@@ -82299,16 +82512,22 @@
         <v>46234</v>
       </c>
       <c r="M1044" s="105" t="n">
-        <v>18309</v>
+        <v>4175000</v>
       </c>
       <c r="N1044" s="105" t="n">
-        <v>156073086.756468</v>
-      </c>
-      <c r="O1044" s="103" t="n"/>
-      <c r="P1044" s="103" t="n"/>
+        <v>1070726250</v>
+      </c>
+      <c r="O1044" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1044" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1044" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82320,21 +82539,29 @@
       </c>
       <c r="B1045" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1045" s="103" t="n"/>
-      <c r="D1045" s="103" t="n"/>
-      <c r="E1045" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1045" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
+        </is>
+      </c>
+      <c r="D1045" s="104" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E1045" s="104" t="n">
+        <v>46312</v>
+      </c>
       <c r="F1045" s="103" t="n"/>
       <c r="G1045" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1045" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Rental WH</t>
         </is>
       </c>
       <c r="I1045" s="103" t="inlineStr">
@@ -82342,7 +82569,11 @@
           <t>Rental</t>
         </is>
       </c>
-      <c r="J1045" s="103" t="n"/>
+      <c r="J1045" s="103" t="inlineStr">
+        <is>
+          <t>zero material</t>
+        </is>
+      </c>
       <c r="K1045" s="104" t="n">
         <v>46204</v>
       </c>
@@ -82350,16 +82581,22 @@
         <v>46234</v>
       </c>
       <c r="M1045" s="105" t="n">
-        <v>1654962.70767742</v>
+        <v>3600000</v>
       </c>
       <c r="N1045" s="105" t="n">
-        <v>593353779.5835853</v>
-      </c>
-      <c r="O1045" s="103" t="n"/>
-      <c r="P1045" s="103" t="n"/>
+        <v>272700000</v>
+      </c>
+      <c r="O1045" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1045" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1045" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82371,7 +82608,7 @@
       </c>
       <c r="B1046" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1046" s="103" t="n"/>
@@ -82385,7 +82622,7 @@
       </c>
       <c r="H1046" s="103" t="inlineStr">
         <is>
-          <t>Reprocessing</t>
+          <t>FIELD CORN</t>
         </is>
       </c>
       <c r="I1046" s="103" t="inlineStr">
@@ -82401,10 +82638,10 @@
         <v>46234</v>
       </c>
       <c r="M1046" s="105" t="n">
-        <v>140049</v>
+        <v>1034082</v>
       </c>
       <c r="N1046" s="105" t="n">
-        <v>46711943.46</v>
+        <v>4206172069.8522</v>
       </c>
       <c r="O1046" s="103" t="n"/>
       <c r="P1046" s="103" t="n"/>
@@ -82422,7 +82659,7 @@
       </c>
       <c r="B1047" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1047" s="103" t="n"/>
@@ -82436,7 +82673,7 @@
       </c>
       <c r="H1047" s="103" t="inlineStr">
         <is>
-          <t>Reprocessing</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="I1047" s="103" t="inlineStr">
@@ -82452,10 +82689,10 @@
         <v>46234</v>
       </c>
       <c r="M1047" s="105" t="n">
-        <v>165711</v>
+        <v>1816</v>
       </c>
       <c r="N1047" s="105" t="n">
-        <v>40821247.74</v>
+        <v>9231791.4496</v>
       </c>
       <c r="O1047" s="103" t="n"/>
       <c r="P1047" s="103" t="n"/>
@@ -82473,7 +82710,7 @@
       </c>
       <c r="B1048" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1048" s="103" t="n"/>
@@ -82487,7 +82724,7 @@
       </c>
       <c r="H1048" s="103" t="inlineStr">
         <is>
-          <t>Reprocessing</t>
+          <t>SWEET CORN</t>
         </is>
       </c>
       <c r="I1048" s="103" t="inlineStr">
@@ -82503,10 +82740,10 @@
         <v>46234</v>
       </c>
       <c r="M1048" s="105" t="n">
-        <v>64695</v>
+        <v>18309</v>
       </c>
       <c r="N1048" s="105" t="n">
-        <v>20026984.2</v>
+        <v>156073086.756468</v>
       </c>
       <c r="O1048" s="103" t="n"/>
       <c r="P1048" s="103" t="n"/>
@@ -82538,12 +82775,12 @@
       </c>
       <c r="H1049" s="103" t="inlineStr">
         <is>
-          <t>Reprocessing</t>
+          <t>RENTAL CS</t>
         </is>
       </c>
       <c r="I1049" s="103" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1049" s="103" t="n"/>
@@ -82554,10 +82791,10 @@
         <v>46234</v>
       </c>
       <c r="M1049" s="105" t="n">
-        <v>40273</v>
+        <v>1654962.70767742</v>
       </c>
       <c r="N1049" s="105" t="n">
-        <v>12027934.18</v>
+        <v>593353779.5835853</v>
       </c>
       <c r="O1049" s="103" t="n"/>
       <c r="P1049" s="103" t="n"/>
@@ -82605,10 +82842,10 @@
         <v>46234</v>
       </c>
       <c r="M1050" s="105" t="n">
-        <v>19235</v>
+        <v>140049</v>
       </c>
       <c r="N1050" s="105" t="n">
-        <v>5535063.600000001</v>
+        <v>46711943.46</v>
       </c>
       <c r="O1050" s="103" t="n"/>
       <c r="P1050" s="103" t="n"/>
@@ -82626,7 +82863,7 @@
       </c>
       <c r="B1051" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1051" s="103" t="n"/>
@@ -82640,12 +82877,12 @@
       </c>
       <c r="H1051" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Reprocessing</t>
         </is>
       </c>
       <c r="I1051" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="J1051" s="103" t="n"/>
@@ -82656,10 +82893,10 @@
         <v>46234</v>
       </c>
       <c r="M1051" s="105" t="n">
-        <v>1660000</v>
+        <v>165711</v>
       </c>
       <c r="N1051" s="105" t="n">
-        <v>552691555.2</v>
+        <v>40821247.74</v>
       </c>
       <c r="O1051" s="103" t="n"/>
       <c r="P1051" s="103" t="n"/>
@@ -82677,7 +82914,7 @@
       </c>
       <c r="B1052" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1052" s="103" t="n"/>
@@ -82691,12 +82928,12 @@
       </c>
       <c r="H1052" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Reprocessing</t>
         </is>
       </c>
       <c r="I1052" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="J1052" s="103" t="n"/>
@@ -82707,10 +82944,10 @@
         <v>46234</v>
       </c>
       <c r="M1052" s="105" t="n">
-        <v>1660000</v>
+        <v>64695</v>
       </c>
       <c r="N1052" s="105" t="n">
-        <v>552691555.2</v>
+        <v>20026984.2</v>
       </c>
       <c r="O1052" s="103" t="n"/>
       <c r="P1052" s="103" t="n"/>
@@ -82728,7 +82965,7 @@
       </c>
       <c r="B1053" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1053" s="103" t="n"/>
@@ -82742,12 +82979,12 @@
       </c>
       <c r="H1053" s="103" t="inlineStr">
         <is>
-          <t>RENTAL</t>
+          <t>Reprocessing</t>
         </is>
       </c>
       <c r="I1053" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="J1053" s="103" t="n"/>
@@ -82758,10 +82995,10 @@
         <v>46234</v>
       </c>
       <c r="M1053" s="105" t="n">
-        <v>855000</v>
+        <v>40273</v>
       </c>
       <c r="N1053" s="105" t="n">
-        <v>71167361.40000001</v>
+        <v>12027934.18</v>
       </c>
       <c r="O1053" s="103" t="n"/>
       <c r="P1053" s="103" t="n"/>
@@ -82779,7 +83016,7 @@
       </c>
       <c r="B1054" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1054" s="103" t="n"/>
@@ -82793,12 +83030,12 @@
       </c>
       <c r="H1054" s="103" t="inlineStr">
         <is>
-          <t>RENTAL</t>
+          <t>Reprocessing</t>
         </is>
       </c>
       <c r="I1054" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="J1054" s="103" t="n"/>
@@ -82809,10 +83046,10 @@
         <v>46234</v>
       </c>
       <c r="M1054" s="105" t="n">
-        <v>3600000</v>
+        <v>19235</v>
       </c>
       <c r="N1054" s="105" t="n">
-        <v>299652048</v>
+        <v>5535063.600000001</v>
       </c>
       <c r="O1054" s="103" t="n"/>
       <c r="P1054" s="103" t="n"/>
@@ -82860,10 +83097,10 @@
         <v>46234</v>
       </c>
       <c r="M1055" s="105" t="n">
-        <v>4000000</v>
+        <v>1660000</v>
       </c>
       <c r="N1055" s="105" t="n">
-        <v>1605326400</v>
+        <v>552691555.2</v>
       </c>
       <c r="O1055" s="103" t="n"/>
       <c r="P1055" s="103" t="n"/>
@@ -82873,8 +83110,212 @@
         </is>
       </c>
     </row>
+    <row r="1056">
+      <c r="A1056" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1056" s="103" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1056" s="103" t="n"/>
+      <c r="D1056" s="103" t="n"/>
+      <c r="E1056" s="103" t="n"/>
+      <c r="F1056" s="103" t="n"/>
+      <c r="G1056" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1056" s="103" t="inlineStr">
+        <is>
+          <t>RENTAL CS</t>
+        </is>
+      </c>
+      <c r="I1056" s="103" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1056" s="103" t="n"/>
+      <c r="K1056" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1056" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1056" s="105" t="n">
+        <v>1660000</v>
+      </c>
+      <c r="N1056" s="105" t="n">
+        <v>552691555.2</v>
+      </c>
+      <c r="O1056" s="103" t="n"/>
+      <c r="P1056" s="103" t="n"/>
+      <c r="Q1056" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1057" s="103" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1057" s="103" t="n"/>
+      <c r="D1057" s="103" t="n"/>
+      <c r="E1057" s="103" t="n"/>
+      <c r="F1057" s="103" t="n"/>
+      <c r="G1057" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1057" s="103" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="I1057" s="103" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1057" s="103" t="n"/>
+      <c r="K1057" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1057" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1057" s="105" t="n">
+        <v>855000</v>
+      </c>
+      <c r="N1057" s="105" t="n">
+        <v>71167361.40000001</v>
+      </c>
+      <c r="O1057" s="103" t="n"/>
+      <c r="P1057" s="103" t="n"/>
+      <c r="Q1057" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1058" s="103" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1058" s="103" t="n"/>
+      <c r="D1058" s="103" t="n"/>
+      <c r="E1058" s="103" t="n"/>
+      <c r="F1058" s="103" t="n"/>
+      <c r="G1058" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1058" s="103" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="I1058" s="103" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1058" s="103" t="n"/>
+      <c r="K1058" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1058" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1058" s="105" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="N1058" s="105" t="n">
+        <v>299652048</v>
+      </c>
+      <c r="O1058" s="103" t="n"/>
+      <c r="P1058" s="103" t="n"/>
+      <c r="Q1058" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1059" s="103" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1059" s="103" t="n"/>
+      <c r="D1059" s="103" t="n"/>
+      <c r="E1059" s="103" t="n"/>
+      <c r="F1059" s="103" t="n"/>
+      <c r="G1059" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1059" s="103" t="inlineStr">
+        <is>
+          <t>RENTAL CS</t>
+        </is>
+      </c>
+      <c r="I1059" s="103" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1059" s="103" t="n"/>
+      <c r="K1059" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1059" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1059" s="105" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="N1059" s="105" t="n">
+        <v>1605326400</v>
+      </c>
+      <c r="O1059" s="103" t="n"/>
+      <c r="P1059" s="103" t="n"/>
+      <c r="Q1059" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q1055"/>
+  <autoFilter ref="A1:Q1059"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto-deploy AR dashboard 2026-08-20 17:10
</commit_message>
<xml_diff>
--- a/AR Movement Report.xlsx
+++ b/AR Movement Report.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$120</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1054</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1063</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1320,7 +1320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J78"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1346,7 +1346,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data as of Thursday, 20 August 2026 - 13:09  |  Source: PSI AR Monitoring Master.xlsx</t>
+          <t>Data as of Thursday, 20 August 2026 - 17:10  |  Source: PSI AR Monitoring Master.xlsx</t>
         </is>
       </c>
     </row>
@@ -1383,13 +1383,13 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="9" t="n">
-        <v>67943929583.94227</v>
+        <v>75731521342.77567</v>
       </c>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="10" t="n"/>
       <c r="D7" s="11" t="n"/>
       <c r="E7" s="12" t="n">
-        <v>57494500642.55869</v>
+        <v>65282092401.39208</v>
       </c>
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="11" t="n"/>
@@ -1440,7 +1440,7 @@
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="19" t="n">
-        <v>32222341970.56546</v>
+        <v>40009933729.39886</v>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="10" t="n"/>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="26" t="n">
-        <v>25740005068.59342</v>
+        <v>32495661670.68282</v>
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="27" t="n">
@@ -1600,7 +1600,7 @@
         </is>
       </c>
       <c r="B23" s="34" t="n">
-        <v>1473357319.28</v>
+        <v>2299760631.12</v>
       </c>
       <c r="C23" s="35" t="n">
         <v>4371476948.058269</v>
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="B30" s="34" t="n">
-        <v>20657878057.79124</v>
+        <v>27619066504.78464</v>
       </c>
       <c r="C30" s="36" t="n">
         <v>0</v>
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="B41" s="49" t="n">
-        <v>22366266808.76546</v>
+        <v>30153858567.59886</v>
       </c>
       <c r="C41" s="49" t="n">
         <v>9856075161.799999</v>
@@ -2603,7 +2603,7 @@
         <v>46284</v>
       </c>
       <c r="B63" s="36" t="n">
-        <v>0</v>
+        <v>826403311.84</v>
       </c>
       <c r="C63" s="36" t="n">
         <v>0</v>
@@ -2991,75 +2991,108 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="59" t="inlineStr">
+      <c r="A75" s="58" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B75" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C75" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="36" t="n">
+        <v>6961188446.9934</v>
+      </c>
+      <c r="J75" s="37">
+        <f>SUM(B75:I75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="59" t="inlineStr">
         <is>
           <t>Total upcoming in October</t>
         </is>
       </c>
-      <c r="B75" s="40">
-        <f>SUM(B70:B74)</f>
+      <c r="B76" s="40">
+        <f>SUM(B70:B75)</f>
         <v/>
       </c>
-      <c r="C75" s="40">
-        <f>SUM(C70:C74)</f>
+      <c r="C76" s="40">
+        <f>SUM(C70:C75)</f>
         <v/>
       </c>
-      <c r="D75" s="40">
-        <f>SUM(D70:D74)</f>
+      <c r="D76" s="40">
+        <f>SUM(D70:D75)</f>
         <v/>
       </c>
-      <c r="E75" s="40">
-        <f>SUM(E70:E74)</f>
+      <c r="E76" s="40">
+        <f>SUM(E70:E75)</f>
         <v/>
       </c>
-      <c r="F75" s="40">
-        <f>SUM(F70:F74)</f>
+      <c r="F76" s="40">
+        <f>SUM(F70:F75)</f>
         <v/>
       </c>
-      <c r="G75" s="40">
-        <f>SUM(G70:G74)</f>
+      <c r="G76" s="40">
+        <f>SUM(G70:G75)</f>
         <v/>
       </c>
-      <c r="H75" s="40">
-        <f>SUM(H70:H74)</f>
+      <c r="H76" s="40">
+        <f>SUM(H70:H75)</f>
         <v/>
       </c>
-      <c r="I75" s="40">
-        <f>SUM(I70:I74)</f>
+      <c r="I76" s="40">
+        <f>SUM(I70:I75)</f>
         <v/>
       </c>
-      <c r="J75" s="40">
-        <f>SUM(J70:J74)</f>
+      <c r="J76" s="40">
+        <f>SUM(J70:J75)</f>
         <v/>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="60" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="60" t="inlineStr">
         <is>
           <t>Detail Sheets:</t>
         </is>
       </c>
-      <c r="B78" s="61" t="inlineStr">
+      <c r="B79" s="61" t="inlineStr">
         <is>
           <t>Daily Projection</t>
         </is>
       </c>
-      <c r="C78" s="61" t="inlineStr">
+      <c r="C79" s="61" t="inlineStr">
         <is>
           <t>Aging</t>
         </is>
       </c>
-      <c r="D78" s="61" t="inlineStr">
+      <c r="D79" s="61" t="inlineStr">
         <is>
           <t>Invoice vs Service</t>
         </is>
       </c>
-      <c r="E78" s="61" t="inlineStr">
+      <c r="E79" s="61" t="inlineStr">
         <is>
           <t>Service &amp; Billing</t>
         </is>
       </c>
-      <c r="F78" s="61" t="inlineStr">
+      <c r="F79" s="61" t="inlineStr">
         <is>
           <t>Raw Data</t>
         </is>
@@ -3095,11 +3128,11 @@
     <mergeCell ref="H6:J6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3230,7 +3263,7 @@
         </is>
       </c>
       <c r="C7" s="36" t="n">
-        <v>0</v>
+        <v>826403311.84</v>
       </c>
       <c r="D7" s="36" t="n">
         <v>1473357319.28</v>
@@ -3430,7 +3463,7 @@
         </is>
       </c>
       <c r="C15" s="36" t="n">
-        <v>13809707763.51124</v>
+        <v>20770896210.50464</v>
       </c>
       <c r="D15" s="36" t="n">
         <v>6848170294.28</v>
@@ -3478,7 +3511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H120"/>
+  <dimension ref="A1:H129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6355,12 +6388,12 @@
       </c>
       <c r="B89" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C89" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
+          <t>PT.PSI/PT.ASI/FC_LMB_PGB/02/2026</t>
         </is>
       </c>
       <c r="D89" s="76" t="inlineStr">
@@ -6369,7 +6402,7 @@
         </is>
       </c>
       <c r="E89" s="77" t="n">
-        <v>326395903.6008</v>
+        <v>51019085</v>
       </c>
       <c r="F89" s="75" t="n">
         <v>46284</v>
@@ -6389,12 +6422,12 @@
       </c>
       <c r="B90" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C90" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
+          <t>PT.PSI/PT.ASI/FC_PAS2/03/26</t>
         </is>
       </c>
       <c r="D90" s="76" t="inlineStr">
@@ -6403,7 +6436,7 @@
         </is>
       </c>
       <c r="E90" s="77" t="n">
-        <v>240049.20888</v>
+        <v>119160408.84</v>
       </c>
       <c r="F90" s="75" t="n">
         <v>46284</v>
@@ -6419,16 +6452,16 @@
     </row>
     <row r="91">
       <c r="A91" s="75" t="n">
-        <v>46286</v>
+        <v>46284</v>
       </c>
       <c r="B91" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C91" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/51/2026 </t>
         </is>
       </c>
       <c r="D91" s="76" t="inlineStr">
@@ -6437,13 +6470,13 @@
         </is>
       </c>
       <c r="E91" s="77" t="n">
-        <v>570800977.7184</v>
+        <v>587478172</v>
       </c>
       <c r="F91" s="75" t="n">
-        <v>46286</v>
+        <v>46284</v>
       </c>
       <c r="G91" s="78" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H91" s="76" t="inlineStr">
         <is>
@@ -6453,16 +6486,16 @@
     </row>
     <row r="92">
       <c r="A92" s="75" t="n">
-        <v>46292</v>
+        <v>46284</v>
       </c>
       <c r="B92" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C92" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/43/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/52/2026 </t>
         </is>
       </c>
       <c r="D92" s="76" t="inlineStr">
@@ -6471,13 +6504,13 @@
         </is>
       </c>
       <c r="E92" s="77" t="n">
-        <v>103679056</v>
+        <v>68745646</v>
       </c>
       <c r="F92" s="75" t="n">
-        <v>46292</v>
+        <v>46284</v>
       </c>
       <c r="G92" s="78" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="H92" s="76" t="inlineStr">
         <is>
@@ -6487,16 +6520,16 @@
     </row>
     <row r="93">
       <c r="A93" s="75" t="n">
-        <v>46292</v>
+        <v>46284</v>
       </c>
       <c r="B93" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C93" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/44/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
         </is>
       </c>
       <c r="D93" s="76" t="inlineStr">
@@ -6505,13 +6538,13 @@
         </is>
       </c>
       <c r="E93" s="77" t="n">
-        <v>92863095</v>
+        <v>326395903.6008</v>
       </c>
       <c r="F93" s="75" t="n">
-        <v>46292</v>
+        <v>46284</v>
       </c>
       <c r="G93" s="78" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="H93" s="76" t="inlineStr">
         <is>
@@ -6521,16 +6554,16 @@
     </row>
     <row r="94">
       <c r="A94" s="75" t="n">
-        <v>46292</v>
+        <v>46284</v>
       </c>
       <c r="B94" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C94" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/45/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
         </is>
       </c>
       <c r="D94" s="76" t="inlineStr">
@@ -6539,13 +6572,13 @@
         </is>
       </c>
       <c r="E94" s="77" t="n">
-        <v>17392258</v>
+        <v>240049.20888</v>
       </c>
       <c r="F94" s="75" t="n">
-        <v>46292</v>
+        <v>46284</v>
       </c>
       <c r="G94" s="78" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="H94" s="76" t="inlineStr">
         <is>
@@ -6555,16 +6588,16 @@
     </row>
     <row r="95">
       <c r="A95" s="75" t="n">
-        <v>46292</v>
+        <v>46286</v>
       </c>
       <c r="B95" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C95" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/46/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
         </is>
       </c>
       <c r="D95" s="76" t="inlineStr">
@@ -6573,13 +6606,13 @@
         </is>
       </c>
       <c r="E95" s="77" t="n">
-        <v>197734556.5</v>
+        <v>570800977.7184</v>
       </c>
       <c r="F95" s="75" t="n">
-        <v>46292</v>
+        <v>46286</v>
       </c>
       <c r="G95" s="78" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="H95" s="76" t="inlineStr">
         <is>
@@ -6598,7 +6631,7 @@
       </c>
       <c r="C96" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/47/2026</t>
+          <t>PT.PSI/PT.BI/FC/43/2026</t>
         </is>
       </c>
       <c r="D96" s="76" t="inlineStr">
@@ -6607,7 +6640,7 @@
         </is>
       </c>
       <c r="E96" s="77" t="n">
-        <v>254755628.4</v>
+        <v>103679056</v>
       </c>
       <c r="F96" s="75" t="n">
         <v>46292</v>
@@ -6632,7 +6665,7 @@
       </c>
       <c r="C97" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/48/2026</t>
+          <t>PT.PSI/PT.BI/FC/44/2026</t>
         </is>
       </c>
       <c r="D97" s="76" t="inlineStr">
@@ -6641,7 +6674,7 @@
         </is>
       </c>
       <c r="E97" s="77" t="n">
-        <v>10599160</v>
+        <v>92863095</v>
       </c>
       <c r="F97" s="75" t="n">
         <v>46292</v>
@@ -6666,7 +6699,7 @@
       </c>
       <c r="C98" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/49/2026</t>
+          <t>PT.PSI/PT.BI/FC/45/2026</t>
         </is>
       </c>
       <c r="D98" s="76" t="inlineStr">
@@ -6675,7 +6708,7 @@
         </is>
       </c>
       <c r="E98" s="77" t="n">
-        <v>54405006.5</v>
+        <v>17392258</v>
       </c>
       <c r="F98" s="75" t="n">
         <v>46292</v>
@@ -6700,7 +6733,7 @@
       </c>
       <c r="C99" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/50/2026</t>
+          <t>PT.PSI/PT.BI/FC/46/2026</t>
         </is>
       </c>
       <c r="D99" s="76" t="inlineStr">
@@ -6709,7 +6742,7 @@
         </is>
       </c>
       <c r="E99" s="77" t="n">
-        <v>1075481.2</v>
+        <v>197734556.5</v>
       </c>
       <c r="F99" s="75" t="n">
         <v>46292</v>
@@ -6734,7 +6767,7 @@
       </c>
       <c r="C100" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/51/2026</t>
+          <t>PT.PSI/PT.BI/FC/47/2026</t>
         </is>
       </c>
       <c r="D100" s="76" t="inlineStr">
@@ -6743,7 +6776,7 @@
         </is>
       </c>
       <c r="E100" s="77" t="n">
-        <v>803447.72</v>
+        <v>254755628.4</v>
       </c>
       <c r="F100" s="75" t="n">
         <v>46292</v>
@@ -6768,7 +6801,7 @@
       </c>
       <c r="C101" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/52/2026</t>
+          <t>PT.PSI/PT.BI/FC/48/2026</t>
         </is>
       </c>
       <c r="D101" s="76" t="inlineStr">
@@ -6777,7 +6810,7 @@
         </is>
       </c>
       <c r="E101" s="77" t="n">
-        <v>7250789</v>
+        <v>10599160</v>
       </c>
       <c r="F101" s="75" t="n">
         <v>46292</v>
@@ -6802,7 +6835,7 @@
       </c>
       <c r="C102" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/53/2026</t>
+          <t>PT.PSI/PT.BI/FC/49/2026</t>
         </is>
       </c>
       <c r="D102" s="76" t="inlineStr">
@@ -6811,7 +6844,7 @@
         </is>
       </c>
       <c r="E102" s="77" t="n">
-        <v>101318334</v>
+        <v>54405006.5</v>
       </c>
       <c r="F102" s="75" t="n">
         <v>46292</v>
@@ -6827,7 +6860,7 @@
     </row>
     <row r="103">
       <c r="A103" s="75" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B103" s="76" t="inlineStr">
         <is>
@@ -6836,7 +6869,7 @@
       </c>
       <c r="C103" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/54/2026</t>
+          <t>PT.PSI/PT.BI/FC/50/2026</t>
         </is>
       </c>
       <c r="D103" s="76" t="inlineStr">
@@ -6845,13 +6878,13 @@
         </is>
       </c>
       <c r="E103" s="77" t="n">
-        <v>156400274.1</v>
+        <v>1075481.2</v>
       </c>
       <c r="F103" s="75" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="G103" s="78" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H103" s="76" t="inlineStr">
         <is>
@@ -6861,7 +6894,7 @@
     </row>
     <row r="104">
       <c r="A104" s="75" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B104" s="76" t="inlineStr">
         <is>
@@ -6870,7 +6903,7 @@
       </c>
       <c r="C104" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/55/2026</t>
+          <t>PT.PSI/PT.BI/FC/51/2026</t>
         </is>
       </c>
       <c r="D104" s="76" t="inlineStr">
@@ -6879,13 +6912,13 @@
         </is>
       </c>
       <c r="E104" s="77" t="n">
-        <v>50838199.5</v>
+        <v>803447.72</v>
       </c>
       <c r="F104" s="75" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="G104" s="78" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H104" s="76" t="inlineStr">
         <is>
@@ -6895,7 +6928,7 @@
     </row>
     <row r="105">
       <c r="A105" s="75" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B105" s="76" t="inlineStr">
         <is>
@@ -6904,7 +6937,7 @@
       </c>
       <c r="C105" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/56/2026</t>
+          <t>PT.PSI/PT.BI/FC/52/2026</t>
         </is>
       </c>
       <c r="D105" s="76" t="inlineStr">
@@ -6913,13 +6946,13 @@
         </is>
       </c>
       <c r="E105" s="77" t="n">
-        <v>376884765.6</v>
+        <v>7250789</v>
       </c>
       <c r="F105" s="75" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="G105" s="78" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H105" s="76" t="inlineStr">
         <is>
@@ -6929,7 +6962,7 @@
     </row>
     <row r="106">
       <c r="A106" s="75" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B106" s="76" t="inlineStr">
         <is>
@@ -6938,7 +6971,7 @@
       </c>
       <c r="C106" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/57/2026</t>
+          <t>PT.PSI/PT.BI/FC/53/2026</t>
         </is>
       </c>
       <c r="D106" s="76" t="inlineStr">
@@ -6947,13 +6980,13 @@
         </is>
       </c>
       <c r="E106" s="77" t="n">
-        <v>100336789</v>
+        <v>101318334</v>
       </c>
       <c r="F106" s="75" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="G106" s="78" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H106" s="76" t="inlineStr">
         <is>
@@ -6972,7 +7005,7 @@
       </c>
       <c r="C107" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/58/2026</t>
+          <t>PT.PSI/PT.BI/FC/54/2026</t>
         </is>
       </c>
       <c r="D107" s="76" t="inlineStr">
@@ -6981,7 +7014,7 @@
         </is>
       </c>
       <c r="E107" s="77" t="n">
-        <v>787756603.1999999</v>
+        <v>156400274.1</v>
       </c>
       <c r="F107" s="75" t="n">
         <v>46293</v>
@@ -7006,7 +7039,7 @@
       </c>
       <c r="C108" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/59/2026</t>
+          <t>PT.PSI/PT.BI/FC/55/2026</t>
         </is>
       </c>
       <c r="D108" s="76" t="inlineStr">
@@ -7015,7 +7048,7 @@
         </is>
       </c>
       <c r="E108" s="77" t="n">
-        <v>140859991.5</v>
+        <v>50838199.5</v>
       </c>
       <c r="F108" s="75" t="n">
         <v>46293</v>
@@ -7031,16 +7064,16 @@
     </row>
     <row r="109">
       <c r="A109" s="75" t="n">
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="B109" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C109" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
+          <t>PT.PSI/PT.BI/FC/56/2026</t>
         </is>
       </c>
       <c r="D109" s="76" t="inlineStr">
@@ -7049,13 +7082,13 @@
         </is>
       </c>
       <c r="E109" s="77" t="n">
-        <v>18871809.6</v>
+        <v>376884765.6</v>
       </c>
       <c r="F109" s="75" t="n">
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="G109" s="78" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="H109" s="76" t="inlineStr">
         <is>
@@ -7065,16 +7098,16 @@
     </row>
     <row r="110">
       <c r="A110" s="75" t="n">
-        <v>46301</v>
+        <v>46293</v>
       </c>
       <c r="B110" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C110" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
+          <t>PT.PSI/PT.BI/FC/57/2026</t>
         </is>
       </c>
       <c r="D110" s="76" t="inlineStr">
@@ -7083,13 +7116,13 @@
         </is>
       </c>
       <c r="E110" s="77" t="n">
-        <v>226017285.066</v>
+        <v>100336789</v>
       </c>
       <c r="F110" s="75" t="n">
-        <v>46301</v>
+        <v>46293</v>
       </c>
       <c r="G110" s="78" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H110" s="76" t="inlineStr">
         <is>
@@ -7099,16 +7132,16 @@
     </row>
     <row r="111">
       <c r="A111" s="75" t="n">
-        <v>46301</v>
+        <v>46293</v>
       </c>
       <c r="B111" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C111" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
+          <t>PT.PSI/PT.BI/FC/58/2026</t>
         </is>
       </c>
       <c r="D111" s="76" t="inlineStr">
@@ -7117,13 +7150,13 @@
         </is>
       </c>
       <c r="E111" s="77" t="n">
-        <v>3356193038.598001</v>
+        <v>787756603.1999999</v>
       </c>
       <c r="F111" s="75" t="n">
-        <v>46301</v>
+        <v>46293</v>
       </c>
       <c r="G111" s="78" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H111" s="76" t="inlineStr">
         <is>
@@ -7133,16 +7166,16 @@
     </row>
     <row r="112">
       <c r="A112" s="75" t="n">
-        <v>46301</v>
+        <v>46293</v>
       </c>
       <c r="B112" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C112" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
+          <t>PT.PSI/PT.BI/FC/59/2026</t>
         </is>
       </c>
       <c r="D112" s="76" t="inlineStr">
@@ -7151,13 +7184,13 @@
         </is>
       </c>
       <c r="E112" s="77" t="n">
-        <v>999055757.8296</v>
+        <v>140859991.5</v>
       </c>
       <c r="F112" s="75" t="n">
-        <v>46301</v>
+        <v>46293</v>
       </c>
       <c r="G112" s="78" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H112" s="76" t="inlineStr">
         <is>
@@ -7167,7 +7200,7 @@
     </row>
     <row r="113">
       <c r="A113" s="75" t="n">
-        <v>46305</v>
+        <v>46300</v>
       </c>
       <c r="B113" s="76" t="inlineStr">
         <is>
@@ -7176,7 +7209,7 @@
       </c>
       <c r="C113" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
         </is>
       </c>
       <c r="D113" s="76" t="inlineStr">
@@ -7185,13 +7218,13 @@
         </is>
       </c>
       <c r="E113" s="77" t="n">
-        <v>886307502.1920002</v>
+        <v>18871809.6</v>
       </c>
       <c r="F113" s="75" t="n">
-        <v>46305</v>
+        <v>46300</v>
       </c>
       <c r="G113" s="78" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="H113" s="76" t="inlineStr">
         <is>
@@ -7201,7 +7234,7 @@
     </row>
     <row r="114">
       <c r="A114" s="75" t="n">
-        <v>46308</v>
+        <v>46301</v>
       </c>
       <c r="B114" s="76" t="inlineStr">
         <is>
@@ -7210,7 +7243,7 @@
       </c>
       <c r="C114" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
         </is>
       </c>
       <c r="D114" s="76" t="inlineStr">
@@ -7219,13 +7252,13 @@
         </is>
       </c>
       <c r="E114" s="77" t="n">
-        <v>5676698527.872001</v>
+        <v>226017285.066</v>
       </c>
       <c r="F114" s="75" t="n">
-        <v>46308</v>
+        <v>46301</v>
       </c>
       <c r="G114" s="78" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="H114" s="76" t="inlineStr">
         <is>
@@ -7235,7 +7268,7 @@
     </row>
     <row r="115">
       <c r="A115" s="75" t="n">
-        <v>46308</v>
+        <v>46301</v>
       </c>
       <c r="B115" s="76" t="inlineStr">
         <is>
@@ -7244,7 +7277,7 @@
       </c>
       <c r="C115" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
         </is>
       </c>
       <c r="D115" s="76" t="inlineStr">
@@ -7253,13 +7286,13 @@
         </is>
       </c>
       <c r="E115" s="77" t="n">
-        <v>564189103.6416</v>
+        <v>3356193038.598001</v>
       </c>
       <c r="F115" s="75" t="n">
-        <v>46308</v>
+        <v>46301</v>
       </c>
       <c r="G115" s="78" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="H115" s="76" t="inlineStr">
         <is>
@@ -7269,7 +7302,7 @@
     </row>
     <row r="116">
       <c r="A116" s="75" t="n">
-        <v>46312</v>
+        <v>46301</v>
       </c>
       <c r="B116" s="76" t="inlineStr">
         <is>
@@ -7278,22 +7311,22 @@
       </c>
       <c r="C116" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
         </is>
       </c>
       <c r="D116" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E116" s="77" t="n">
-        <v>1365520000</v>
+        <v>999055757.8296</v>
       </c>
       <c r="F116" s="75" t="n">
-        <v>46312</v>
+        <v>46301</v>
       </c>
       <c r="G116" s="78" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="H116" s="76" t="inlineStr">
         <is>
@@ -7303,7 +7336,7 @@
     </row>
     <row r="117">
       <c r="A117" s="75" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="B117" s="76" t="inlineStr">
         <is>
@@ -7312,22 +7345,22 @@
       </c>
       <c r="C117" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
         </is>
       </c>
       <c r="D117" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E117" s="77" t="n">
-        <v>25780415.64</v>
+        <v>886307502.1920002</v>
       </c>
       <c r="F117" s="75" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="G117" s="78" t="n">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="H117" s="76" t="inlineStr">
         <is>
@@ -7337,7 +7370,7 @@
     </row>
     <row r="118">
       <c r="A118" s="75" t="n">
-        <v>46312</v>
+        <v>46308</v>
       </c>
       <c r="B118" s="76" t="inlineStr">
         <is>
@@ -7346,22 +7379,22 @@
       </c>
       <c r="C118" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
         </is>
       </c>
       <c r="D118" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E118" s="77" t="n">
-        <v>1070726250</v>
+        <v>5676698527.872001</v>
       </c>
       <c r="F118" s="75" t="n">
-        <v>46312</v>
+        <v>46308</v>
       </c>
       <c r="G118" s="78" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H118" s="76" t="inlineStr">
         <is>
@@ -7371,57 +7404,363 @@
     </row>
     <row r="119">
       <c r="A119" s="75" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B119" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C119" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
+        </is>
+      </c>
+      <c r="D119" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E119" s="77" t="n">
+        <v>564189103.6416</v>
+      </c>
+      <c r="F119" s="75" t="n">
+        <v>46308</v>
+      </c>
+      <c r="G119" s="78" t="n">
+        <v>54</v>
+      </c>
+      <c r="H119" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="75" t="n">
         <v>46312</v>
       </c>
-      <c r="B119" s="76" t="inlineStr">
+      <c r="B120" s="76" t="inlineStr">
         <is>
           <t>PT Syngenta Indonesia</t>
         </is>
       </c>
-      <c r="C119" s="76" t="inlineStr">
+      <c r="C120" s="76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
+        </is>
+      </c>
+      <c r="D120" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E120" s="77" t="n">
+        <v>1365520000</v>
+      </c>
+      <c r="F120" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G120" s="78" t="n">
+        <v>58</v>
+      </c>
+      <c r="H120" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B121" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C121" s="76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
+        </is>
+      </c>
+      <c r="D121" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E121" s="77" t="n">
+        <v>25780415.64</v>
+      </c>
+      <c r="F121" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G121" s="78" t="n">
+        <v>58</v>
+      </c>
+      <c r="H121" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B122" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C122" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
+        </is>
+      </c>
+      <c r="D122" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E122" s="77" t="n">
+        <v>1070726250</v>
+      </c>
+      <c r="F122" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G122" s="78" t="n">
+        <v>58</v>
+      </c>
+      <c r="H122" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B123" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C123" s="76" t="inlineStr">
         <is>
           <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
         </is>
       </c>
-      <c r="D119" s="76" t="inlineStr">
+      <c r="D123" s="76" t="inlineStr">
         <is>
           <t>Rental</t>
         </is>
       </c>
-      <c r="E119" s="77" t="n">
+      <c r="E123" s="77" t="n">
         <v>272700000</v>
       </c>
-      <c r="F119" s="75" t="n">
+      <c r="F123" s="75" t="n">
         <v>46312</v>
       </c>
-      <c r="G119" s="78" t="n">
+      <c r="G123" s="78" t="n">
         <v>58</v>
       </c>
-      <c r="H119" s="76" t="inlineStr">
+      <c r="H123" s="76" t="inlineStr">
         <is>
           <t>Future</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="39" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B124" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C124" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
+        </is>
+      </c>
+      <c r="D124" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E124" s="77" t="n">
+        <v>545818781.4912</v>
+      </c>
+      <c r="F124" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G124" s="78" t="n">
+        <v>60</v>
+      </c>
+      <c r="H124" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B125" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C125" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
+        </is>
+      </c>
+      <c r="D125" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E125" s="77" t="n">
+        <v>767367847.5204</v>
+      </c>
+      <c r="F125" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G125" s="78" t="n">
+        <v>60</v>
+      </c>
+      <c r="H125" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B126" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C126" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
+        </is>
+      </c>
+      <c r="D126" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E126" s="77" t="n">
+        <v>4761468367.9458</v>
+      </c>
+      <c r="F126" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G126" s="78" t="n">
+        <v>60</v>
+      </c>
+      <c r="H126" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B127" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C127" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+        </is>
+      </c>
+      <c r="D127" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E127" s="77" t="n">
+        <v>442076465.292</v>
+      </c>
+      <c r="F127" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G127" s="78" t="n">
+        <v>60</v>
+      </c>
+      <c r="H127" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B128" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C128" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+        </is>
+      </c>
+      <c r="D128" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E128" s="77" t="n">
+        <v>444456984.744</v>
+      </c>
+      <c r="F128" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G128" s="78" t="n">
+        <v>60</v>
+      </c>
+      <c r="H128" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="39" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B120" s="79" t="n"/>
-      <c r="C120" s="79" t="n"/>
-      <c r="D120" s="79" t="n"/>
-      <c r="E120" s="80">
-        <f>SUM(E5:E119)</f>
+      <c r="B129" s="79" t="n"/>
+      <c r="C129" s="79" t="n"/>
+      <c r="D129" s="79" t="n"/>
+      <c r="E129" s="80">
+        <f>SUM(E5:E128)</f>
         <v/>
       </c>
-      <c r="F120" s="79" t="n"/>
-      <c r="G120" s="79" t="n"/>
-      <c r="H120" s="79" t="n"/>
+      <c r="F129" s="79" t="n"/>
+      <c r="G129" s="79" t="n"/>
+      <c r="H129" s="79" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H120"/>
+  <autoFilter ref="A4:H129"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8303,25 +8642,25 @@
         <v>1440563725.87</v>
       </c>
       <c r="BQ8" s="86" t="n">
-        <v>751829762.9799999</v>
+        <v>990754902.8199999</v>
       </c>
       <c r="BR8" s="36" t="n">
-        <v>688733962.8900005</v>
+        <v>449808823.0500004</v>
       </c>
       <c r="BS8" s="85" t="n">
-        <v>0</v>
+        <v>238925139.84</v>
       </c>
       <c r="BT8" s="86" t="n">
         <v>0</v>
       </c>
       <c r="BU8" s="36" t="n">
-        <v>0</v>
+        <v>238925139.84</v>
       </c>
       <c r="BV8" s="40" t="n">
-        <v>147052801562.1454</v>
+        <v>147291726701.9854</v>
       </c>
       <c r="BW8" s="40" t="n">
-        <v>147052801562.1454</v>
+        <v>147291726701.9854</v>
       </c>
       <c r="BX8" s="40" t="n">
         <v>0</v>
@@ -9463,25 +9802,25 @@
         <v>1975035839.45968</v>
       </c>
       <c r="BQ13" s="86" t="n">
-        <v>5384826565.984081</v>
+        <v>5826903031.276081</v>
       </c>
       <c r="BR13" s="36" t="n">
-        <v>-3409790726.524402</v>
+        <v>-3851867191.816401</v>
       </c>
       <c r="BS13" s="85" t="n">
-        <v>11727333024.7992</v>
+        <v>18244064487.0486</v>
       </c>
       <c r="BT13" s="86" t="n">
-        <v>7239943389.343201</v>
+        <v>13314598386.3006</v>
       </c>
       <c r="BU13" s="36" t="n">
-        <v>4487389635.455999</v>
+        <v>4929466100.747999</v>
       </c>
       <c r="BV13" s="40" t="n">
-        <v>134023511784.8631</v>
+        <v>140540243247.1125</v>
       </c>
       <c r="BW13" s="40" t="n">
-        <v>134023511784.8631</v>
+        <v>140540243247.1125</v>
       </c>
       <c r="BX13" s="40" t="n">
         <v>0</v>
@@ -10569,25 +10908,25 @@
         <v>1070910</v>
       </c>
       <c r="BQ19" s="90" t="n">
-        <v>364864</v>
+        <v>534051</v>
       </c>
       <c r="BR19" s="91" t="n">
-        <v>706046</v>
+        <v>536859</v>
       </c>
       <c r="BS19" s="89" t="n">
-        <v>0</v>
+        <v>169187</v>
       </c>
       <c r="BT19" s="90" t="n">
         <v>0</v>
       </c>
       <c r="BU19" s="91" t="n">
-        <v>0</v>
+        <v>169187</v>
       </c>
       <c r="BV19" s="92" t="n">
-        <v>51996733</v>
+        <v>52165920</v>
       </c>
       <c r="BW19" s="92" t="n">
-        <v>51996733</v>
+        <v>52165920</v>
       </c>
       <c r="BX19" s="92" t="n">
         <v>0</v>
@@ -11729,25 +12068,25 @@
         <v>579104.28</v>
       </c>
       <c r="BQ24" s="90" t="n">
-        <v>1267275.28</v>
+        <v>1393555.28</v>
       </c>
       <c r="BR24" s="91" t="n">
-        <v>-688171</v>
+        <v>-814451</v>
       </c>
       <c r="BS24" s="89" t="n">
-        <v>2775914</v>
+        <v>4362603</v>
       </c>
       <c r="BT24" s="90" t="n">
-        <v>1572250</v>
+        <v>3032659</v>
       </c>
       <c r="BU24" s="91" t="n">
-        <v>1203664</v>
+        <v>1329944</v>
       </c>
       <c r="BV24" s="92" t="n">
-        <v>38645159.01</v>
+        <v>40231848.01</v>
       </c>
       <c r="BW24" s="92" t="n">
-        <v>38645159.01</v>
+        <v>40231848.01</v>
       </c>
       <c r="BX24" s="92" t="n">
         <v>0</v>
@@ -16092,16 +16431,16 @@
         </is>
       </c>
       <c r="B16" s="36" t="n">
-        <v>18818087082.88478</v>
+        <v>19499088688.01678</v>
       </c>
       <c r="C16" s="36" t="n">
         <v>11917212675.50339</v>
       </c>
       <c r="D16" s="97" t="n">
-        <v>6900874407.38139</v>
+        <v>7581876012.51339</v>
       </c>
       <c r="E16" s="98" t="n">
-        <v>0.6332850211083465</v>
+        <v>0.6111676738424779</v>
       </c>
       <c r="F16" s="99" t="inlineStr">
         <is>
@@ -16116,16 +16455,16 @@
         </is>
       </c>
       <c r="B17" s="36" t="n">
-        <v>8853020012.243202</v>
+        <v>14927675009.2006</v>
       </c>
       <c r="C17" s="36" t="n">
-        <v>25740005068.59342</v>
+        <v>32495661670.68282</v>
       </c>
       <c r="D17" s="100" t="n">
-        <v>-16886985056.35022</v>
+        <v>-17567986661.48222</v>
       </c>
       <c r="E17" s="98" t="n">
-        <v>2.907482986935138</v>
+        <v>2.176873602262527</v>
       </c>
       <c r="F17" s="99" t="inlineStr">
         <is>
@@ -16212,7 +16551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1054"/>
+  <dimension ref="A1:Q1063"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -82370,18 +82709,26 @@
           <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
-      <c r="C1046" s="103" t="n"/>
-      <c r="D1046" s="103" t="n"/>
-      <c r="E1046" s="103" t="n"/>
+      <c r="C1046" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.ASI/FC_LMB_PGB/02/2026</t>
+        </is>
+      </c>
+      <c r="D1046" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1046" s="104" t="n">
+        <v>46284</v>
+      </c>
       <c r="F1046" s="103" t="n"/>
       <c r="G1046" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1046" s="103" t="inlineStr">
         <is>
-          <t>FIELD CORN</t>
+          <t>Processing - LMB</t>
         </is>
       </c>
       <c r="I1046" s="103" t="inlineStr">
@@ -82391,22 +82738,28 @@
       </c>
       <c r="J1046" s="103" t="n"/>
       <c r="K1046" s="104" t="n">
-        <v>46204</v>
+        <v>46217</v>
       </c>
       <c r="L1046" s="104" t="n">
-        <v>46234</v>
+        <v>46231</v>
       </c>
       <c r="M1046" s="105" t="n">
-        <v>1034082</v>
+        <v>9854</v>
       </c>
       <c r="N1046" s="105" t="n">
-        <v>4206172069.8522</v>
-      </c>
-      <c r="O1046" s="103" t="n"/>
-      <c r="P1046" s="103" t="n"/>
+        <v>51019085</v>
+      </c>
+      <c r="O1046" s="103" t="n">
+        <v>-30</v>
+      </c>
+      <c r="P1046" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1046" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82421,18 +82774,26 @@
           <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
-      <c r="C1047" s="103" t="n"/>
-      <c r="D1047" s="103" t="n"/>
-      <c r="E1047" s="103" t="n"/>
+      <c r="C1047" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.ASI/FC_PAS2/03/26</t>
+        </is>
+      </c>
+      <c r="D1047" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1047" s="104" t="n">
+        <v>46284</v>
+      </c>
       <c r="F1047" s="103" t="n"/>
       <c r="G1047" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1047" s="103" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1047" s="103" t="inlineStr">
@@ -82442,22 +82803,28 @@
       </c>
       <c r="J1047" s="103" t="n"/>
       <c r="K1047" s="104" t="n">
-        <v>46204</v>
+        <v>46203</v>
       </c>
       <c r="L1047" s="104" t="n">
-        <v>46234</v>
+        <v>46220</v>
       </c>
       <c r="M1047" s="105" t="n">
-        <v>1816</v>
+        <v>29293</v>
       </c>
       <c r="N1047" s="105" t="n">
-        <v>9231791.4496</v>
-      </c>
-      <c r="O1047" s="103" t="n"/>
-      <c r="P1047" s="103" t="n"/>
+        <v>119160408.84</v>
+      </c>
+      <c r="O1047" s="103" t="n">
+        <v>-30</v>
+      </c>
+      <c r="P1047" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1047" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82472,18 +82839,26 @@
           <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
-      <c r="C1048" s="103" t="n"/>
-      <c r="D1048" s="103" t="n"/>
-      <c r="E1048" s="103" t="n"/>
+      <c r="C1048" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/51/2026 </t>
+        </is>
+      </c>
+      <c r="D1048" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1048" s="104" t="n">
+        <v>46284</v>
+      </c>
       <c r="F1048" s="103" t="n"/>
       <c r="G1048" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1048" s="103" t="inlineStr">
         <is>
-          <t>SWEET CORN</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1048" s="103" t="inlineStr">
@@ -82499,16 +82874,22 @@
         <v>46234</v>
       </c>
       <c r="M1048" s="105" t="n">
-        <v>18309</v>
+        <v>555640</v>
       </c>
       <c r="N1048" s="105" t="n">
-        <v>156073086.756468</v>
-      </c>
-      <c r="O1048" s="103" t="n"/>
-      <c r="P1048" s="103" t="n"/>
+        <v>587478172</v>
+      </c>
+      <c r="O1048" s="103" t="n">
+        <v>-30</v>
+      </c>
+      <c r="P1048" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1048" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82520,46 +82901,60 @@
       </c>
       <c r="B1049" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1049" s="103" t="n"/>
-      <c r="D1049" s="103" t="n"/>
-      <c r="E1049" s="103" t="n"/>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C1049" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/52/2026 </t>
+        </is>
+      </c>
+      <c r="D1049" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1049" s="104" t="n">
+        <v>46284</v>
+      </c>
       <c r="F1049" s="103" t="n"/>
       <c r="G1049" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1049" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1049" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="J1049" s="103" t="n"/>
       <c r="K1049" s="104" t="n">
-        <v>46204</v>
+        <v>46230</v>
       </c>
       <c r="L1049" s="104" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="M1049" s="105" t="n">
-        <v>1654962.70767742</v>
+        <v>130040</v>
       </c>
       <c r="N1049" s="105" t="n">
-        <v>593353779.5835853</v>
-      </c>
-      <c r="O1049" s="103" t="n"/>
-      <c r="P1049" s="103" t="n"/>
+        <v>68745646</v>
+      </c>
+      <c r="O1049" s="103" t="n">
+        <v>-30</v>
+      </c>
+      <c r="P1049" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1049" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82571,21 +82966,29 @@
       </c>
       <c r="B1050" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1050" s="103" t="n"/>
-      <c r="D1050" s="103" t="n"/>
-      <c r="E1050" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1050" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
+        </is>
+      </c>
+      <c r="D1050" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1050" s="104" t="n">
+        <v>46314</v>
+      </c>
       <c r="F1050" s="103" t="n"/>
       <c r="G1050" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1050" s="103" t="inlineStr">
         <is>
-          <t>Reprocessing</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1050" s="103" t="inlineStr">
@@ -82595,22 +82998,28 @@
       </c>
       <c r="J1050" s="103" t="n"/>
       <c r="K1050" s="104" t="n">
-        <v>46204</v>
+        <v>46245</v>
       </c>
       <c r="L1050" s="104" t="n">
-        <v>46234</v>
+        <v>46247</v>
       </c>
       <c r="M1050" s="105" t="n">
-        <v>140049</v>
+        <v>38976</v>
       </c>
       <c r="N1050" s="105" t="n">
-        <v>46711943.46</v>
-      </c>
-      <c r="O1050" s="103" t="n"/>
-      <c r="P1050" s="103" t="n"/>
+        <v>545818781.4912</v>
+      </c>
+      <c r="O1050" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1050" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1050" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82622,21 +83031,29 @@
       </c>
       <c r="B1051" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1051" s="103" t="n"/>
-      <c r="D1051" s="103" t="n"/>
-      <c r="E1051" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1051" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
+        </is>
+      </c>
+      <c r="D1051" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1051" s="104" t="n">
+        <v>46314</v>
+      </c>
       <c r="F1051" s="103" t="n"/>
       <c r="G1051" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1051" s="103" t="inlineStr">
         <is>
-          <t>Reprocessing</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1051" s="103" t="inlineStr">
@@ -82646,22 +83063,28 @@
       </c>
       <c r="J1051" s="103" t="n"/>
       <c r="K1051" s="104" t="n">
-        <v>46204</v>
+        <v>46242</v>
       </c>
       <c r="L1051" s="104" t="n">
-        <v>46234</v>
+        <v>46243</v>
       </c>
       <c r="M1051" s="105" t="n">
-        <v>165711</v>
+        <v>197286</v>
       </c>
       <c r="N1051" s="105" t="n">
-        <v>40821247.74</v>
-      </c>
-      <c r="O1051" s="103" t="n"/>
-      <c r="P1051" s="103" t="n"/>
+        <v>767367847.5204</v>
+      </c>
+      <c r="O1051" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1051" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1051" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82673,21 +83096,29 @@
       </c>
       <c r="B1052" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1052" s="103" t="n"/>
-      <c r="D1052" s="103" t="n"/>
-      <c r="E1052" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1052" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
+        </is>
+      </c>
+      <c r="D1052" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1052" s="104" t="n">
+        <v>46314</v>
+      </c>
       <c r="F1052" s="103" t="n"/>
       <c r="G1052" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1052" s="103" t="inlineStr">
         <is>
-          <t>Reprocessing</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1052" s="103" t="inlineStr">
@@ -82697,22 +83128,28 @@
       </c>
       <c r="J1052" s="103" t="n"/>
       <c r="K1052" s="104" t="n">
-        <v>46204</v>
+        <v>46242</v>
       </c>
       <c r="L1052" s="104" t="n">
-        <v>46234</v>
+        <v>46248</v>
       </c>
       <c r="M1052" s="105" t="n">
-        <v>64695</v>
+        <v>1224147</v>
       </c>
       <c r="N1052" s="105" t="n">
-        <v>20026984.2</v>
-      </c>
-      <c r="O1052" s="103" t="n"/>
-      <c r="P1052" s="103" t="n"/>
+        <v>4761468367.9458</v>
+      </c>
+      <c r="O1052" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1052" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1052" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82724,21 +83161,29 @@
       </c>
       <c r="B1053" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1053" s="103" t="n"/>
-      <c r="D1053" s="103" t="n"/>
-      <c r="E1053" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1053" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+        </is>
+      </c>
+      <c r="D1053" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1053" s="104" t="n">
+        <v>46314</v>
+      </c>
       <c r="F1053" s="103" t="n"/>
       <c r="G1053" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1053" s="103" t="inlineStr">
         <is>
-          <t>Reprocessing</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1053" s="103" t="inlineStr">
@@ -82748,22 +83193,28 @@
       </c>
       <c r="J1053" s="103" t="n"/>
       <c r="K1053" s="104" t="n">
-        <v>46204</v>
+        <v>46226</v>
       </c>
       <c r="L1053" s="104" t="n">
-        <v>46234</v>
+        <v>46229</v>
       </c>
       <c r="M1053" s="105" t="n">
-        <v>40273</v>
+        <v>126280</v>
       </c>
       <c r="N1053" s="105" t="n">
-        <v>12027934.18</v>
-      </c>
-      <c r="O1053" s="103" t="n"/>
-      <c r="P1053" s="103" t="n"/>
+        <v>442076465.292</v>
+      </c>
+      <c r="O1053" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1053" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1053" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -82775,21 +83226,29 @@
       </c>
       <c r="B1054" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1054" s="103" t="n"/>
-      <c r="D1054" s="103" t="n"/>
-      <c r="E1054" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1054" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+        </is>
+      </c>
+      <c r="D1054" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1054" s="104" t="n">
+        <v>46314</v>
+      </c>
       <c r="F1054" s="103" t="n"/>
       <c r="G1054" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1054" s="103" t="inlineStr">
         <is>
-          <t>Reprocessing</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1054" s="103" t="inlineStr">
@@ -82799,27 +83258,492 @@
       </c>
       <c r="J1054" s="103" t="n"/>
       <c r="K1054" s="104" t="n">
+        <v>46247</v>
+      </c>
+      <c r="L1054" s="104" t="n">
+        <v>46252</v>
+      </c>
+      <c r="M1054" s="105" t="n">
+        <v>126960</v>
+      </c>
+      <c r="N1054" s="105" t="n">
+        <v>444456984.744</v>
+      </c>
+      <c r="O1054" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1054" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+      <c r="Q1054" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B1055" s="103" t="inlineStr">
+        <is>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C1055" s="103" t="n"/>
+      <c r="D1055" s="103" t="n"/>
+      <c r="E1055" s="103" t="n"/>
+      <c r="F1055" s="103" t="n"/>
+      <c r="G1055" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1055" s="103" t="inlineStr">
+        <is>
+          <t>FIELD CORN</t>
+        </is>
+      </c>
+      <c r="I1055" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1055" s="103" t="n"/>
+      <c r="K1055" s="104" t="n">
         <v>46204</v>
       </c>
-      <c r="L1054" s="104" t="n">
+      <c r="L1055" s="104" t="n">
         <v>46234</v>
       </c>
-      <c r="M1054" s="105" t="n">
+      <c r="M1055" s="105" t="n">
+        <v>1034082</v>
+      </c>
+      <c r="N1055" s="105" t="n">
+        <v>4206172069.8522</v>
+      </c>
+      <c r="O1055" s="103" t="n"/>
+      <c r="P1055" s="103" t="n"/>
+      <c r="Q1055" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B1056" s="103" t="inlineStr">
+        <is>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C1056" s="103" t="n"/>
+      <c r="D1056" s="103" t="n"/>
+      <c r="E1056" s="103" t="n"/>
+      <c r="F1056" s="103" t="n"/>
+      <c r="G1056" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1056" s="103" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="I1056" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1056" s="103" t="n"/>
+      <c r="K1056" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1056" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1056" s="105" t="n">
+        <v>1816</v>
+      </c>
+      <c r="N1056" s="105" t="n">
+        <v>9231791.4496</v>
+      </c>
+      <c r="O1056" s="103" t="n"/>
+      <c r="P1056" s="103" t="n"/>
+      <c r="Q1056" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B1057" s="103" t="inlineStr">
+        <is>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C1057" s="103" t="n"/>
+      <c r="D1057" s="103" t="n"/>
+      <c r="E1057" s="103" t="n"/>
+      <c r="F1057" s="103" t="n"/>
+      <c r="G1057" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1057" s="103" t="inlineStr">
+        <is>
+          <t>SWEET CORN</t>
+        </is>
+      </c>
+      <c r="I1057" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1057" s="103" t="n"/>
+      <c r="K1057" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1057" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1057" s="105" t="n">
+        <v>18309</v>
+      </c>
+      <c r="N1057" s="105" t="n">
+        <v>156073086.756468</v>
+      </c>
+      <c r="O1057" s="103" t="n"/>
+      <c r="P1057" s="103" t="n"/>
+      <c r="Q1057" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B1058" s="103" t="inlineStr">
+        <is>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1058" s="103" t="n"/>
+      <c r="D1058" s="103" t="n"/>
+      <c r="E1058" s="103" t="n"/>
+      <c r="F1058" s="103" t="n"/>
+      <c r="G1058" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1058" s="103" t="inlineStr">
+        <is>
+          <t>RENTAL CS</t>
+        </is>
+      </c>
+      <c r="I1058" s="103" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1058" s="103" t="n"/>
+      <c r="K1058" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1058" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1058" s="105" t="n">
+        <v>1654962.70767742</v>
+      </c>
+      <c r="N1058" s="105" t="n">
+        <v>593353779.5835853</v>
+      </c>
+      <c r="O1058" s="103" t="n"/>
+      <c r="P1058" s="103" t="n"/>
+      <c r="Q1058" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B1059" s="103" t="inlineStr">
+        <is>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1059" s="103" t="n"/>
+      <c r="D1059" s="103" t="n"/>
+      <c r="E1059" s="103" t="n"/>
+      <c r="F1059" s="103" t="n"/>
+      <c r="G1059" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1059" s="103" t="inlineStr">
+        <is>
+          <t>Reprocessing</t>
+        </is>
+      </c>
+      <c r="I1059" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1059" s="103" t="n"/>
+      <c r="K1059" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1059" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1059" s="105" t="n">
+        <v>140049</v>
+      </c>
+      <c r="N1059" s="105" t="n">
+        <v>46711943.46</v>
+      </c>
+      <c r="O1059" s="103" t="n"/>
+      <c r="P1059" s="103" t="n"/>
+      <c r="Q1059" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B1060" s="103" t="inlineStr">
+        <is>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1060" s="103" t="n"/>
+      <c r="D1060" s="103" t="n"/>
+      <c r="E1060" s="103" t="n"/>
+      <c r="F1060" s="103" t="n"/>
+      <c r="G1060" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1060" s="103" t="inlineStr">
+        <is>
+          <t>Reprocessing</t>
+        </is>
+      </c>
+      <c r="I1060" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1060" s="103" t="n"/>
+      <c r="K1060" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1060" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1060" s="105" t="n">
+        <v>165711</v>
+      </c>
+      <c r="N1060" s="105" t="n">
+        <v>40821247.74</v>
+      </c>
+      <c r="O1060" s="103" t="n"/>
+      <c r="P1060" s="103" t="n"/>
+      <c r="Q1060" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B1061" s="103" t="inlineStr">
+        <is>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1061" s="103" t="n"/>
+      <c r="D1061" s="103" t="n"/>
+      <c r="E1061" s="103" t="n"/>
+      <c r="F1061" s="103" t="n"/>
+      <c r="G1061" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1061" s="103" t="inlineStr">
+        <is>
+          <t>Reprocessing</t>
+        </is>
+      </c>
+      <c r="I1061" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1061" s="103" t="n"/>
+      <c r="K1061" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1061" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1061" s="105" t="n">
+        <v>64695</v>
+      </c>
+      <c r="N1061" s="105" t="n">
+        <v>20026984.2</v>
+      </c>
+      <c r="O1061" s="103" t="n"/>
+      <c r="P1061" s="103" t="n"/>
+      <c r="Q1061" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B1062" s="103" t="inlineStr">
+        <is>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1062" s="103" t="n"/>
+      <c r="D1062" s="103" t="n"/>
+      <c r="E1062" s="103" t="n"/>
+      <c r="F1062" s="103" t="n"/>
+      <c r="G1062" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1062" s="103" t="inlineStr">
+        <is>
+          <t>Reprocessing</t>
+        </is>
+      </c>
+      <c r="I1062" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1062" s="103" t="n"/>
+      <c r="K1062" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1062" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1062" s="105" t="n">
+        <v>40273</v>
+      </c>
+      <c r="N1062" s="105" t="n">
+        <v>12027934.18</v>
+      </c>
+      <c r="O1062" s="103" t="n"/>
+      <c r="P1062" s="103" t="n"/>
+      <c r="Q1062" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B1063" s="103" t="inlineStr">
+        <is>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1063" s="103" t="n"/>
+      <c r="D1063" s="103" t="n"/>
+      <c r="E1063" s="103" t="n"/>
+      <c r="F1063" s="103" t="n"/>
+      <c r="G1063" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1063" s="103" t="inlineStr">
+        <is>
+          <t>Reprocessing</t>
+        </is>
+      </c>
+      <c r="I1063" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1063" s="103" t="n"/>
+      <c r="K1063" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1063" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1063" s="105" t="n">
         <v>19235</v>
       </c>
-      <c r="N1054" s="105" t="n">
+      <c r="N1063" s="105" t="n">
         <v>5535063.600000001</v>
       </c>
-      <c r="O1054" s="103" t="n"/>
-      <c r="P1054" s="103" t="n"/>
-      <c r="Q1054" s="103" t="inlineStr">
+      <c r="O1063" s="103" t="n"/>
+      <c r="P1063" s="103" t="n"/>
+      <c r="Q1063" s="103" t="inlineStr">
         <is>
           <t>0-30</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q1054"/>
+  <autoFilter ref="A1:Q1063"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto-deploy AR dashboard 2026-08-24 19:24
</commit_message>
<xml_diff>
--- a/AR Movement Report.xlsx
+++ b/AR Movement Report.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$133</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1067</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1062</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1346,7 +1346,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data as of Monday, 24 August 2026 - 09:17  |  Source: PSI AR Monitoring Master.xlsx</t>
+          <t>Data as of Monday, 24 August 2026 - 19:24  |  Source: PSI AR Monitoring Master.xlsx</t>
         </is>
       </c>
     </row>
@@ -1383,18 +1383,18 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="9" t="n">
-        <v>75853386332.42767</v>
+        <v>75712169774.80766</v>
       </c>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="10" t="n"/>
       <c r="D7" s="11" t="n"/>
       <c r="E7" s="12" t="n">
-        <v>65403957391.04408</v>
+        <v>65278834217.86408</v>
       </c>
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="11" t="n"/>
       <c r="H7" s="13" t="n">
-        <v>10449428941.38358</v>
+        <v>10433335556.94358</v>
       </c>
       <c r="I7" s="10" t="n"/>
       <c r="J7" s="11" t="n"/>
@@ -1440,14 +1440,14 @@
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="19" t="n">
-        <v>40131798719.05087</v>
+        <v>40115705334.61087</v>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="10" t="n"/>
       <c r="D12" s="10" t="n"/>
       <c r="E12" s="11" t="n"/>
       <c r="F12" s="20" t="n">
-        <v>35721587613.37681</v>
+        <v>35596464440.19682</v>
       </c>
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="10" t="n"/>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="26" t="n">
-        <v>32583930585.50482</v>
+        <v>32567837201.06482</v>
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="27" t="n">
@@ -1667,7 +1667,7 @@
         <v>7289350202.20622</v>
       </c>
       <c r="C25" s="35" t="n">
-        <v>718476952.7635853</v>
+        <v>593353779.5835853</v>
       </c>
       <c r="D25" s="36" t="n">
         <v>0</v>
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="B30" s="34" t="n">
-        <v>27619066504.78464</v>
+        <v>27602973120.34464</v>
       </c>
       <c r="C30" s="36" t="n">
         <v>0</v>
@@ -2029,7 +2029,7 @@
         <v>30275723557.25086</v>
       </c>
       <c r="C41" s="49" t="n">
-        <v>9856075161.799999</v>
+        <v>9839981777.360001</v>
       </c>
       <c r="D41" s="50">
         <f>SUM(B41:C41)</f>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B42" s="36" t="n">
-        <v>4496600121.238269</v>
+        <v>4371476948.058269</v>
       </c>
       <c r="C42" s="36" t="n">
         <v>593353779.5835853</v>
@@ -2151,7 +2151,7 @@
         <v>209900924.97</v>
       </c>
       <c r="D49" s="57" t="n">
-        <v>718476952.7635853</v>
+        <v>593353779.5835853</v>
       </c>
       <c r="E49" s="36" t="n">
         <v>0</v>
@@ -3016,7 +3016,7 @@
         <v>0</v>
       </c>
       <c r="I75" s="36" t="n">
-        <v>2734726665.64</v>
+        <v>2718633281.2</v>
       </c>
       <c r="J75" s="37">
         <f>SUM(B75:I75)</f>
@@ -3446,7 +3446,7 @@
         </is>
       </c>
       <c r="C13" s="36" t="n">
-        <v>125123173.18</v>
+        <v>0</v>
       </c>
       <c r="D13" s="36" t="n">
         <v>593353779.5835853</v>
@@ -3499,7 +3499,7 @@
         <v>20770896210.50464</v>
       </c>
       <c r="D15" s="36" t="n">
-        <v>6848170294.28</v>
+        <v>6832076909.839999</v>
       </c>
       <c r="E15" s="36" t="n">
         <v>0</v>
@@ -3544,7 +3544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H133"/>
+  <dimension ref="A1:H128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5052,148 +5052,178 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="71" t="n">
-        <v>46258</v>
-      </c>
-      <c r="B48" s="72" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C48" s="72" t="n"/>
-      <c r="D48" s="72" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E48" s="73" t="n">
-        <v>46711943.46</v>
-      </c>
-      <c r="F48" s="71" t="n"/>
-      <c r="G48" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="72" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+      <c r="A48" s="75" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B48" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C48" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/26/2026</t>
+        </is>
+      </c>
+      <c r="D48" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E48" s="77" t="n">
+        <v>1105158867</v>
+      </c>
+      <c r="F48" s="75" t="n">
+        <v>46259</v>
+      </c>
+      <c r="G48" s="78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="71" t="n">
-        <v>46258</v>
-      </c>
-      <c r="B49" s="72" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C49" s="72" t="n"/>
-      <c r="D49" s="72" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E49" s="73" t="n">
-        <v>40821247.74</v>
-      </c>
-      <c r="F49" s="71" t="n"/>
-      <c r="G49" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="72" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+      <c r="A49" s="75" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B49" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C49" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/27/2026</t>
+        </is>
+      </c>
+      <c r="D49" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E49" s="77" t="n">
+        <v>272700000</v>
+      </c>
+      <c r="F49" s="75" t="n">
+        <v>46259</v>
+      </c>
+      <c r="G49" s="78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="71" t="n">
-        <v>46258</v>
-      </c>
-      <c r="B50" s="72" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C50" s="72" t="n"/>
-      <c r="D50" s="72" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E50" s="73" t="n">
-        <v>20026984.2</v>
-      </c>
-      <c r="F50" s="71" t="n"/>
-      <c r="G50" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="72" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+      <c r="A50" s="75" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B50" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C50" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL/28/2026</t>
+        </is>
+      </c>
+      <c r="D50" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E50" s="77" t="n">
+        <v>15492035.49</v>
+      </c>
+      <c r="F50" s="75" t="n">
+        <v>46259</v>
+      </c>
+      <c r="G50" s="78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="71" t="n">
-        <v>46258</v>
-      </c>
-      <c r="B51" s="72" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C51" s="72" t="n"/>
-      <c r="D51" s="72" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E51" s="73" t="n">
-        <v>12027934.18</v>
-      </c>
-      <c r="F51" s="71" t="n"/>
-      <c r="G51" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" s="72" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+      <c r="A51" s="75" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B51" s="76" t="inlineStr">
+        <is>
+          <t>PT Bayer Indonesia</t>
+        </is>
+      </c>
+      <c r="C51" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.BI/FC/42/2026</t>
+        </is>
+      </c>
+      <c r="D51" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E51" s="77" t="n">
+        <v>213514.65</v>
+      </c>
+      <c r="F51" s="75" t="n">
+        <v>46261</v>
+      </c>
+      <c r="G51" s="78" t="n">
+        <v>3</v>
+      </c>
+      <c r="H51" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="71" t="n">
-        <v>46258</v>
-      </c>
-      <c r="B52" s="72" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C52" s="72" t="n"/>
-      <c r="D52" s="72" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E52" s="73" t="n">
-        <v>5535063.600000001</v>
-      </c>
-      <c r="F52" s="71" t="n"/>
-      <c r="G52" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H52" s="72" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+      <c r="A52" s="75" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B52" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C52" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/28/2026</t>
+        </is>
+      </c>
+      <c r="D52" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E52" s="77" t="n">
+        <v>360730.411008</v>
+      </c>
+      <c r="F52" s="75" t="n">
+        <v>46262</v>
+      </c>
+      <c r="G52" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="H52" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="75" t="n">
-        <v>46259</v>
+        <v>46262</v>
       </c>
       <c r="B53" s="76" t="inlineStr">
         <is>
@@ -5202,22 +5232,22 @@
       </c>
       <c r="C53" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/26/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/29/2026</t>
         </is>
       </c>
       <c r="D53" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E53" s="77" t="n">
-        <v>1105158867</v>
+        <v>91486133.35135135</v>
       </c>
       <c r="F53" s="75" t="n">
-        <v>46259</v>
+        <v>46262</v>
       </c>
       <c r="G53" s="78" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H53" s="76" t="inlineStr">
         <is>
@@ -5227,16 +5257,16 @@
     </row>
     <row r="54">
       <c r="A54" s="75" t="n">
-        <v>46259</v>
+        <v>46268</v>
       </c>
       <c r="B54" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C54" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/27/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/11/2026</t>
         </is>
       </c>
       <c r="D54" s="76" t="inlineStr">
@@ -5245,13 +5275,13 @@
         </is>
       </c>
       <c r="E54" s="77" t="n">
-        <v>272700000</v>
+        <v>872911811.2</v>
       </c>
       <c r="F54" s="75" t="n">
-        <v>46259</v>
+        <v>46267</v>
       </c>
       <c r="G54" s="78" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H54" s="76" t="inlineStr">
         <is>
@@ -5261,31 +5291,31 @@
     </row>
     <row r="55">
       <c r="A55" s="75" t="n">
-        <v>46259</v>
+        <v>46268</v>
       </c>
       <c r="B55" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C55" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/28/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/12/2026</t>
         </is>
       </c>
       <c r="D55" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E55" s="77" t="n">
-        <v>15492035.49</v>
+        <v>302161780.8</v>
       </c>
       <c r="F55" s="75" t="n">
-        <v>46259</v>
+        <v>46267</v>
       </c>
       <c r="G55" s="78" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H55" s="76" t="inlineStr">
         <is>
@@ -5295,31 +5325,31 @@
     </row>
     <row r="56">
       <c r="A56" s="75" t="n">
-        <v>46261</v>
+        <v>46270</v>
       </c>
       <c r="B56" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Alam Semesta Agro</t>
         </is>
       </c>
       <c r="C56" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/42/2026</t>
+          <t>PT.PSI/PT.ASA/Rental CS/09/2026</t>
         </is>
       </c>
       <c r="D56" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E56" s="77" t="n">
-        <v>213514.65</v>
+        <v>142652400</v>
       </c>
       <c r="F56" s="75" t="n">
-        <v>46261</v>
+        <v>46270</v>
       </c>
       <c r="G56" s="78" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H56" s="76" t="inlineStr">
         <is>
@@ -5329,31 +5359,31 @@
     </row>
     <row r="57">
       <c r="A57" s="75" t="n">
-        <v>46262</v>
+        <v>46270</v>
       </c>
       <c r="B57" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Alam Semesta Agro</t>
         </is>
       </c>
       <c r="C57" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/28/2026</t>
+          <t>PT.PSI/PT.ASA/Rental CS/10/2026</t>
         </is>
       </c>
       <c r="D57" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E57" s="77" t="n">
-        <v>360730.411008</v>
+        <v>6920631.27</v>
       </c>
       <c r="F57" s="75" t="n">
-        <v>46262</v>
+        <v>46270</v>
       </c>
       <c r="G57" s="78" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H57" s="76" t="inlineStr">
         <is>
@@ -5363,7 +5393,7 @@
     </row>
     <row r="58">
       <c r="A58" s="75" t="n">
-        <v>46262</v>
+        <v>46273</v>
       </c>
       <c r="B58" s="76" t="inlineStr">
         <is>
@@ -5372,22 +5402,22 @@
       </c>
       <c r="C58" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/29/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/29/2026 </t>
         </is>
       </c>
       <c r="D58" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E58" s="77" t="n">
-        <v>91486133.35135135</v>
+        <v>1365520000</v>
       </c>
       <c r="F58" s="75" t="n">
-        <v>46262</v>
+        <v>46273</v>
       </c>
       <c r="G58" s="78" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="H58" s="76" t="inlineStr">
         <is>
@@ -5397,16 +5427,16 @@
     </row>
     <row r="59">
       <c r="A59" s="75" t="n">
-        <v>46268</v>
+        <v>46273</v>
       </c>
       <c r="B59" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C59" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/11/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/30/2026</t>
         </is>
       </c>
       <c r="D59" s="76" t="inlineStr">
@@ -5415,13 +5445,13 @@
         </is>
       </c>
       <c r="E59" s="77" t="n">
-        <v>872911811.2</v>
+        <v>1071584346</v>
       </c>
       <c r="F59" s="75" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="G59" s="78" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H59" s="76" t="inlineStr">
         <is>
@@ -5431,16 +5461,16 @@
     </row>
     <row r="60">
       <c r="A60" s="75" t="n">
-        <v>46268</v>
+        <v>46273</v>
       </c>
       <c r="B60" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C60" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/12/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/31/2026</t>
         </is>
       </c>
       <c r="D60" s="76" t="inlineStr">
@@ -5449,13 +5479,13 @@
         </is>
       </c>
       <c r="E60" s="77" t="n">
-        <v>302161780.8</v>
+        <v>272700000</v>
       </c>
       <c r="F60" s="75" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="G60" s="78" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H60" s="76" t="inlineStr">
         <is>
@@ -5465,16 +5495,16 @@
     </row>
     <row r="61">
       <c r="A61" s="75" t="n">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B61" s="76" t="inlineStr">
         <is>
-          <t>PT Alam Semesta Agro</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C61" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASA/Rental CS/09/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/32/2026 </t>
         </is>
       </c>
       <c r="D61" s="76" t="inlineStr">
@@ -5483,13 +5513,13 @@
         </is>
       </c>
       <c r="E61" s="77" t="n">
-        <v>142652400</v>
+        <v>25780415.64</v>
       </c>
       <c r="F61" s="75" t="n">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="G61" s="78" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H61" s="76" t="inlineStr">
         <is>
@@ -5499,16 +5529,16 @@
     </row>
     <row r="62">
       <c r="A62" s="75" t="n">
-        <v>46270</v>
+        <v>46276</v>
       </c>
       <c r="B62" s="76" t="inlineStr">
         <is>
-          <t>PT Alam Semesta Agro</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C62" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASA/Rental CS/10/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-22/2026</t>
         </is>
       </c>
       <c r="D62" s="76" t="inlineStr">
@@ -5517,13 +5547,13 @@
         </is>
       </c>
       <c r="E62" s="77" t="n">
-        <v>6920631.27</v>
+        <v>707000000</v>
       </c>
       <c r="F62" s="75" t="n">
-        <v>46270</v>
+        <v>46276</v>
       </c>
       <c r="G62" s="78" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H62" s="76" t="inlineStr">
         <is>
@@ -5533,16 +5563,16 @@
     </row>
     <row r="63">
       <c r="A63" s="75" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="B63" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C63" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/29/2026 </t>
+          <t>PT.PSI/PT.ASI/HANDLING-CS-PAS2/23/2026</t>
         </is>
       </c>
       <c r="D63" s="76" t="inlineStr">
@@ -5551,13 +5581,13 @@
         </is>
       </c>
       <c r="E63" s="77" t="n">
-        <v>1365520000</v>
+        <v>9857624.279999999</v>
       </c>
       <c r="F63" s="75" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="G63" s="78" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H63" s="76" t="inlineStr">
         <is>
@@ -5567,16 +5597,16 @@
     </row>
     <row r="64">
       <c r="A64" s="75" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="B64" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C64" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/30/2026</t>
+          <t>PT.PSI/PT.ASI/HANDLING-CS-PAS2/23/2026</t>
         </is>
       </c>
       <c r="D64" s="76" t="inlineStr">
@@ -5585,13 +5615,13 @@
         </is>
       </c>
       <c r="E64" s="77" t="n">
-        <v>1071584346</v>
+        <v>1019695</v>
       </c>
       <c r="F64" s="75" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="G64" s="78" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H64" s="76" t="inlineStr">
         <is>
@@ -5601,16 +5631,16 @@
     </row>
     <row r="65">
       <c r="A65" s="75" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="B65" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C65" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/31/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/24/2026</t>
         </is>
       </c>
       <c r="D65" s="76" t="inlineStr">
@@ -5619,13 +5649,13 @@
         </is>
       </c>
       <c r="E65" s="77" t="n">
-        <v>272700000</v>
+        <v>755480000</v>
       </c>
       <c r="F65" s="75" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="G65" s="78" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H65" s="76" t="inlineStr">
         <is>
@@ -5635,7 +5665,7 @@
     </row>
     <row r="66">
       <c r="A66" s="75" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="B66" s="76" t="inlineStr">
         <is>
@@ -5644,22 +5674,22 @@
       </c>
       <c r="C66" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/32/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/30/2026</t>
         </is>
       </c>
       <c r="D66" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E66" s="77" t="n">
-        <v>25780415.64</v>
+        <v>536105249.4995999</v>
       </c>
       <c r="F66" s="75" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="G66" s="78" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H66" s="76" t="inlineStr">
         <is>
@@ -5673,21 +5703,21 @@
       </c>
       <c r="B67" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C67" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-22/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/31/2026</t>
         </is>
       </c>
       <c r="D67" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E67" s="77" t="n">
-        <v>707000000</v>
+        <v>513650866.212</v>
       </c>
       <c r="F67" s="75" t="n">
         <v>46276</v>
@@ -5703,31 +5733,31 @@
     </row>
     <row r="68">
       <c r="A68" s="75" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="B68" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C68" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/HANDLING-CS-PAS2/23/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL/33/2026</t>
         </is>
       </c>
       <c r="D68" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E68" s="77" t="n">
-        <v>9857624.279999999</v>
+        <v>27842793.22</v>
       </c>
       <c r="F68" s="75" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="G68" s="78" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H68" s="76" t="inlineStr">
         <is>
@@ -5737,31 +5767,31 @@
     </row>
     <row r="69">
       <c r="A69" s="75" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="B69" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C69" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/HANDLING-CS-PAS2/23/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/01/2026</t>
         </is>
       </c>
       <c r="D69" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E69" s="77" t="n">
-        <v>1019695</v>
+        <v>24468320</v>
       </c>
       <c r="F69" s="75" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="G69" s="78" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H69" s="76" t="inlineStr">
         <is>
@@ -5771,31 +5801,31 @@
     </row>
     <row r="70">
       <c r="A70" s="75" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="B70" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C70" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/24/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/02/2026</t>
         </is>
       </c>
       <c r="D70" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E70" s="77" t="n">
-        <v>755480000</v>
+        <v>7298640</v>
       </c>
       <c r="F70" s="75" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="G70" s="78" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H70" s="76" t="inlineStr">
         <is>
@@ -5805,16 +5835,16 @@
     </row>
     <row r="71">
       <c r="A71" s="75" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="B71" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C71" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/30/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/03/2026</t>
         </is>
       </c>
       <c r="D71" s="76" t="inlineStr">
@@ -5823,13 +5853,13 @@
         </is>
       </c>
       <c r="E71" s="77" t="n">
-        <v>536105249.4995999</v>
+        <v>1430080</v>
       </c>
       <c r="F71" s="75" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="G71" s="78" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H71" s="76" t="inlineStr">
         <is>
@@ -5839,16 +5869,16 @@
     </row>
     <row r="72">
       <c r="A72" s="75" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="B72" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C72" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/31/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/04/2026</t>
         </is>
       </c>
       <c r="D72" s="76" t="inlineStr">
@@ -5857,13 +5887,13 @@
         </is>
       </c>
       <c r="E72" s="77" t="n">
-        <v>513650866.212</v>
+        <v>2450320</v>
       </c>
       <c r="F72" s="75" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="G72" s="78" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H72" s="76" t="inlineStr">
         <is>
@@ -5873,16 +5903,16 @@
     </row>
     <row r="73">
       <c r="A73" s="75" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="B73" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C73" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/33/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/05/2026</t>
         </is>
       </c>
       <c r="D73" s="76" t="inlineStr">
@@ -5891,13 +5921,13 @@
         </is>
       </c>
       <c r="E73" s="77" t="n">
-        <v>27842793.22</v>
+        <v>2450320</v>
       </c>
       <c r="F73" s="75" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="G73" s="78" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H73" s="76" t="inlineStr">
         <is>
@@ -5916,7 +5946,7 @@
       </c>
       <c r="C74" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/01/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/06/2026</t>
         </is>
       </c>
       <c r="D74" s="76" t="inlineStr">
@@ -5925,7 +5955,7 @@
         </is>
       </c>
       <c r="E74" s="77" t="n">
-        <v>24468320</v>
+        <v>10961040</v>
       </c>
       <c r="F74" s="75" t="n">
         <v>46279</v>
@@ -5950,7 +5980,7 @@
       </c>
       <c r="C75" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/02/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/07/2026</t>
         </is>
       </c>
       <c r="D75" s="76" t="inlineStr">
@@ -5959,7 +5989,7 @@
         </is>
       </c>
       <c r="E75" s="77" t="n">
-        <v>7298640</v>
+        <v>2249760</v>
       </c>
       <c r="F75" s="75" t="n">
         <v>46279</v>
@@ -5984,7 +6014,7 @@
       </c>
       <c r="C76" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/03/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/08/2026</t>
         </is>
       </c>
       <c r="D76" s="76" t="inlineStr">
@@ -5993,7 +6023,7 @@
         </is>
       </c>
       <c r="E76" s="77" t="n">
-        <v>1430080</v>
+        <v>4019920</v>
       </c>
       <c r="F76" s="75" t="n">
         <v>46279</v>
@@ -6018,7 +6048,7 @@
       </c>
       <c r="C77" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/04/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/09/2026</t>
         </is>
       </c>
       <c r="D77" s="76" t="inlineStr">
@@ -6027,7 +6057,7 @@
         </is>
       </c>
       <c r="E77" s="77" t="n">
-        <v>2450320</v>
+        <v>12609120</v>
       </c>
       <c r="F77" s="75" t="n">
         <v>46279</v>
@@ -6052,7 +6082,7 @@
       </c>
       <c r="C78" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/05/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/10/2026</t>
         </is>
       </c>
       <c r="D78" s="76" t="inlineStr">
@@ -6061,7 +6091,7 @@
         </is>
       </c>
       <c r="E78" s="77" t="n">
-        <v>2450320</v>
+        <v>2180000</v>
       </c>
       <c r="F78" s="75" t="n">
         <v>46279</v>
@@ -6086,7 +6116,7 @@
       </c>
       <c r="C79" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/06/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/11/2026</t>
         </is>
       </c>
       <c r="D79" s="76" t="inlineStr">
@@ -6095,7 +6125,7 @@
         </is>
       </c>
       <c r="E79" s="77" t="n">
-        <v>10961040</v>
+        <v>5266880</v>
       </c>
       <c r="F79" s="75" t="n">
         <v>46279</v>
@@ -6111,16 +6141,16 @@
     </row>
     <row r="80">
       <c r="A80" s="75" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="B80" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C80" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/07/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/49/2026</t>
         </is>
       </c>
       <c r="D80" s="76" t="inlineStr">
@@ -6129,13 +6159,13 @@
         </is>
       </c>
       <c r="E80" s="77" t="n">
-        <v>2249760</v>
+        <v>3981599123.659349</v>
       </c>
       <c r="F80" s="75" t="n">
-        <v>46279</v>
+        <v>46276</v>
       </c>
       <c r="G80" s="78" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H80" s="76" t="inlineStr">
         <is>
@@ -6145,16 +6175,16 @@
     </row>
     <row r="81">
       <c r="A81" s="75" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="B81" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C81" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/08/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/50/2026</t>
         </is>
       </c>
       <c r="D81" s="76" t="inlineStr">
@@ -6163,13 +6193,13 @@
         </is>
       </c>
       <c r="E81" s="77" t="n">
-        <v>4019920</v>
+        <v>1542175442.6694</v>
       </c>
       <c r="F81" s="75" t="n">
-        <v>46279</v>
+        <v>46276</v>
       </c>
       <c r="G81" s="78" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H81" s="76" t="inlineStr">
         <is>
@@ -6179,16 +6209,16 @@
     </row>
     <row r="82">
       <c r="A82" s="75" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="B82" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C82" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/09/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/51/2026</t>
         </is>
       </c>
       <c r="D82" s="76" t="inlineStr">
@@ -6197,13 +6227,13 @@
         </is>
       </c>
       <c r="E82" s="77" t="n">
-        <v>12609120</v>
+        <v>487978078.30875</v>
       </c>
       <c r="F82" s="75" t="n">
-        <v>46279</v>
+        <v>46276</v>
       </c>
       <c r="G82" s="78" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H82" s="76" t="inlineStr">
         <is>
@@ -6213,16 +6243,16 @@
     </row>
     <row r="83">
       <c r="A83" s="75" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="B83" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C83" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/10/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/52/2026</t>
         </is>
       </c>
       <c r="D83" s="76" t="inlineStr">
@@ -6231,13 +6261,13 @@
         </is>
       </c>
       <c r="E83" s="77" t="n">
-        <v>2180000</v>
+        <v>14255050.74672</v>
       </c>
       <c r="F83" s="75" t="n">
-        <v>46279</v>
+        <v>46276</v>
       </c>
       <c r="G83" s="78" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H83" s="76" t="inlineStr">
         <is>
@@ -6247,16 +6277,16 @@
     </row>
     <row r="84">
       <c r="A84" s="75" t="n">
-        <v>46279</v>
+        <v>46284</v>
       </c>
       <c r="B84" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C84" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/11/2026</t>
+          <t>PT.PSI/PT.ASI/FC_LMB_PGB/02/2026</t>
         </is>
       </c>
       <c r="D84" s="76" t="inlineStr">
@@ -6265,13 +6295,13 @@
         </is>
       </c>
       <c r="E84" s="77" t="n">
-        <v>5266880</v>
+        <v>51019085</v>
       </c>
       <c r="F84" s="75" t="n">
-        <v>46279</v>
+        <v>46284</v>
       </c>
       <c r="G84" s="78" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="H84" s="76" t="inlineStr">
         <is>
@@ -6281,16 +6311,16 @@
     </row>
     <row r="85">
       <c r="A85" s="75" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="B85" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C85" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/49/2026</t>
+          <t>PT.PSI/PT.ASI/FC_PAS2/03/26</t>
         </is>
       </c>
       <c r="D85" s="76" t="inlineStr">
@@ -6299,13 +6329,13 @@
         </is>
       </c>
       <c r="E85" s="77" t="n">
-        <v>3981599123.659349</v>
+        <v>119160408.84</v>
       </c>
       <c r="F85" s="75" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
       <c r="G85" s="78" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H85" s="76" t="inlineStr">
         <is>
@@ -6315,16 +6345,16 @@
     </row>
     <row r="86">
       <c r="A86" s="75" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="B86" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C86" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/50/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/51/2026 </t>
         </is>
       </c>
       <c r="D86" s="76" t="inlineStr">
@@ -6333,13 +6363,13 @@
         </is>
       </c>
       <c r="E86" s="77" t="n">
-        <v>1542175442.6694</v>
+        <v>587478172</v>
       </c>
       <c r="F86" s="75" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
       <c r="G86" s="78" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H86" s="76" t="inlineStr">
         <is>
@@ -6349,16 +6379,16 @@
     </row>
     <row r="87">
       <c r="A87" s="75" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="B87" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C87" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/51/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/52/2026 </t>
         </is>
       </c>
       <c r="D87" s="76" t="inlineStr">
@@ -6367,13 +6397,13 @@
         </is>
       </c>
       <c r="E87" s="77" t="n">
-        <v>487978078.30875</v>
+        <v>68745646</v>
       </c>
       <c r="F87" s="75" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
       <c r="G87" s="78" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H87" s="76" t="inlineStr">
         <is>
@@ -6383,16 +6413,16 @@
     </row>
     <row r="88">
       <c r="A88" s="75" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="B88" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C88" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/52/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/53/2026 </t>
         </is>
       </c>
       <c r="D88" s="76" t="inlineStr">
@@ -6401,13 +6431,13 @@
         </is>
       </c>
       <c r="E88" s="77" t="n">
-        <v>14255050.74672</v>
+        <v>33596074.83</v>
       </c>
       <c r="F88" s="75" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
       <c r="G88" s="78" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H88" s="76" t="inlineStr">
         <is>
@@ -6421,12 +6451,12 @@
       </c>
       <c r="B89" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C89" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/FC_LMB_PGB/02/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
         </is>
       </c>
       <c r="D89" s="76" t="inlineStr">
@@ -6435,7 +6465,7 @@
         </is>
       </c>
       <c r="E89" s="77" t="n">
-        <v>51019085</v>
+        <v>326395903.6008</v>
       </c>
       <c r="F89" s="75" t="n">
         <v>46284</v>
@@ -6455,12 +6485,12 @@
       </c>
       <c r="B90" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C90" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/FC_PAS2/03/26</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
         </is>
       </c>
       <c r="D90" s="76" t="inlineStr">
@@ -6469,7 +6499,7 @@
         </is>
       </c>
       <c r="E90" s="77" t="n">
-        <v>119160408.84</v>
+        <v>240049.20888</v>
       </c>
       <c r="F90" s="75" t="n">
         <v>46284</v>
@@ -6485,16 +6515,16 @@
     </row>
     <row r="91">
       <c r="A91" s="75" t="n">
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="B91" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C91" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/51/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
         </is>
       </c>
       <c r="D91" s="76" t="inlineStr">
@@ -6503,13 +6533,13 @@
         </is>
       </c>
       <c r="E91" s="77" t="n">
-        <v>587478172</v>
+        <v>570800977.7184</v>
       </c>
       <c r="F91" s="75" t="n">
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="G91" s="78" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H91" s="76" t="inlineStr">
         <is>
@@ -6519,16 +6549,16 @@
     </row>
     <row r="92">
       <c r="A92" s="75" t="n">
-        <v>46284</v>
+        <v>46289</v>
       </c>
       <c r="B92" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C92" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/52/2026 </t>
+          <t>PT.PSI/PT.CASI/REP/53/2026</t>
         </is>
       </c>
       <c r="D92" s="76" t="inlineStr">
@@ -6537,13 +6567,13 @@
         </is>
       </c>
       <c r="E92" s="77" t="n">
-        <v>68745646</v>
+        <v>36849832.74</v>
       </c>
       <c r="F92" s="75" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="G92" s="78" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="H92" s="76" t="inlineStr">
         <is>
@@ -6553,16 +6583,16 @@
     </row>
     <row r="93">
       <c r="A93" s="75" t="n">
-        <v>46284</v>
+        <v>46289</v>
       </c>
       <c r="B93" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C93" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/53/2026 </t>
+          <t>PT.PSI/PT.CASI/REP/54/2026</t>
         </is>
       </c>
       <c r="D93" s="76" t="inlineStr">
@@ -6571,13 +6601,13 @@
         </is>
       </c>
       <c r="E93" s="77" t="n">
-        <v>33596074.83</v>
+        <v>31988016.36</v>
       </c>
       <c r="F93" s="75" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="G93" s="78" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="H93" s="76" t="inlineStr">
         <is>
@@ -6587,16 +6617,16 @@
     </row>
     <row r="94">
       <c r="A94" s="75" t="n">
-        <v>46284</v>
+        <v>46289</v>
       </c>
       <c r="B94" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C94" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
+          <t>PT.PSI/PT.CASI/REP/55/2026</t>
         </is>
       </c>
       <c r="D94" s="76" t="inlineStr">
@@ -6605,13 +6635,13 @@
         </is>
       </c>
       <c r="E94" s="77" t="n">
-        <v>326395903.6008</v>
+        <v>19431065.722</v>
       </c>
       <c r="F94" s="75" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="G94" s="78" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="H94" s="76" t="inlineStr">
         <is>
@@ -6621,16 +6651,16 @@
     </row>
     <row r="95">
       <c r="A95" s="75" t="n">
-        <v>46284</v>
+        <v>46292</v>
       </c>
       <c r="B95" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C95" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
+          <t>PT.PSI/PT.BI/FC/43/2026</t>
         </is>
       </c>
       <c r="D95" s="76" t="inlineStr">
@@ -6639,13 +6669,13 @@
         </is>
       </c>
       <c r="E95" s="77" t="n">
-        <v>240049.20888</v>
+        <v>103679056</v>
       </c>
       <c r="F95" s="75" t="n">
-        <v>46284</v>
+        <v>46292</v>
       </c>
       <c r="G95" s="78" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="H95" s="76" t="inlineStr">
         <is>
@@ -6655,16 +6685,16 @@
     </row>
     <row r="96">
       <c r="A96" s="75" t="n">
-        <v>46286</v>
+        <v>46292</v>
       </c>
       <c r="B96" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C96" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
+          <t>PT.PSI/PT.BI/FC/44/2026</t>
         </is>
       </c>
       <c r="D96" s="76" t="inlineStr">
@@ -6673,13 +6703,13 @@
         </is>
       </c>
       <c r="E96" s="77" t="n">
-        <v>570800977.7184</v>
+        <v>92863095</v>
       </c>
       <c r="F96" s="75" t="n">
-        <v>46286</v>
+        <v>46292</v>
       </c>
       <c r="G96" s="78" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H96" s="76" t="inlineStr">
         <is>
@@ -6689,16 +6719,16 @@
     </row>
     <row r="97">
       <c r="A97" s="75" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="B97" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C97" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/53/2026</t>
+          <t>PT.PSI/PT.BI/FC/45/2026</t>
         </is>
       </c>
       <c r="D97" s="76" t="inlineStr">
@@ -6707,13 +6737,13 @@
         </is>
       </c>
       <c r="E97" s="77" t="n">
-        <v>36849832.74</v>
+        <v>17392258</v>
       </c>
       <c r="F97" s="75" t="n">
-        <v>46285</v>
+        <v>46292</v>
       </c>
       <c r="G97" s="78" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H97" s="76" t="inlineStr">
         <is>
@@ -6723,16 +6753,16 @@
     </row>
     <row r="98">
       <c r="A98" s="75" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="B98" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C98" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/54/2026</t>
+          <t>PT.PSI/PT.BI/FC/46/2026</t>
         </is>
       </c>
       <c r="D98" s="76" t="inlineStr">
@@ -6741,13 +6771,13 @@
         </is>
       </c>
       <c r="E98" s="77" t="n">
-        <v>31988016.36</v>
+        <v>197734556.5</v>
       </c>
       <c r="F98" s="75" t="n">
-        <v>46285</v>
+        <v>46292</v>
       </c>
       <c r="G98" s="78" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H98" s="76" t="inlineStr">
         <is>
@@ -6757,16 +6787,16 @@
     </row>
     <row r="99">
       <c r="A99" s="75" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="B99" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C99" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/55/2026</t>
+          <t>PT.PSI/PT.BI/FC/47/2026</t>
         </is>
       </c>
       <c r="D99" s="76" t="inlineStr">
@@ -6775,13 +6805,13 @@
         </is>
       </c>
       <c r="E99" s="77" t="n">
-        <v>19431065.722</v>
+        <v>254755628.4</v>
       </c>
       <c r="F99" s="75" t="n">
-        <v>46285</v>
+        <v>46292</v>
       </c>
       <c r="G99" s="78" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H99" s="76" t="inlineStr">
         <is>
@@ -6800,7 +6830,7 @@
       </c>
       <c r="C100" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/43/2026</t>
+          <t>PT.PSI/PT.BI/FC/48/2026</t>
         </is>
       </c>
       <c r="D100" s="76" t="inlineStr">
@@ -6809,7 +6839,7 @@
         </is>
       </c>
       <c r="E100" s="77" t="n">
-        <v>103679056</v>
+        <v>10599160</v>
       </c>
       <c r="F100" s="75" t="n">
         <v>46292</v>
@@ -6834,7 +6864,7 @@
       </c>
       <c r="C101" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/44/2026</t>
+          <t>PT.PSI/PT.BI/FC/49/2026</t>
         </is>
       </c>
       <c r="D101" s="76" t="inlineStr">
@@ -6843,7 +6873,7 @@
         </is>
       </c>
       <c r="E101" s="77" t="n">
-        <v>92863095</v>
+        <v>54405006.5</v>
       </c>
       <c r="F101" s="75" t="n">
         <v>46292</v>
@@ -6868,7 +6898,7 @@
       </c>
       <c r="C102" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/45/2026</t>
+          <t>PT.PSI/PT.BI/FC/50/2026</t>
         </is>
       </c>
       <c r="D102" s="76" t="inlineStr">
@@ -6877,7 +6907,7 @@
         </is>
       </c>
       <c r="E102" s="77" t="n">
-        <v>17392258</v>
+        <v>1075481.2</v>
       </c>
       <c r="F102" s="75" t="n">
         <v>46292</v>
@@ -6902,7 +6932,7 @@
       </c>
       <c r="C103" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/46/2026</t>
+          <t>PT.PSI/PT.BI/FC/51/2026</t>
         </is>
       </c>
       <c r="D103" s="76" t="inlineStr">
@@ -6911,7 +6941,7 @@
         </is>
       </c>
       <c r="E103" s="77" t="n">
-        <v>197734556.5</v>
+        <v>803447.72</v>
       </c>
       <c r="F103" s="75" t="n">
         <v>46292</v>
@@ -6936,7 +6966,7 @@
       </c>
       <c r="C104" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/47/2026</t>
+          <t>PT.PSI/PT.BI/FC/52/2026</t>
         </is>
       </c>
       <c r="D104" s="76" t="inlineStr">
@@ -6945,7 +6975,7 @@
         </is>
       </c>
       <c r="E104" s="77" t="n">
-        <v>254755628.4</v>
+        <v>7250789</v>
       </c>
       <c r="F104" s="75" t="n">
         <v>46292</v>
@@ -6970,7 +7000,7 @@
       </c>
       <c r="C105" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/48/2026</t>
+          <t>PT.PSI/PT.BI/FC/53/2026</t>
         </is>
       </c>
       <c r="D105" s="76" t="inlineStr">
@@ -6979,7 +7009,7 @@
         </is>
       </c>
       <c r="E105" s="77" t="n">
-        <v>10599160</v>
+        <v>101318334</v>
       </c>
       <c r="F105" s="75" t="n">
         <v>46292</v>
@@ -6995,7 +7025,7 @@
     </row>
     <row r="106">
       <c r="A106" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B106" s="76" t="inlineStr">
         <is>
@@ -7004,7 +7034,7 @@
       </c>
       <c r="C106" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/49/2026</t>
+          <t>PT.PSI/PT.BI/FC/54/2026</t>
         </is>
       </c>
       <c r="D106" s="76" t="inlineStr">
@@ -7013,13 +7043,13 @@
         </is>
       </c>
       <c r="E106" s="77" t="n">
-        <v>54405006.5</v>
+        <v>156400274.1</v>
       </c>
       <c r="F106" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G106" s="78" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H106" s="76" t="inlineStr">
         <is>
@@ -7029,7 +7059,7 @@
     </row>
     <row r="107">
       <c r="A107" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B107" s="76" t="inlineStr">
         <is>
@@ -7038,7 +7068,7 @@
       </c>
       <c r="C107" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/50/2026</t>
+          <t>PT.PSI/PT.BI/FC/55/2026</t>
         </is>
       </c>
       <c r="D107" s="76" t="inlineStr">
@@ -7047,13 +7077,13 @@
         </is>
       </c>
       <c r="E107" s="77" t="n">
-        <v>1075481.2</v>
+        <v>50838199.5</v>
       </c>
       <c r="F107" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G107" s="78" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H107" s="76" t="inlineStr">
         <is>
@@ -7063,7 +7093,7 @@
     </row>
     <row r="108">
       <c r="A108" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B108" s="76" t="inlineStr">
         <is>
@@ -7072,7 +7102,7 @@
       </c>
       <c r="C108" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/51/2026</t>
+          <t>PT.PSI/PT.BI/FC/56/2026</t>
         </is>
       </c>
       <c r="D108" s="76" t="inlineStr">
@@ -7081,13 +7111,13 @@
         </is>
       </c>
       <c r="E108" s="77" t="n">
-        <v>803447.72</v>
+        <v>376884765.6</v>
       </c>
       <c r="F108" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G108" s="78" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H108" s="76" t="inlineStr">
         <is>
@@ -7097,7 +7127,7 @@
     </row>
     <row r="109">
       <c r="A109" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B109" s="76" t="inlineStr">
         <is>
@@ -7106,7 +7136,7 @@
       </c>
       <c r="C109" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/52/2026</t>
+          <t>PT.PSI/PT.BI/FC/57/2026</t>
         </is>
       </c>
       <c r="D109" s="76" t="inlineStr">
@@ -7115,13 +7145,13 @@
         </is>
       </c>
       <c r="E109" s="77" t="n">
-        <v>7250789</v>
+        <v>100336789</v>
       </c>
       <c r="F109" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G109" s="78" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H109" s="76" t="inlineStr">
         <is>
@@ -7131,7 +7161,7 @@
     </row>
     <row r="110">
       <c r="A110" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B110" s="76" t="inlineStr">
         <is>
@@ -7140,7 +7170,7 @@
       </c>
       <c r="C110" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/53/2026</t>
+          <t>PT.PSI/PT.BI/FC/58/2026</t>
         </is>
       </c>
       <c r="D110" s="76" t="inlineStr">
@@ -7149,13 +7179,13 @@
         </is>
       </c>
       <c r="E110" s="77" t="n">
-        <v>101318334</v>
+        <v>787756603.1999999</v>
       </c>
       <c r="F110" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G110" s="78" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H110" s="76" t="inlineStr">
         <is>
@@ -7174,7 +7204,7 @@
       </c>
       <c r="C111" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/54/2026</t>
+          <t>PT.PSI/PT.BI/FC/59/2026</t>
         </is>
       </c>
       <c r="D111" s="76" t="inlineStr">
@@ -7183,7 +7213,7 @@
         </is>
       </c>
       <c r="E111" s="77" t="n">
-        <v>156400274.1</v>
+        <v>140859991.5</v>
       </c>
       <c r="F111" s="75" t="n">
         <v>46293</v>
@@ -7199,16 +7229,16 @@
     </row>
     <row r="112">
       <c r="A112" s="75" t="n">
-        <v>46293</v>
+        <v>46300</v>
       </c>
       <c r="B112" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C112" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/55/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
         </is>
       </c>
       <c r="D112" s="76" t="inlineStr">
@@ -7217,13 +7247,13 @@
         </is>
       </c>
       <c r="E112" s="77" t="n">
-        <v>50838199.5</v>
+        <v>18871809.6</v>
       </c>
       <c r="F112" s="75" t="n">
-        <v>46293</v>
+        <v>46300</v>
       </c>
       <c r="G112" s="78" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="H112" s="76" t="inlineStr">
         <is>
@@ -7233,16 +7263,16 @@
     </row>
     <row r="113">
       <c r="A113" s="75" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="B113" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C113" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/56/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
         </is>
       </c>
       <c r="D113" s="76" t="inlineStr">
@@ -7251,13 +7281,13 @@
         </is>
       </c>
       <c r="E113" s="77" t="n">
-        <v>376884765.6</v>
+        <v>226017285.066</v>
       </c>
       <c r="F113" s="75" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="G113" s="78" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H113" s="76" t="inlineStr">
         <is>
@@ -7267,16 +7297,16 @@
     </row>
     <row r="114">
       <c r="A114" s="75" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="B114" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C114" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/57/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
         </is>
       </c>
       <c r="D114" s="76" t="inlineStr">
@@ -7285,13 +7315,13 @@
         </is>
       </c>
       <c r="E114" s="77" t="n">
-        <v>100336789</v>
+        <v>3356193038.598001</v>
       </c>
       <c r="F114" s="75" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="G114" s="78" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H114" s="76" t="inlineStr">
         <is>
@@ -7301,16 +7331,16 @@
     </row>
     <row r="115">
       <c r="A115" s="75" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="B115" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C115" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/58/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
         </is>
       </c>
       <c r="D115" s="76" t="inlineStr">
@@ -7319,13 +7349,13 @@
         </is>
       </c>
       <c r="E115" s="77" t="n">
-        <v>787756603.1999999</v>
+        <v>999055757.8296</v>
       </c>
       <c r="F115" s="75" t="n">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="G115" s="78" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H115" s="76" t="inlineStr">
         <is>
@@ -7335,16 +7365,16 @@
     </row>
     <row r="116">
       <c r="A116" s="75" t="n">
-        <v>46293</v>
+        <v>46305</v>
       </c>
       <c r="B116" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C116" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/59/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
         </is>
       </c>
       <c r="D116" s="76" t="inlineStr">
@@ -7353,13 +7383,13 @@
         </is>
       </c>
       <c r="E116" s="77" t="n">
-        <v>140859991.5</v>
+        <v>886307502.1920002</v>
       </c>
       <c r="F116" s="75" t="n">
-        <v>46293</v>
+        <v>46305</v>
       </c>
       <c r="G116" s="78" t="n">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="H116" s="76" t="inlineStr">
         <is>
@@ -7369,7 +7399,7 @@
     </row>
     <row r="117">
       <c r="A117" s="75" t="n">
-        <v>46300</v>
+        <v>46308</v>
       </c>
       <c r="B117" s="76" t="inlineStr">
         <is>
@@ -7378,7 +7408,7 @@
       </c>
       <c r="C117" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
         </is>
       </c>
       <c r="D117" s="76" t="inlineStr">
@@ -7387,13 +7417,13 @@
         </is>
       </c>
       <c r="E117" s="77" t="n">
-        <v>18871809.6</v>
+        <v>5676698527.872001</v>
       </c>
       <c r="F117" s="75" t="n">
-        <v>46300</v>
+        <v>46308</v>
       </c>
       <c r="G117" s="78" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="H117" s="76" t="inlineStr">
         <is>
@@ -7403,7 +7433,7 @@
     </row>
     <row r="118">
       <c r="A118" s="75" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="B118" s="76" t="inlineStr">
         <is>
@@ -7412,7 +7442,7 @@
       </c>
       <c r="C118" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
         </is>
       </c>
       <c r="D118" s="76" t="inlineStr">
@@ -7421,13 +7451,13 @@
         </is>
       </c>
       <c r="E118" s="77" t="n">
-        <v>226017285.066</v>
+        <v>564189103.6416</v>
       </c>
       <c r="F118" s="75" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="G118" s="78" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="H118" s="76" t="inlineStr">
         <is>
@@ -7437,7 +7467,7 @@
     </row>
     <row r="119">
       <c r="A119" s="75" t="n">
-        <v>46301</v>
+        <v>46312</v>
       </c>
       <c r="B119" s="76" t="inlineStr">
         <is>
@@ -7446,22 +7476,22 @@
       </c>
       <c r="C119" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
         </is>
       </c>
       <c r="D119" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E119" s="77" t="n">
-        <v>3356193038.598001</v>
+        <v>1365520000</v>
       </c>
       <c r="F119" s="75" t="n">
-        <v>46301</v>
+        <v>46312</v>
       </c>
       <c r="G119" s="78" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="H119" s="76" t="inlineStr">
         <is>
@@ -7471,7 +7501,7 @@
     </row>
     <row r="120">
       <c r="A120" s="75" t="n">
-        <v>46301</v>
+        <v>46312</v>
       </c>
       <c r="B120" s="76" t="inlineStr">
         <is>
@@ -7480,22 +7510,22 @@
       </c>
       <c r="C120" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
         </is>
       </c>
       <c r="D120" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E120" s="77" t="n">
-        <v>999055757.8296</v>
+        <v>9687031.199999999</v>
       </c>
       <c r="F120" s="75" t="n">
-        <v>46301</v>
+        <v>46312</v>
       </c>
       <c r="G120" s="78" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="H120" s="76" t="inlineStr">
         <is>
@@ -7505,7 +7535,7 @@
     </row>
     <row r="121">
       <c r="A121" s="75" t="n">
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="B121" s="76" t="inlineStr">
         <is>
@@ -7514,22 +7544,22 @@
       </c>
       <c r="C121" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
         </is>
       </c>
       <c r="D121" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E121" s="77" t="n">
-        <v>886307502.1920002</v>
+        <v>1070726250</v>
       </c>
       <c r="F121" s="75" t="n">
-        <v>46305</v>
+        <v>46312</v>
       </c>
       <c r="G121" s="78" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="H121" s="76" t="inlineStr">
         <is>
@@ -7539,7 +7569,7 @@
     </row>
     <row r="122">
       <c r="A122" s="75" t="n">
-        <v>46308</v>
+        <v>46312</v>
       </c>
       <c r="B122" s="76" t="inlineStr">
         <is>
@@ -7548,22 +7578,22 @@
       </c>
       <c r="C122" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
         </is>
       </c>
       <c r="D122" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E122" s="77" t="n">
-        <v>5676698527.872001</v>
+        <v>272700000</v>
       </c>
       <c r="F122" s="75" t="n">
-        <v>46308</v>
+        <v>46312</v>
       </c>
       <c r="G122" s="78" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H122" s="76" t="inlineStr">
         <is>
@@ -7573,7 +7603,7 @@
     </row>
     <row r="123">
       <c r="A123" s="75" t="n">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="B123" s="76" t="inlineStr">
         <is>
@@ -7582,7 +7612,7 @@
       </c>
       <c r="C123" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
         </is>
       </c>
       <c r="D123" s="76" t="inlineStr">
@@ -7591,13 +7621,13 @@
         </is>
       </c>
       <c r="E123" s="77" t="n">
-        <v>564189103.6416</v>
+        <v>545818781.4912</v>
       </c>
       <c r="F123" s="75" t="n">
-        <v>46308</v>
+        <v>46314</v>
       </c>
       <c r="G123" s="78" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="H123" s="76" t="inlineStr">
         <is>
@@ -7607,7 +7637,7 @@
     </row>
     <row r="124">
       <c r="A124" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B124" s="76" t="inlineStr">
         <is>
@@ -7616,22 +7646,22 @@
       </c>
       <c r="C124" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
         </is>
       </c>
       <c r="D124" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E124" s="77" t="n">
-        <v>1365520000</v>
+        <v>767367847.5204</v>
       </c>
       <c r="F124" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="G124" s="78" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H124" s="76" t="inlineStr">
         <is>
@@ -7641,7 +7671,7 @@
     </row>
     <row r="125">
       <c r="A125" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B125" s="76" t="inlineStr">
         <is>
@@ -7650,22 +7680,22 @@
       </c>
       <c r="C125" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
         </is>
       </c>
       <c r="D125" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E125" s="77" t="n">
-        <v>25780415.64</v>
+        <v>4761468367.9458</v>
       </c>
       <c r="F125" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="G125" s="78" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H125" s="76" t="inlineStr">
         <is>
@@ -7675,7 +7705,7 @@
     </row>
     <row r="126">
       <c r="A126" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B126" s="76" t="inlineStr">
         <is>
@@ -7684,22 +7714,22 @@
       </c>
       <c r="C126" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
         </is>
       </c>
       <c r="D126" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E126" s="77" t="n">
-        <v>1070726250</v>
+        <v>442076465.292</v>
       </c>
       <c r="F126" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="G126" s="78" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H126" s="76" t="inlineStr">
         <is>
@@ -7709,7 +7739,7 @@
     </row>
     <row r="127">
       <c r="A127" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B127" s="76" t="inlineStr">
         <is>
@@ -7718,22 +7748,22 @@
       </c>
       <c r="C127" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
         </is>
       </c>
       <c r="D127" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E127" s="77" t="n">
-        <v>272700000</v>
+        <v>444456984.744</v>
       </c>
       <c r="F127" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="G127" s="78" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H127" s="76" t="inlineStr">
         <is>
@@ -7742,194 +7772,24 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="75" t="n">
-        <v>46314</v>
-      </c>
-      <c r="B128" s="76" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="C128" s="76" t="inlineStr">
-        <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
-        </is>
-      </c>
-      <c r="D128" s="76" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E128" s="77" t="n">
-        <v>545818781.4912</v>
-      </c>
-      <c r="F128" s="75" t="n">
-        <v>46314</v>
-      </c>
-      <c r="G128" s="78" t="n">
-        <v>56</v>
-      </c>
-      <c r="H128" s="76" t="inlineStr">
-        <is>
-          <t>Future</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="75" t="n">
-        <v>46314</v>
-      </c>
-      <c r="B129" s="76" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="C129" s="76" t="inlineStr">
-        <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
-        </is>
-      </c>
-      <c r="D129" s="76" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E129" s="77" t="n">
-        <v>767367847.5204</v>
-      </c>
-      <c r="F129" s="75" t="n">
-        <v>46314</v>
-      </c>
-      <c r="G129" s="78" t="n">
-        <v>56</v>
-      </c>
-      <c r="H129" s="76" t="inlineStr">
-        <is>
-          <t>Future</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="75" t="n">
-        <v>46314</v>
-      </c>
-      <c r="B130" s="76" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="C130" s="76" t="inlineStr">
-        <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
-        </is>
-      </c>
-      <c r="D130" s="76" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E130" s="77" t="n">
-        <v>4761468367.9458</v>
-      </c>
-      <c r="F130" s="75" t="n">
-        <v>46314</v>
-      </c>
-      <c r="G130" s="78" t="n">
-        <v>56</v>
-      </c>
-      <c r="H130" s="76" t="inlineStr">
-        <is>
-          <t>Future</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="75" t="n">
-        <v>46314</v>
-      </c>
-      <c r="B131" s="76" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="C131" s="76" t="inlineStr">
-        <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
-        </is>
-      </c>
-      <c r="D131" s="76" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E131" s="77" t="n">
-        <v>442076465.292</v>
-      </c>
-      <c r="F131" s="75" t="n">
-        <v>46314</v>
-      </c>
-      <c r="G131" s="78" t="n">
-        <v>56</v>
-      </c>
-      <c r="H131" s="76" t="inlineStr">
-        <is>
-          <t>Future</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="75" t="n">
-        <v>46314</v>
-      </c>
-      <c r="B132" s="76" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="C132" s="76" t="inlineStr">
-        <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
-        </is>
-      </c>
-      <c r="D132" s="76" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E132" s="77" t="n">
-        <v>444456984.744</v>
-      </c>
-      <c r="F132" s="75" t="n">
-        <v>46314</v>
-      </c>
-      <c r="G132" s="78" t="n">
-        <v>56</v>
-      </c>
-      <c r="H132" s="76" t="inlineStr">
-        <is>
-          <t>Future</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="39" t="inlineStr">
+      <c r="A128" s="39" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B133" s="79" t="n"/>
-      <c r="C133" s="79" t="n"/>
-      <c r="D133" s="79" t="n"/>
-      <c r="E133" s="80">
-        <f>SUM(E5:E132)</f>
+      <c r="B128" s="79" t="n"/>
+      <c r="C128" s="79" t="n"/>
+      <c r="D128" s="79" t="n"/>
+      <c r="E128" s="80">
+        <f>SUM(E5:E127)</f>
         <v/>
       </c>
-      <c r="F133" s="79" t="n"/>
-      <c r="G133" s="79" t="n"/>
-      <c r="H133" s="79" t="n"/>
+      <c r="F128" s="79" t="n"/>
+      <c r="G128" s="79" t="n"/>
+      <c r="H128" s="79" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H133"/>
+  <autoFilter ref="A4:H128"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9266,28 +9126,28 @@
         <v>325598968.5</v>
       </c>
       <c r="BN10" s="86" t="n">
-        <v>179512192.65</v>
+        <v>180315640.37</v>
       </c>
       <c r="BO10" s="36" t="n">
-        <v>146086775.85</v>
+        <v>145283328.13</v>
       </c>
       <c r="BP10" s="85" t="n">
         <v>180591379.85</v>
       </c>
       <c r="BQ10" s="86" t="n">
-        <v>841876812.3200001</v>
+        <v>530837248.5</v>
       </c>
       <c r="BR10" s="36" t="n">
-        <v>-661285432.47</v>
+        <v>-350245868.65</v>
       </c>
       <c r="BS10" s="85" t="n">
         <v>2454953435.22</v>
       </c>
       <c r="BT10" s="86" t="n">
-        <v>1613076622.9</v>
+        <v>1923312739</v>
       </c>
       <c r="BU10" s="36" t="n">
-        <v>841876812.3199999</v>
+        <v>531640696.2199998</v>
       </c>
       <c r="BV10" s="40" t="n">
         <v>34322220584.8</v>
@@ -11532,28 +11392,28 @@
         <v>135165</v>
       </c>
       <c r="BN21" s="90" t="n">
-        <v>74790</v>
+        <v>75298</v>
       </c>
       <c r="BO21" s="91" t="n">
-        <v>60375</v>
+        <v>59867</v>
       </c>
       <c r="BP21" s="89" t="n">
         <v>75238</v>
       </c>
       <c r="BQ21" s="90" t="n">
-        <v>349894</v>
+        <v>220365</v>
       </c>
       <c r="BR21" s="91" t="n">
-        <v>-274656</v>
+        <v>-145127</v>
       </c>
       <c r="BS21" s="89" t="n">
         <v>570703</v>
       </c>
       <c r="BT21" s="90" t="n">
-        <v>220809</v>
+        <v>349830</v>
       </c>
       <c r="BU21" s="91" t="n">
-        <v>349894</v>
+        <v>220873</v>
       </c>
       <c r="BV21" s="92" t="n">
         <v>6961456</v>
@@ -14039,25 +13899,25 @@
         <v>2735584761.64</v>
       </c>
       <c r="BQ33" s="86" t="n">
-        <v>2734726665.64</v>
+        <v>2718633281.2</v>
       </c>
       <c r="BR33" s="36" t="n">
-        <v>858095.9999995232</v>
+        <v>16951480.44000006</v>
       </c>
       <c r="BS33" s="85" t="n">
-        <v>2734726665.64</v>
+        <v>2718633281.2</v>
       </c>
       <c r="BT33" s="86" t="n">
         <v>0</v>
       </c>
       <c r="BU33" s="36" t="n">
-        <v>2734726665.64</v>
+        <v>2718633281.2</v>
       </c>
       <c r="BV33" s="40" t="n">
-        <v>57561859786.83</v>
+        <v>57545766402.39</v>
       </c>
       <c r="BW33" s="40" t="n">
-        <v>57561859786.83</v>
+        <v>57545766402.39</v>
       </c>
       <c r="BX33" s="40" t="n">
         <v>0</v>
@@ -15841,25 +15701,25 @@
         <v>12385574</v>
       </c>
       <c r="BQ42" s="90" t="n">
-        <v>12382742</v>
+        <v>12003360</v>
       </c>
       <c r="BR42" s="91" t="n">
-        <v>2832</v>
+        <v>382214</v>
       </c>
       <c r="BS42" s="89" t="n">
-        <v>12382742</v>
+        <v>12003360</v>
       </c>
       <c r="BT42" s="90" t="n">
         <v>0</v>
       </c>
       <c r="BU42" s="91" t="n">
-        <v>12382742</v>
+        <v>12003360</v>
       </c>
       <c r="BV42" s="92" t="n">
-        <v>255507147.5</v>
+        <v>255127765.5</v>
       </c>
       <c r="BW42" s="92" t="n">
-        <v>255507147.5</v>
+        <v>255127765.5</v>
       </c>
       <c r="BX42" s="92" t="n">
         <v>0</v>
@@ -16576,16 +16436,16 @@
         </is>
       </c>
       <c r="B15" s="36" t="n">
-        <v>8687984237.840969</v>
+        <v>8688787685.560968</v>
       </c>
       <c r="C15" s="36" t="n">
         <v>9767838169.155153</v>
       </c>
       <c r="D15" s="100" t="n">
-        <v>-1079853931.314184</v>
+        <v>-1079050483.594185</v>
       </c>
       <c r="E15" s="98" t="n">
-        <v>1.124292805068732</v>
+        <v>1.124188842292389</v>
       </c>
       <c r="F15" s="99" t="inlineStr">
         <is>
@@ -16600,16 +16460,16 @@
         </is>
       </c>
       <c r="B16" s="36" t="n">
-        <v>19587357602.83878</v>
+        <v>19260224654.57878</v>
       </c>
       <c r="C16" s="36" t="n">
         <v>11917212675.50339</v>
       </c>
       <c r="D16" s="97" t="n">
-        <v>7670144927.335392</v>
+        <v>7343011979.07539</v>
       </c>
       <c r="E16" s="98" t="n">
-        <v>0.6084134939046724</v>
+        <v>0.6187473349471176</v>
       </c>
       <c r="F16" s="99" t="inlineStr">
         <is>
@@ -16624,16 +16484,16 @@
         </is>
       </c>
       <c r="B17" s="36" t="n">
-        <v>14927675009.2006</v>
+        <v>15237911125.3006</v>
       </c>
       <c r="C17" s="36" t="n">
-        <v>32583930585.50482</v>
+        <v>32567837201.06482</v>
       </c>
       <c r="D17" s="100" t="n">
-        <v>-17656255576.30421</v>
+        <v>-17329926075.76422</v>
       </c>
       <c r="E17" s="98" t="n">
-        <v>2.182786707603285</v>
+        <v>2.137290139918856</v>
       </c>
       <c r="F17" s="99" t="inlineStr">
         <is>
@@ -16720,7 +16580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1067"/>
+  <dimension ref="A1:Q1062"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -81400,10 +81260,10 @@
       </c>
       <c r="J1023" s="103" t="n"/>
       <c r="K1023" s="104" t="n">
-        <v>46204</v>
+        <v>46217</v>
       </c>
       <c r="L1023" s="104" t="n">
-        <v>46234</v>
+        <v>46219</v>
       </c>
       <c r="M1023" s="105" t="n">
         <v>43040</v>
@@ -81465,10 +81325,10 @@
       </c>
       <c r="J1024" s="103" t="n"/>
       <c r="K1024" s="104" t="n">
-        <v>46204</v>
+        <v>46220</v>
       </c>
       <c r="L1024" s="104" t="n">
-        <v>46234</v>
+        <v>46223</v>
       </c>
       <c r="M1024" s="105" t="n">
         <v>38550</v>
@@ -81530,10 +81390,10 @@
       </c>
       <c r="J1025" s="103" t="n"/>
       <c r="K1025" s="104" t="n">
-        <v>46204</v>
+        <v>46230</v>
       </c>
       <c r="L1025" s="104" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="M1025" s="105" t="n">
         <v>7220</v>
@@ -81595,10 +81455,10 @@
       </c>
       <c r="J1026" s="103" t="n"/>
       <c r="K1026" s="104" t="n">
-        <v>46204</v>
+        <v>46225</v>
       </c>
       <c r="L1026" s="104" t="n">
-        <v>46234</v>
+        <v>46229</v>
       </c>
       <c r="M1026" s="105" t="n">
         <v>82085</v>
@@ -81660,10 +81520,10 @@
       </c>
       <c r="J1027" s="103" t="n"/>
       <c r="K1027" s="104" t="n">
-        <v>46204</v>
+        <v>46234</v>
       </c>
       <c r="L1027" s="104" t="n">
-        <v>46234</v>
+        <v>46238</v>
       </c>
       <c r="M1027" s="105" t="n">
         <v>105756</v>
@@ -81725,10 +81585,10 @@
       </c>
       <c r="J1028" s="103" t="n"/>
       <c r="K1028" s="104" t="n">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="L1028" s="104" t="n">
-        <v>46234</v>
+        <v>46206</v>
       </c>
       <c r="M1028" s="105" t="n">
         <v>4400</v>
@@ -81790,10 +81650,10 @@
       </c>
       <c r="J1029" s="103" t="n"/>
       <c r="K1029" s="104" t="n">
-        <v>46204</v>
+        <v>46238</v>
       </c>
       <c r="L1029" s="104" t="n">
-        <v>46234</v>
+        <v>46239</v>
       </c>
       <c r="M1029" s="105" t="n">
         <v>22585</v>
@@ -81855,10 +81715,10 @@
       </c>
       <c r="J1030" s="103" t="n"/>
       <c r="K1030" s="104" t="n">
-        <v>46204</v>
+        <v>46240</v>
       </c>
       <c r="L1030" s="104" t="n">
-        <v>46234</v>
+        <v>46240</v>
       </c>
       <c r="M1030" s="105" t="n">
         <v>680</v>
@@ -81920,10 +81780,10 @@
       </c>
       <c r="J1031" s="103" t="n"/>
       <c r="K1031" s="104" t="n">
-        <v>46204</v>
+        <v>46203</v>
       </c>
       <c r="L1031" s="104" t="n">
-        <v>46234</v>
+        <v>46203</v>
       </c>
       <c r="M1031" s="105" t="n">
         <v>508</v>
@@ -81985,10 +81845,10 @@
       </c>
       <c r="J1032" s="103" t="n"/>
       <c r="K1032" s="104" t="n">
-        <v>46204</v>
+        <v>46230</v>
       </c>
       <c r="L1032" s="104" t="n">
-        <v>46234</v>
+        <v>46230</v>
       </c>
       <c r="M1032" s="105" t="n">
         <v>3010</v>
@@ -82050,10 +81910,10 @@
       </c>
       <c r="J1033" s="103" t="n"/>
       <c r="K1033" s="104" t="n">
-        <v>46204</v>
+        <v>46224</v>
       </c>
       <c r="L1033" s="104" t="n">
-        <v>46234</v>
+        <v>46225</v>
       </c>
       <c r="M1033" s="105" t="n">
         <v>42060</v>
@@ -82714,10 +82574,10 @@
         <v>46234</v>
       </c>
       <c r="M1043" s="105" t="n">
-        <v>607742</v>
+        <v>228360</v>
       </c>
       <c r="N1043" s="105" t="n">
-        <v>25780415.64</v>
+        <v>9687031.199999999</v>
       </c>
       <c r="O1043" s="103" t="n">
         <v>-54</v>
@@ -83916,263 +83776,8 @@
         </is>
       </c>
     </row>
-    <row r="1063">
-      <c r="A1063" s="103" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B1063" s="103" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1063" s="103" t="n"/>
-      <c r="D1063" s="103" t="n"/>
-      <c r="E1063" s="103" t="n"/>
-      <c r="F1063" s="103" t="n"/>
-      <c r="G1063" s="103" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H1063" s="103" t="inlineStr">
-        <is>
-          <t>Reprocessing</t>
-        </is>
-      </c>
-      <c r="I1063" s="103" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="J1063" s="103" t="n"/>
-      <c r="K1063" s="104" t="n">
-        <v>46204</v>
-      </c>
-      <c r="L1063" s="104" t="n">
-        <v>46234</v>
-      </c>
-      <c r="M1063" s="105" t="n">
-        <v>140049</v>
-      </c>
-      <c r="N1063" s="105" t="n">
-        <v>46711943.46</v>
-      </c>
-      <c r="O1063" s="103" t="n"/>
-      <c r="P1063" s="103" t="n"/>
-      <c r="Q1063" s="103" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="1064">
-      <c r="A1064" s="103" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B1064" s="103" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1064" s="103" t="n"/>
-      <c r="D1064" s="103" t="n"/>
-      <c r="E1064" s="103" t="n"/>
-      <c r="F1064" s="103" t="n"/>
-      <c r="G1064" s="103" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H1064" s="103" t="inlineStr">
-        <is>
-          <t>Reprocessing</t>
-        </is>
-      </c>
-      <c r="I1064" s="103" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="J1064" s="103" t="n"/>
-      <c r="K1064" s="104" t="n">
-        <v>46204</v>
-      </c>
-      <c r="L1064" s="104" t="n">
-        <v>46234</v>
-      </c>
-      <c r="M1064" s="105" t="n">
-        <v>165711</v>
-      </c>
-      <c r="N1064" s="105" t="n">
-        <v>40821247.74</v>
-      </c>
-      <c r="O1064" s="103" t="n"/>
-      <c r="P1064" s="103" t="n"/>
-      <c r="Q1064" s="103" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="1065">
-      <c r="A1065" s="103" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B1065" s="103" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1065" s="103" t="n"/>
-      <c r="D1065" s="103" t="n"/>
-      <c r="E1065" s="103" t="n"/>
-      <c r="F1065" s="103" t="n"/>
-      <c r="G1065" s="103" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H1065" s="103" t="inlineStr">
-        <is>
-          <t>Reprocessing</t>
-        </is>
-      </c>
-      <c r="I1065" s="103" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="J1065" s="103" t="n"/>
-      <c r="K1065" s="104" t="n">
-        <v>46204</v>
-      </c>
-      <c r="L1065" s="104" t="n">
-        <v>46234</v>
-      </c>
-      <c r="M1065" s="105" t="n">
-        <v>64695</v>
-      </c>
-      <c r="N1065" s="105" t="n">
-        <v>20026984.2</v>
-      </c>
-      <c r="O1065" s="103" t="n"/>
-      <c r="P1065" s="103" t="n"/>
-      <c r="Q1065" s="103" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="1066">
-      <c r="A1066" s="103" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B1066" s="103" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1066" s="103" t="n"/>
-      <c r="D1066" s="103" t="n"/>
-      <c r="E1066" s="103" t="n"/>
-      <c r="F1066" s="103" t="n"/>
-      <c r="G1066" s="103" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H1066" s="103" t="inlineStr">
-        <is>
-          <t>Reprocessing</t>
-        </is>
-      </c>
-      <c r="I1066" s="103" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="J1066" s="103" t="n"/>
-      <c r="K1066" s="104" t="n">
-        <v>46204</v>
-      </c>
-      <c r="L1066" s="104" t="n">
-        <v>46234</v>
-      </c>
-      <c r="M1066" s="105" t="n">
-        <v>40273</v>
-      </c>
-      <c r="N1066" s="105" t="n">
-        <v>12027934.18</v>
-      </c>
-      <c r="O1066" s="103" t="n"/>
-      <c r="P1066" s="103" t="n"/>
-      <c r="Q1066" s="103" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="1067">
-      <c r="A1067" s="103" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B1067" s="103" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1067" s="103" t="n"/>
-      <c r="D1067" s="103" t="n"/>
-      <c r="E1067" s="103" t="n"/>
-      <c r="F1067" s="103" t="n"/>
-      <c r="G1067" s="103" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H1067" s="103" t="inlineStr">
-        <is>
-          <t>Reprocessing</t>
-        </is>
-      </c>
-      <c r="I1067" s="103" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="J1067" s="103" t="n"/>
-      <c r="K1067" s="104" t="n">
-        <v>46204</v>
-      </c>
-      <c r="L1067" s="104" t="n">
-        <v>46234</v>
-      </c>
-      <c r="M1067" s="105" t="n">
-        <v>19235</v>
-      </c>
-      <c r="N1067" s="105" t="n">
-        <v>5535063.600000001</v>
-      </c>
-      <c r="O1067" s="103" t="n"/>
-      <c r="P1067" s="103" t="n"/>
-      <c r="Q1067" s="103" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Q1067"/>
+  <autoFilter ref="A1:Q1062"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto-deploy AR dashboard 2026-08-27 16:58
</commit_message>
<xml_diff>
--- a/AR Movement Report.xlsx
+++ b/AR Movement Report.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$123</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1062</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1071</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1346,7 +1346,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data as of Thursday, 27 August 2026 - 13:27  |  Source: PSI AR Monitoring Master.xlsx</t>
+          <t>Data as of Thursday, 27 August 2026 - 16:58  |  Source: PSI AR Monitoring Master.xlsx</t>
         </is>
       </c>
     </row>
@@ -1383,13 +1383,13 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="9" t="n">
-        <v>74226972008.55531</v>
+        <v>74332160676.26884</v>
       </c>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="10" t="n"/>
       <c r="D7" s="11" t="n"/>
       <c r="E7" s="12" t="n">
-        <v>65171495318.61172</v>
+        <v>65276683986.32526</v>
       </c>
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="11" t="n"/>
@@ -1440,14 +1440,14 @@
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="19" t="n">
-        <v>38630507568.35851</v>
+        <v>38891769322.82851</v>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="10" t="n"/>
       <c r="D12" s="10" t="n"/>
       <c r="E12" s="11" t="n"/>
       <c r="F12" s="20" t="n">
-        <v>35596464440.19682</v>
+        <v>35440391353.44035</v>
       </c>
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="10" t="n"/>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="26" t="n">
-        <v>32567837201.06482</v>
+        <v>32829098955.53482</v>
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="27" t="n">
@@ -1600,10 +1600,10 @@
         </is>
       </c>
       <c r="B23" s="34" t="n">
-        <v>2333356705.95</v>
+        <v>2462658700.42</v>
       </c>
       <c r="C23" s="35" t="n">
-        <v>4371476948.058269</v>
+        <v>4215403861.3018</v>
       </c>
       <c r="D23" s="36" t="n">
         <v>0</v>
@@ -1792,7 +1792,7 @@
         </is>
       </c>
       <c r="B29" s="34" t="n">
-        <v>75384400</v>
+        <v>207344160</v>
       </c>
       <c r="C29" s="36" t="n">
         <v>0</v>
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="B41" s="49" t="n">
-        <v>30168384657.9985</v>
+        <v>30429646412.4685</v>
       </c>
       <c r="C41" s="49" t="n">
         <v>8462122910.359999</v>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B42" s="36" t="n">
-        <v>4371476948.058269</v>
+        <v>4215403861.3018</v>
       </c>
       <c r="C42" s="36" t="n">
         <v>593353779.5835853</v>
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="B49" s="57" t="n">
-        <v>4371476948.058269</v>
+        <v>4215403861.3018</v>
       </c>
       <c r="C49" s="57" t="n">
         <v>209900924.97</v>
@@ -2409,7 +2409,7 @@
         <v>46284</v>
       </c>
       <c r="B57" s="36" t="n">
-        <v>859999386.6700001</v>
+        <v>989301381.1400001</v>
       </c>
       <c r="C57" s="36" t="n">
         <v>0</v>
@@ -2753,7 +2753,7 @@
         <v>0</v>
       </c>
       <c r="H67" s="36" t="n">
-        <v>0</v>
+        <v>131959760</v>
       </c>
       <c r="I67" s="36" t="n">
         <v>886307502.1920002</v>
@@ -3102,7 +3102,7 @@
         </is>
       </c>
       <c r="C7" s="36" t="n">
-        <v>859999386.6700001</v>
+        <v>989301381.1400001</v>
       </c>
       <c r="D7" s="36" t="n">
         <v>1473357319.28</v>
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="C8" s="36" t="n">
-        <v>4371476948.058269</v>
+        <v>4215403861.3018</v>
       </c>
       <c r="D8" s="36" t="n">
         <v>0</v>
@@ -3302,7 +3302,7 @@
         </is>
       </c>
       <c r="C15" s="36" t="n">
-        <v>75384400</v>
+        <v>207344160</v>
       </c>
       <c r="D15" s="36" t="n">
         <v>0</v>
@@ -3375,7 +3375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H123"/>
+  <dimension ref="A1:H132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4832,19 +4832,25 @@
       </c>
       <c r="B46" s="72" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C46" s="72" t="n"/>
+          <t>PT Bayer Indonesia</t>
+        </is>
+      </c>
+      <c r="C46" s="72" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.BI/FC/42/2026</t>
+        </is>
+      </c>
       <c r="D46" s="72" t="inlineStr">
         <is>
           <t>Tooling</t>
         </is>
       </c>
       <c r="E46" s="73" t="n">
-        <v>156073086.756468</v>
-      </c>
-      <c r="F46" s="71" t="n"/>
+        <v>213514.65</v>
+      </c>
+      <c r="F46" s="71" t="n">
+        <v>46261</v>
+      </c>
       <c r="G46" s="74" t="n">
         <v>0</v>
       </c>
@@ -4860,25 +4866,19 @@
       </c>
       <c r="B47" s="72" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
-        </is>
-      </c>
-      <c r="C47" s="72" t="inlineStr">
-        <is>
-          <t>PT.PSI/PT.BI/FC/42/2026</t>
-        </is>
-      </c>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C47" s="72" t="n"/>
       <c r="D47" s="72" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E47" s="73" t="n">
-        <v>213514.65</v>
-      </c>
-      <c r="F47" s="71" t="n">
-        <v>46261</v>
-      </c>
+        <v>593353779.5835853</v>
+      </c>
+      <c r="F47" s="71" t="n"/>
       <c r="G47" s="74" t="n">
         <v>0</v>
       </c>
@@ -4889,30 +4889,36 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="71" t="n">
-        <v>46261</v>
-      </c>
-      <c r="B48" s="72" t="inlineStr">
+      <c r="A48" s="75" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B48" s="76" t="inlineStr">
         <is>
           <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
-      <c r="C48" s="72" t="n"/>
-      <c r="D48" s="72" t="inlineStr">
+      <c r="C48" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/11/2026</t>
+        </is>
+      </c>
+      <c r="D48" s="76" t="inlineStr">
         <is>
           <t>Rental</t>
         </is>
       </c>
-      <c r="E48" s="73" t="n">
-        <v>593353779.5835853</v>
-      </c>
-      <c r="F48" s="71" t="n"/>
-      <c r="G48" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="72" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+      <c r="E48" s="77" t="n">
+        <v>872911811.2</v>
+      </c>
+      <c r="F48" s="75" t="n">
+        <v>46267</v>
+      </c>
+      <c r="G48" s="78" t="n">
+        <v>7</v>
+      </c>
+      <c r="H48" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4933,7 @@
       </c>
       <c r="C49" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/11/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/12/2026</t>
         </is>
       </c>
       <c r="D49" s="76" t="inlineStr">
@@ -4936,7 +4942,7 @@
         </is>
       </c>
       <c r="E49" s="77" t="n">
-        <v>872911811.2</v>
+        <v>302161780.8</v>
       </c>
       <c r="F49" s="75" t="n">
         <v>46267</v>
@@ -4952,16 +4958,16 @@
     </row>
     <row r="50">
       <c r="A50" s="75" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="B50" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Alam Semesta Agro</t>
         </is>
       </c>
       <c r="C50" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/12/2026</t>
+          <t>PT.PSI/PT.ASA/Rental CS/09/2026</t>
         </is>
       </c>
       <c r="D50" s="76" t="inlineStr">
@@ -4970,13 +4976,13 @@
         </is>
       </c>
       <c r="E50" s="77" t="n">
-        <v>302161780.8</v>
+        <v>142652400</v>
       </c>
       <c r="F50" s="75" t="n">
-        <v>46267</v>
+        <v>46270</v>
       </c>
       <c r="G50" s="78" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H50" s="76" t="inlineStr">
         <is>
@@ -4995,7 +5001,7 @@
       </c>
       <c r="C51" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASA/Rental CS/09/2026</t>
+          <t>PT.PSI/PT.ASA/Rental CS/10/2026</t>
         </is>
       </c>
       <c r="D51" s="76" t="inlineStr">
@@ -5004,7 +5010,7 @@
         </is>
       </c>
       <c r="E51" s="77" t="n">
-        <v>142652400</v>
+        <v>6920631.27</v>
       </c>
       <c r="F51" s="75" t="n">
         <v>46270</v>
@@ -5020,16 +5026,16 @@
     </row>
     <row r="52">
       <c r="A52" s="75" t="n">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="B52" s="76" t="inlineStr">
         <is>
-          <t>PT Alam Semesta Agro</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C52" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASA/Rental CS/10/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/29/2026 </t>
         </is>
       </c>
       <c r="D52" s="76" t="inlineStr">
@@ -5038,13 +5044,13 @@
         </is>
       </c>
       <c r="E52" s="77" t="n">
-        <v>6920631.27</v>
+        <v>1365520000</v>
       </c>
       <c r="F52" s="75" t="n">
-        <v>46270</v>
+        <v>46273</v>
       </c>
       <c r="G52" s="78" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H52" s="76" t="inlineStr">
         <is>
@@ -5063,7 +5069,7 @@
       </c>
       <c r="C53" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/29/2026 </t>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/30/2026</t>
         </is>
       </c>
       <c r="D53" s="76" t="inlineStr">
@@ -5072,7 +5078,7 @@
         </is>
       </c>
       <c r="E53" s="77" t="n">
-        <v>1365520000</v>
+        <v>1071584346</v>
       </c>
       <c r="F53" s="75" t="n">
         <v>46273</v>
@@ -5097,7 +5103,7 @@
       </c>
       <c r="C54" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/30/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/31/2026</t>
         </is>
       </c>
       <c r="D54" s="76" t="inlineStr">
@@ -5106,7 +5112,7 @@
         </is>
       </c>
       <c r="E54" s="77" t="n">
-        <v>1071584346</v>
+        <v>272700000</v>
       </c>
       <c r="F54" s="75" t="n">
         <v>46273</v>
@@ -5131,7 +5137,7 @@
       </c>
       <c r="C55" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/31/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/32/2026 </t>
         </is>
       </c>
       <c r="D55" s="76" t="inlineStr">
@@ -5140,7 +5146,7 @@
         </is>
       </c>
       <c r="E55" s="77" t="n">
-        <v>272700000</v>
+        <v>25780415.64</v>
       </c>
       <c r="F55" s="75" t="n">
         <v>46273</v>
@@ -5156,16 +5162,16 @@
     </row>
     <row r="56">
       <c r="A56" s="75" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="B56" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C56" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/32/2026 </t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-22/2026</t>
         </is>
       </c>
       <c r="D56" s="76" t="inlineStr">
@@ -5174,13 +5180,13 @@
         </is>
       </c>
       <c r="E56" s="77" t="n">
-        <v>25780415.64</v>
+        <v>707000000</v>
       </c>
       <c r="F56" s="75" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="G56" s="78" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H56" s="76" t="inlineStr">
         <is>
@@ -5199,7 +5205,7 @@
       </c>
       <c r="C57" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-22/2026</t>
+          <t>PT.PSI/PT.ASI/HANDLING-CS-PAS2/23/2026</t>
         </is>
       </c>
       <c r="D57" s="76" t="inlineStr">
@@ -5208,7 +5214,7 @@
         </is>
       </c>
       <c r="E57" s="77" t="n">
-        <v>707000000</v>
+        <v>9857624.279999999</v>
       </c>
       <c r="F57" s="75" t="n">
         <v>46276</v>
@@ -5242,7 +5248,7 @@
         </is>
       </c>
       <c r="E58" s="77" t="n">
-        <v>9857624.279999999</v>
+        <v>1019695</v>
       </c>
       <c r="F58" s="75" t="n">
         <v>46276</v>
@@ -5267,7 +5273,7 @@
       </c>
       <c r="C59" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/HANDLING-CS-PAS2/23/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/24/2026</t>
         </is>
       </c>
       <c r="D59" s="76" t="inlineStr">
@@ -5276,7 +5282,7 @@
         </is>
       </c>
       <c r="E59" s="77" t="n">
-        <v>1019695</v>
+        <v>755480000</v>
       </c>
       <c r="F59" s="75" t="n">
         <v>46276</v>
@@ -5296,21 +5302,21 @@
       </c>
       <c r="B60" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C60" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/24/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/30/2026</t>
         </is>
       </c>
       <c r="D60" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E60" s="77" t="n">
-        <v>755480000</v>
+        <v>536105249.4995999</v>
       </c>
       <c r="F60" s="75" t="n">
         <v>46276</v>
@@ -5335,7 +5341,7 @@
       </c>
       <c r="C61" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/30/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/31/2026</t>
         </is>
       </c>
       <c r="D61" s="76" t="inlineStr">
@@ -5344,7 +5350,7 @@
         </is>
       </c>
       <c r="E61" s="77" t="n">
-        <v>536105249.4995999</v>
+        <v>513650866.212</v>
       </c>
       <c r="F61" s="75" t="n">
         <v>46276</v>
@@ -5360,7 +5366,7 @@
     </row>
     <row r="62">
       <c r="A62" s="75" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="B62" s="76" t="inlineStr">
         <is>
@@ -5369,7 +5375,7 @@
       </c>
       <c r="C62" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/31/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL/33/2026</t>
         </is>
       </c>
       <c r="D62" s="76" t="inlineStr">
@@ -5378,13 +5384,13 @@
         </is>
       </c>
       <c r="E62" s="77" t="n">
-        <v>513650866.212</v>
+        <v>27842793.22</v>
       </c>
       <c r="F62" s="75" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="G62" s="78" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H62" s="76" t="inlineStr">
         <is>
@@ -5394,16 +5400,16 @@
     </row>
     <row r="63">
       <c r="A63" s="75" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="B63" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C63" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/33/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/01/2026</t>
         </is>
       </c>
       <c r="D63" s="76" t="inlineStr">
@@ -5412,13 +5418,13 @@
         </is>
       </c>
       <c r="E63" s="77" t="n">
-        <v>27842793.22</v>
+        <v>24468320</v>
       </c>
       <c r="F63" s="75" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="G63" s="78" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H63" s="76" t="inlineStr">
         <is>
@@ -5437,7 +5443,7 @@
       </c>
       <c r="C64" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/01/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/02/2026</t>
         </is>
       </c>
       <c r="D64" s="76" t="inlineStr">
@@ -5446,7 +5452,7 @@
         </is>
       </c>
       <c r="E64" s="77" t="n">
-        <v>24468320</v>
+        <v>7298640</v>
       </c>
       <c r="F64" s="75" t="n">
         <v>46279</v>
@@ -5471,7 +5477,7 @@
       </c>
       <c r="C65" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/02/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/03/2026</t>
         </is>
       </c>
       <c r="D65" s="76" t="inlineStr">
@@ -5480,7 +5486,7 @@
         </is>
       </c>
       <c r="E65" s="77" t="n">
-        <v>7298640</v>
+        <v>1430080</v>
       </c>
       <c r="F65" s="75" t="n">
         <v>46279</v>
@@ -5505,7 +5511,7 @@
       </c>
       <c r="C66" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/03/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/04/2026</t>
         </is>
       </c>
       <c r="D66" s="76" t="inlineStr">
@@ -5514,7 +5520,7 @@
         </is>
       </c>
       <c r="E66" s="77" t="n">
-        <v>1430080</v>
+        <v>2450320</v>
       </c>
       <c r="F66" s="75" t="n">
         <v>46279</v>
@@ -5539,7 +5545,7 @@
       </c>
       <c r="C67" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/04/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/05/2026</t>
         </is>
       </c>
       <c r="D67" s="76" t="inlineStr">
@@ -5573,7 +5579,7 @@
       </c>
       <c r="C68" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/05/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/06/2026</t>
         </is>
       </c>
       <c r="D68" s="76" t="inlineStr">
@@ -5582,7 +5588,7 @@
         </is>
       </c>
       <c r="E68" s="77" t="n">
-        <v>2450320</v>
+        <v>10961040</v>
       </c>
       <c r="F68" s="75" t="n">
         <v>46279</v>
@@ -5607,7 +5613,7 @@
       </c>
       <c r="C69" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/06/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/07/2026</t>
         </is>
       </c>
       <c r="D69" s="76" t="inlineStr">
@@ -5616,7 +5622,7 @@
         </is>
       </c>
       <c r="E69" s="77" t="n">
-        <v>10961040</v>
+        <v>2249760</v>
       </c>
       <c r="F69" s="75" t="n">
         <v>46279</v>
@@ -5641,7 +5647,7 @@
       </c>
       <c r="C70" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/07/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/08/2026</t>
         </is>
       </c>
       <c r="D70" s="76" t="inlineStr">
@@ -5650,7 +5656,7 @@
         </is>
       </c>
       <c r="E70" s="77" t="n">
-        <v>2249760</v>
+        <v>4019920</v>
       </c>
       <c r="F70" s="75" t="n">
         <v>46279</v>
@@ -5675,7 +5681,7 @@
       </c>
       <c r="C71" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/08/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/09/2026</t>
         </is>
       </c>
       <c r="D71" s="76" t="inlineStr">
@@ -5684,7 +5690,7 @@
         </is>
       </c>
       <c r="E71" s="77" t="n">
-        <v>4019920</v>
+        <v>12609120</v>
       </c>
       <c r="F71" s="75" t="n">
         <v>46279</v>
@@ -5709,7 +5715,7 @@
       </c>
       <c r="C72" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/09/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/10/2026</t>
         </is>
       </c>
       <c r="D72" s="76" t="inlineStr">
@@ -5718,7 +5724,7 @@
         </is>
       </c>
       <c r="E72" s="77" t="n">
-        <v>12609120</v>
+        <v>2180000</v>
       </c>
       <c r="F72" s="75" t="n">
         <v>46279</v>
@@ -5743,7 +5749,7 @@
       </c>
       <c r="C73" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/10/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/11/2026</t>
         </is>
       </c>
       <c r="D73" s="76" t="inlineStr">
@@ -5752,7 +5758,7 @@
         </is>
       </c>
       <c r="E73" s="77" t="n">
-        <v>2180000</v>
+        <v>5266880</v>
       </c>
       <c r="F73" s="75" t="n">
         <v>46279</v>
@@ -5768,16 +5774,16 @@
     </row>
     <row r="74">
       <c r="A74" s="75" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="B74" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C74" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/11/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/49/2026</t>
         </is>
       </c>
       <c r="D74" s="76" t="inlineStr">
@@ -5786,13 +5792,13 @@
         </is>
       </c>
       <c r="E74" s="77" t="n">
-        <v>5266880</v>
+        <v>3981599123.659349</v>
       </c>
       <c r="F74" s="75" t="n">
-        <v>46279</v>
+        <v>46276</v>
       </c>
       <c r="G74" s="78" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H74" s="76" t="inlineStr">
         <is>
@@ -5811,7 +5817,7 @@
       </c>
       <c r="C75" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/49/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/50/2026</t>
         </is>
       </c>
       <c r="D75" s="76" t="inlineStr">
@@ -5820,7 +5826,7 @@
         </is>
       </c>
       <c r="E75" s="77" t="n">
-        <v>3981599123.659349</v>
+        <v>1542175442.6694</v>
       </c>
       <c r="F75" s="75" t="n">
         <v>46276</v>
@@ -5845,7 +5851,7 @@
       </c>
       <c r="C76" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/50/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/51/2026</t>
         </is>
       </c>
       <c r="D76" s="76" t="inlineStr">
@@ -5854,7 +5860,7 @@
         </is>
       </c>
       <c r="E76" s="77" t="n">
-        <v>1542175442.6694</v>
+        <v>487978078.30875</v>
       </c>
       <c r="F76" s="75" t="n">
         <v>46276</v>
@@ -5879,7 +5885,7 @@
       </c>
       <c r="C77" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/51/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/52/2026</t>
         </is>
       </c>
       <c r="D77" s="76" t="inlineStr">
@@ -5888,7 +5894,7 @@
         </is>
       </c>
       <c r="E77" s="77" t="n">
-        <v>487978078.30875</v>
+        <v>14255050.74672</v>
       </c>
       <c r="F77" s="75" t="n">
         <v>46276</v>
@@ -5904,16 +5910,16 @@
     </row>
     <row r="78">
       <c r="A78" s="75" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="B78" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C78" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/52/2026</t>
+          <t>PT.PSI/PT.ASI/FC_LMB_PGB/02/2026</t>
         </is>
       </c>
       <c r="D78" s="76" t="inlineStr">
@@ -5922,13 +5928,13 @@
         </is>
       </c>
       <c r="E78" s="77" t="n">
-        <v>14255050.74672</v>
+        <v>51019085</v>
       </c>
       <c r="F78" s="75" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
       <c r="G78" s="78" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H78" s="76" t="inlineStr">
         <is>
@@ -5947,7 +5953,7 @@
       </c>
       <c r="C79" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/FC_LMB_PGB/02/2026</t>
+          <t>PT.PSI/PT.ASI/FC_PAS2/03/26</t>
         </is>
       </c>
       <c r="D79" s="76" t="inlineStr">
@@ -5956,7 +5962,7 @@
         </is>
       </c>
       <c r="E79" s="77" t="n">
-        <v>51019085</v>
+        <v>119160408.84</v>
       </c>
       <c r="F79" s="75" t="n">
         <v>46284</v>
@@ -5981,7 +5987,7 @@
       </c>
       <c r="C80" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/FC_PAS2/03/26</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/51/2026 </t>
         </is>
       </c>
       <c r="D80" s="76" t="inlineStr">
@@ -5990,7 +5996,7 @@
         </is>
       </c>
       <c r="E80" s="77" t="n">
-        <v>119160408.84</v>
+        <v>587478172</v>
       </c>
       <c r="F80" s="75" t="n">
         <v>46284</v>
@@ -6015,7 +6021,7 @@
       </c>
       <c r="C81" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/51/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/52/2026 </t>
         </is>
       </c>
       <c r="D81" s="76" t="inlineStr">
@@ -6024,7 +6030,7 @@
         </is>
       </c>
       <c r="E81" s="77" t="n">
-        <v>587478172</v>
+        <v>68745646</v>
       </c>
       <c r="F81" s="75" t="n">
         <v>46284</v>
@@ -6049,7 +6055,7 @@
       </c>
       <c r="C82" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/52/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/53/2026 </t>
         </is>
       </c>
       <c r="D82" s="76" t="inlineStr">
@@ -6058,7 +6064,7 @@
         </is>
       </c>
       <c r="E82" s="77" t="n">
-        <v>68745646</v>
+        <v>33596074.83</v>
       </c>
       <c r="F82" s="75" t="n">
         <v>46284</v>
@@ -6083,7 +6089,7 @@
       </c>
       <c r="C83" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/53/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/SC/64/2026 </t>
         </is>
       </c>
       <c r="D83" s="76" t="inlineStr">
@@ -6092,7 +6098,7 @@
         </is>
       </c>
       <c r="E83" s="77" t="n">
-        <v>33596074.83</v>
+        <v>127114309.97</v>
       </c>
       <c r="F83" s="75" t="n">
         <v>46284</v>
@@ -6112,12 +6118,12 @@
       </c>
       <c r="B84" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C84" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/SC/65/2026 </t>
         </is>
       </c>
       <c r="D84" s="76" t="inlineStr">
@@ -6126,7 +6132,7 @@
         </is>
       </c>
       <c r="E84" s="77" t="n">
-        <v>326395903.6008</v>
+        <v>2187684.5</v>
       </c>
       <c r="F84" s="75" t="n">
         <v>46284</v>
@@ -6151,7 +6157,7 @@
       </c>
       <c r="C85" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
         </is>
       </c>
       <c r="D85" s="76" t="inlineStr">
@@ -6160,7 +6166,7 @@
         </is>
       </c>
       <c r="E85" s="77" t="n">
-        <v>240049.20888</v>
+        <v>326395903.6008</v>
       </c>
       <c r="F85" s="75" t="n">
         <v>46284</v>
@@ -6176,7 +6182,7 @@
     </row>
     <row r="86">
       <c r="A86" s="75" t="n">
-        <v>46286</v>
+        <v>46284</v>
       </c>
       <c r="B86" s="76" t="inlineStr">
         <is>
@@ -6185,7 +6191,7 @@
       </c>
       <c r="C86" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
         </is>
       </c>
       <c r="D86" s="76" t="inlineStr">
@@ -6194,13 +6200,13 @@
         </is>
       </c>
       <c r="E86" s="77" t="n">
-        <v>570800977.7184</v>
+        <v>240049.20888</v>
       </c>
       <c r="F86" s="75" t="n">
-        <v>46286</v>
+        <v>46284</v>
       </c>
       <c r="G86" s="78" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H86" s="76" t="inlineStr">
         <is>
@@ -6210,16 +6216,16 @@
     </row>
     <row r="87">
       <c r="A87" s="75" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="B87" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C87" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/53/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
         </is>
       </c>
       <c r="D87" s="76" t="inlineStr">
@@ -6228,13 +6234,13 @@
         </is>
       </c>
       <c r="E87" s="77" t="n">
-        <v>36849832.74</v>
+        <v>570800977.7184</v>
       </c>
       <c r="F87" s="75" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="G87" s="78" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H87" s="76" t="inlineStr">
         <is>
@@ -6253,7 +6259,7 @@
       </c>
       <c r="C88" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/54/2026</t>
+          <t>PT.PSI/PT.CASI/REP/53/2026</t>
         </is>
       </c>
       <c r="D88" s="76" t="inlineStr">
@@ -6262,7 +6268,7 @@
         </is>
       </c>
       <c r="E88" s="77" t="n">
-        <v>31988016.36</v>
+        <v>36849832.74</v>
       </c>
       <c r="F88" s="75" t="n">
         <v>46285</v>
@@ -6287,7 +6293,7 @@
       </c>
       <c r="C89" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/55/2026</t>
+          <t>PT.PSI/PT.CASI/REP/54/2026</t>
         </is>
       </c>
       <c r="D89" s="76" t="inlineStr">
@@ -6296,7 +6302,7 @@
         </is>
       </c>
       <c r="E89" s="77" t="n">
-        <v>19431065.722</v>
+        <v>31988016.36</v>
       </c>
       <c r="F89" s="75" t="n">
         <v>46285</v>
@@ -6312,16 +6318,16 @@
     </row>
     <row r="90">
       <c r="A90" s="75" t="n">
-        <v>46292</v>
+        <v>46289</v>
       </c>
       <c r="B90" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C90" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/43/2026</t>
+          <t>PT.PSI/PT.CASI/REP/55/2026</t>
         </is>
       </c>
       <c r="D90" s="76" t="inlineStr">
@@ -6330,13 +6336,13 @@
         </is>
       </c>
       <c r="E90" s="77" t="n">
-        <v>103679056</v>
+        <v>19431065.722</v>
       </c>
       <c r="F90" s="75" t="n">
-        <v>46292</v>
+        <v>46285</v>
       </c>
       <c r="G90" s="78" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H90" s="76" t="inlineStr">
         <is>
@@ -6355,7 +6361,7 @@
       </c>
       <c r="C91" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/44/2026</t>
+          <t>PT.PSI/PT.BI/FC/43/2026</t>
         </is>
       </c>
       <c r="D91" s="76" t="inlineStr">
@@ -6364,7 +6370,7 @@
         </is>
       </c>
       <c r="E91" s="77" t="n">
-        <v>92863095</v>
+        <v>103679056</v>
       </c>
       <c r="F91" s="75" t="n">
         <v>46292</v>
@@ -6389,7 +6395,7 @@
       </c>
       <c r="C92" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/45/2026</t>
+          <t>PT.PSI/PT.BI/FC/44/2026</t>
         </is>
       </c>
       <c r="D92" s="76" t="inlineStr">
@@ -6398,7 +6404,7 @@
         </is>
       </c>
       <c r="E92" s="77" t="n">
-        <v>17392258</v>
+        <v>92863095</v>
       </c>
       <c r="F92" s="75" t="n">
         <v>46292</v>
@@ -6423,7 +6429,7 @@
       </c>
       <c r="C93" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/46/2026</t>
+          <t>PT.PSI/PT.BI/FC/45/2026</t>
         </is>
       </c>
       <c r="D93" s="76" t="inlineStr">
@@ -6432,7 +6438,7 @@
         </is>
       </c>
       <c r="E93" s="77" t="n">
-        <v>197734556.5</v>
+        <v>17392258</v>
       </c>
       <c r="F93" s="75" t="n">
         <v>46292</v>
@@ -6457,7 +6463,7 @@
       </c>
       <c r="C94" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/47/2026</t>
+          <t>PT.PSI/PT.BI/FC/46/2026</t>
         </is>
       </c>
       <c r="D94" s="76" t="inlineStr">
@@ -6466,7 +6472,7 @@
         </is>
       </c>
       <c r="E94" s="77" t="n">
-        <v>254755628.4</v>
+        <v>197734556.5</v>
       </c>
       <c r="F94" s="75" t="n">
         <v>46292</v>
@@ -6491,7 +6497,7 @@
       </c>
       <c r="C95" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/48/2026</t>
+          <t>PT.PSI/PT.BI/FC/47/2026</t>
         </is>
       </c>
       <c r="D95" s="76" t="inlineStr">
@@ -6500,7 +6506,7 @@
         </is>
       </c>
       <c r="E95" s="77" t="n">
-        <v>10599160</v>
+        <v>254755628.4</v>
       </c>
       <c r="F95" s="75" t="n">
         <v>46292</v>
@@ -6525,7 +6531,7 @@
       </c>
       <c r="C96" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/49/2026</t>
+          <t>PT.PSI/PT.BI/FC/48/2026</t>
         </is>
       </c>
       <c r="D96" s="76" t="inlineStr">
@@ -6534,7 +6540,7 @@
         </is>
       </c>
       <c r="E96" s="77" t="n">
-        <v>54405006.5</v>
+        <v>10599160</v>
       </c>
       <c r="F96" s="75" t="n">
         <v>46292</v>
@@ -6559,7 +6565,7 @@
       </c>
       <c r="C97" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/50/2026</t>
+          <t>PT.PSI/PT.BI/FC/49/2026</t>
         </is>
       </c>
       <c r="D97" s="76" t="inlineStr">
@@ -6568,7 +6574,7 @@
         </is>
       </c>
       <c r="E97" s="77" t="n">
-        <v>1075481.2</v>
+        <v>54405006.5</v>
       </c>
       <c r="F97" s="75" t="n">
         <v>46292</v>
@@ -6593,7 +6599,7 @@
       </c>
       <c r="C98" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/51/2026</t>
+          <t>PT.PSI/PT.BI/FC/50/2026</t>
         </is>
       </c>
       <c r="D98" s="76" t="inlineStr">
@@ -6602,7 +6608,7 @@
         </is>
       </c>
       <c r="E98" s="77" t="n">
-        <v>803447.72</v>
+        <v>1075481.2</v>
       </c>
       <c r="F98" s="75" t="n">
         <v>46292</v>
@@ -6627,7 +6633,7 @@
       </c>
       <c r="C99" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/52/2026</t>
+          <t>PT.PSI/PT.BI/FC/51/2026</t>
         </is>
       </c>
       <c r="D99" s="76" t="inlineStr">
@@ -6636,7 +6642,7 @@
         </is>
       </c>
       <c r="E99" s="77" t="n">
-        <v>7250789</v>
+        <v>803447.72</v>
       </c>
       <c r="F99" s="75" t="n">
         <v>46292</v>
@@ -6661,7 +6667,7 @@
       </c>
       <c r="C100" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/53/2026</t>
+          <t>PT.PSI/PT.BI/FC/52/2026</t>
         </is>
       </c>
       <c r="D100" s="76" t="inlineStr">
@@ -6670,7 +6676,7 @@
         </is>
       </c>
       <c r="E100" s="77" t="n">
-        <v>101318334</v>
+        <v>7250789</v>
       </c>
       <c r="F100" s="75" t="n">
         <v>46292</v>
@@ -6686,7 +6692,7 @@
     </row>
     <row r="101">
       <c r="A101" s="75" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B101" s="76" t="inlineStr">
         <is>
@@ -6695,7 +6701,7 @@
       </c>
       <c r="C101" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/54/2026</t>
+          <t>PT.PSI/PT.BI/FC/53/2026</t>
         </is>
       </c>
       <c r="D101" s="76" t="inlineStr">
@@ -6704,13 +6710,13 @@
         </is>
       </c>
       <c r="E101" s="77" t="n">
-        <v>156400274.1</v>
+        <v>101318334</v>
       </c>
       <c r="F101" s="75" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="G101" s="78" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H101" s="76" t="inlineStr">
         <is>
@@ -6729,7 +6735,7 @@
       </c>
       <c r="C102" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/55/2026</t>
+          <t>PT.PSI/PT.BI/FC/54/2026</t>
         </is>
       </c>
       <c r="D102" s="76" t="inlineStr">
@@ -6738,7 +6744,7 @@
         </is>
       </c>
       <c r="E102" s="77" t="n">
-        <v>50838199.5</v>
+        <v>156400274.1</v>
       </c>
       <c r="F102" s="75" t="n">
         <v>46293</v>
@@ -6763,7 +6769,7 @@
       </c>
       <c r="C103" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/56/2026</t>
+          <t>PT.PSI/PT.BI/FC/55/2026</t>
         </is>
       </c>
       <c r="D103" s="76" t="inlineStr">
@@ -6772,7 +6778,7 @@
         </is>
       </c>
       <c r="E103" s="77" t="n">
-        <v>376884765.6</v>
+        <v>50838199.5</v>
       </c>
       <c r="F103" s="75" t="n">
         <v>46293</v>
@@ -6797,7 +6803,7 @@
       </c>
       <c r="C104" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/57/2026</t>
+          <t>PT.PSI/PT.BI/FC/56/2026</t>
         </is>
       </c>
       <c r="D104" s="76" t="inlineStr">
@@ -6806,7 +6812,7 @@
         </is>
       </c>
       <c r="E104" s="77" t="n">
-        <v>100336789</v>
+        <v>376884765.6</v>
       </c>
       <c r="F104" s="75" t="n">
         <v>46293</v>
@@ -6831,7 +6837,7 @@
       </c>
       <c r="C105" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/58/2026</t>
+          <t>PT.PSI/PT.BI/FC/57/2026</t>
         </is>
       </c>
       <c r="D105" s="76" t="inlineStr">
@@ -6840,7 +6846,7 @@
         </is>
       </c>
       <c r="E105" s="77" t="n">
-        <v>787756603.1999999</v>
+        <v>100336789</v>
       </c>
       <c r="F105" s="75" t="n">
         <v>46293</v>
@@ -6865,7 +6871,7 @@
       </c>
       <c r="C106" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/59/2026</t>
+          <t>PT.PSI/PT.BI/FC/58/2026</t>
         </is>
       </c>
       <c r="D106" s="76" t="inlineStr">
@@ -6874,7 +6880,7 @@
         </is>
       </c>
       <c r="E106" s="77" t="n">
-        <v>140859991.5</v>
+        <v>787756603.1999999</v>
       </c>
       <c r="F106" s="75" t="n">
         <v>46293</v>
@@ -6890,16 +6896,16 @@
     </row>
     <row r="107">
       <c r="A107" s="75" t="n">
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="B107" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C107" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
+          <t>PT.PSI/PT.BI/FC/59/2026</t>
         </is>
       </c>
       <c r="D107" s="76" t="inlineStr">
@@ -6908,13 +6914,13 @@
         </is>
       </c>
       <c r="E107" s="77" t="n">
-        <v>18871809.6</v>
+        <v>140859991.5</v>
       </c>
       <c r="F107" s="75" t="n">
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="G107" s="78" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="H107" s="76" t="inlineStr">
         <is>
@@ -6924,7 +6930,7 @@
     </row>
     <row r="108">
       <c r="A108" s="75" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="B108" s="76" t="inlineStr">
         <is>
@@ -6933,7 +6939,7 @@
       </c>
       <c r="C108" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
         </is>
       </c>
       <c r="D108" s="76" t="inlineStr">
@@ -6942,13 +6948,13 @@
         </is>
       </c>
       <c r="E108" s="77" t="n">
-        <v>226017285.066</v>
+        <v>18871809.6</v>
       </c>
       <c r="F108" s="75" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="G108" s="78" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H108" s="76" t="inlineStr">
         <is>
@@ -6967,7 +6973,7 @@
       </c>
       <c r="C109" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
         </is>
       </c>
       <c r="D109" s="76" t="inlineStr">
@@ -6976,7 +6982,7 @@
         </is>
       </c>
       <c r="E109" s="77" t="n">
-        <v>3356193038.598001</v>
+        <v>226017285.066</v>
       </c>
       <c r="F109" s="75" t="n">
         <v>46301</v>
@@ -7001,7 +7007,7 @@
       </c>
       <c r="C110" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
         </is>
       </c>
       <c r="D110" s="76" t="inlineStr">
@@ -7010,7 +7016,7 @@
         </is>
       </c>
       <c r="E110" s="77" t="n">
-        <v>999055757.8296</v>
+        <v>3356193038.598001</v>
       </c>
       <c r="F110" s="75" t="n">
         <v>46301</v>
@@ -7026,7 +7032,7 @@
     </row>
     <row r="111">
       <c r="A111" s="75" t="n">
-        <v>46305</v>
+        <v>46301</v>
       </c>
       <c r="B111" s="76" t="inlineStr">
         <is>
@@ -7035,7 +7041,7 @@
       </c>
       <c r="C111" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
         </is>
       </c>
       <c r="D111" s="76" t="inlineStr">
@@ -7044,13 +7050,13 @@
         </is>
       </c>
       <c r="E111" s="77" t="n">
-        <v>886307502.1920002</v>
+        <v>999055757.8296</v>
       </c>
       <c r="F111" s="75" t="n">
-        <v>46305</v>
+        <v>46301</v>
       </c>
       <c r="G111" s="78" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H111" s="76" t="inlineStr">
         <is>
@@ -7060,16 +7066,16 @@
     </row>
     <row r="112">
       <c r="A112" s="75" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="B112" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C112" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/12/2026</t>
         </is>
       </c>
       <c r="D112" s="76" t="inlineStr">
@@ -7078,13 +7084,13 @@
         </is>
       </c>
       <c r="E112" s="77" t="n">
-        <v>5676698527.872001</v>
+        <v>802240</v>
       </c>
       <c r="F112" s="75" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="G112" s="78" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H112" s="76" t="inlineStr">
         <is>
@@ -7094,16 +7100,16 @@
     </row>
     <row r="113">
       <c r="A113" s="75" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="B113" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C113" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/13/2026</t>
         </is>
       </c>
       <c r="D113" s="76" t="inlineStr">
@@ -7112,13 +7118,13 @@
         </is>
       </c>
       <c r="E113" s="77" t="n">
-        <v>564189103.6416</v>
+        <v>8632800</v>
       </c>
       <c r="F113" s="75" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="G113" s="78" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H113" s="76" t="inlineStr">
         <is>
@@ -7128,31 +7134,31 @@
     </row>
     <row r="114">
       <c r="A114" s="75" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="B114" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C114" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
+          <t>PT.PSI/PT.EWINDO_LMB/14/2026</t>
         </is>
       </c>
       <c r="D114" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E114" s="77" t="n">
-        <v>1365520000</v>
+        <v>967920</v>
       </c>
       <c r="F114" s="75" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="G114" s="78" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H114" s="76" t="inlineStr">
         <is>
@@ -7162,31 +7168,31 @@
     </row>
     <row r="115">
       <c r="A115" s="75" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="B115" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C115" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
+          <t>PT.PSI/PT.EWINDO_LMB/15/2026</t>
         </is>
       </c>
       <c r="D115" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E115" s="77" t="n">
-        <v>9687031.199999999</v>
+        <v>20509440</v>
       </c>
       <c r="F115" s="75" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="G115" s="78" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H115" s="76" t="inlineStr">
         <is>
@@ -7196,31 +7202,31 @@
     </row>
     <row r="116">
       <c r="A116" s="75" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="B116" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C116" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/16/2026</t>
         </is>
       </c>
       <c r="D116" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E116" s="77" t="n">
-        <v>1070726250</v>
+        <v>2180000</v>
       </c>
       <c r="F116" s="75" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="G116" s="78" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H116" s="76" t="inlineStr">
         <is>
@@ -7230,31 +7236,31 @@
     </row>
     <row r="117">
       <c r="A117" s="75" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="B117" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C117" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/17/2026</t>
         </is>
       </c>
       <c r="D117" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E117" s="77" t="n">
-        <v>272700000</v>
+        <v>540640</v>
       </c>
       <c r="F117" s="75" t="n">
-        <v>46312</v>
+        <v>46305</v>
       </c>
       <c r="G117" s="78" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H117" s="76" t="inlineStr">
         <is>
@@ -7264,16 +7270,16 @@
     </row>
     <row r="118">
       <c r="A118" s="75" t="n">
-        <v>46314</v>
+        <v>46305</v>
       </c>
       <c r="B118" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C118" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/18/2026</t>
         </is>
       </c>
       <c r="D118" s="76" t="inlineStr">
@@ -7282,13 +7288,13 @@
         </is>
       </c>
       <c r="E118" s="77" t="n">
-        <v>545818781.4912</v>
+        <v>47532720</v>
       </c>
       <c r="F118" s="75" t="n">
-        <v>46314</v>
+        <v>46305</v>
       </c>
       <c r="G118" s="78" t="n">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="H118" s="76" t="inlineStr">
         <is>
@@ -7298,16 +7304,16 @@
     </row>
     <row r="119">
       <c r="A119" s="75" t="n">
-        <v>46314</v>
+        <v>46305</v>
       </c>
       <c r="B119" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C119" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/19/2026</t>
         </is>
       </c>
       <c r="D119" s="76" t="inlineStr">
@@ -7316,13 +7322,13 @@
         </is>
       </c>
       <c r="E119" s="77" t="n">
-        <v>767367847.5204</v>
+        <v>50794000</v>
       </c>
       <c r="F119" s="75" t="n">
-        <v>46314</v>
+        <v>46305</v>
       </c>
       <c r="G119" s="78" t="n">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="H119" s="76" t="inlineStr">
         <is>
@@ -7332,7 +7338,7 @@
     </row>
     <row r="120">
       <c r="A120" s="75" t="n">
-        <v>46314</v>
+        <v>46305</v>
       </c>
       <c r="B120" s="76" t="inlineStr">
         <is>
@@ -7341,7 +7347,7 @@
       </c>
       <c r="C120" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
         </is>
       </c>
       <c r="D120" s="76" t="inlineStr">
@@ -7350,13 +7356,13 @@
         </is>
       </c>
       <c r="E120" s="77" t="n">
-        <v>4761468367.9458</v>
+        <v>886307502.1920002</v>
       </c>
       <c r="F120" s="75" t="n">
-        <v>46314</v>
+        <v>46305</v>
       </c>
       <c r="G120" s="78" t="n">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="H120" s="76" t="inlineStr">
         <is>
@@ -7366,7 +7372,7 @@
     </row>
     <row r="121">
       <c r="A121" s="75" t="n">
-        <v>46314</v>
+        <v>46308</v>
       </c>
       <c r="B121" s="76" t="inlineStr">
         <is>
@@ -7375,7 +7381,7 @@
       </c>
       <c r="C121" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
         </is>
       </c>
       <c r="D121" s="76" t="inlineStr">
@@ -7384,13 +7390,13 @@
         </is>
       </c>
       <c r="E121" s="77" t="n">
-        <v>442076465.292</v>
+        <v>5676698527.872001</v>
       </c>
       <c r="F121" s="75" t="n">
-        <v>46314</v>
+        <v>46308</v>
       </c>
       <c r="G121" s="78" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="H121" s="76" t="inlineStr">
         <is>
@@ -7400,57 +7406,363 @@
     </row>
     <row r="122">
       <c r="A122" s="75" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B122" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C122" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
+        </is>
+      </c>
+      <c r="D122" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E122" s="77" t="n">
+        <v>564189103.6416</v>
+      </c>
+      <c r="F122" s="75" t="n">
+        <v>46308</v>
+      </c>
+      <c r="G122" s="78" t="n">
+        <v>47</v>
+      </c>
+      <c r="H122" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B123" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C123" s="76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
+        </is>
+      </c>
+      <c r="D123" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E123" s="77" t="n">
+        <v>1365520000</v>
+      </c>
+      <c r="F123" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G123" s="78" t="n">
+        <v>51</v>
+      </c>
+      <c r="H123" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B124" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C124" s="76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
+        </is>
+      </c>
+      <c r="D124" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E124" s="77" t="n">
+        <v>9687031.199999999</v>
+      </c>
+      <c r="F124" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G124" s="78" t="n">
+        <v>51</v>
+      </c>
+      <c r="H124" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B125" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C125" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
+        </is>
+      </c>
+      <c r="D125" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E125" s="77" t="n">
+        <v>1070726250</v>
+      </c>
+      <c r="F125" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G125" s="78" t="n">
+        <v>51</v>
+      </c>
+      <c r="H125" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B126" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C126" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
+        </is>
+      </c>
+      <c r="D126" s="76" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="E126" s="77" t="n">
+        <v>272700000</v>
+      </c>
+      <c r="F126" s="75" t="n">
+        <v>46312</v>
+      </c>
+      <c r="G126" s="78" t="n">
+        <v>51</v>
+      </c>
+      <c r="H126" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="75" t="n">
         <v>46314</v>
       </c>
-      <c r="B122" s="76" t="inlineStr">
+      <c r="B127" s="76" t="inlineStr">
         <is>
           <t>PT Syngenta Indonesia</t>
         </is>
       </c>
-      <c r="C122" s="76" t="inlineStr">
+      <c r="C127" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
+        </is>
+      </c>
+      <c r="D127" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E127" s="77" t="n">
+        <v>545818781.4912</v>
+      </c>
+      <c r="F127" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G127" s="78" t="n">
+        <v>53</v>
+      </c>
+      <c r="H127" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B128" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C128" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
+        </is>
+      </c>
+      <c r="D128" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E128" s="77" t="n">
+        <v>767367847.5204</v>
+      </c>
+      <c r="F128" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G128" s="78" t="n">
+        <v>53</v>
+      </c>
+      <c r="H128" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B129" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C129" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
+        </is>
+      </c>
+      <c r="D129" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E129" s="77" t="n">
+        <v>4761468367.9458</v>
+      </c>
+      <c r="F129" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G129" s="78" t="n">
+        <v>53</v>
+      </c>
+      <c r="H129" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B130" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C130" s="76" t="inlineStr">
         <is>
           <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
         </is>
       </c>
-      <c r="D122" s="76" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E122" s="77" t="n">
+      <c r="D130" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E130" s="77" t="n">
+        <v>442076465.292</v>
+      </c>
+      <c r="F130" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G130" s="78" t="n">
+        <v>53</v>
+      </c>
+      <c r="H130" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="75" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B131" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C131" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+        </is>
+      </c>
+      <c r="D131" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E131" s="77" t="n">
         <v>444456984.744</v>
       </c>
-      <c r="F122" s="75" t="n">
+      <c r="F131" s="75" t="n">
         <v>46314</v>
       </c>
-      <c r="G122" s="78" t="n">
+      <c r="G131" s="78" t="n">
         <v>53</v>
       </c>
-      <c r="H122" s="76" t="inlineStr">
+      <c r="H131" s="76" t="inlineStr">
         <is>
           <t>Future</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="39" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="39" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B123" s="79" t="n"/>
-      <c r="C123" s="79" t="n"/>
-      <c r="D123" s="79" t="n"/>
-      <c r="E123" s="80">
-        <f>SUM(E5:E122)</f>
+      <c r="B132" s="79" t="n"/>
+      <c r="C132" s="79" t="n"/>
+      <c r="D132" s="79" t="n"/>
+      <c r="E132" s="80">
+        <f>SUM(E5:E131)</f>
         <v/>
       </c>
-      <c r="F123" s="79" t="n"/>
-      <c r="G123" s="79" t="n"/>
-      <c r="H123" s="79" t="n"/>
+      <c r="F132" s="79" t="n"/>
+      <c r="G132" s="79" t="n"/>
+      <c r="H132" s="79" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H123"/>
+  <autoFilter ref="A4:H132"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8323,34 +8635,34 @@
         <v>1274206673.07</v>
       </c>
       <c r="BN8" s="86" t="n">
-        <v>718601162.73</v>
+        <v>720788847.23</v>
       </c>
       <c r="BO8" s="36" t="n">
-        <v>555605510.3399999</v>
+        <v>553417825.8399999</v>
       </c>
       <c r="BP8" s="85" t="n">
         <v>1440563725.87</v>
       </c>
       <c r="BQ8" s="86" t="n">
-        <v>990754902.8199999</v>
+        <v>1117869212.79</v>
       </c>
       <c r="BR8" s="36" t="n">
-        <v>449808823.0500004</v>
+        <v>322694513.0800004</v>
       </c>
       <c r="BS8" s="85" t="n">
-        <v>238925139.84</v>
+        <v>368227134.31</v>
       </c>
       <c r="BT8" s="86" t="n">
         <v>0</v>
       </c>
       <c r="BU8" s="36" t="n">
-        <v>238925139.84</v>
+        <v>368227134.31</v>
       </c>
       <c r="BV8" s="40" t="n">
-        <v>147291726701.9854</v>
+        <v>147421028696.4554</v>
       </c>
       <c r="BW8" s="40" t="n">
-        <v>147291726701.9854</v>
+        <v>147421028696.4554</v>
       </c>
       <c r="BX8" s="40" t="n">
         <v>0</v>
@@ -9260,25 +9572,25 @@
         <v>75384400</v>
       </c>
       <c r="BQ12" s="86" t="n">
-        <v>24075920</v>
+        <v>105241680</v>
       </c>
       <c r="BR12" s="36" t="n">
-        <v>51308480</v>
+        <v>-29857280</v>
       </c>
       <c r="BS12" s="85" t="n">
-        <v>0</v>
+        <v>131959760</v>
       </c>
       <c r="BT12" s="86" t="n">
-        <v>0</v>
+        <v>50794000</v>
       </c>
       <c r="BU12" s="36" t="n">
-        <v>0</v>
+        <v>81165760</v>
       </c>
       <c r="BV12" s="40" t="n">
-        <v>75384400</v>
+        <v>207344160</v>
       </c>
       <c r="BW12" s="40" t="n">
-        <v>75384400</v>
+        <v>207344160</v>
       </c>
       <c r="BX12" s="40" t="n">
         <v>0</v>
@@ -10589,34 +10901,34 @@
         <v>993895</v>
       </c>
       <c r="BN19" s="90" t="n">
-        <v>698900</v>
+        <v>699585</v>
       </c>
       <c r="BO19" s="91" t="n">
-        <v>294995</v>
+        <v>294310</v>
       </c>
       <c r="BP19" s="89" t="n">
         <v>1070910</v>
       </c>
       <c r="BQ19" s="90" t="n">
-        <v>534051</v>
+        <v>549214</v>
       </c>
       <c r="BR19" s="91" t="n">
-        <v>536859</v>
+        <v>521696</v>
       </c>
       <c r="BS19" s="89" t="n">
-        <v>169187</v>
+        <v>185035</v>
       </c>
       <c r="BT19" s="90" t="n">
         <v>0</v>
       </c>
       <c r="BU19" s="91" t="n">
-        <v>169187</v>
+        <v>185035</v>
       </c>
       <c r="BV19" s="92" t="n">
-        <v>52165920</v>
+        <v>52181768</v>
       </c>
       <c r="BW19" s="92" t="n">
-        <v>52165920</v>
+        <v>52181768</v>
       </c>
       <c r="BX19" s="92" t="n">
         <v>0</v>
@@ -11526,25 +11838,25 @@
         <v>8645</v>
       </c>
       <c r="BQ23" s="90" t="n">
-        <v>2761</v>
+        <v>12069</v>
       </c>
       <c r="BR23" s="91" t="n">
-        <v>5884</v>
+        <v>-3424</v>
       </c>
       <c r="BS23" s="89" t="n">
-        <v>0</v>
+        <v>15133</v>
       </c>
       <c r="BT23" s="90" t="n">
-        <v>0</v>
+        <v>5825</v>
       </c>
       <c r="BU23" s="91" t="n">
-        <v>0</v>
+        <v>9308</v>
       </c>
       <c r="BV23" s="92" t="n">
-        <v>8645</v>
+        <v>23778</v>
       </c>
       <c r="BW23" s="92" t="n">
-        <v>8645</v>
+        <v>23778</v>
       </c>
       <c r="BX23" s="92" t="n">
         <v>0</v>
@@ -16097,16 +16409,16 @@
         </is>
       </c>
       <c r="B15" s="36" t="n">
-        <v>8688787685.560968</v>
+        <v>8690975370.060968</v>
       </c>
       <c r="C15" s="36" t="n">
         <v>9767838169.155153</v>
       </c>
       <c r="D15" s="100" t="n">
-        <v>-1079050483.594185</v>
+        <v>-1076862799.094185</v>
       </c>
       <c r="E15" s="98" t="n">
-        <v>1.124188842292389</v>
+        <v>1.123905862488554</v>
       </c>
       <c r="F15" s="99" t="inlineStr">
         <is>
@@ -16121,16 +16433,16 @@
         </is>
       </c>
       <c r="B16" s="36" t="n">
-        <v>19260224654.57878</v>
+        <v>19468504724.54878</v>
       </c>
       <c r="C16" s="36" t="n">
         <v>11917212675.50339</v>
       </c>
       <c r="D16" s="97" t="n">
-        <v>7343011979.07539</v>
+        <v>7551292049.045391</v>
       </c>
       <c r="E16" s="98" t="n">
-        <v>0.6187473349471176</v>
+        <v>0.612127785061808</v>
       </c>
       <c r="F16" s="99" t="inlineStr">
         <is>
@@ -16145,16 +16457,16 @@
         </is>
       </c>
       <c r="B17" s="36" t="n">
-        <v>15237911125.3006</v>
+        <v>15288705125.3006</v>
       </c>
       <c r="C17" s="36" t="n">
-        <v>32567837201.06482</v>
+        <v>32829098955.53482</v>
       </c>
       <c r="D17" s="100" t="n">
-        <v>-17329926075.76422</v>
+        <v>-17540393830.23421</v>
       </c>
       <c r="E17" s="98" t="n">
-        <v>2.137290139918856</v>
+        <v>2.147277920954038</v>
       </c>
       <c r="F17" s="99" t="inlineStr">
         <is>
@@ -16241,7 +16553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1062"/>
+  <dimension ref="A1:Q1071"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -83221,21 +83533,29 @@
       </c>
       <c r="B1059" s="103" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C1059" s="103" t="n"/>
-      <c r="D1059" s="103" t="n"/>
-      <c r="E1059" s="103" t="n"/>
+          <t>PT East West Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1059" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.EWINDO_LMB/12/2026</t>
+        </is>
+      </c>
+      <c r="D1059" s="104" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E1059" s="104" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1059" s="103" t="n"/>
       <c r="G1059" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1059" s="103" t="inlineStr">
         <is>
-          <t>FIELD CORN</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1059" s="103" t="inlineStr">
@@ -83245,22 +83565,28 @@
       </c>
       <c r="J1059" s="103" t="n"/>
       <c r="K1059" s="104" t="n">
-        <v>46204</v>
+        <v>46214</v>
       </c>
       <c r="L1059" s="104" t="n">
-        <v>46234</v>
+        <v>46214</v>
       </c>
       <c r="M1059" s="105" t="n">
-        <v>1034082</v>
+        <v>92</v>
       </c>
       <c r="N1059" s="105" t="n">
-        <v>4206172069.8522</v>
-      </c>
-      <c r="O1059" s="103" t="n"/>
-      <c r="P1059" s="103" t="n"/>
+        <v>802240</v>
+      </c>
+      <c r="O1059" s="103" t="n">
+        <v>-44</v>
+      </c>
+      <c r="P1059" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1059" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -83272,21 +83598,29 @@
       </c>
       <c r="B1060" s="103" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C1060" s="103" t="n"/>
-      <c r="D1060" s="103" t="n"/>
-      <c r="E1060" s="103" t="n"/>
+          <t>PT East West Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1060" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.EWINDO_LMB/13/2026</t>
+        </is>
+      </c>
+      <c r="D1060" s="104" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E1060" s="104" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1060" s="103" t="n"/>
       <c r="G1060" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1060" s="103" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1060" s="103" t="inlineStr">
@@ -83296,22 +83630,28 @@
       </c>
       <c r="J1060" s="103" t="n"/>
       <c r="K1060" s="104" t="n">
-        <v>46204</v>
+        <v>46215</v>
       </c>
       <c r="L1060" s="104" t="n">
-        <v>46234</v>
+        <v>46215</v>
       </c>
       <c r="M1060" s="105" t="n">
-        <v>1816</v>
+        <v>990</v>
       </c>
       <c r="N1060" s="105" t="n">
-        <v>9231791.4496</v>
-      </c>
-      <c r="O1060" s="103" t="n"/>
-      <c r="P1060" s="103" t="n"/>
+        <v>8632800</v>
+      </c>
+      <c r="O1060" s="103" t="n">
+        <v>-44</v>
+      </c>
+      <c r="P1060" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1060" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -83323,21 +83663,29 @@
       </c>
       <c r="B1061" s="103" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C1061" s="103" t="n"/>
-      <c r="D1061" s="103" t="n"/>
-      <c r="E1061" s="103" t="n"/>
+          <t>PT East West Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1061" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.EWINDO_LMB/14/2026</t>
+        </is>
+      </c>
+      <c r="D1061" s="104" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E1061" s="104" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1061" s="103" t="n"/>
       <c r="G1061" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1061" s="103" t="inlineStr">
         <is>
-          <t>SWEET CORN</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1061" s="103" t="inlineStr">
@@ -83347,22 +83695,28 @@
       </c>
       <c r="J1061" s="103" t="n"/>
       <c r="K1061" s="104" t="n">
-        <v>46204</v>
+        <v>46219</v>
       </c>
       <c r="L1061" s="104" t="n">
-        <v>46234</v>
+        <v>46219</v>
       </c>
       <c r="M1061" s="105" t="n">
-        <v>18309</v>
+        <v>111</v>
       </c>
       <c r="N1061" s="105" t="n">
-        <v>156073086.756468</v>
-      </c>
-      <c r="O1061" s="103" t="n"/>
-      <c r="P1061" s="103" t="n"/>
+        <v>967920</v>
+      </c>
+      <c r="O1061" s="103" t="n">
+        <v>-44</v>
+      </c>
+      <c r="P1061" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1061" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -83374,51 +83728,608 @@
       </c>
       <c r="B1062" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1062" s="103" t="n"/>
-      <c r="D1062" s="103" t="n"/>
-      <c r="E1062" s="103" t="n"/>
+          <t>PT East West Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1062" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.EWINDO_LMB/15/2026</t>
+        </is>
+      </c>
+      <c r="D1062" s="104" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E1062" s="104" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1062" s="103" t="n"/>
       <c r="G1062" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1062" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1062" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="J1062" s="103" t="n"/>
       <c r="K1062" s="104" t="n">
+        <v>46228</v>
+      </c>
+      <c r="L1062" s="104" t="n">
+        <v>46228</v>
+      </c>
+      <c r="M1062" s="105" t="n">
+        <v>2352</v>
+      </c>
+      <c r="N1062" s="105" t="n">
+        <v>20509440</v>
+      </c>
+      <c r="O1062" s="103" t="n">
+        <v>-44</v>
+      </c>
+      <c r="P1062" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+      <c r="Q1062" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1063" s="103" t="inlineStr">
+        <is>
+          <t>PT East West Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1063" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.EWINDO_LMB/16/2026</t>
+        </is>
+      </c>
+      <c r="D1063" s="104" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E1063" s="104" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F1063" s="103" t="n"/>
+      <c r="G1063" s="103" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H1063" s="103" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="I1063" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1063" s="103" t="n"/>
+      <c r="K1063" s="104" t="n">
+        <v>46228</v>
+      </c>
+      <c r="L1063" s="104" t="n">
+        <v>46228</v>
+      </c>
+      <c r="M1063" s="105" t="n">
+        <v>250</v>
+      </c>
+      <c r="N1063" s="105" t="n">
+        <v>2180000</v>
+      </c>
+      <c r="O1063" s="103" t="n">
+        <v>-44</v>
+      </c>
+      <c r="P1063" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+      <c r="Q1063" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1064" s="103" t="inlineStr">
+        <is>
+          <t>PT East West Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1064" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.EWINDO_LMB/17/2026</t>
+        </is>
+      </c>
+      <c r="D1064" s="104" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E1064" s="104" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F1064" s="103" t="n"/>
+      <c r="G1064" s="103" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H1064" s="103" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="I1064" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1064" s="103" t="n"/>
+      <c r="K1064" s="104" t="n">
+        <v>46233</v>
+      </c>
+      <c r="L1064" s="104" t="n">
+        <v>46233</v>
+      </c>
+      <c r="M1064" s="105" t="n">
+        <v>62</v>
+      </c>
+      <c r="N1064" s="105" t="n">
+        <v>540640</v>
+      </c>
+      <c r="O1064" s="103" t="n">
+        <v>-44</v>
+      </c>
+      <c r="P1064" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+      <c r="Q1064" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1065" s="103" t="inlineStr">
+        <is>
+          <t>PT East West Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1065" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.EWINDO_LMB/18/2026</t>
+        </is>
+      </c>
+      <c r="D1065" s="104" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E1065" s="104" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F1065" s="103" t="n"/>
+      <c r="G1065" s="103" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H1065" s="103" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="I1065" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1065" s="103" t="n"/>
+      <c r="K1065" s="104" t="n">
+        <v>46233</v>
+      </c>
+      <c r="L1065" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1065" s="105" t="n">
+        <v>5451</v>
+      </c>
+      <c r="N1065" s="105" t="n">
+        <v>47532720</v>
+      </c>
+      <c r="O1065" s="103" t="n">
+        <v>-44</v>
+      </c>
+      <c r="P1065" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+      <c r="Q1065" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1066" s="103" t="inlineStr">
+        <is>
+          <t>PT East West Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1066" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.EWINDO_LMB/19/2026</t>
+        </is>
+      </c>
+      <c r="D1066" s="104" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E1066" s="104" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F1066" s="103" t="n"/>
+      <c r="G1066" s="103" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H1066" s="103" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="I1066" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1066" s="103" t="n"/>
+      <c r="K1066" s="104" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1066" s="104" t="n">
+        <v>46238</v>
+      </c>
+      <c r="M1066" s="105" t="n">
+        <v>5825</v>
+      </c>
+      <c r="N1066" s="105" t="n">
+        <v>50794000</v>
+      </c>
+      <c r="O1066" s="103" t="n">
+        <v>-44</v>
+      </c>
+      <c r="P1066" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+      <c r="Q1066" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1067" s="103" t="inlineStr">
+        <is>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C1067" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.ASI/SC/64/2026 </t>
+        </is>
+      </c>
+      <c r="D1067" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1067" s="104" t="n">
+        <v>46284</v>
+      </c>
+      <c r="F1067" s="103" t="n"/>
+      <c r="G1067" s="103" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H1067" s="103" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="I1067" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1067" s="103" t="n"/>
+      <c r="K1067" s="104" t="n">
+        <v>46223</v>
+      </c>
+      <c r="L1067" s="104" t="n">
+        <v>46230</v>
+      </c>
+      <c r="M1067" s="105" t="n">
+        <v>15163</v>
+      </c>
+      <c r="N1067" s="105" t="n">
+        <v>127114309.97</v>
+      </c>
+      <c r="O1067" s="103" t="n">
+        <v>-23</v>
+      </c>
+      <c r="P1067" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+      <c r="Q1067" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1068" s="103" t="inlineStr">
+        <is>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C1068" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT.PSI/PT.ASI/SC/65/2026 </t>
+        </is>
+      </c>
+      <c r="D1068" s="104" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E1068" s="104" t="n">
+        <v>46284</v>
+      </c>
+      <c r="F1068" s="103" t="n"/>
+      <c r="G1068" s="103" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H1068" s="103" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="I1068" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1068" s="103" t="n"/>
+      <c r="K1068" s="104" t="n">
+        <v>46193</v>
+      </c>
+      <c r="L1068" s="104" t="n">
+        <v>46193</v>
+      </c>
+      <c r="M1068" s="105" t="n">
+        <v>685</v>
+      </c>
+      <c r="N1068" s="105" t="n">
+        <v>2187684.5</v>
+      </c>
+      <c r="O1068" s="103" t="n">
+        <v>-23</v>
+      </c>
+      <c r="P1068" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+      <c r="Q1068" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1069" s="103" t="inlineStr">
+        <is>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C1069" s="103" t="n"/>
+      <c r="D1069" s="103" t="n"/>
+      <c r="E1069" s="103" t="n"/>
+      <c r="F1069" s="103" t="n"/>
+      <c r="G1069" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1069" s="103" t="inlineStr">
+        <is>
+          <t>FIELD CORN</t>
+        </is>
+      </c>
+      <c r="I1069" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1069" s="103" t="n"/>
+      <c r="K1069" s="104" t="n">
         <v>46204</v>
       </c>
-      <c r="L1062" s="104" t="n">
+      <c r="L1069" s="104" t="n">
         <v>46234</v>
       </c>
-      <c r="M1062" s="105" t="n">
+      <c r="M1069" s="105" t="n">
+        <v>1034082</v>
+      </c>
+      <c r="N1069" s="105" t="n">
+        <v>4206172069.8522</v>
+      </c>
+      <c r="O1069" s="103" t="n"/>
+      <c r="P1069" s="103" t="n"/>
+      <c r="Q1069" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1070" s="103" t="inlineStr">
+        <is>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C1070" s="103" t="n"/>
+      <c r="D1070" s="103" t="n"/>
+      <c r="E1070" s="103" t="n"/>
+      <c r="F1070" s="103" t="n"/>
+      <c r="G1070" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1070" s="103" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="I1070" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1070" s="103" t="n"/>
+      <c r="K1070" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1070" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1070" s="105" t="n">
+        <v>1816</v>
+      </c>
+      <c r="N1070" s="105" t="n">
+        <v>9231791.4496</v>
+      </c>
+      <c r="O1070" s="103" t="n"/>
+      <c r="P1070" s="103" t="n"/>
+      <c r="Q1070" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1071" s="103" t="inlineStr">
+        <is>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C1071" s="103" t="n"/>
+      <c r="D1071" s="103" t="n"/>
+      <c r="E1071" s="103" t="n"/>
+      <c r="F1071" s="103" t="n"/>
+      <c r="G1071" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1071" s="103" t="inlineStr">
+        <is>
+          <t>RENTAL CS</t>
+        </is>
+      </c>
+      <c r="I1071" s="103" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1071" s="103" t="n"/>
+      <c r="K1071" s="104" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L1071" s="104" t="n">
+        <v>46234</v>
+      </c>
+      <c r="M1071" s="105" t="n">
         <v>1654962.70767742</v>
       </c>
-      <c r="N1062" s="105" t="n">
+      <c r="N1071" s="105" t="n">
         <v>593353779.5835853</v>
       </c>
-      <c r="O1062" s="103" t="n"/>
-      <c r="P1062" s="103" t="n"/>
-      <c r="Q1062" s="103" t="inlineStr">
+      <c r="O1071" s="103" t="n"/>
+      <c r="P1071" s="103" t="n"/>
+      <c r="Q1071" s="103" t="inlineStr">
         <is>
           <t>0-30</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q1062"/>
+  <autoFilter ref="A1:Q1071"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto-deploy AR dashboard 2026-09-07 12:00
</commit_message>
<xml_diff>
--- a/AR Movement Report.xlsx
+++ b/AR Movement Report.xlsx
@@ -1346,7 +1346,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data as of Monday, 07 September 2026 - 10:55  |  Source: PSI AR Monitoring Master.xlsx</t>
+          <t>Data as of Monday, 07 September 2026 - 12:00  |  Source: PSI AR Monitoring Master.xlsx</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="9" t="n">
-        <v>128143925430.9986</v>
+        <v>128297857570.7547</v>
       </c>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="10" t="n"/>
@@ -1394,7 +1394,7 @@
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="11" t="n"/>
       <c r="H7" s="13" t="n">
-        <v>12732624513.64691</v>
+        <v>12886556653.40296</v>
       </c>
       <c r="I7" s="10" t="n"/>
       <c r="J7" s="11" t="n"/>
@@ -1440,7 +1440,7 @@
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="19" t="n">
-        <v>56020856682.52223</v>
+        <v>56174788822.27828</v>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="10" t="n"/>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="26" t="n">
-        <v>8302741469.802128</v>
+        <v>8456673609.558172</v>
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="27" t="n">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="D17" s="11" t="n"/>
       <c r="E17" s="28" t="n">
-        <v>172894573690.6945</v>
+        <v>173282145580.1879</v>
       </c>
       <c r="F17" s="11" t="n"/>
       <c r="G17" s="29" t="n">
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="B25" s="34" t="n">
-        <v>7699431425.389547</v>
+        <v>7853363565.145592</v>
       </c>
       <c r="C25" s="35" t="n">
         <v>23694713679.40245</v>
@@ -2029,7 +2029,7 @@
         <v>48622009868.2589</v>
       </c>
       <c r="C41" s="49" t="n">
-        <v>7398846814.263327</v>
+        <v>7552778954.01937</v>
       </c>
       <c r="D41" s="50">
         <f>SUM(B41:C41)</f>
@@ -2675,7 +2675,7 @@
         <v>0</v>
       </c>
       <c r="D65" s="36" t="n">
-        <v>410081223.1833281</v>
+        <v>564013362.9393721</v>
       </c>
       <c r="E65" s="36" t="n">
         <v>0</v>
@@ -3333,7 +3333,7 @@
         <v>6114276610.20622</v>
       </c>
       <c r="D11" s="36" t="n">
-        <v>1585154815.183328</v>
+        <v>1739086954.939372</v>
       </c>
       <c r="E11" s="36" t="n">
         <v>0</v>
@@ -6927,7 +6927,7 @@
         </is>
       </c>
       <c r="E107" s="77" t="n">
-        <v>387571889.4933281</v>
+        <v>541504029.249372</v>
       </c>
       <c r="F107" s="75" t="n">
         <v>46298</v>
@@ -13771,19 +13771,19 @@
         <v>669012817.1507928</v>
       </c>
       <c r="BK32" s="86" t="n">
-        <v>1175073592</v>
+        <v>1562645481.493328</v>
       </c>
       <c r="BL32" s="36" t="n">
-        <v>-506060774.8492072</v>
+        <v>-893632664.3425353</v>
       </c>
       <c r="BM32" s="85" t="n">
-        <v>1175073592</v>
+        <v>1562645481.493328</v>
       </c>
       <c r="BN32" s="86" t="n">
-        <v>1562645481.493328</v>
+        <v>1716577621.249372</v>
       </c>
       <c r="BO32" s="36" t="n">
-        <v>-387571889.4933281</v>
+        <v>-153932139.7560439</v>
       </c>
       <c r="BP32" s="85" t="n">
         <v>2350147184</v>
@@ -13795,22 +13795,22 @@
         <v>1152564258.31</v>
       </c>
       <c r="BS32" s="85" t="n">
-        <v>410081223.1833281</v>
+        <v>564013362.9393721</v>
       </c>
       <c r="BT32" s="86" t="n">
         <v>0</v>
       </c>
       <c r="BU32" s="36" t="n">
-        <v>410081223.1833281</v>
+        <v>564013362.9393721</v>
       </c>
       <c r="BV32" s="40" t="n">
-        <v>26847855610.63563</v>
+        <v>27389359639.88501</v>
       </c>
       <c r="BW32" s="40" t="n">
-        <v>26847855610.63563</v>
+        <v>27389359639.885</v>
       </c>
       <c r="BX32" s="40" t="n">
-        <v>0</v>
+        <v>3.814697265625e-06</v>
       </c>
     </row>
     <row r="33">
@@ -15573,19 +15573,19 @@
         <v>1979149.878406686</v>
       </c>
       <c r="BK41" s="90" t="n">
-        <v>7000</v>
+        <v>1193489.84</v>
       </c>
       <c r="BL41" s="91" t="n">
-        <v>1972149.878406686</v>
+        <v>785660.0384066855</v>
       </c>
       <c r="BM41" s="89" t="n">
-        <v>7000</v>
+        <v>1193489.84</v>
       </c>
       <c r="BN41" s="90" t="n">
-        <v>1193489.84</v>
+        <v>1664728.66</v>
       </c>
       <c r="BO41" s="91" t="n">
-        <v>-1186489.84</v>
+        <v>-471238.8199999998</v>
       </c>
       <c r="BP41" s="89" t="n">
         <v>14000</v>
@@ -15597,19 +15597,19 @@
         <v>6997</v>
       </c>
       <c r="BS41" s="89" t="n">
-        <v>1186492.84</v>
+        <v>1657731.66</v>
       </c>
       <c r="BT41" s="90" t="n">
         <v>0</v>
       </c>
       <c r="BU41" s="91" t="n">
-        <v>1186492.84</v>
+        <v>1657731.66</v>
       </c>
       <c r="BV41" s="92" t="n">
-        <v>165075186.6213745</v>
+        <v>166732915.2813745</v>
       </c>
       <c r="BW41" s="92" t="n">
-        <v>165075186.6213745</v>
+        <v>166732915.2813745</v>
       </c>
       <c r="BX41" s="92" t="n">
         <v>2.980232238769531e-08</v>
@@ -16534,20 +16534,20 @@
         </is>
       </c>
       <c r="B14" s="36" t="n">
-        <v>8690975370.060968</v>
+        <v>9078547259.554296</v>
       </c>
       <c r="C14" s="36" t="n">
         <v>9767838169.155153</v>
       </c>
       <c r="D14" s="100" t="n">
-        <v>-1076862799.094185</v>
+        <v>-689290909.6008568</v>
       </c>
       <c r="E14" s="98" t="n">
-        <v>1.123905862488554</v>
+        <v>1.075925243311968</v>
       </c>
       <c r="F14" s="99" t="inlineStr">
         <is>
-          <t>Catch-up: prior-month invoices issued</t>
+          <t>On track</t>
         </is>
       </c>
     </row>
@@ -16558,16 +16558,16 @@
         </is>
       </c>
       <c r="B15" s="36" t="n">
-        <v>22985075607.06211</v>
+        <v>23139007746.81815</v>
       </c>
       <c r="C15" s="36" t="n">
-        <v>11917212675.50339</v>
+        <v>12304784564.99672</v>
       </c>
       <c r="D15" s="97" t="n">
-        <v>11067862931.55872</v>
+        <v>10834223181.82143</v>
       </c>
       <c r="E15" s="98" t="n">
-        <v>0.5184761137719232</v>
+        <v>0.5317766733834449</v>
       </c>
       <c r="F15" s="99" t="inlineStr">
         <is>
@@ -16609,10 +16609,10 @@
         <v>0</v>
       </c>
       <c r="C17" s="36" t="n">
-        <v>8302741469.802128</v>
+        <v>8456673609.558172</v>
       </c>
       <c r="D17" s="100" t="n">
-        <v>-8302741469.802128</v>
+        <v>-8456673609.558172</v>
       </c>
       <c r="E17" s="98" t="n">
         <v>0</v>
@@ -76214,7 +76214,7 @@
       </c>
       <c r="C942" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/08/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL COLD STORAGE_ PAS/10/2026</t>
         </is>
       </c>
       <c r="D942" s="104" t="n">
@@ -76249,15 +76249,15 @@
         <v>46203</v>
       </c>
       <c r="M942" s="105" t="n">
-        <v>5200</v>
+        <v>1186489.84</v>
       </c>
       <c r="N942" s="105" t="n">
-        <v>872911811.2</v>
+        <v>387571889.4933281</v>
       </c>
       <c r="O942" s="103" t="n"/>
       <c r="P942" s="103" t="inlineStr">
         <is>
-          <t>NOT YET DUE</t>
+          <t>PAID</t>
         </is>
       </c>
       <c r="Q942" s="103" t="n"/>
@@ -76270,24 +76270,26 @@
       </c>
       <c r="B943" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C943" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/29/2026 </t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/08/2026</t>
         </is>
       </c>
       <c r="D943" s="104" t="n">
         <v>46213</v>
       </c>
       <c r="E943" s="104" t="n">
-        <v>46273</v>
-      </c>
-      <c r="F943" s="103" t="n"/>
+        <v>46243</v>
+      </c>
+      <c r="F943" s="104" t="n">
+        <v>46241</v>
+      </c>
       <c r="G943" s="103" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H943" s="103" t="inlineStr">
@@ -76300,11 +76302,7 @@
           <t>Rental</t>
         </is>
       </c>
-      <c r="J943" s="103" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
+      <c r="J943" s="103" t="n"/>
       <c r="K943" s="104" t="n">
         <v>46174</v>
       </c>
@@ -76312,24 +76310,18 @@
         <v>46203</v>
       </c>
       <c r="M943" s="105" t="n">
-        <v>4000000</v>
+        <v>5200</v>
       </c>
       <c r="N943" s="105" t="n">
-        <v>1365520000</v>
-      </c>
-      <c r="O943" s="103" t="n">
-        <v>-1</v>
-      </c>
+        <v>872911811.2</v>
+      </c>
+      <c r="O943" s="103" t="n"/>
       <c r="P943" s="103" t="inlineStr">
         <is>
           <t>NOT YET DUE</t>
         </is>
       </c>
-      <c r="Q943" s="103" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
+      <c r="Q943" s="103" t="n"/>
     </row>
     <row r="944">
       <c r="A944" s="103" t="inlineStr">
@@ -76344,7 +76336,7 @@
       </c>
       <c r="C944" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/30/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/29/2026 </t>
         </is>
       </c>
       <c r="D944" s="104" t="n">
@@ -76369,7 +76361,11 @@
           <t>Rental</t>
         </is>
       </c>
-      <c r="J944" s="103" t="n"/>
+      <c r="J944" s="103" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
       <c r="K944" s="104" t="n">
         <v>46174</v>
       </c>
@@ -76377,10 +76373,10 @@
         <v>46203</v>
       </c>
       <c r="M944" s="105" t="n">
-        <v>4177832</v>
+        <v>4000000</v>
       </c>
       <c r="N944" s="105" t="n">
-        <v>1071584346</v>
+        <v>1365520000</v>
       </c>
       <c r="O944" s="103" t="n">
         <v>-1</v>
@@ -76409,7 +76405,7 @@
       </c>
       <c r="C945" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/31/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/30/2026</t>
         </is>
       </c>
       <c r="D945" s="104" t="n">
@@ -76426,7 +76422,7 @@
       </c>
       <c r="H945" s="103" t="inlineStr">
         <is>
-          <t>Rental WH</t>
+          <t>Rental CS</t>
         </is>
       </c>
       <c r="I945" s="103" t="inlineStr">
@@ -76434,11 +76430,7 @@
           <t>Rental</t>
         </is>
       </c>
-      <c r="J945" s="103" t="inlineStr">
-        <is>
-          <t>zero material</t>
-        </is>
-      </c>
+      <c r="J945" s="103" t="n"/>
       <c r="K945" s="104" t="n">
         <v>46174</v>
       </c>
@@ -76446,10 +76438,10 @@
         <v>46203</v>
       </c>
       <c r="M945" s="105" t="n">
-        <v>3600000</v>
+        <v>4177832</v>
       </c>
       <c r="N945" s="105" t="n">
-        <v>272700000</v>
+        <v>1071584346</v>
       </c>
       <c r="O945" s="103" t="n">
         <v>-1</v>
@@ -76478,7 +76470,7 @@
       </c>
       <c r="C946" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/32/2026 </t>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/31/2026</t>
         </is>
       </c>
       <c r="D946" s="104" t="n">
@@ -76495,7 +76487,7 @@
       </c>
       <c r="H946" s="103" t="inlineStr">
         <is>
-          <t>Rental CS</t>
+          <t>Rental WH</t>
         </is>
       </c>
       <c r="I946" s="103" t="inlineStr">
@@ -76505,7 +76497,7 @@
       </c>
       <c r="J946" s="103" t="inlineStr">
         <is>
-          <t>Handling</t>
+          <t>zero material</t>
         </is>
       </c>
       <c r="K946" s="104" t="n">
@@ -76515,10 +76507,10 @@
         <v>46203</v>
       </c>
       <c r="M946" s="105" t="n">
-        <v>607742</v>
+        <v>3600000</v>
       </c>
       <c r="N946" s="105" t="n">
-        <v>25780415.64</v>
+        <v>272700000</v>
       </c>
       <c r="O946" s="103" t="n">
         <v>-1</v>
@@ -76542,58 +76534,66 @@
       </c>
       <c r="B947" s="103" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C947" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/27/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/32/2026 </t>
         </is>
       </c>
       <c r="D947" s="104" t="n">
-        <v>46217</v>
+        <v>46213</v>
       </c>
       <c r="E947" s="104" t="n">
-        <v>46262</v>
-      </c>
-      <c r="F947" s="104" t="n">
-        <v>46247</v>
-      </c>
+        <v>46273</v>
+      </c>
+      <c r="F947" s="103" t="n"/>
       <c r="G947" s="103" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H947" s="103" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Rental CS</t>
         </is>
       </c>
       <c r="I947" s="103" t="inlineStr">
         <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="J947" s="103" t="n"/>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J947" s="103" t="inlineStr">
+        <is>
+          <t>Handling</t>
+        </is>
+      </c>
       <c r="K947" s="104" t="n">
-        <v>46178</v>
+        <v>46174</v>
       </c>
       <c r="L947" s="104" t="n">
-        <v>46178</v>
+        <v>46203</v>
       </c>
       <c r="M947" s="105" t="n">
-        <v>120</v>
+        <v>607742</v>
       </c>
       <c r="N947" s="105" t="n">
-        <v>289068</v>
-      </c>
-      <c r="O947" s="103" t="n"/>
+        <v>25780415.64</v>
+      </c>
+      <c r="O947" s="103" t="n">
+        <v>-1</v>
+      </c>
       <c r="P947" s="103" t="inlineStr">
         <is>
           <t>NOT YET DUE</t>
         </is>
       </c>
-      <c r="Q947" s="103" t="n"/>
+      <c r="Q947" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
     </row>
     <row r="948">
       <c r="A948" s="103" t="inlineStr">
@@ -76608,7 +76608,7 @@
       </c>
       <c r="C948" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/28/2026</t>
+          <t>PT.PSI/PT.BI/FC/27/2026</t>
         </is>
       </c>
       <c r="D948" s="104" t="n">
@@ -76637,16 +76637,16 @@
       </c>
       <c r="J948" s="103" t="n"/>
       <c r="K948" s="104" t="n">
-        <v>46171</v>
+        <v>46178</v>
       </c>
       <c r="L948" s="104" t="n">
-        <v>46171</v>
+        <v>46178</v>
       </c>
       <c r="M948" s="105" t="n">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="N948" s="105" t="n">
-        <v>269796.8</v>
+        <v>289068</v>
       </c>
       <c r="O948" s="103" t="n"/>
       <c r="P948" s="103" t="inlineStr">
@@ -76669,7 +76669,7 @@
       </c>
       <c r="C949" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/29/2026</t>
+          <t>PT.PSI/PT.BI/FC/28/2026</t>
         </is>
       </c>
       <c r="D949" s="104" t="n">
@@ -76730,7 +76730,7 @@
       </c>
       <c r="C950" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/30/2026</t>
+          <t>PT.PSI/PT.BI/FC/29/2026</t>
         </is>
       </c>
       <c r="D950" s="104" t="n">
@@ -76791,7 +76791,7 @@
       </c>
       <c r="C951" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/31/2026</t>
+          <t>PT.PSI/PT.BI/FC/30/2026</t>
         </is>
       </c>
       <c r="D951" s="104" t="n">
@@ -76852,14 +76852,14 @@
       </c>
       <c r="C952" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/32/2026</t>
+          <t>PT.PSI/PT.BI/FC/31/2026</t>
         </is>
       </c>
       <c r="D952" s="104" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="E952" s="104" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="F952" s="104" t="n">
         <v>46247</v>
@@ -76881,16 +76881,16 @@
       </c>
       <c r="J952" s="103" t="n"/>
       <c r="K952" s="104" t="n">
-        <v>46184</v>
+        <v>46171</v>
       </c>
       <c r="L952" s="104" t="n">
-        <v>46184</v>
+        <v>46171</v>
       </c>
       <c r="M952" s="105" t="n">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="N952" s="105" t="n">
-        <v>180667.5</v>
+        <v>269796.8</v>
       </c>
       <c r="O952" s="103" t="n"/>
       <c r="P952" s="103" t="inlineStr">
@@ -76913,7 +76913,7 @@
       </c>
       <c r="C953" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/33/2026</t>
+          <t>PT.PSI/PT.BI/FC/32/2026</t>
         </is>
       </c>
       <c r="D953" s="104" t="n">
@@ -76974,7 +76974,7 @@
       </c>
       <c r="C954" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/34/2026</t>
+          <t>PT.PSI/PT.BI/FC/33/2026</t>
         </is>
       </c>
       <c r="D954" s="104" t="n">
@@ -77035,7 +77035,7 @@
       </c>
       <c r="C955" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/35/2026</t>
+          <t>PT.PSI/PT.BI/FC/34/2026</t>
         </is>
       </c>
       <c r="D955" s="104" t="n">
@@ -77064,16 +77064,16 @@
       </c>
       <c r="J955" s="103" t="n"/>
       <c r="K955" s="104" t="n">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="L955" s="104" t="n">
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="M955" s="105" t="n">
-        <v>500</v>
+        <v>75</v>
       </c>
       <c r="N955" s="105" t="n">
-        <v>790795</v>
+        <v>180667.5</v>
       </c>
       <c r="O955" s="103" t="n"/>
       <c r="P955" s="103" t="inlineStr">
@@ -77096,7 +77096,7 @@
       </c>
       <c r="C956" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/36/2026</t>
+          <t>PT.PSI/PT.BI/FC/35/2026</t>
         </is>
       </c>
       <c r="D956" s="104" t="n">
@@ -77131,10 +77131,10 @@
         <v>46182</v>
       </c>
       <c r="M956" s="105" t="n">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="N956" s="105" t="n">
-        <v>237238.5</v>
+        <v>790795</v>
       </c>
       <c r="O956" s="103" t="n"/>
       <c r="P956" s="103" t="inlineStr">
@@ -77157,7 +77157,7 @@
       </c>
       <c r="C957" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/37/2026</t>
+          <t>PT.PSI/PT.BI/FC/36/2026</t>
         </is>
       </c>
       <c r="D957" s="104" t="n">
@@ -77186,16 +77186,16 @@
       </c>
       <c r="J957" s="103" t="n"/>
       <c r="K957" s="104" t="n">
-        <v>46197</v>
+        <v>46182</v>
       </c>
       <c r="L957" s="104" t="n">
-        <v>46198</v>
+        <v>46182</v>
       </c>
       <c r="M957" s="105" t="n">
-        <v>36550</v>
+        <v>150</v>
       </c>
       <c r="N957" s="105" t="n">
-        <v>88045295</v>
+        <v>237238.5</v>
       </c>
       <c r="O957" s="103" t="n"/>
       <c r="P957" s="103" t="inlineStr">
@@ -77218,7 +77218,7 @@
       </c>
       <c r="C958" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/38/2026</t>
+          <t>PT.PSI/PT.BI/FC/37/2026</t>
         </is>
       </c>
       <c r="D958" s="104" t="n">
@@ -77247,16 +77247,16 @@
       </c>
       <c r="J958" s="103" t="n"/>
       <c r="K958" s="104" t="n">
-        <v>46203</v>
+        <v>46197</v>
       </c>
       <c r="L958" s="104" t="n">
-        <v>46203</v>
+        <v>46198</v>
       </c>
       <c r="M958" s="105" t="n">
-        <v>10475</v>
+        <v>36550</v>
       </c>
       <c r="N958" s="105" t="n">
-        <v>25233227.5</v>
+        <v>88045295</v>
       </c>
       <c r="O958" s="103" t="n"/>
       <c r="P958" s="103" t="inlineStr">
@@ -77279,7 +77279,7 @@
       </c>
       <c r="C959" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/39/2026</t>
+          <t>PT.PSI/PT.BI/FC/38/2026</t>
         </is>
       </c>
       <c r="D959" s="104" t="n">
@@ -77308,16 +77308,16 @@
       </c>
       <c r="J959" s="103" t="n"/>
       <c r="K959" s="104" t="n">
-        <v>46199</v>
+        <v>46203</v>
       </c>
       <c r="L959" s="104" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="M959" s="105" t="n">
-        <v>24519</v>
+        <v>10475</v>
       </c>
       <c r="N959" s="105" t="n">
-        <v>59063819.1</v>
+        <v>25233227.5</v>
       </c>
       <c r="O959" s="103" t="n"/>
       <c r="P959" s="103" t="inlineStr">
@@ -77340,7 +77340,7 @@
       </c>
       <c r="C960" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/40/2026</t>
+          <t>PT.PSI/PT.BI/FC/39/2026</t>
         </is>
       </c>
       <c r="D960" s="104" t="n">
@@ -77369,16 +77369,16 @@
       </c>
       <c r="J960" s="103" t="n"/>
       <c r="K960" s="104" t="n">
-        <v>46203</v>
+        <v>46199</v>
       </c>
       <c r="L960" s="104" t="n">
-        <v>46203</v>
+        <v>46200</v>
       </c>
       <c r="M960" s="105" t="n">
-        <v>1058</v>
+        <v>24519</v>
       </c>
       <c r="N960" s="105" t="n">
-        <v>2548616.2</v>
+        <v>59063819.1</v>
       </c>
       <c r="O960" s="103" t="n"/>
       <c r="P960" s="103" t="inlineStr">
@@ -77401,7 +77401,7 @@
       </c>
       <c r="C961" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/41/2026</t>
+          <t>PT.PSI/PT.BI/FC/40/2026</t>
         </is>
       </c>
       <c r="D961" s="104" t="n">
@@ -77462,7 +77462,7 @@
       </c>
       <c r="C962" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/42/2026</t>
+          <t>PT.PSI/PT.BI/FC/41/2026</t>
         </is>
       </c>
       <c r="D962" s="104" t="n">
@@ -77472,7 +77472,7 @@
         <v>46261</v>
       </c>
       <c r="F962" s="104" t="n">
-        <v>46253</v>
+        <v>46247</v>
       </c>
       <c r="G962" s="103" t="inlineStr">
         <is>
@@ -77491,16 +77491,16 @@
       </c>
       <c r="J962" s="103" t="n"/>
       <c r="K962" s="104" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="L962" s="104" t="n">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="M962" s="105" t="n">
-        <v>135</v>
+        <v>1058</v>
       </c>
       <c r="N962" s="105" t="n">
-        <v>213514.65</v>
+        <v>2548616.2</v>
       </c>
       <c r="O962" s="103" t="n"/>
       <c r="P962" s="103" t="inlineStr">
@@ -77518,24 +77518,26 @@
       </c>
       <c r="B963" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C963" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/30/2026</t>
+          <t>PT.PSI/PT.BI/FC/42/2026</t>
         </is>
       </c>
       <c r="D963" s="104" t="n">
         <v>46216</v>
       </c>
       <c r="E963" s="104" t="n">
-        <v>46276</v>
-      </c>
-      <c r="F963" s="103" t="n"/>
+        <v>46261</v>
+      </c>
+      <c r="F963" s="104" t="n">
+        <v>46253</v>
+      </c>
       <c r="G963" s="103" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H963" s="103" t="inlineStr">
@@ -77550,30 +77552,24 @@
       </c>
       <c r="J963" s="103" t="n"/>
       <c r="K963" s="104" t="n">
-        <v>46197</v>
+        <v>46202</v>
       </c>
       <c r="L963" s="104" t="n">
-        <v>46203</v>
+        <v>46202</v>
       </c>
       <c r="M963" s="105" t="n">
-        <v>37939</v>
+        <v>135</v>
       </c>
       <c r="N963" s="105" t="n">
-        <v>536105249.4995999</v>
-      </c>
-      <c r="O963" s="103" t="n">
-        <v>-4</v>
-      </c>
+        <v>213514.65</v>
+      </c>
+      <c r="O963" s="103" t="n"/>
       <c r="P963" s="103" t="inlineStr">
         <is>
           <t>NOT YET DUE</t>
         </is>
       </c>
-      <c r="Q963" s="103" t="inlineStr">
-        <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
+      <c r="Q963" s="103" t="n"/>
     </row>
     <row r="964">
       <c r="A964" s="103" t="inlineStr">
@@ -77588,7 +77584,7 @@
       </c>
       <c r="C964" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/31/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/30/2026</t>
         </is>
       </c>
       <c r="D964" s="104" t="n">
@@ -77615,16 +77611,16 @@
       </c>
       <c r="J964" s="103" t="n"/>
       <c r="K964" s="104" t="n">
-        <v>46200</v>
+        <v>46197</v>
       </c>
       <c r="L964" s="104" t="n">
         <v>46203</v>
       </c>
       <c r="M964" s="105" t="n">
-        <v>145420</v>
+        <v>37939</v>
       </c>
       <c r="N964" s="105" t="n">
-        <v>513650866.212</v>
+        <v>536105249.4995999</v>
       </c>
       <c r="O964" s="103" t="n">
         <v>-4</v>
@@ -77648,26 +77644,24 @@
       </c>
       <c r="B965" s="103" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C965" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/50/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-MLG/31/2026</t>
         </is>
       </c>
       <c r="D965" s="104" t="n">
-        <v>46217</v>
+        <v>46216</v>
       </c>
       <c r="E965" s="104" t="n">
-        <v>46247</v>
-      </c>
-      <c r="F965" s="104" t="n">
-        <v>46234</v>
-      </c>
+        <v>46276</v>
+      </c>
+      <c r="F965" s="103" t="n"/>
       <c r="G965" s="103" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H965" s="103" t="inlineStr">
@@ -77682,24 +77676,30 @@
       </c>
       <c r="J965" s="103" t="n"/>
       <c r="K965" s="104" t="n">
+        <v>46200</v>
+      </c>
+      <c r="L965" s="104" t="n">
         <v>46203</v>
       </c>
-      <c r="L965" s="104" t="n">
-        <v>46204</v>
-      </c>
       <c r="M965" s="105" t="n">
-        <v>78248</v>
+        <v>145420</v>
       </c>
       <c r="N965" s="105" t="n">
-        <v>318303474.2399999</v>
-      </c>
-      <c r="O965" s="103" t="n"/>
+        <v>513650866.212</v>
+      </c>
+      <c r="O965" s="103" t="n">
+        <v>-4</v>
+      </c>
       <c r="P965" s="103" t="inlineStr">
         <is>
           <t>NOT YET DUE</t>
         </is>
       </c>
-      <c r="Q965" s="103" t="n"/>
+      <c r="Q965" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
     </row>
     <row r="966">
       <c r="A966" s="103" t="inlineStr">
@@ -77714,7 +77714,7 @@
       </c>
       <c r="C966" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/51/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/50/2026 </t>
         </is>
       </c>
       <c r="D966" s="104" t="n">
@@ -77743,16 +77743,16 @@
       </c>
       <c r="J966" s="103" t="n"/>
       <c r="K966" s="104" t="n">
-        <v>46165</v>
+        <v>46203</v>
       </c>
       <c r="L966" s="104" t="n">
         <v>46204</v>
       </c>
       <c r="M966" s="105" t="n">
-        <v>217990</v>
+        <v>78248</v>
       </c>
       <c r="N966" s="105" t="n">
-        <v>345483631.4</v>
+        <v>318303474.2399999</v>
       </c>
       <c r="O966" s="103" t="n"/>
       <c r="P966" s="103" t="inlineStr">
@@ -77775,7 +77775,7 @@
       </c>
       <c r="C967" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/SC/52/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/51/2026 </t>
         </is>
       </c>
       <c r="D967" s="104" t="n">
@@ -77804,16 +77804,16 @@
       </c>
       <c r="J967" s="103" t="n"/>
       <c r="K967" s="104" t="n">
-        <v>46125</v>
+        <v>46165</v>
       </c>
       <c r="L967" s="104" t="n">
-        <v>46195</v>
+        <v>46204</v>
       </c>
       <c r="M967" s="105" t="n">
-        <v>15909</v>
+        <v>217990</v>
       </c>
       <c r="N967" s="105" t="n">
-        <v>51692954.61</v>
+        <v>345483631.4</v>
       </c>
       <c r="O967" s="103" t="n"/>
       <c r="P967" s="103" t="inlineStr">
@@ -77836,7 +77836,7 @@
       </c>
       <c r="C968" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/53/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/SC/52/2026 </t>
         </is>
       </c>
       <c r="D968" s="104" t="n">
@@ -77865,16 +77865,16 @@
       </c>
       <c r="J968" s="103" t="n"/>
       <c r="K968" s="104" t="n">
-        <v>46167</v>
+        <v>46125</v>
       </c>
       <c r="L968" s="104" t="n">
-        <v>46203</v>
+        <v>46195</v>
       </c>
       <c r="M968" s="105" t="n">
-        <v>492873</v>
+        <v>15909</v>
       </c>
       <c r="N968" s="105" t="n">
-        <v>521114622.9</v>
+        <v>51692954.61</v>
       </c>
       <c r="O968" s="103" t="n"/>
       <c r="P968" s="103" t="inlineStr">
@@ -77897,7 +77897,7 @@
       </c>
       <c r="C969" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/SC/54/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/53/2026 </t>
         </is>
       </c>
       <c r="D969" s="104" t="n">
@@ -77926,16 +77926,16 @@
       </c>
       <c r="J969" s="103" t="n"/>
       <c r="K969" s="104" t="n">
-        <v>46168</v>
+        <v>46167</v>
       </c>
       <c r="L969" s="104" t="n">
-        <v>46200</v>
+        <v>46203</v>
       </c>
       <c r="M969" s="105" t="n">
-        <v>13694</v>
+        <v>492873</v>
       </c>
       <c r="N969" s="105" t="n">
-        <v>30599243</v>
+        <v>521114622.9</v>
       </c>
       <c r="O969" s="103" t="n"/>
       <c r="P969" s="103" t="inlineStr">
@@ -77958,7 +77958,7 @@
       </c>
       <c r="C970" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/55/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/SC/54/2026 </t>
         </is>
       </c>
       <c r="D970" s="104" t="n">
@@ -77987,16 +77987,16 @@
       </c>
       <c r="J970" s="103" t="n"/>
       <c r="K970" s="104" t="n">
-        <v>46184</v>
+        <v>46168</v>
       </c>
       <c r="L970" s="104" t="n">
-        <v>46203</v>
+        <v>46200</v>
       </c>
       <c r="M970" s="105" t="n">
-        <v>87083</v>
+        <v>13694</v>
       </c>
       <c r="N970" s="105" t="n">
-        <v>46036427.95</v>
+        <v>30599243</v>
       </c>
       <c r="O970" s="103" t="n"/>
       <c r="P970" s="103" t="inlineStr">
@@ -78019,7 +78019,7 @@
       </c>
       <c r="C971" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/56/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/55/2026 </t>
         </is>
       </c>
       <c r="D971" s="104" t="n">
@@ -78048,16 +78048,16 @@
       </c>
       <c r="J971" s="103" t="n"/>
       <c r="K971" s="104" t="n">
-        <v>46192</v>
+        <v>46184</v>
       </c>
       <c r="L971" s="104" t="n">
-        <v>46199</v>
+        <v>46203</v>
       </c>
       <c r="M971" s="105" t="n">
-        <v>85411</v>
+        <v>87083</v>
       </c>
       <c r="N971" s="105" t="n">
-        <v>22064223.63</v>
+        <v>46036427.95</v>
       </c>
       <c r="O971" s="103" t="n"/>
       <c r="P971" s="103" t="inlineStr">
@@ -78075,62 +78075,58 @@
       </c>
       <c r="B972" s="103" t="inlineStr">
         <is>
-          <t>PT Alam Semesta Agro</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C972" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/Rental CS/07/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/56/2026 </t>
         </is>
       </c>
       <c r="D972" s="104" t="n">
         <v>46217</v>
       </c>
       <c r="E972" s="104" t="n">
-        <v>46248</v>
-      </c>
-      <c r="F972" s="103" t="n"/>
+        <v>46247</v>
+      </c>
+      <c r="F972" s="104" t="n">
+        <v>46234</v>
+      </c>
       <c r="G972" s="103" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H972" s="103" t="inlineStr">
         <is>
-          <t>Rental CS</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I972" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="J972" s="103" t="n"/>
       <c r="K972" s="104" t="n">
-        <v>46174</v>
+        <v>46192</v>
       </c>
       <c r="L972" s="104" t="n">
-        <v>46203</v>
+        <v>46199</v>
       </c>
       <c r="M972" s="105" t="n">
-        <v>510000</v>
+        <v>85411</v>
       </c>
       <c r="N972" s="105" t="n">
-        <v>206040000</v>
-      </c>
-      <c r="O972" s="103" t="n">
-        <v>24</v>
-      </c>
+        <v>22064223.63</v>
+      </c>
+      <c r="O972" s="103" t="n"/>
       <c r="P972" s="103" t="inlineStr">
         <is>
           <t>NOT YET DUE</t>
         </is>
       </c>
-      <c r="Q972" s="103" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
+      <c r="Q972" s="103" t="n"/>
     </row>
     <row r="973">
       <c r="A973" s="103" t="inlineStr">
@@ -78145,7 +78141,7 @@
       </c>
       <c r="C973" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/Rental CS/08/2026</t>
+          <t>PT.PSI/PT.ASI/Rental CS/07/2026</t>
         </is>
       </c>
       <c r="D973" s="104" t="n">
@@ -78178,10 +78174,10 @@
         <v>46203</v>
       </c>
       <c r="M973" s="105" t="n">
-        <v>168673</v>
+        <v>510000</v>
       </c>
       <c r="N973" s="105" t="n">
-        <v>3860924.97</v>
+        <v>206040000</v>
       </c>
       <c r="O973" s="103" t="n">
         <v>24</v>
@@ -78205,26 +78201,24 @@
       </c>
       <c r="B974" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Alam Semesta Agro</t>
         </is>
       </c>
       <c r="C974" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/09/2026</t>
+          <t>PT.PSI/PT.ASI/Rental CS/08/2026</t>
         </is>
       </c>
       <c r="D974" s="104" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="E974" s="104" t="n">
-        <v>46246</v>
-      </c>
-      <c r="F974" s="104" t="n">
-        <v>46241</v>
-      </c>
+        <v>46248</v>
+      </c>
+      <c r="F974" s="103" t="n"/>
       <c r="G974" s="103" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H974" s="103" t="inlineStr">
@@ -78245,18 +78239,24 @@
         <v>46203</v>
       </c>
       <c r="M974" s="105" t="n">
-        <v>1800</v>
+        <v>168673</v>
       </c>
       <c r="N974" s="105" t="n">
-        <v>302161780.8</v>
-      </c>
-      <c r="O974" s="103" t="n"/>
+        <v>3860924.97</v>
+      </c>
+      <c r="O974" s="103" t="n">
+        <v>24</v>
+      </c>
       <c r="P974" s="103" t="inlineStr">
         <is>
           <t>NOT YET DUE</t>
         </is>
       </c>
-      <c r="Q974" s="103" t="n"/>
+      <c r="Q974" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
     </row>
     <row r="975">
       <c r="A975" s="103" t="inlineStr">
@@ -78271,7 +78271,7 @@
       </c>
       <c r="C975" s="103" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL COLD STORAGE_ PAS/07/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/09/2026</t>
         </is>
       </c>
       <c r="D975" s="104" t="n">
@@ -78306,10 +78306,10 @@
         <v>46203</v>
       </c>
       <c r="M975" s="105" t="n">
-        <v>1186489.84</v>
+        <v>1800</v>
       </c>
       <c r="N975" s="105" t="n">
-        <v>387571889.4933281</v>
+        <v>302161780.8</v>
       </c>
       <c r="O975" s="103" t="n"/>
       <c r="P975" s="103" t="inlineStr">
@@ -84855,10 +84855,10 @@
         <v>46234</v>
       </c>
       <c r="M1078" s="105" t="n">
-        <v>1186489.84</v>
+        <v>1657728.66</v>
       </c>
       <c r="N1078" s="105" t="n">
-        <v>387571889.4933281</v>
+        <v>541504029.249372</v>
       </c>
       <c r="O1078" s="103" t="n">
         <v>-26</v>
@@ -85369,8 +85369,12 @@
         </is>
       </c>
       <c r="J1087" s="103" t="n"/>
-      <c r="K1087" s="103" t="n"/>
-      <c r="L1087" s="103" t="n"/>
+      <c r="K1087" s="104" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1087" s="104" t="n">
+        <v>46265</v>
+      </c>
       <c r="M1087" s="105" t="n">
         <v>972186.75</v>
       </c>
@@ -85467,8 +85471,12 @@
         </is>
       </c>
       <c r="J1089" s="103" t="n"/>
-      <c r="K1089" s="103" t="n"/>
-      <c r="L1089" s="103" t="n"/>
+      <c r="K1089" s="104" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1089" s="104" t="n">
+        <v>46265</v>
+      </c>
       <c r="M1089" s="105" t="n">
         <v>198569</v>
       </c>

</xml_diff>

<commit_message>
Auto-deploy AR dashboard 2026-09-10 10:05
</commit_message>
<xml_diff>
--- a/AR Movement Report.xlsx
+++ b/AR Movement Report.xlsx
@@ -1346,7 +1346,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data as of Thursday, 10 September 2026 - 09:51  |  Source: PSI AR Monitoring Master.xlsx</t>
+          <t>Data as of Thursday, 10 September 2026 - 10:05  |  Source: PSI AR Monitoring Master.xlsx</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="26" t="n">
-        <v>20815718109.45918</v>
+        <v>21228658137.03918</v>
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="27" t="n">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="D17" s="11" t="n"/>
       <c r="E17" s="28" t="n">
-        <v>176562423778.4995</v>
+        <v>173958157025.0544</v>
       </c>
       <c r="F17" s="11" t="n"/>
       <c r="G17" s="29" t="n">
@@ -8765,73 +8765,73 @@
         <v>10392322771.50451</v>
       </c>
       <c r="AJ8" s="86" t="n">
-        <v>10897102486.38739</v>
+        <v>10878208486.38739</v>
       </c>
       <c r="AK8" s="36" t="n">
-        <v>-504779714.8828831</v>
+        <v>-485885714.8828831</v>
       </c>
       <c r="AL8" s="85" t="n">
         <v>20300886772.72072</v>
       </c>
       <c r="AM8" s="86" t="n">
-        <v>19627060208.88288</v>
+        <v>19624708508.88288</v>
       </c>
       <c r="AN8" s="36" t="n">
-        <v>673826563.8378372</v>
+        <v>676178263.8378372</v>
       </c>
       <c r="AO8" s="85" t="n">
         <v>11727429.8018018</v>
       </c>
       <c r="AP8" s="86" t="n">
-        <v>60512974933.39641</v>
+        <v>58166768866.39641</v>
       </c>
       <c r="AQ8" s="36" t="n">
-        <v>-60501247503.5946</v>
+        <v>-58155041436.5946</v>
       </c>
       <c r="AR8" s="85" t="n">
-        <v>60570832135.36037</v>
+        <v>58051988188.36037</v>
       </c>
       <c r="AS8" s="86" t="n">
-        <v>5755510383.882882</v>
+        <v>4678451594.801802</v>
       </c>
       <c r="AT8" s="36" t="n">
-        <v>54815321751.47749</v>
+        <v>53373536593.55856</v>
       </c>
       <c r="AU8" s="85" t="n">
-        <v>7766643367.252254</v>
+        <v>6840958179.252254</v>
       </c>
       <c r="AV8" s="86" t="n">
-        <v>1862011022.772613</v>
+        <v>1827192737.813153</v>
       </c>
       <c r="AW8" s="36" t="n">
-        <v>5904632344.479641</v>
+        <v>5013765441.4391</v>
       </c>
       <c r="AX8" s="85" t="n">
         <v>330957527.8108109</v>
       </c>
       <c r="AY8" s="86" t="n">
-        <v>1566384709.990991</v>
+        <v>1314152775.95045</v>
       </c>
       <c r="AZ8" s="36" t="n">
-        <v>-1235427182.18018</v>
+        <v>-983195248.1396396</v>
       </c>
       <c r="BA8" s="85" t="n">
-        <v>1719092359.765766</v>
+        <v>1422127376.414414</v>
       </c>
       <c r="BB8" s="86" t="n">
-        <v>2710432239.517478</v>
+        <v>2472995552.967928</v>
       </c>
       <c r="BC8" s="36" t="n">
-        <v>-991339879.7517118</v>
+        <v>-1050868176.553514</v>
       </c>
       <c r="BD8" s="85" t="n">
-        <v>2530489748.441442</v>
+        <v>2290816052.441442</v>
       </c>
       <c r="BE8" s="86" t="n">
-        <v>271658880.6427027</v>
+        <v>269347434.8913513</v>
       </c>
       <c r="BF8" s="36" t="n">
-        <v>2258830867.798739</v>
+        <v>2021468617.55009</v>
       </c>
       <c r="BG8" s="85" t="n">
         <v>0</v>
@@ -8843,49 +8843,49 @@
         <v>-882085415.7499999</v>
       </c>
       <c r="BJ8" s="85" t="n">
-        <v>1274206673.07</v>
+        <v>1284065580.03937</v>
       </c>
       <c r="BK8" s="86" t="n">
-        <v>990203785.35</v>
+        <v>1301637724.25</v>
       </c>
       <c r="BL8" s="36" t="n">
-        <v>284002887.7199999</v>
+        <v>-17572144.21063089</v>
       </c>
       <c r="BM8" s="85" t="n">
-        <v>1023319689.27</v>
+        <v>1415004365.87</v>
       </c>
       <c r="BN8" s="86" t="n">
-        <v>3375878033.99</v>
+        <v>4314238536.54</v>
       </c>
       <c r="BO8" s="36" t="n">
-        <v>-2352558344.72</v>
+        <v>-2899234170.67</v>
       </c>
       <c r="BP8" s="85" t="n">
-        <v>273596041.87</v>
+        <v>989301381.1400001</v>
       </c>
       <c r="BQ8" s="86" t="n">
-        <v>0</v>
+        <v>270535602</v>
       </c>
       <c r="BR8" s="36" t="n">
-        <v>273596041.87</v>
+        <v>718765779.1400001</v>
       </c>
       <c r="BS8" s="85" t="n">
-        <v>3129236722.02</v>
+        <v>3542176749.6</v>
       </c>
       <c r="BT8" s="86" t="n">
         <v>0</v>
       </c>
       <c r="BU8" s="36" t="n">
-        <v>3129236722.02</v>
+        <v>3542176749.6</v>
       </c>
       <c r="BV8" s="40" t="n">
-        <v>150038390289.4354</v>
+        <v>147587411425.5034</v>
       </c>
       <c r="BW8" s="40" t="n">
-        <v>150038390289.4354</v>
+        <v>147587411425.5034</v>
       </c>
       <c r="BX8" s="40" t="n">
-        <v>0</v>
+        <v>-3.0517578125e-05</v>
       </c>
     </row>
     <row r="9">
@@ -9033,10 +9033,10 @@
         <v>0</v>
       </c>
       <c r="AV9" s="86" t="n">
-        <v>539255590.4932972</v>
+        <v>980501521.682153</v>
       </c>
       <c r="AW9" s="36" t="n">
-        <v>-539255590.4932972</v>
+        <v>-980501521.682153</v>
       </c>
       <c r="AX9" s="85" t="n">
         <v>476716225.7332972</v>
@@ -9048,13 +9048,13 @@
         <v>-601633023.8732792</v>
       </c>
       <c r="BA9" s="85" t="n">
-        <v>1015488535.406576</v>
+        <v>1456734466.595432</v>
       </c>
       <c r="BB9" s="86" t="n">
         <v>905291107.8238831</v>
       </c>
       <c r="BC9" s="36" t="n">
-        <v>110197427.5826933</v>
+        <v>551443358.771549</v>
       </c>
       <c r="BD9" s="85" t="n">
         <v>1799432161.288153</v>
@@ -9111,13 +9111,13 @@
         <v>12771984527.48101</v>
       </c>
       <c r="BV9" s="40" t="n">
-        <v>119883644393.2256</v>
+        <v>120324890324.4144</v>
       </c>
       <c r="BW9" s="40" t="n">
-        <v>107135324198.2064</v>
+        <v>107576570129.3952</v>
       </c>
       <c r="BX9" s="40" t="n">
-        <v>12748320195.01915</v>
+        <v>12748320195.01917</v>
       </c>
     </row>
     <row r="10">
@@ -10021,10 +10021,10 @@
         <v>-4619356997.126001</v>
       </c>
       <c r="BP13" s="85" t="n">
-        <v>29377101039.4902</v>
+        <v>30053123976.7542</v>
       </c>
       <c r="BQ13" s="86" t="n">
-        <v>28030628630.4514</v>
+        <v>28706651567.7154</v>
       </c>
       <c r="BR13" s="36" t="n">
         <v>1346472409.038807</v>
@@ -10039,13 +10039,13 @@
         <v>4350483497.0188</v>
       </c>
       <c r="BV13" s="40" t="n">
-        <v>156023763296.5729</v>
+        <v>156699786233.8369</v>
       </c>
       <c r="BW13" s="40" t="n">
-        <v>156023763296.5729</v>
+        <v>156699786233.8369</v>
       </c>
       <c r="BX13" s="40" t="n">
-        <v>0</v>
+        <v>3.0517578125e-05</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -11031,10 +11031,10 @@
         <v>3701324</v>
       </c>
       <c r="AJ19" s="90" t="n">
-        <v>3667487</v>
+        <v>3690987</v>
       </c>
       <c r="AK19" s="91" t="n">
-        <v>33837</v>
+        <v>10337</v>
       </c>
       <c r="AL19" s="89" t="n">
         <v>6638413</v>
@@ -11049,37 +11049,37 @@
         <v>2456</v>
       </c>
       <c r="AP19" s="90" t="n">
-        <v>17235212.5</v>
+        <v>20125908.5</v>
       </c>
       <c r="AQ19" s="91" t="n">
-        <v>-17232756.5</v>
+        <v>-20123452.5</v>
       </c>
       <c r="AR19" s="89" t="n">
-        <v>17674831.5</v>
+        <v>20685887.5</v>
       </c>
       <c r="AS19" s="90" t="n">
-        <v>2193670</v>
+        <v>3375285</v>
       </c>
       <c r="AT19" s="91" t="n">
-        <v>15481161.5</v>
+        <v>17310602.5</v>
       </c>
       <c r="AU19" s="89" t="n">
-        <v>2706025</v>
+        <v>3790780</v>
       </c>
       <c r="AV19" s="90" t="n">
         <v>1103200.5</v>
       </c>
       <c r="AW19" s="91" t="n">
-        <v>1602824.5</v>
+        <v>2687579.5</v>
       </c>
       <c r="AX19" s="89" t="n">
         <v>228135.5</v>
       </c>
       <c r="AY19" s="90" t="n">
-        <v>1477070</v>
+        <v>1621270</v>
       </c>
       <c r="AZ19" s="91" t="n">
-        <v>-1248934.5</v>
+        <v>-1393134.5</v>
       </c>
       <c r="BA19" s="89" t="n">
         <v>1564252</v>
@@ -11094,10 +11094,10 @@
         <v>2125651</v>
       </c>
       <c r="BE19" s="90" t="n">
-        <v>211848</v>
+        <v>210389.6</v>
       </c>
       <c r="BF19" s="91" t="n">
-        <v>1913803</v>
+        <v>1915261.4</v>
       </c>
       <c r="BG19" s="89" t="n">
         <v>0</v>
@@ -11109,46 +11109,46 @@
         <v>-751392</v>
       </c>
       <c r="BJ19" s="89" t="n">
-        <v>993895</v>
+        <v>1136636.6</v>
       </c>
       <c r="BK19" s="90" t="n">
-        <v>765556</v>
+        <v>983101</v>
       </c>
       <c r="BL19" s="91" t="n">
-        <v>228339</v>
+        <v>153535.6000000001</v>
       </c>
       <c r="BM19" s="89" t="n">
-        <v>822918</v>
+        <v>1070909</v>
       </c>
       <c r="BN19" s="90" t="n">
-        <v>953516</v>
+        <v>1782769</v>
       </c>
       <c r="BO19" s="91" t="n">
-        <v>-130598</v>
+        <v>-711860</v>
       </c>
       <c r="BP19" s="89" t="n">
-        <v>161772</v>
+        <v>870726</v>
       </c>
       <c r="BQ19" s="90" t="n">
-        <v>0</v>
+        <v>170700</v>
       </c>
       <c r="BR19" s="91" t="n">
-        <v>161772</v>
+        <v>700026</v>
       </c>
       <c r="BS19" s="89" t="n">
-        <v>798609</v>
+        <v>1059162</v>
       </c>
       <c r="BT19" s="90" t="n">
         <v>0</v>
       </c>
       <c r="BU19" s="91" t="n">
-        <v>798609</v>
+        <v>1059162</v>
       </c>
       <c r="BV19" s="92" t="n">
-        <v>52709122</v>
+        <v>58165172.6</v>
       </c>
       <c r="BW19" s="92" t="n">
-        <v>52709122</v>
+        <v>58165172.6</v>
       </c>
       <c r="BX19" s="92" t="n">
         <v>0</v>
@@ -12287,10 +12287,10 @@
         <v>-868972</v>
       </c>
       <c r="BP24" s="89" t="n">
-        <v>7131689</v>
+        <v>7275099</v>
       </c>
       <c r="BQ24" s="90" t="n">
-        <v>6773940</v>
+        <v>6917350</v>
       </c>
       <c r="BR24" s="91" t="n">
         <v>357749</v>
@@ -12305,10 +12305,10 @@
         <v>1026716</v>
       </c>
       <c r="BV24" s="92" t="n">
-        <v>44027650.01</v>
+        <v>44171060.01</v>
       </c>
       <c r="BW24" s="92" t="n">
-        <v>44027650.01</v>
+        <v>44171060.01</v>
       </c>
       <c r="BX24" s="92" t="n">
         <v>0</v>
@@ -13360,46 +13360,46 @@
         <v>2074058758.45874</v>
       </c>
       <c r="BE30" s="86" t="n">
-        <v>1964200596.61874</v>
+        <v>1776075581.61874</v>
       </c>
       <c r="BF30" s="36" t="n">
-        <v>109858161.8400002</v>
+        <v>297983176.8400002</v>
       </c>
       <c r="BG30" s="85" t="n">
-        <v>1960230710.637296</v>
+        <v>1960521195.637296</v>
       </c>
       <c r="BH30" s="86" t="n">
-        <v>1737219331.417296</v>
+        <v>1738461386.417296</v>
       </c>
       <c r="BI30" s="36" t="n">
-        <v>223011379.22</v>
+        <v>222059809.22</v>
       </c>
       <c r="BJ30" s="85" t="n">
-        <v>1738781466.77128</v>
+        <v>1551608021.77128</v>
       </c>
       <c r="BK30" s="86" t="n">
-        <v>1687520425.79128</v>
+        <v>1687625065.79128</v>
       </c>
       <c r="BL30" s="36" t="n">
-        <v>51261040.98000002</v>
+        <v>-136017044.02</v>
       </c>
       <c r="BM30" s="85" t="n">
-        <v>1730529151.596482</v>
+        <v>1730633791.596482</v>
       </c>
       <c r="BN30" s="86" t="n">
-        <v>1736909487.306482</v>
+        <v>1737929182.306482</v>
       </c>
       <c r="BO30" s="36" t="n">
-        <v>-6380335.7099998</v>
+        <v>-7295390.7099998</v>
       </c>
       <c r="BP30" s="85" t="n">
-        <v>1472337624.28</v>
+        <v>1473357319.28</v>
       </c>
       <c r="BQ30" s="86" t="n">
         <v>0</v>
       </c>
       <c r="BR30" s="36" t="n">
-        <v>1472337624.28</v>
+        <v>1473357319.28</v>
       </c>
       <c r="BS30" s="85" t="n">
         <v>0</v>
@@ -13411,10 +13411,10 @@
         <v>0</v>
       </c>
       <c r="BV30" s="40" t="n">
-        <v>26521753016.13084</v>
+        <v>26335994391.13084</v>
       </c>
       <c r="BW30" s="40" t="n">
-        <v>26511753016.13084</v>
+        <v>26325994391.13084</v>
       </c>
       <c r="BX30" s="40" t="n">
         <v>10000000</v>
@@ -13779,19 +13779,19 @@
         <v>1068248720</v>
       </c>
       <c r="AP32" s="86" t="n">
-        <v>2023941495.386072</v>
+        <v>2028106327.264181</v>
       </c>
       <c r="AQ32" s="36" t="n">
-        <v>-955692775.3860725</v>
+        <v>-959857607.2641808</v>
       </c>
       <c r="AR32" s="85" t="n">
-        <v>3525141157.457236</v>
+        <v>3529305989.335344</v>
       </c>
       <c r="AS32" s="86" t="n">
         <v>1984504875.105441</v>
       </c>
       <c r="AT32" s="36" t="n">
-        <v>1540636282.351795</v>
+        <v>1544801114.229903</v>
       </c>
       <c r="AU32" s="85" t="n">
         <v>0</v>
@@ -13875,13 +13875,13 @@
         <v>564013362.9393721</v>
       </c>
       <c r="BV32" s="40" t="n">
-        <v>27389359639.88501</v>
+        <v>27393524471.76311</v>
       </c>
       <c r="BW32" s="40" t="n">
-        <v>27389359639.885</v>
+        <v>27393524471.76311</v>
       </c>
       <c r="BX32" s="40" t="n">
-        <v>3.814697265625e-06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -15162,46 +15162,46 @@
         <v>5406868.1</v>
       </c>
       <c r="BE39" s="90" t="n">
-        <v>5243812.1</v>
+        <v>4711260.1</v>
       </c>
       <c r="BF39" s="91" t="n">
-        <v>163056</v>
+        <v>695608</v>
       </c>
       <c r="BG39" s="89" t="n">
-        <v>5240314.44</v>
+        <v>5240762.44</v>
       </c>
       <c r="BH39" s="90" t="n">
-        <v>4625816.439999999</v>
+        <v>4628095.439999999</v>
       </c>
       <c r="BI39" s="91" t="n">
-        <v>614498.0000000009</v>
+        <v>612667.0000000009</v>
       </c>
       <c r="BJ39" s="89" t="n">
-        <v>4627206.2</v>
+        <v>4096485.2</v>
       </c>
       <c r="BK39" s="90" t="n">
-        <v>4369524.2</v>
+        <v>4369716.2</v>
       </c>
       <c r="BL39" s="91" t="n">
-        <v>257682</v>
+        <v>-273231</v>
       </c>
       <c r="BM39" s="89" t="n">
-        <v>4403332.23</v>
+        <v>4403524.23</v>
       </c>
       <c r="BN39" s="90" t="n">
-        <v>4682071.23</v>
+        <v>4683942.23</v>
       </c>
       <c r="BO39" s="91" t="n">
-        <v>-278739.0000000009</v>
+        <v>-280418.0000000009</v>
       </c>
       <c r="BP39" s="89" t="n">
-        <v>4630652</v>
+        <v>4632523</v>
       </c>
       <c r="BQ39" s="90" t="n">
         <v>0</v>
       </c>
       <c r="BR39" s="91" t="n">
-        <v>4630652</v>
+        <v>4632523</v>
       </c>
       <c r="BS39" s="89" t="n">
         <v>0</v>
@@ -15213,10 +15213,10 @@
         <v>0</v>
       </c>
       <c r="BV39" s="92" t="n">
-        <v>37588374.53</v>
+        <v>37060164.53</v>
       </c>
       <c r="BW39" s="92" t="n">
-        <v>37588374.53</v>
+        <v>37060164.53</v>
       </c>
       <c r="BX39" s="92" t="n">
         <v>0</v>
@@ -15581,19 +15581,19 @@
         <v>0</v>
       </c>
       <c r="AP41" s="90" t="n">
-        <v>85676089.14000006</v>
+        <v>86523717.19000007</v>
       </c>
       <c r="AQ41" s="91" t="n">
-        <v>-85676089.14000006</v>
+        <v>-86523717.19000007</v>
       </c>
       <c r="AR41" s="89" t="n">
-        <v>125990966.5520001</v>
+        <v>126838594.6020001</v>
       </c>
       <c r="AS41" s="90" t="n">
         <v>2784332.014193548</v>
       </c>
       <c r="AT41" s="91" t="n">
-        <v>123206634.5378065</v>
+        <v>124054262.5878065</v>
       </c>
       <c r="AU41" s="89" t="n">
         <v>0</v>
@@ -15677,10 +15677,10 @@
         <v>1657731.66</v>
       </c>
       <c r="BV41" s="92" t="n">
-        <v>166732915.2813745</v>
+        <v>167580543.3313745</v>
       </c>
       <c r="BW41" s="92" t="n">
-        <v>166732915.2813745</v>
+        <v>167580543.3313745</v>
       </c>
       <c r="BX41" s="92" t="n">
         <v>2.980232238769531e-08</v>
@@ -16413,16 +16413,16 @@
         </is>
       </c>
       <c r="B6" s="36" t="n">
-        <v>66793712354.01656</v>
+        <v>66791360654.01656</v>
       </c>
       <c r="C6" s="36" t="n">
         <v>63827327546.06796</v>
       </c>
       <c r="D6" s="97" t="n">
-        <v>2966384807.948601</v>
+        <v>2964033107.948601</v>
       </c>
       <c r="E6" s="98" t="n">
-        <v>0.9555888615349553</v>
+        <v>0.9556225074781382</v>
       </c>
       <c r="F6" s="99" t="inlineStr">
         <is>
@@ -16437,16 +16437,16 @@
         </is>
       </c>
       <c r="B7" s="36" t="n">
-        <v>84371132941.67935</v>
+        <v>82029091706.55746</v>
       </c>
       <c r="C7" s="36" t="n">
         <v>31245109766.04071</v>
       </c>
       <c r="D7" s="97" t="n">
-        <v>53126023175.63864</v>
+        <v>50783981940.51675</v>
       </c>
       <c r="E7" s="98" t="n">
-        <v>0.3703293849051258</v>
+        <v>0.3809027884620957</v>
       </c>
       <c r="F7" s="99" t="inlineStr">
         <is>
@@ -16461,16 +16461,16 @@
         </is>
       </c>
       <c r="B8" s="36" t="n">
-        <v>15421312930.92924</v>
+        <v>14344254141.84816</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>86240159201.30141</v>
+        <v>83725480086.17952</v>
       </c>
       <c r="D8" s="100" t="n">
-        <v>-70818846270.37216</v>
+        <v>-69381225944.33136</v>
       </c>
       <c r="E8" s="98" t="n">
-        <v>5.592270877814608</v>
+        <v>5.836865357949666</v>
       </c>
       <c r="F8" s="99" t="inlineStr">
         <is>
@@ -16485,16 +16485,16 @@
         </is>
       </c>
       <c r="B9" s="36" t="n">
-        <v>9281134641.667723</v>
+        <v>9687562287.897118</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>13827779290.76451</v>
+        <v>12902094102.76451</v>
       </c>
       <c r="D9" s="100" t="n">
-        <v>-4546644649.096786</v>
+        <v>-3214531814.867392</v>
       </c>
       <c r="E9" s="98" t="n">
-        <v>1.489880259756667</v>
+        <v>1.33182050544164</v>
       </c>
       <c r="F9" s="99" t="inlineStr">
         <is>
@@ -16509,16 +16509,16 @@
         </is>
       </c>
       <c r="B10" s="36" t="n">
-        <v>13136105644.05059</v>
+        <v>12883873710.01005</v>
       </c>
       <c r="C10" s="36" t="n">
         <v>10232991763.92059</v>
       </c>
       <c r="D10" s="97" t="n">
-        <v>2903113880.129999</v>
+        <v>2650881946.08946</v>
       </c>
       <c r="E10" s="98" t="n">
-        <v>0.7789973711543015</v>
+        <v>0.7942480650031618</v>
       </c>
       <c r="F10" s="99" t="inlineStr">
         <is>
@@ -16533,16 +16533,16 @@
         </is>
       </c>
       <c r="B11" s="36" t="n">
-        <v>14953567134.55988</v>
+        <v>14716130448.01033</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>14795617887.56988</v>
-      </c>
-      <c r="D11" s="97" t="n">
-        <v>157949246.9900017</v>
+        <v>14939898835.40739</v>
+      </c>
+      <c r="D11" s="100" t="n">
+        <v>-223768387.3970528</v>
       </c>
       <c r="E11" s="98" t="n">
-        <v>0.9894373532703807</v>
+        <v>1.01520565397185</v>
       </c>
       <c r="F11" s="99" t="inlineStr">
         <is>
@@ -16557,16 +16557,16 @@
         </is>
       </c>
       <c r="B12" s="36" t="n">
-        <v>9284375265.819054</v>
+        <v>9093938805.067703</v>
       </c>
       <c r="C12" s="36" t="n">
-        <v>14358678838.51815</v>
+        <v>14119005142.51815</v>
       </c>
       <c r="D12" s="100" t="n">
-        <v>-5074303572.6991</v>
+        <v>-5025066337.450451</v>
       </c>
       <c r="E12" s="98" t="n">
-        <v>1.546542274242235</v>
+        <v>1.552573141865676</v>
       </c>
       <c r="F12" s="99" t="inlineStr">
         <is>
@@ -16581,16 +16581,16 @@
         </is>
       </c>
       <c r="B13" s="36" t="n">
-        <v>12041589098.57968</v>
+        <v>12042831153.57968</v>
       </c>
       <c r="C13" s="36" t="n">
-        <v>8523861993.219052</v>
+        <v>8524152478.219052</v>
       </c>
       <c r="D13" s="97" t="n">
-        <v>3517727105.360625</v>
+        <v>3518678675.360625</v>
       </c>
       <c r="E13" s="98" t="n">
-        <v>0.7078685315897761</v>
+        <v>0.7078196455229123</v>
       </c>
       <c r="F13" s="99" t="inlineStr">
         <is>
@@ -16605,16 +16605,16 @@
         </is>
       </c>
       <c r="B14" s="36" t="n">
-        <v>9347962197.674297</v>
+        <v>9659500776.574297</v>
       </c>
       <c r="C14" s="36" t="n">
-        <v>9767838169.155153</v>
-      </c>
-      <c r="D14" s="100" t="n">
-        <v>-419875971.4808559</v>
+        <v>9590523631.124523</v>
+      </c>
+      <c r="D14" s="36" t="n">
+        <v>68977145.44977379</v>
       </c>
       <c r="E14" s="98" t="n">
-        <v>1.044916310378889</v>
+        <v>0.9928591397169247</v>
       </c>
       <c r="F14" s="99" t="inlineStr">
         <is>
@@ -16629,16 +16629,16 @@
         </is>
       </c>
       <c r="B15" s="36" t="n">
-        <v>23065984162.76961</v>
+        <v>24005364360.31962</v>
       </c>
       <c r="C15" s="36" t="n">
-        <v>11894352978.39672</v>
+        <v>12286142294.99672</v>
       </c>
       <c r="D15" s="97" t="n">
-        <v>11171631184.37289</v>
+        <v>11719222065.3229</v>
       </c>
       <c r="E15" s="98" t="n">
-        <v>0.5156663983839537</v>
+        <v>0.5118081988084907</v>
       </c>
       <c r="F15" s="99" t="inlineStr">
         <is>
@@ -16653,16 +16653,16 @@
         </is>
       </c>
       <c r="B16" s="36" t="n">
-        <v>31202318295.1414</v>
+        <v>32148876834.4054</v>
       </c>
       <c r="C16" s="36" t="n">
-        <v>45042578007.53642</v>
+        <v>46435325979.07043</v>
       </c>
       <c r="D16" s="100" t="n">
-        <v>-13840259712.39503</v>
+        <v>-14286449144.66503</v>
       </c>
       <c r="E16" s="98" t="n">
-        <v>1.443565108896095</v>
+        <v>1.44438408278624</v>
       </c>
       <c r="F16" s="99" t="inlineStr">
         <is>
@@ -16680,10 +16680,10 @@
         <v>0</v>
       </c>
       <c r="C17" s="36" t="n">
-        <v>20815718109.45918</v>
+        <v>21228658137.03918</v>
       </c>
       <c r="D17" s="100" t="n">
-        <v>-20815718109.45918</v>
+        <v>-21228658137.03918</v>
       </c>
       <c r="E17" s="98" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Auto-deploy AR dashboard 2026-09-10 15:54
</commit_message>
<xml_diff>
--- a/AR Movement Report.xlsx
+++ b/AR Movement Report.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$138</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1118</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1320,7 +1320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1346,7 +1346,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data as of Thursday, 10 September 2026 - 14:50  |  Source: PSI AR Monitoring Master.xlsx</t>
+          <t>Data as of Thursday, 10 September 2026 - 15:54  |  Source: PSI AR Monitoring Master.xlsx</t>
         </is>
       </c>
     </row>
@@ -1383,18 +1383,18 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="9" t="n">
-        <v>128553544603.3722</v>
+        <v>130823792442.2642</v>
       </c>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="10" t="n"/>
       <c r="D7" s="11" t="n"/>
       <c r="E7" s="12" t="n">
-        <v>118402572711.6093</v>
+        <v>120748351115.5612</v>
       </c>
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="11" t="n"/>
       <c r="H7" s="13" t="n">
-        <v>10150971891.76296</v>
+        <v>10075441326.70296</v>
       </c>
       <c r="I7" s="10" t="n"/>
       <c r="J7" s="11" t="n"/>
@@ -1440,14 +1440,14 @@
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="19" t="n">
-        <v>65161432472.40769</v>
+        <v>69090575311.29965</v>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="10" t="n"/>
       <c r="D12" s="10" t="n"/>
       <c r="E12" s="11" t="n"/>
       <c r="F12" s="20" t="n">
-        <v>63392112130.96454</v>
+        <v>61733217130.96454</v>
       </c>
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="10" t="n"/>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="26" t="n">
-        <v>21228658137.03918</v>
+        <v>25157800975.93113</v>
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="27" t="n">
@@ -1600,10 +1600,10 @@
         </is>
       </c>
       <c r="B23" s="34" t="n">
-        <v>3542176749.6</v>
+        <v>5125541184.54</v>
       </c>
       <c r="C23" s="35" t="n">
-        <v>16029298282.307</v>
+        <v>14370403282.307</v>
       </c>
       <c r="D23" s="36" t="n">
         <v>0</v>
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="B30" s="34" t="n">
-        <v>38047520478.72108</v>
+        <v>40393298882.67303</v>
       </c>
       <c r="C30" s="35" t="n">
         <v>16137826356.519</v>
@@ -2026,10 +2026,10 @@
         </is>
       </c>
       <c r="B41" s="49" t="n">
-        <v>60344238280.02831</v>
+        <v>62690016683.98026</v>
       </c>
       <c r="C41" s="49" t="n">
-        <v>4817194192.379373</v>
+        <v>6400558627.319372</v>
       </c>
       <c r="D41" s="50">
         <f>SUM(B41:C41)</f>
@@ -2046,7 +2046,7 @@
         <v>27426700719.026</v>
       </c>
       <c r="C42" s="36" t="n">
-        <v>5333777699.383585</v>
+        <v>3674882699.383585</v>
       </c>
       <c r="D42" s="36">
         <f>SUM(B42:C42)</f>
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="B49" s="57" t="n">
-        <v>16029298282.307</v>
+        <v>14370403282.307</v>
       </c>
       <c r="C49" s="57" t="n">
         <v>359473956.24</v>
@@ -2636,7 +2636,7 @@
         <v>46305</v>
       </c>
       <c r="B64" s="36" t="n">
-        <v>0</v>
+        <v>1583364434.94</v>
       </c>
       <c r="C64" s="36" t="n">
         <v>0</v>
@@ -2958,75 +2958,108 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="59" t="inlineStr">
+      <c r="A74" s="58" t="n">
+        <v>46335</v>
+      </c>
+      <c r="B74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="36" t="n">
+        <v>2345778403.95195</v>
+      </c>
+      <c r="J74" s="37">
+        <f>SUM(B74:I74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="59" t="inlineStr">
         <is>
           <t>Total upcoming in November</t>
         </is>
       </c>
-      <c r="B74" s="40">
-        <f>SUM(B73:B73)</f>
+      <c r="B75" s="40">
+        <f>SUM(B73:B74)</f>
         <v/>
       </c>
-      <c r="C74" s="40">
-        <f>SUM(C73:C73)</f>
+      <c r="C75" s="40">
+        <f>SUM(C73:C74)</f>
         <v/>
       </c>
-      <c r="D74" s="40">
-        <f>SUM(D73:D73)</f>
+      <c r="D75" s="40">
+        <f>SUM(D73:D74)</f>
         <v/>
       </c>
-      <c r="E74" s="40">
-        <f>SUM(E73:E73)</f>
+      <c r="E75" s="40">
+        <f>SUM(E73:E74)</f>
         <v/>
       </c>
-      <c r="F74" s="40">
-        <f>SUM(F73:F73)</f>
+      <c r="F75" s="40">
+        <f>SUM(F73:F74)</f>
         <v/>
       </c>
-      <c r="G74" s="40">
-        <f>SUM(G73:G73)</f>
+      <c r="G75" s="40">
+        <f>SUM(G73:G74)</f>
         <v/>
       </c>
-      <c r="H74" s="40">
-        <f>SUM(H73:H73)</f>
+      <c r="H75" s="40">
+        <f>SUM(H73:H74)</f>
         <v/>
       </c>
-      <c r="I74" s="40">
-        <f>SUM(I73:I73)</f>
+      <c r="I75" s="40">
+        <f>SUM(I73:I74)</f>
         <v/>
       </c>
-      <c r="J74" s="40">
-        <f>SUM(J73:J73)</f>
+      <c r="J75" s="40">
+        <f>SUM(J73:J74)</f>
         <v/>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="60" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="60" t="inlineStr">
         <is>
           <t>Detail Sheets:</t>
         </is>
       </c>
-      <c r="B77" s="61" t="inlineStr">
+      <c r="B78" s="61" t="inlineStr">
         <is>
           <t>Daily Projection</t>
         </is>
       </c>
-      <c r="C77" s="61" t="inlineStr">
+      <c r="C78" s="61" t="inlineStr">
         <is>
           <t>Aging</t>
         </is>
       </c>
-      <c r="D77" s="61" t="inlineStr">
+      <c r="D78" s="61" t="inlineStr">
         <is>
           <t>Invoice vs Service</t>
         </is>
       </c>
-      <c r="E77" s="61" t="inlineStr">
+      <c r="E78" s="61" t="inlineStr">
         <is>
           <t>Service &amp; Billing</t>
         </is>
       </c>
-      <c r="F77" s="61" t="inlineStr">
+      <c r="F78" s="61" t="inlineStr">
         <is>
           <t>Raw Data</t>
         </is>
@@ -3062,11 +3095,11 @@
     <mergeCell ref="H6:J6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3200,7 +3233,7 @@
         <v>3542176749.6</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>0</v>
+        <v>1583364434.94</v>
       </c>
       <c r="E7" s="36" t="n">
         <v>0</v>
@@ -3225,7 +3258,7 @@
         <v>14370403282.307</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>1658895000</v>
+        <v>0</v>
       </c>
       <c r="E8" s="36" t="n">
         <v>0</v>
@@ -3372,7 +3405,7 @@
         </is>
       </c>
       <c r="C14" s="36" t="n">
-        <v>35328887197.52108</v>
+        <v>37674665601.47303</v>
       </c>
       <c r="D14" s="36" t="n">
         <v>2718633281.2</v>
@@ -3445,7 +3478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H138"/>
+  <dimension ref="A1:H141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4920,11 +4953,11 @@
       <c r="C46" s="72" t="n"/>
       <c r="D46" s="72" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E46" s="73" t="n">
-        <v>777000000</v>
+        <v>13247943944.279</v>
       </c>
       <c r="F46" s="71" t="n"/>
       <c r="G46" s="74" t="n">
@@ -4948,11 +4981,11 @@
       <c r="C47" s="72" t="n"/>
       <c r="D47" s="72" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E47" s="73" t="n">
-        <v>881895000</v>
+        <v>1122459338.028</v>
       </c>
       <c r="F47" s="71" t="n"/>
       <c r="G47" s="74" t="n">
@@ -4970,17 +5003,17 @@
       </c>
       <c r="B48" s="72" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C48" s="72" t="n"/>
       <c r="D48" s="72" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E48" s="73" t="n">
-        <v>13247943944.279</v>
+        <v>593353779.5835853</v>
       </c>
       <c r="F48" s="71" t="n"/>
       <c r="G48" s="74" t="n">
@@ -4998,7 +5031,7 @@
       </c>
       <c r="B49" s="72" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C49" s="72" t="n"/>
@@ -5008,7 +5041,7 @@
         </is>
       </c>
       <c r="E49" s="73" t="n">
-        <v>1122459338.028</v>
+        <v>7266583243.008001</v>
       </c>
       <c r="F49" s="71" t="n"/>
       <c r="G49" s="74" t="n">
@@ -5026,7 +5059,7 @@
       </c>
       <c r="B50" s="72" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C50" s="72" t="n"/>
@@ -5036,7 +5069,7 @@
         </is>
       </c>
       <c r="E50" s="73" t="n">
-        <v>593353779.5835853</v>
+        <v>552691555.2</v>
       </c>
       <c r="F50" s="71" t="n"/>
       <c r="G50" s="74" t="n">
@@ -5060,11 +5093,11 @@
       <c r="C51" s="72" t="n"/>
       <c r="D51" s="72" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E51" s="73" t="n">
-        <v>7266583243.008001</v>
+        <v>552691555.2</v>
       </c>
       <c r="F51" s="71" t="n"/>
       <c r="G51" s="74" t="n">
@@ -5092,7 +5125,7 @@
         </is>
       </c>
       <c r="E52" s="73" t="n">
-        <v>552691555.2</v>
+        <v>71167361.40000001</v>
       </c>
       <c r="F52" s="71" t="n"/>
       <c r="G52" s="74" t="n">
@@ -5120,7 +5153,7 @@
         </is>
       </c>
       <c r="E53" s="73" t="n">
-        <v>552691555.2</v>
+        <v>299652048</v>
       </c>
       <c r="F53" s="71" t="n"/>
       <c r="G53" s="74" t="n">
@@ -5144,11 +5177,11 @@
       <c r="C54" s="72" t="n"/>
       <c r="D54" s="72" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E54" s="73" t="n">
-        <v>71167361.40000001</v>
+        <v>5789714193.710999</v>
       </c>
       <c r="F54" s="71" t="n"/>
       <c r="G54" s="74" t="n">
@@ -5176,7 +5209,7 @@
         </is>
       </c>
       <c r="E55" s="73" t="n">
-        <v>299652048</v>
+        <v>1605326400</v>
       </c>
       <c r="F55" s="71" t="n"/>
       <c r="G55" s="74" t="n">
@@ -5189,73 +5222,85 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="71" t="n">
-        <v>46275</v>
-      </c>
-      <c r="B56" s="72" t="inlineStr">
+      <c r="A56" s="75" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B56" s="76" t="inlineStr">
         <is>
           <t>PT Syngenta Indonesia</t>
         </is>
       </c>
-      <c r="C56" s="72" t="n"/>
-      <c r="D56" s="72" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="E56" s="73" t="n">
-        <v>5789714193.710999</v>
-      </c>
-      <c r="F56" s="71" t="n"/>
-      <c r="G56" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="72" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+      <c r="C56" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL/33/2026</t>
+        </is>
+      </c>
+      <c r="D56" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E56" s="77" t="n">
+        <v>27842793.22</v>
+      </c>
+      <c r="F56" s="75" t="n">
+        <v>46278</v>
+      </c>
+      <c r="G56" s="78" t="n">
+        <v>3</v>
+      </c>
+      <c r="H56" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="71" t="n">
-        <v>46275</v>
-      </c>
-      <c r="B57" s="72" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="C57" s="72" t="n"/>
-      <c r="D57" s="72" t="inlineStr">
-        <is>
-          <t>Rental</t>
-        </is>
-      </c>
-      <c r="E57" s="73" t="n">
-        <v>1605326400</v>
-      </c>
-      <c r="F57" s="71" t="n"/>
-      <c r="G57" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H57" s="72" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+      <c r="A57" s="75" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B57" s="76" t="inlineStr">
+        <is>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="C57" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.CASI/FC-C/49/2026</t>
+        </is>
+      </c>
+      <c r="D57" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E57" s="77" t="n">
+        <v>3981599123.659349</v>
+      </c>
+      <c r="F57" s="75" t="n">
+        <v>46276</v>
+      </c>
+      <c r="G57" s="78" t="n">
+        <v>7</v>
+      </c>
+      <c r="H57" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="75" t="n">
-        <v>46278</v>
+        <v>46282</v>
       </c>
       <c r="B58" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C58" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/33/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/50/2026</t>
         </is>
       </c>
       <c r="D58" s="76" t="inlineStr">
@@ -5264,13 +5309,13 @@
         </is>
       </c>
       <c r="E58" s="77" t="n">
-        <v>27842793.22</v>
+        <v>1542175442.6694</v>
       </c>
       <c r="F58" s="75" t="n">
-        <v>46278</v>
+        <v>46276</v>
       </c>
       <c r="G58" s="78" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H58" s="76" t="inlineStr">
         <is>
@@ -5289,7 +5334,7 @@
       </c>
       <c r="C59" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/49/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/51/2026</t>
         </is>
       </c>
       <c r="D59" s="76" t="inlineStr">
@@ -5298,7 +5343,7 @@
         </is>
       </c>
       <c r="E59" s="77" t="n">
-        <v>3981599123.659349</v>
+        <v>487978078.30875</v>
       </c>
       <c r="F59" s="75" t="n">
         <v>46276</v>
@@ -5323,7 +5368,7 @@
       </c>
       <c r="C60" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/50/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/52/2026</t>
         </is>
       </c>
       <c r="D60" s="76" t="inlineStr">
@@ -5332,7 +5377,7 @@
         </is>
       </c>
       <c r="E60" s="77" t="n">
-        <v>1542175442.6694</v>
+        <v>14255050.74672</v>
       </c>
       <c r="F60" s="75" t="n">
         <v>46276</v>
@@ -5348,16 +5393,16 @@
     </row>
     <row r="61">
       <c r="A61" s="75" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="B61" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C61" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/51/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
         </is>
       </c>
       <c r="D61" s="76" t="inlineStr">
@@ -5366,13 +5411,13 @@
         </is>
       </c>
       <c r="E61" s="77" t="n">
-        <v>487978078.30875</v>
+        <v>326395903.6008</v>
       </c>
       <c r="F61" s="75" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
       <c r="G61" s="78" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H61" s="76" t="inlineStr">
         <is>
@@ -5382,16 +5427,16 @@
     </row>
     <row r="62">
       <c r="A62" s="75" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="B62" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C62" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/52/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
         </is>
       </c>
       <c r="D62" s="76" t="inlineStr">
@@ -5400,13 +5445,13 @@
         </is>
       </c>
       <c r="E62" s="77" t="n">
-        <v>14255050.74672</v>
+        <v>240049.20888</v>
       </c>
       <c r="F62" s="75" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
       <c r="G62" s="78" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H62" s="76" t="inlineStr">
         <is>
@@ -5416,7 +5461,7 @@
     </row>
     <row r="63">
       <c r="A63" s="75" t="n">
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="B63" s="76" t="inlineStr">
         <is>
@@ -5425,7 +5470,7 @@
       </c>
       <c r="C63" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
         </is>
       </c>
       <c r="D63" s="76" t="inlineStr">
@@ -5434,13 +5479,13 @@
         </is>
       </c>
       <c r="E63" s="77" t="n">
-        <v>326395903.6008</v>
+        <v>570800977.7184</v>
       </c>
       <c r="F63" s="75" t="n">
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="G63" s="78" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H63" s="76" t="inlineStr">
         <is>
@@ -5450,16 +5495,16 @@
     </row>
     <row r="64">
       <c r="A64" s="75" t="n">
-        <v>46284</v>
+        <v>46289</v>
       </c>
       <c r="B64" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C64" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
+          <t>PT.PSI/PT.CASI/REP/53/2026</t>
         </is>
       </c>
       <c r="D64" s="76" t="inlineStr">
@@ -5468,13 +5513,13 @@
         </is>
       </c>
       <c r="E64" s="77" t="n">
-        <v>240049.20888</v>
+        <v>36849832.74</v>
       </c>
       <c r="F64" s="75" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="G64" s="78" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H64" s="76" t="inlineStr">
         <is>
@@ -5484,16 +5529,16 @@
     </row>
     <row r="65">
       <c r="A65" s="75" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="B65" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C65" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
+          <t>PT.PSI/PT.CASI/REP/54/2026</t>
         </is>
       </c>
       <c r="D65" s="76" t="inlineStr">
@@ -5502,13 +5547,13 @@
         </is>
       </c>
       <c r="E65" s="77" t="n">
-        <v>570800977.7184</v>
+        <v>31988016.36</v>
       </c>
       <c r="F65" s="75" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="G65" s="78" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H65" s="76" t="inlineStr">
         <is>
@@ -5527,7 +5572,7 @@
       </c>
       <c r="C66" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/53/2026</t>
+          <t>PT.PSI/PT.CASI/REP/55/2026</t>
         </is>
       </c>
       <c r="D66" s="76" t="inlineStr">
@@ -5536,7 +5581,7 @@
         </is>
       </c>
       <c r="E66" s="77" t="n">
-        <v>36849832.74</v>
+        <v>19431065.722</v>
       </c>
       <c r="F66" s="75" t="n">
         <v>46285</v>
@@ -5552,16 +5597,16 @@
     </row>
     <row r="67">
       <c r="A67" s="75" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="B67" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C67" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/54/2026</t>
+          <t>PT.PSI/PT.BI/FC/43/2026</t>
         </is>
       </c>
       <c r="D67" s="76" t="inlineStr">
@@ -5570,13 +5615,13 @@
         </is>
       </c>
       <c r="E67" s="77" t="n">
-        <v>31988016.36</v>
+        <v>103679056</v>
       </c>
       <c r="F67" s="75" t="n">
-        <v>46285</v>
+        <v>46292</v>
       </c>
       <c r="G67" s="78" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H67" s="76" t="inlineStr">
         <is>
@@ -5586,16 +5631,16 @@
     </row>
     <row r="68">
       <c r="A68" s="75" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="B68" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C68" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/55/2026</t>
+          <t>PT.PSI/PT.BI/FC/44/2026</t>
         </is>
       </c>
       <c r="D68" s="76" t="inlineStr">
@@ -5604,13 +5649,13 @@
         </is>
       </c>
       <c r="E68" s="77" t="n">
-        <v>19431065.722</v>
+        <v>92863095</v>
       </c>
       <c r="F68" s="75" t="n">
-        <v>46285</v>
+        <v>46292</v>
       </c>
       <c r="G68" s="78" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H68" s="76" t="inlineStr">
         <is>
@@ -5629,7 +5674,7 @@
       </c>
       <c r="C69" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/43/2026</t>
+          <t>PT.PSI/PT.BI/FC/45/2026</t>
         </is>
       </c>
       <c r="D69" s="76" t="inlineStr">
@@ -5638,7 +5683,7 @@
         </is>
       </c>
       <c r="E69" s="77" t="n">
-        <v>103679056</v>
+        <v>17392258</v>
       </c>
       <c r="F69" s="75" t="n">
         <v>46292</v>
@@ -5663,7 +5708,7 @@
       </c>
       <c r="C70" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/44/2026</t>
+          <t>PT.PSI/PT.BI/FC/46/2026</t>
         </is>
       </c>
       <c r="D70" s="76" t="inlineStr">
@@ -5672,7 +5717,7 @@
         </is>
       </c>
       <c r="E70" s="77" t="n">
-        <v>92863095</v>
+        <v>197734556.5</v>
       </c>
       <c r="F70" s="75" t="n">
         <v>46292</v>
@@ -5697,7 +5742,7 @@
       </c>
       <c r="C71" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/45/2026</t>
+          <t>PT.PSI/PT.BI/FC/47/2026</t>
         </is>
       </c>
       <c r="D71" s="76" t="inlineStr">
@@ -5706,7 +5751,7 @@
         </is>
       </c>
       <c r="E71" s="77" t="n">
-        <v>17392258</v>
+        <v>254755628.4</v>
       </c>
       <c r="F71" s="75" t="n">
         <v>46292</v>
@@ -5731,7 +5776,7 @@
       </c>
       <c r="C72" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/46/2026</t>
+          <t>PT.PSI/PT.BI/FC/48/2026</t>
         </is>
       </c>
       <c r="D72" s="76" t="inlineStr">
@@ -5740,7 +5785,7 @@
         </is>
       </c>
       <c r="E72" s="77" t="n">
-        <v>197734556.5</v>
+        <v>10599160</v>
       </c>
       <c r="F72" s="75" t="n">
         <v>46292</v>
@@ -5765,7 +5810,7 @@
       </c>
       <c r="C73" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/47/2026</t>
+          <t>PT.PSI/PT.BI/FC/49/2026</t>
         </is>
       </c>
       <c r="D73" s="76" t="inlineStr">
@@ -5774,7 +5819,7 @@
         </is>
       </c>
       <c r="E73" s="77" t="n">
-        <v>254755628.4</v>
+        <v>54405006.5</v>
       </c>
       <c r="F73" s="75" t="n">
         <v>46292</v>
@@ -5799,7 +5844,7 @@
       </c>
       <c r="C74" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/48/2026</t>
+          <t>PT.PSI/PT.BI/FC/50/2026</t>
         </is>
       </c>
       <c r="D74" s="76" t="inlineStr">
@@ -5808,7 +5853,7 @@
         </is>
       </c>
       <c r="E74" s="77" t="n">
-        <v>10599160</v>
+        <v>1075481.2</v>
       </c>
       <c r="F74" s="75" t="n">
         <v>46292</v>
@@ -5833,7 +5878,7 @@
       </c>
       <c r="C75" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/49/2026</t>
+          <t>PT.PSI/PT.BI/FC/51/2026</t>
         </is>
       </c>
       <c r="D75" s="76" t="inlineStr">
@@ -5842,7 +5887,7 @@
         </is>
       </c>
       <c r="E75" s="77" t="n">
-        <v>54405006.5</v>
+        <v>803447.72</v>
       </c>
       <c r="F75" s="75" t="n">
         <v>46292</v>
@@ -5867,7 +5912,7 @@
       </c>
       <c r="C76" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/50/2026</t>
+          <t>PT.PSI/PT.BI/FC/52/2026</t>
         </is>
       </c>
       <c r="D76" s="76" t="inlineStr">
@@ -5876,7 +5921,7 @@
         </is>
       </c>
       <c r="E76" s="77" t="n">
-        <v>1075481.2</v>
+        <v>7250789</v>
       </c>
       <c r="F76" s="75" t="n">
         <v>46292</v>
@@ -5901,7 +5946,7 @@
       </c>
       <c r="C77" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/51/2026</t>
+          <t>PT.PSI/PT.BI/FC/53/2026</t>
         </is>
       </c>
       <c r="D77" s="76" t="inlineStr">
@@ -5910,7 +5955,7 @@
         </is>
       </c>
       <c r="E77" s="77" t="n">
-        <v>803447.72</v>
+        <v>101318334</v>
       </c>
       <c r="F77" s="75" t="n">
         <v>46292</v>
@@ -5926,7 +5971,7 @@
     </row>
     <row r="78">
       <c r="A78" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B78" s="76" t="inlineStr">
         <is>
@@ -5935,7 +5980,7 @@
       </c>
       <c r="C78" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/52/2026</t>
+          <t>PT.PSI/PT.BI/FC/54/2026</t>
         </is>
       </c>
       <c r="D78" s="76" t="inlineStr">
@@ -5944,13 +5989,13 @@
         </is>
       </c>
       <c r="E78" s="77" t="n">
-        <v>7250789</v>
+        <v>156400274.1</v>
       </c>
       <c r="F78" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G78" s="78" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H78" s="76" t="inlineStr">
         <is>
@@ -5960,7 +6005,7 @@
     </row>
     <row r="79">
       <c r="A79" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B79" s="76" t="inlineStr">
         <is>
@@ -5969,7 +6014,7 @@
       </c>
       <c r="C79" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/53/2026</t>
+          <t>PT.PSI/PT.BI/FC/55/2026</t>
         </is>
       </c>
       <c r="D79" s="76" t="inlineStr">
@@ -5978,13 +6023,13 @@
         </is>
       </c>
       <c r="E79" s="77" t="n">
-        <v>101318334</v>
+        <v>50838199.5</v>
       </c>
       <c r="F79" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G79" s="78" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H79" s="76" t="inlineStr">
         <is>
@@ -6003,7 +6048,7 @@
       </c>
       <c r="C80" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/54/2026</t>
+          <t>PT.PSI/PT.BI/FC/56/2026</t>
         </is>
       </c>
       <c r="D80" s="76" t="inlineStr">
@@ -6012,7 +6057,7 @@
         </is>
       </c>
       <c r="E80" s="77" t="n">
-        <v>156400274.1</v>
+        <v>376884765.6</v>
       </c>
       <c r="F80" s="75" t="n">
         <v>46293</v>
@@ -6037,7 +6082,7 @@
       </c>
       <c r="C81" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/55/2026</t>
+          <t>PT.PSI/PT.BI/FC/57/2026</t>
         </is>
       </c>
       <c r="D81" s="76" t="inlineStr">
@@ -6046,7 +6091,7 @@
         </is>
       </c>
       <c r="E81" s="77" t="n">
-        <v>50838199.5</v>
+        <v>100336789</v>
       </c>
       <c r="F81" s="75" t="n">
         <v>46293</v>
@@ -6071,7 +6116,7 @@
       </c>
       <c r="C82" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/56/2026</t>
+          <t>PT.PSI/PT.BI/FC/58/2026</t>
         </is>
       </c>
       <c r="D82" s="76" t="inlineStr">
@@ -6080,7 +6125,7 @@
         </is>
       </c>
       <c r="E82" s="77" t="n">
-        <v>376884765.6</v>
+        <v>787756603.1999999</v>
       </c>
       <c r="F82" s="75" t="n">
         <v>46293</v>
@@ -6105,7 +6150,7 @@
       </c>
       <c r="C83" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/57/2026</t>
+          <t>PT.PSI/PT.BI/FC/59/2026</t>
         </is>
       </c>
       <c r="D83" s="76" t="inlineStr">
@@ -6114,7 +6159,7 @@
         </is>
       </c>
       <c r="E83" s="77" t="n">
-        <v>100336789</v>
+        <v>140859991.5</v>
       </c>
       <c r="F83" s="75" t="n">
         <v>46293</v>
@@ -6130,16 +6175,16 @@
     </row>
     <row r="84">
       <c r="A84" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="B84" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C84" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/58/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/66/2026 </t>
         </is>
       </c>
       <c r="D84" s="76" t="inlineStr">
@@ -6148,13 +6193,13 @@
         </is>
       </c>
       <c r="E84" s="77" t="n">
-        <v>787756603.1999999</v>
+        <v>3100200501.96</v>
       </c>
       <c r="F84" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="G84" s="78" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H84" s="76" t="inlineStr">
         <is>
@@ -6164,16 +6209,16 @@
     </row>
     <row r="85">
       <c r="A85" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="B85" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C85" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/59/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
         </is>
       </c>
       <c r="D85" s="76" t="inlineStr">
@@ -6182,13 +6227,13 @@
         </is>
       </c>
       <c r="E85" s="77" t="n">
-        <v>140859991.5</v>
+        <v>237729</v>
       </c>
       <c r="F85" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="G85" s="78" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H85" s="76" t="inlineStr">
         <is>
@@ -6207,7 +6252,7 @@
       </c>
       <c r="C86" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/66/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
         </is>
       </c>
       <c r="D86" s="76" t="inlineStr">
@@ -6216,7 +6261,7 @@
         </is>
       </c>
       <c r="E86" s="77" t="n">
-        <v>3100200501.96</v>
+        <v>142404425.58</v>
       </c>
       <c r="F86" s="75" t="n">
         <v>46296</v>
@@ -6250,7 +6295,7 @@
         </is>
       </c>
       <c r="E87" s="77" t="n">
-        <v>237729</v>
+        <v>270535602</v>
       </c>
       <c r="F87" s="75" t="n">
         <v>46296</v>
@@ -6275,7 +6320,7 @@
       </c>
       <c r="C88" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/68/2026 </t>
         </is>
       </c>
       <c r="D88" s="76" t="inlineStr">
@@ -6284,7 +6329,7 @@
         </is>
       </c>
       <c r="E88" s="77" t="n">
-        <v>142404425.58</v>
+        <v>28798491.06</v>
       </c>
       <c r="F88" s="75" t="n">
         <v>46296</v>
@@ -6304,24 +6349,24 @@
       </c>
       <c r="B89" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C89" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/13/2026</t>
         </is>
       </c>
       <c r="D89" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E89" s="77" t="n">
-        <v>270535602</v>
+        <v>872911811.2</v>
       </c>
       <c r="F89" s="75" t="n">
-        <v>46296</v>
+        <v>46295</v>
       </c>
       <c r="G89" s="78" t="n">
         <v>21</v>
@@ -6338,24 +6383,24 @@
       </c>
       <c r="B90" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C90" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/68/2026 </t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/14/2026</t>
         </is>
       </c>
       <c r="D90" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E90" s="77" t="n">
-        <v>28798491.06</v>
+        <v>302161780.8</v>
       </c>
       <c r="F90" s="75" t="n">
-        <v>46296</v>
+        <v>46295</v>
       </c>
       <c r="G90" s="78" t="n">
         <v>21</v>
@@ -6368,31 +6413,31 @@
     </row>
     <row r="91">
       <c r="A91" s="75" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="B91" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C91" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/13/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
         </is>
       </c>
       <c r="D91" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E91" s="77" t="n">
-        <v>872911811.2</v>
+        <v>18871809.6</v>
       </c>
       <c r="F91" s="75" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="G91" s="78" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H91" s="76" t="inlineStr">
         <is>
@@ -6402,31 +6447,31 @@
     </row>
     <row r="92">
       <c r="A92" s="75" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="B92" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C92" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/14/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
         </is>
       </c>
       <c r="D92" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E92" s="77" t="n">
-        <v>302161780.8</v>
+        <v>226017285.066</v>
       </c>
       <c r="F92" s="75" t="n">
-        <v>46295</v>
+        <v>46301</v>
       </c>
       <c r="G92" s="78" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="H92" s="76" t="inlineStr">
         <is>
@@ -6436,7 +6481,7 @@
     </row>
     <row r="93">
       <c r="A93" s="75" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B93" s="76" t="inlineStr">
         <is>
@@ -6445,7 +6490,7 @@
       </c>
       <c r="C93" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
         </is>
       </c>
       <c r="D93" s="76" t="inlineStr">
@@ -6454,13 +6499,13 @@
         </is>
       </c>
       <c r="E93" s="77" t="n">
-        <v>18871809.6</v>
+        <v>3356193038.598001</v>
       </c>
       <c r="F93" s="75" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="G93" s="78" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H93" s="76" t="inlineStr">
         <is>
@@ -6479,7 +6524,7 @@
       </c>
       <c r="C94" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
         </is>
       </c>
       <c r="D94" s="76" t="inlineStr">
@@ -6488,7 +6533,7 @@
         </is>
       </c>
       <c r="E94" s="77" t="n">
-        <v>226017285.066</v>
+        <v>767489805.3095999</v>
       </c>
       <c r="F94" s="75" t="n">
         <v>46301</v>
@@ -6513,7 +6558,7 @@
       </c>
       <c r="C95" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
         </is>
       </c>
       <c r="D95" s="76" t="inlineStr">
@@ -6522,7 +6567,7 @@
         </is>
       </c>
       <c r="E95" s="77" t="n">
-        <v>3356193038.598001</v>
+        <v>231565952.52</v>
       </c>
       <c r="F95" s="75" t="n">
         <v>46301</v>
@@ -6538,31 +6583,31 @@
     </row>
     <row r="96">
       <c r="A96" s="75" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="B96" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C96" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL COLD STORAGE_ PAS/15/2026</t>
         </is>
       </c>
       <c r="D96" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E96" s="77" t="n">
-        <v>767489805.3095999</v>
+        <v>541504029.249372</v>
       </c>
       <c r="F96" s="75" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G96" s="78" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H96" s="76" t="inlineStr">
         <is>
@@ -6572,31 +6617,31 @@
     </row>
     <row r="97">
       <c r="A97" s="75" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="B97" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C97" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL OFFICE/03/2026</t>
         </is>
       </c>
       <c r="D97" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E97" s="77" t="n">
-        <v>231565952.52</v>
+        <v>22509333.69</v>
       </c>
       <c r="F97" s="75" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G97" s="78" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H97" s="76" t="inlineStr">
         <is>
@@ -6606,16 +6651,16 @@
     </row>
     <row r="98">
       <c r="A98" s="75" t="n">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="B98" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C98" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL COLD STORAGE_ PAS/15/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-25/IX/2026</t>
         </is>
       </c>
       <c r="D98" s="76" t="inlineStr">
@@ -6624,13 +6669,13 @@
         </is>
       </c>
       <c r="E98" s="77" t="n">
-        <v>541504029.249372</v>
+        <v>816231500</v>
       </c>
       <c r="F98" s="75" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="G98" s="78" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H98" s="76" t="inlineStr">
         <is>
@@ -6640,16 +6685,16 @@
     </row>
     <row r="99">
       <c r="A99" s="75" t="n">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="B99" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C99" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL OFFICE/03/2026</t>
+          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
         </is>
       </c>
       <c r="D99" s="76" t="inlineStr">
@@ -6658,13 +6703,13 @@
         </is>
       </c>
       <c r="E99" s="77" t="n">
-        <v>22509333.69</v>
+        <v>11590259.94</v>
       </c>
       <c r="F99" s="75" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="G99" s="78" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H99" s="76" t="inlineStr">
         <is>
@@ -6678,21 +6723,21 @@
       </c>
       <c r="B100" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C100" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/12/2026</t>
+          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
         </is>
       </c>
       <c r="D100" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E100" s="77" t="n">
-        <v>802240</v>
+        <v>62675</v>
       </c>
       <c r="F100" s="75" t="n">
         <v>46305</v>
@@ -6712,21 +6757,21 @@
       </c>
       <c r="B101" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C101" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/13/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/27/IX/2026</t>
         </is>
       </c>
       <c r="D101" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E101" s="77" t="n">
-        <v>8632800</v>
+        <v>755480000</v>
       </c>
       <c r="F101" s="75" t="n">
         <v>46305</v>
@@ -6751,7 +6796,7 @@
       </c>
       <c r="C102" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/14/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/12/2026</t>
         </is>
       </c>
       <c r="D102" s="76" t="inlineStr">
@@ -6760,7 +6805,7 @@
         </is>
       </c>
       <c r="E102" s="77" t="n">
-        <v>967920</v>
+        <v>802240</v>
       </c>
       <c r="F102" s="75" t="n">
         <v>46305</v>
@@ -6785,7 +6830,7 @@
       </c>
       <c r="C103" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/15/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/13/2026</t>
         </is>
       </c>
       <c r="D103" s="76" t="inlineStr">
@@ -6794,7 +6839,7 @@
         </is>
       </c>
       <c r="E103" s="77" t="n">
-        <v>20509440</v>
+        <v>8632800</v>
       </c>
       <c r="F103" s="75" t="n">
         <v>46305</v>
@@ -6819,7 +6864,7 @@
       </c>
       <c r="C104" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/16/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/14/2026</t>
         </is>
       </c>
       <c r="D104" s="76" t="inlineStr">
@@ -6828,7 +6873,7 @@
         </is>
       </c>
       <c r="E104" s="77" t="n">
-        <v>2180000</v>
+        <v>967920</v>
       </c>
       <c r="F104" s="75" t="n">
         <v>46305</v>
@@ -6853,7 +6898,7 @@
       </c>
       <c r="C105" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/17/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/15/2026</t>
         </is>
       </c>
       <c r="D105" s="76" t="inlineStr">
@@ -6862,7 +6907,7 @@
         </is>
       </c>
       <c r="E105" s="77" t="n">
-        <v>540640</v>
+        <v>20509440</v>
       </c>
       <c r="F105" s="75" t="n">
         <v>46305</v>
@@ -6887,7 +6932,7 @@
       </c>
       <c r="C106" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/18/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/16/2026</t>
         </is>
       </c>
       <c r="D106" s="76" t="inlineStr">
@@ -6896,7 +6941,7 @@
         </is>
       </c>
       <c r="E106" s="77" t="n">
-        <v>47532720</v>
+        <v>2180000</v>
       </c>
       <c r="F106" s="75" t="n">
         <v>46305</v>
@@ -6921,7 +6966,7 @@
       </c>
       <c r="C107" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/19/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/17/2026</t>
         </is>
       </c>
       <c r="D107" s="76" t="inlineStr">
@@ -6930,7 +6975,7 @@
         </is>
       </c>
       <c r="E107" s="77" t="n">
-        <v>50794000</v>
+        <v>540640</v>
       </c>
       <c r="F107" s="75" t="n">
         <v>46305</v>
@@ -6950,12 +6995,12 @@
       </c>
       <c r="B108" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C108" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/18/2026</t>
         </is>
       </c>
       <c r="D108" s="76" t="inlineStr">
@@ -6964,7 +7009,7 @@
         </is>
       </c>
       <c r="E108" s="77" t="n">
-        <v>886307502.1920002</v>
+        <v>47532720</v>
       </c>
       <c r="F108" s="75" t="n">
         <v>46305</v>
@@ -6980,16 +7025,16 @@
     </row>
     <row r="109">
       <c r="A109" s="75" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="B109" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C109" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/19/2026</t>
         </is>
       </c>
       <c r="D109" s="76" t="inlineStr">
@@ -6998,13 +7043,13 @@
         </is>
       </c>
       <c r="E109" s="77" t="n">
-        <v>5676698527.872001</v>
+        <v>50794000</v>
       </c>
       <c r="F109" s="75" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="G109" s="78" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H109" s="76" t="inlineStr">
         <is>
@@ -7014,7 +7059,7 @@
     </row>
     <row r="110">
       <c r="A110" s="75" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="B110" s="76" t="inlineStr">
         <is>
@@ -7023,7 +7068,7 @@
       </c>
       <c r="C110" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
         </is>
       </c>
       <c r="D110" s="76" t="inlineStr">
@@ -7032,13 +7077,13 @@
         </is>
       </c>
       <c r="E110" s="77" t="n">
-        <v>564189103.6416</v>
+        <v>886307502.1920002</v>
       </c>
       <c r="F110" s="75" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="G110" s="78" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H110" s="76" t="inlineStr">
         <is>
@@ -7048,16 +7093,16 @@
     </row>
     <row r="111">
       <c r="A111" s="75" t="n">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="B111" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C111" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/56/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
         </is>
       </c>
       <c r="D111" s="76" t="inlineStr">
@@ -7066,13 +7111,13 @@
         </is>
       </c>
       <c r="E111" s="77" t="n">
-        <v>5535207.48</v>
+        <v>5676698527.872001</v>
       </c>
       <c r="F111" s="75" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="G111" s="78" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H111" s="76" t="inlineStr">
         <is>
@@ -7082,16 +7127,16 @@
     </row>
     <row r="112">
       <c r="A112" s="75" t="n">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="B112" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C112" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/57/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
         </is>
       </c>
       <c r="D112" s="76" t="inlineStr">
@@ -7100,13 +7145,13 @@
         </is>
       </c>
       <c r="E112" s="77" t="n">
-        <v>4392388.26</v>
+        <v>564189103.6416</v>
       </c>
       <c r="F112" s="75" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="G112" s="78" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H112" s="76" t="inlineStr">
         <is>
@@ -7125,7 +7170,7 @@
       </c>
       <c r="C113" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/58/2026</t>
+          <t>PT.PSI/PT.CASI/REP/56/2026</t>
         </is>
       </c>
       <c r="D113" s="76" t="inlineStr">
@@ -7134,7 +7179,7 @@
         </is>
       </c>
       <c r="E113" s="77" t="n">
-        <v>18129124.98186</v>
+        <v>5535207.48</v>
       </c>
       <c r="F113" s="75" t="n">
         <v>46304</v>
@@ -7159,7 +7204,7 @@
       </c>
       <c r="C114" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/59/2026</t>
+          <t>PT.PSI/PT.CASI/REP/57/2026</t>
         </is>
       </c>
       <c r="D114" s="76" t="inlineStr">
@@ -7168,7 +7213,7 @@
         </is>
       </c>
       <c r="E114" s="77" t="n">
-        <v>9884824431.36027</v>
+        <v>4392388.26</v>
       </c>
       <c r="F114" s="75" t="n">
         <v>46304</v>
@@ -7193,7 +7238,7 @@
       </c>
       <c r="C115" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/60/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/58/2026</t>
         </is>
       </c>
       <c r="D115" s="76" t="inlineStr">
@@ -7202,7 +7247,7 @@
         </is>
       </c>
       <c r="E115" s="77" t="n">
-        <v>700304033.0543</v>
+        <v>18129124.98186</v>
       </c>
       <c r="F115" s="75" t="n">
         <v>46304</v>
@@ -7227,7 +7272,7 @@
       </c>
       <c r="C116" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/61/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/59/2026</t>
         </is>
       </c>
       <c r="D116" s="76" t="inlineStr">
@@ -7236,7 +7281,7 @@
         </is>
       </c>
       <c r="E116" s="77" t="n">
-        <v>1147400616.7888</v>
+        <v>9884824431.36027</v>
       </c>
       <c r="F116" s="75" t="n">
         <v>46304</v>
@@ -7261,7 +7306,7 @@
       </c>
       <c r="C117" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/62/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/60/2026</t>
         </is>
       </c>
       <c r="D117" s="76" t="inlineStr">
@@ -7270,7 +7315,7 @@
         </is>
       </c>
       <c r="E117" s="77" t="n">
-        <v>4999029.5912</v>
+        <v>700304033.0543</v>
       </c>
       <c r="F117" s="75" t="n">
         <v>46304</v>
@@ -7295,7 +7340,7 @@
       </c>
       <c r="C118" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/63/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/61/2026</t>
         </is>
       </c>
       <c r="D118" s="76" t="inlineStr">
@@ -7304,7 +7349,7 @@
         </is>
       </c>
       <c r="E118" s="77" t="n">
-        <v>34933281.3146</v>
+        <v>1147400616.7888</v>
       </c>
       <c r="F118" s="75" t="n">
         <v>46304</v>
@@ -7329,7 +7374,7 @@
       </c>
       <c r="C119" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/64/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/62/2026</t>
         </is>
       </c>
       <c r="D119" s="76" t="inlineStr">
@@ -7338,7 +7383,7 @@
         </is>
       </c>
       <c r="E119" s="77" t="n">
-        <v>85105002.66900001</v>
+        <v>4999029.5912</v>
       </c>
       <c r="F119" s="75" t="n">
         <v>46304</v>
@@ -7363,7 +7408,7 @@
       </c>
       <c r="C120" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/65/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/63/2026</t>
         </is>
       </c>
       <c r="D120" s="76" t="inlineStr">
@@ -7372,7 +7417,7 @@
         </is>
       </c>
       <c r="E120" s="77" t="n">
-        <v>886098780.5445001</v>
+        <v>34933281.3146</v>
       </c>
       <c r="F120" s="75" t="n">
         <v>46304</v>
@@ -7397,7 +7442,7 @@
       </c>
       <c r="C121" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/66/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/64/2026</t>
         </is>
       </c>
       <c r="D121" s="76" t="inlineStr">
@@ -7406,7 +7451,7 @@
         </is>
       </c>
       <c r="E121" s="77" t="n">
-        <v>262631.43648</v>
+        <v>85105002.66900001</v>
       </c>
       <c r="F121" s="75" t="n">
         <v>46304</v>
@@ -7422,31 +7467,31 @@
     </row>
     <row r="122">
       <c r="A122" s="75" t="n">
-        <v>46312</v>
+        <v>46310</v>
       </c>
       <c r="B122" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C122" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
+          <t>PT.PSI/PT.CASI/FC-PS/65/2026</t>
         </is>
       </c>
       <c r="D122" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E122" s="77" t="n">
-        <v>1365520000</v>
+        <v>886098780.5445001</v>
       </c>
       <c r="F122" s="75" t="n">
-        <v>46312</v>
+        <v>46304</v>
       </c>
       <c r="G122" s="78" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H122" s="76" t="inlineStr">
         <is>
@@ -7456,31 +7501,31 @@
     </row>
     <row r="123">
       <c r="A123" s="75" t="n">
-        <v>46312</v>
+        <v>46310</v>
       </c>
       <c r="B123" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C123" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
+          <t>PT.PSI/PT.CASI/FC-PS/66/2026</t>
         </is>
       </c>
       <c r="D123" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="E123" s="77" t="n">
-        <v>9687031.199999999</v>
+        <v>262631.43648</v>
       </c>
       <c r="F123" s="75" t="n">
-        <v>46312</v>
+        <v>46304</v>
       </c>
       <c r="G123" s="78" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H123" s="76" t="inlineStr">
         <is>
@@ -7499,7 +7544,7 @@
       </c>
       <c r="C124" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
         </is>
       </c>
       <c r="D124" s="76" t="inlineStr">
@@ -7508,7 +7553,7 @@
         </is>
       </c>
       <c r="E124" s="77" t="n">
-        <v>1070726250</v>
+        <v>1365520000</v>
       </c>
       <c r="F124" s="75" t="n">
         <v>46312</v>
@@ -7533,7 +7578,7 @@
       </c>
       <c r="C125" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
         </is>
       </c>
       <c r="D125" s="76" t="inlineStr">
@@ -7542,7 +7587,7 @@
         </is>
       </c>
       <c r="E125" s="77" t="n">
-        <v>272700000</v>
+        <v>9687031.199999999</v>
       </c>
       <c r="F125" s="75" t="n">
         <v>46312</v>
@@ -7558,7 +7603,7 @@
     </row>
     <row r="126">
       <c r="A126" s="75" t="n">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="B126" s="76" t="inlineStr">
         <is>
@@ -7567,22 +7612,22 @@
       </c>
       <c r="C126" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
         </is>
       </c>
       <c r="D126" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E126" s="77" t="n">
-        <v>545818781.4912</v>
+        <v>1070726250</v>
       </c>
       <c r="F126" s="75" t="n">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="G126" s="78" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H126" s="76" t="inlineStr">
         <is>
@@ -7592,7 +7637,7 @@
     </row>
     <row r="127">
       <c r="A127" s="75" t="n">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="B127" s="76" t="inlineStr">
         <is>
@@ -7601,22 +7646,22 @@
       </c>
       <c r="C127" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
         </is>
       </c>
       <c r="D127" s="76" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E127" s="77" t="n">
-        <v>767367847.5204</v>
+        <v>272700000</v>
       </c>
       <c r="F127" s="75" t="n">
-        <v>46314</v>
+        <v>46312</v>
       </c>
       <c r="G127" s="78" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H127" s="76" t="inlineStr">
         <is>
@@ -7635,7 +7680,7 @@
       </c>
       <c r="C128" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
         </is>
       </c>
       <c r="D128" s="76" t="inlineStr">
@@ -7644,7 +7689,7 @@
         </is>
       </c>
       <c r="E128" s="77" t="n">
-        <v>4761468367.9458</v>
+        <v>545818781.4912</v>
       </c>
       <c r="F128" s="75" t="n">
         <v>46314</v>
@@ -7669,7 +7714,7 @@
       </c>
       <c r="C129" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
         </is>
       </c>
       <c r="D129" s="76" t="inlineStr">
@@ -7678,7 +7723,7 @@
         </is>
       </c>
       <c r="E129" s="77" t="n">
-        <v>442076465.292</v>
+        <v>767367847.5204</v>
       </c>
       <c r="F129" s="75" t="n">
         <v>46314</v>
@@ -7703,7 +7748,7 @@
       </c>
       <c r="C130" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
         </is>
       </c>
       <c r="D130" s="76" t="inlineStr">
@@ -7712,7 +7757,7 @@
         </is>
       </c>
       <c r="E130" s="77" t="n">
-        <v>444456984.744</v>
+        <v>4761468367.9458</v>
       </c>
       <c r="F130" s="75" t="n">
         <v>46314</v>
@@ -7728,7 +7773,7 @@
     </row>
     <row r="131">
       <c r="A131" s="75" t="n">
-        <v>46325</v>
+        <v>46314</v>
       </c>
       <c r="B131" s="76" t="inlineStr">
         <is>
@@ -7737,7 +7782,7 @@
       </c>
       <c r="C131" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/45/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
         </is>
       </c>
       <c r="D131" s="76" t="inlineStr">
@@ -7746,13 +7791,13 @@
         </is>
       </c>
       <c r="E131" s="77" t="n">
-        <v>337392787.2479999</v>
+        <v>442076465.292</v>
       </c>
       <c r="F131" s="75" t="n">
-        <v>46325</v>
+        <v>46314</v>
       </c>
       <c r="G131" s="78" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="H131" s="76" t="inlineStr">
         <is>
@@ -7762,7 +7807,7 @@
     </row>
     <row r="132">
       <c r="A132" s="75" t="n">
-        <v>46325</v>
+        <v>46314</v>
       </c>
       <c r="B132" s="76" t="inlineStr">
         <is>
@@ -7771,7 +7816,7 @@
       </c>
       <c r="C132" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/46/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
         </is>
       </c>
       <c r="D132" s="76" t="inlineStr">
@@ -7780,13 +7825,13 @@
         </is>
       </c>
       <c r="E132" s="77" t="n">
-        <v>8211508178.4966</v>
+        <v>444456984.744</v>
       </c>
       <c r="F132" s="75" t="n">
-        <v>46325</v>
+        <v>46314</v>
       </c>
       <c r="G132" s="78" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="H132" s="76" t="inlineStr">
         <is>
@@ -7805,7 +7850,7 @@
       </c>
       <c r="C133" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/47/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/45/2026</t>
         </is>
       </c>
       <c r="D133" s="76" t="inlineStr">
@@ -7814,7 +7859,7 @@
         </is>
       </c>
       <c r="E133" s="77" t="n">
-        <v>903022062.8508</v>
+        <v>337392787.2479999</v>
       </c>
       <c r="F133" s="75" t="n">
         <v>46325</v>
@@ -7839,7 +7884,7 @@
       </c>
       <c r="C134" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/48/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/46/2026</t>
         </is>
       </c>
       <c r="D134" s="76" t="inlineStr">
@@ -7848,7 +7893,7 @@
         </is>
       </c>
       <c r="E134" s="77" t="n">
-        <v>1912679476.3662</v>
+        <v>8211508178.4966</v>
       </c>
       <c r="F134" s="75" t="n">
         <v>46325</v>
@@ -7864,7 +7909,7 @@
     </row>
     <row r="135">
       <c r="A135" s="75" t="n">
-        <v>46328</v>
+        <v>46325</v>
       </c>
       <c r="B135" s="76" t="inlineStr">
         <is>
@@ -7873,7 +7918,7 @@
       </c>
       <c r="C135" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/49/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/47/2026</t>
         </is>
       </c>
       <c r="D135" s="76" t="inlineStr">
@@ -7882,13 +7927,13 @@
         </is>
       </c>
       <c r="E135" s="77" t="n">
-        <v>479734948.6272</v>
+        <v>903022062.8508</v>
       </c>
       <c r="F135" s="75" t="n">
-        <v>46328</v>
+        <v>46325</v>
       </c>
       <c r="G135" s="78" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="H135" s="76" t="inlineStr">
         <is>
@@ -7898,7 +7943,7 @@
     </row>
     <row r="136">
       <c r="A136" s="75" t="n">
-        <v>46328</v>
+        <v>46325</v>
       </c>
       <c r="B136" s="76" t="inlineStr">
         <is>
@@ -7907,7 +7952,7 @@
       </c>
       <c r="C136" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/50/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/48/2026</t>
         </is>
       </c>
       <c r="D136" s="76" t="inlineStr">
@@ -7916,13 +7961,13 @@
         </is>
       </c>
       <c r="E136" s="77" t="n">
-        <v>3340238430.648</v>
+        <v>1912679476.3662</v>
       </c>
       <c r="F136" s="75" t="n">
-        <v>46328</v>
+        <v>46325</v>
       </c>
       <c r="G136" s="78" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="H136" s="76" t="inlineStr">
         <is>
@@ -7941,7 +7986,7 @@
       </c>
       <c r="C137" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/51/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/49/2026</t>
         </is>
       </c>
       <c r="D137" s="76" t="inlineStr">
@@ -7950,7 +7995,7 @@
         </is>
       </c>
       <c r="E137" s="77" t="n">
-        <v>530510117.7436</v>
+        <v>479734948.6272</v>
       </c>
       <c r="F137" s="75" t="n">
         <v>46328</v>
@@ -7965,24 +8010,126 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="39" t="inlineStr">
+      <c r="A138" s="75" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B138" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C138" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/50/2026</t>
+        </is>
+      </c>
+      <c r="D138" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E138" s="77" t="n">
+        <v>3340238430.648</v>
+      </c>
+      <c r="F138" s="75" t="n">
+        <v>46328</v>
+      </c>
+      <c r="G138" s="78" t="n">
+        <v>53</v>
+      </c>
+      <c r="H138" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="75" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B139" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C139" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/51/2026</t>
+        </is>
+      </c>
+      <c r="D139" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E139" s="77" t="n">
+        <v>530510117.7436</v>
+      </c>
+      <c r="F139" s="75" t="n">
+        <v>46328</v>
+      </c>
+      <c r="G139" s="78" t="n">
+        <v>53</v>
+      </c>
+      <c r="H139" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="75" t="n">
+        <v>46335</v>
+      </c>
+      <c r="B140" s="76" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C140" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/SWC/01/2026</t>
+        </is>
+      </c>
+      <c r="D140" s="76" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="E140" s="77" t="n">
+        <v>2345778403.95195</v>
+      </c>
+      <c r="F140" s="75" t="n">
+        <v>46335</v>
+      </c>
+      <c r="G140" s="78" t="n">
+        <v>60</v>
+      </c>
+      <c r="H140" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="39" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B138" s="79" t="n"/>
-      <c r="C138" s="79" t="n"/>
-      <c r="D138" s="79" t="n"/>
-      <c r="E138" s="80">
-        <f>SUM(E5:E137)</f>
+      <c r="B141" s="79" t="n"/>
+      <c r="C141" s="79" t="n"/>
+      <c r="D141" s="79" t="n"/>
+      <c r="E141" s="80">
+        <f>SUM(E5:E140)</f>
         <v/>
       </c>
-      <c r="F138" s="79" t="n"/>
-      <c r="G138" s="79" t="n"/>
-      <c r="H138" s="79" t="n"/>
+      <c r="F141" s="79" t="n"/>
+      <c r="G141" s="79" t="n"/>
+      <c r="H141" s="79" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H138"/>
+  <autoFilter ref="A4:H141"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9997,10 +10144,10 @@
         <v>707040307.7369367</v>
       </c>
       <c r="BH13" s="86" t="n">
-        <v>2504545968.267117</v>
+        <v>4850324372.219067</v>
       </c>
       <c r="BI13" s="36" t="n">
-        <v>-1797505660.53018</v>
+        <v>-4143284064.48213</v>
       </c>
       <c r="BJ13" s="85" t="n">
         <v>1961988714.551999</v>
@@ -10030,22 +10177,22 @@
         <v>1346472409.038807</v>
       </c>
       <c r="BS13" s="85" t="n">
-        <v>4350483497.0188</v>
+        <v>6696261900.97075</v>
       </c>
       <c r="BT13" s="86" t="n">
         <v>0</v>
       </c>
       <c r="BU13" s="36" t="n">
-        <v>4350483497.0188</v>
+        <v>6696261900.97075</v>
       </c>
       <c r="BV13" s="40" t="n">
-        <v>156699786233.8369</v>
+        <v>159045564637.7889</v>
       </c>
       <c r="BW13" s="40" t="n">
-        <v>156699786233.8369</v>
+        <v>159045564637.7889</v>
       </c>
       <c r="BX13" s="40" t="n">
-        <v>3.0517578125e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -12263,10 +12410,10 @@
         <v>383873</v>
       </c>
       <c r="BH24" s="90" t="n">
-        <v>841116.51</v>
+        <v>887855.46</v>
       </c>
       <c r="BI24" s="91" t="n">
-        <v>-457243.51</v>
+        <v>-503982.46</v>
       </c>
       <c r="BJ24" s="89" t="n">
         <v>682905.23</v>
@@ -12296,19 +12443,19 @@
         <v>357749</v>
       </c>
       <c r="BS24" s="89" t="n">
-        <v>1026716</v>
+        <v>1073454.95</v>
       </c>
       <c r="BT24" s="90" t="n">
         <v>0</v>
       </c>
       <c r="BU24" s="91" t="n">
-        <v>1026716</v>
+        <v>1073454.95</v>
       </c>
       <c r="BV24" s="92" t="n">
-        <v>44171060.01</v>
+        <v>44217798.96</v>
       </c>
       <c r="BW24" s="92" t="n">
-        <v>44171060.01</v>
+        <v>44217798.96</v>
       </c>
       <c r="BX24" s="92" t="n">
         <v>0</v>
@@ -13396,25 +13543,25 @@
         <v>1473357319.28</v>
       </c>
       <c r="BQ30" s="86" t="n">
-        <v>0</v>
+        <v>1583364434.94</v>
       </c>
       <c r="BR30" s="36" t="n">
-        <v>1473357319.28</v>
+        <v>-110007115.6600001</v>
       </c>
       <c r="BS30" s="85" t="n">
-        <v>0</v>
+        <v>1583364434.94</v>
       </c>
       <c r="BT30" s="86" t="n">
         <v>0</v>
       </c>
       <c r="BU30" s="36" t="n">
-        <v>0</v>
+        <v>1583364434.94</v>
       </c>
       <c r="BV30" s="40" t="n">
-        <v>26335994391.13084</v>
+        <v>27919358826.07084</v>
       </c>
       <c r="BW30" s="40" t="n">
-        <v>26325994391.13084</v>
+        <v>27909358826.07084</v>
       </c>
       <c r="BX30" s="40" t="n">
         <v>10000000</v>
@@ -15198,25 +15345,25 @@
         <v>4632523</v>
       </c>
       <c r="BQ39" s="90" t="n">
-        <v>0</v>
+        <v>5015461</v>
       </c>
       <c r="BR39" s="91" t="n">
-        <v>4632523</v>
+        <v>-382938</v>
       </c>
       <c r="BS39" s="89" t="n">
-        <v>0</v>
+        <v>5015461</v>
       </c>
       <c r="BT39" s="90" t="n">
         <v>0</v>
       </c>
       <c r="BU39" s="91" t="n">
-        <v>0</v>
+        <v>5015461</v>
       </c>
       <c r="BV39" s="92" t="n">
-        <v>37060164.53</v>
+        <v>42075625.53</v>
       </c>
       <c r="BW39" s="92" t="n">
-        <v>37060164.53</v>
+        <v>42075625.53</v>
       </c>
       <c r="BX39" s="92" t="n">
         <v>0</v>
@@ -16581,20 +16728,20 @@
         </is>
       </c>
       <c r="B13" s="36" t="n">
-        <v>12042831153.57968</v>
+        <v>14388609557.53163</v>
       </c>
       <c r="C13" s="36" t="n">
         <v>8524152478.219052</v>
       </c>
       <c r="D13" s="97" t="n">
-        <v>3518678675.360625</v>
+        <v>5864457079.312575</v>
       </c>
       <c r="E13" s="98" t="n">
-        <v>0.7078196455229123</v>
+        <v>0.5924236420576954</v>
       </c>
       <c r="F13" s="99" t="inlineStr">
         <is>
-          <t>Partially uninvoiced</t>
+          <t>Many services uninvoiced</t>
         </is>
       </c>
     </row>
@@ -16653,16 +16800,16 @@
         </is>
       </c>
       <c r="B16" s="36" t="n">
-        <v>32148876834.4054</v>
+        <v>33732241269.3454</v>
       </c>
       <c r="C16" s="36" t="n">
         <v>46435325979.07043</v>
       </c>
       <c r="D16" s="100" t="n">
-        <v>-14286449144.66503</v>
+        <v>-12703084709.72503</v>
       </c>
       <c r="E16" s="98" t="n">
-        <v>1.44438408278624</v>
+        <v>1.376585848781685</v>
       </c>
       <c r="F16" s="99" t="inlineStr">
         <is>
@@ -16680,10 +16827,10 @@
         <v>0</v>
       </c>
       <c r="C17" s="36" t="n">
-        <v>21228658137.03918</v>
+        <v>25157800975.93113</v>
       </c>
       <c r="D17" s="100" t="n">
-        <v>-21228658137.03918</v>
+        <v>-25157800975.93113</v>
       </c>
       <c r="E17" s="98" t="n">
         <v>0</v>
@@ -16773,7 +16920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1115"/>
+  <dimension ref="A1:Q1118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -86526,46 +86673,60 @@
       </c>
       <c r="B1104" s="103" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C1104" s="103" t="n"/>
-      <c r="D1104" s="103" t="n"/>
-      <c r="E1104" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1104" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/SWC/01/2026</t>
+        </is>
+      </c>
+      <c r="D1104" s="104" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E1104" s="104" t="n">
+        <v>46335</v>
+      </c>
       <c r="F1104" s="103" t="n"/>
       <c r="G1104" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1104" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1104" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="J1104" s="103" t="n"/>
       <c r="K1104" s="104" t="n">
-        <v>46235</v>
+        <v>46143</v>
       </c>
       <c r="L1104" s="104" t="n">
-        <v>46265</v>
+        <v>46173</v>
       </c>
       <c r="M1104" s="105" t="n">
-        <v>2000000</v>
+        <v>46738.95</v>
       </c>
       <c r="N1104" s="105" t="n">
-        <v>777000000</v>
-      </c>
-      <c r="O1104" s="103" t="n"/>
-      <c r="P1104" s="103" t="n"/>
+        <v>2345778403.95195</v>
+      </c>
+      <c r="O1104" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1104" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1104" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -86580,18 +86741,26 @@
           <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
-      <c r="C1105" s="103" t="n"/>
-      <c r="D1105" s="103" t="n"/>
-      <c r="E1105" s="103" t="n"/>
+      <c r="C1105" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-25/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1105" s="104" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E1105" s="104" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1105" s="103" t="n"/>
       <c r="G1105" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1105" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Rental CS -U2</t>
         </is>
       </c>
       <c r="I1105" s="103" t="inlineStr">
@@ -86607,16 +86776,22 @@
         <v>46265</v>
       </c>
       <c r="M1105" s="105" t="n">
-        <v>2270000</v>
+        <v>2309000</v>
       </c>
       <c r="N1105" s="105" t="n">
-        <v>881895000</v>
-      </c>
-      <c r="O1105" s="103" t="n"/>
-      <c r="P1105" s="103" t="n"/>
+        <v>816231500</v>
+      </c>
+      <c r="O1105" s="103" t="n">
+        <v>-30</v>
+      </c>
+      <c r="P1105" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1105" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -86631,23 +86806,31 @@
           <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
-      <c r="C1106" s="103" t="n"/>
-      <c r="D1106" s="103" t="n"/>
-      <c r="E1106" s="103" t="n"/>
+      <c r="C1106" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1106" s="104" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E1106" s="104" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1106" s="103" t="n"/>
       <c r="G1106" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1106" s="103" t="inlineStr">
         <is>
-          <t>FC</t>
+          <t>Rental CS -U2</t>
         </is>
       </c>
       <c r="I1106" s="103" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1106" s="103" t="n"/>
@@ -86658,16 +86841,22 @@
         <v>46265</v>
       </c>
       <c r="M1106" s="105" t="n">
-        <v>3256990</v>
+        <v>506346</v>
       </c>
       <c r="N1106" s="105" t="n">
-        <v>13247943944.279</v>
-      </c>
-      <c r="O1106" s="103" t="n"/>
-      <c r="P1106" s="103" t="n"/>
+        <v>11590259.94</v>
+      </c>
+      <c r="O1106" s="103" t="n">
+        <v>-30</v>
+      </c>
+      <c r="P1106" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1106" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -86682,23 +86871,31 @@
           <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
-      <c r="C1107" s="103" t="n"/>
-      <c r="D1107" s="103" t="n"/>
-      <c r="E1107" s="103" t="n"/>
+      <c r="C1107" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1107" s="104" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E1107" s="104" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1107" s="103" t="n"/>
       <c r="G1107" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1107" s="103" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>Rental CS -U2</t>
         </is>
       </c>
       <c r="I1107" s="103" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1107" s="103" t="n"/>
@@ -86709,16 +86906,22 @@
         <v>46265</v>
       </c>
       <c r="M1107" s="105" t="n">
-        <v>140026</v>
+        <v>115</v>
       </c>
       <c r="N1107" s="105" t="n">
-        <v>1122459338.028</v>
-      </c>
-      <c r="O1107" s="103" t="n"/>
-      <c r="P1107" s="103" t="n"/>
+        <v>62675</v>
+      </c>
+      <c r="O1107" s="103" t="n">
+        <v>-30</v>
+      </c>
+      <c r="P1107" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1107" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -86730,21 +86933,29 @@
       </c>
       <c r="B1108" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1108" s="103" t="n"/>
-      <c r="D1108" s="103" t="n"/>
-      <c r="E1108" s="103" t="n"/>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C1108" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/27/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1108" s="104" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E1108" s="104" t="n">
+        <v>46305</v>
+      </c>
       <c r="F1108" s="103" t="n"/>
       <c r="G1108" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1108" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Rental CS -U2</t>
         </is>
       </c>
       <c r="I1108" s="103" t="inlineStr">
@@ -86760,16 +86971,22 @@
         <v>46265</v>
       </c>
       <c r="M1108" s="105" t="n">
-        <v>1654962.70767742</v>
+        <v>2200000</v>
       </c>
       <c r="N1108" s="105" t="n">
-        <v>593353779.5835853</v>
-      </c>
-      <c r="O1108" s="103" t="n"/>
-      <c r="P1108" s="103" t="n"/>
+        <v>755480000</v>
+      </c>
+      <c r="O1108" s="103" t="n">
+        <v>-30</v>
+      </c>
+      <c r="P1108" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1108" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -86781,7 +86998,7 @@
       </c>
       <c r="B1109" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1109" s="103" t="n"/>
@@ -86795,7 +87012,7 @@
       </c>
       <c r="H1109" s="103" t="inlineStr">
         <is>
-          <t>COMM</t>
+          <t>FC</t>
         </is>
       </c>
       <c r="I1109" s="103" t="inlineStr">
@@ -86811,10 +87028,10 @@
         <v>46265</v>
       </c>
       <c r="M1109" s="105" t="n">
-        <v>1878336</v>
+        <v>3256990</v>
       </c>
       <c r="N1109" s="105" t="n">
-        <v>7266583243.008001</v>
+        <v>13247943944.279</v>
       </c>
       <c r="O1109" s="103" t="n"/>
       <c r="P1109" s="103" t="n"/>
@@ -86832,7 +87049,7 @@
       </c>
       <c r="B1110" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1110" s="103" t="n"/>
@@ -86846,12 +87063,12 @@
       </c>
       <c r="H1110" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="I1110" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="J1110" s="103" t="n"/>
@@ -86862,10 +87079,10 @@
         <v>46265</v>
       </c>
       <c r="M1110" s="105" t="n">
-        <v>1660000</v>
+        <v>140026</v>
       </c>
       <c r="N1110" s="105" t="n">
-        <v>552691555.2</v>
+        <v>1122459338.028</v>
       </c>
       <c r="O1110" s="103" t="n"/>
       <c r="P1110" s="103" t="n"/>
@@ -86883,7 +87100,7 @@
       </c>
       <c r="B1111" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1111" s="103" t="n"/>
@@ -86913,10 +87130,10 @@
         <v>46265</v>
       </c>
       <c r="M1111" s="105" t="n">
-        <v>1660000</v>
+        <v>1654962.70767742</v>
       </c>
       <c r="N1111" s="105" t="n">
-        <v>552691555.2</v>
+        <v>593353779.5835853</v>
       </c>
       <c r="O1111" s="103" t="n"/>
       <c r="P1111" s="103" t="n"/>
@@ -86948,12 +87165,12 @@
       </c>
       <c r="H1112" s="103" t="inlineStr">
         <is>
-          <t>RENTAL</t>
+          <t>COMM</t>
         </is>
       </c>
       <c r="I1112" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tooling</t>
         </is>
       </c>
       <c r="J1112" s="103" t="n"/>
@@ -86964,10 +87181,10 @@
         <v>46265</v>
       </c>
       <c r="M1112" s="105" t="n">
-        <v>855000</v>
+        <v>1878336</v>
       </c>
       <c r="N1112" s="105" t="n">
-        <v>71167361.40000001</v>
+        <v>7266583243.008001</v>
       </c>
       <c r="O1112" s="103" t="n"/>
       <c r="P1112" s="103" t="n"/>
@@ -86999,7 +87216,7 @@
       </c>
       <c r="H1113" s="103" t="inlineStr">
         <is>
-          <t>RENTAL</t>
+          <t>RENTAL CS</t>
         </is>
       </c>
       <c r="I1113" s="103" t="inlineStr">
@@ -87015,10 +87232,10 @@
         <v>46265</v>
       </c>
       <c r="M1113" s="105" t="n">
-        <v>3600000</v>
+        <v>1660000</v>
       </c>
       <c r="N1113" s="105" t="n">
-        <v>299652048</v>
+        <v>552691555.2</v>
       </c>
       <c r="O1113" s="103" t="n"/>
       <c r="P1113" s="103" t="n"/>
@@ -87050,12 +87267,12 @@
       </c>
       <c r="H1114" s="103" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>RENTAL CS</t>
         </is>
       </c>
       <c r="I1114" s="103" t="inlineStr">
         <is>
-          <t>Tooling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1114" s="103" t="n"/>
@@ -87066,10 +87283,10 @@
         <v>46265</v>
       </c>
       <c r="M1114" s="105" t="n">
-        <v>855189</v>
+        <v>1660000</v>
       </c>
       <c r="N1114" s="105" t="n">
-        <v>5789714193.710999</v>
+        <v>552691555.2</v>
       </c>
       <c r="O1114" s="103" t="n"/>
       <c r="P1114" s="103" t="n"/>
@@ -87101,7 +87318,7 @@
       </c>
       <c r="H1115" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>RENTAL</t>
         </is>
       </c>
       <c r="I1115" s="103" t="inlineStr">
@@ -87117,10 +87334,10 @@
         <v>46265</v>
       </c>
       <c r="M1115" s="105" t="n">
-        <v>4000000</v>
+        <v>855000</v>
       </c>
       <c r="N1115" s="105" t="n">
-        <v>1605326400</v>
+        <v>71167361.40000001</v>
       </c>
       <c r="O1115" s="103" t="n"/>
       <c r="P1115" s="103" t="n"/>
@@ -87130,8 +87347,161 @@
         </is>
       </c>
     </row>
+    <row r="1116">
+      <c r="A1116" s="103" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B1116" s="103" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1116" s="103" t="n"/>
+      <c r="D1116" s="103" t="n"/>
+      <c r="E1116" s="103" t="n"/>
+      <c r="F1116" s="103" t="n"/>
+      <c r="G1116" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1116" s="103" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="I1116" s="103" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1116" s="103" t="n"/>
+      <c r="K1116" s="104" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1116" s="104" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1116" s="105" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="N1116" s="105" t="n">
+        <v>299652048</v>
+      </c>
+      <c r="O1116" s="103" t="n"/>
+      <c r="P1116" s="103" t="n"/>
+      <c r="Q1116" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="103" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B1117" s="103" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1117" s="103" t="n"/>
+      <c r="D1117" s="103" t="n"/>
+      <c r="E1117" s="103" t="n"/>
+      <c r="F1117" s="103" t="n"/>
+      <c r="G1117" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1117" s="103" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="I1117" s="103" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="J1117" s="103" t="n"/>
+      <c r="K1117" s="104" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1117" s="104" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1117" s="105" t="n">
+        <v>855189</v>
+      </c>
+      <c r="N1117" s="105" t="n">
+        <v>5789714193.710999</v>
+      </c>
+      <c r="O1117" s="103" t="n"/>
+      <c r="P1117" s="103" t="n"/>
+      <c r="Q1117" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="103" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B1118" s="103" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1118" s="103" t="n"/>
+      <c r="D1118" s="103" t="n"/>
+      <c r="E1118" s="103" t="n"/>
+      <c r="F1118" s="103" t="n"/>
+      <c r="G1118" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1118" s="103" t="inlineStr">
+        <is>
+          <t>RENTAL CS</t>
+        </is>
+      </c>
+      <c r="I1118" s="103" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1118" s="103" t="n"/>
+      <c r="K1118" s="104" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1118" s="104" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1118" s="105" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="N1118" s="105" t="n">
+        <v>1605326400</v>
+      </c>
+      <c r="O1118" s="103" t="n"/>
+      <c r="P1118" s="103" t="n"/>
+      <c r="Q1118" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q1115"/>
+  <autoFilter ref="A1:Q1118"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto-deploy AR dashboard 2026-09-10 15:56
</commit_message>
<xml_diff>
--- a/AR Movement Report.xlsx
+++ b/AR Movement Report.xlsx
@@ -1346,7 +1346,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data as of Thursday, 10 September 2026 - 15:54  |  Source: PSI AR Monitoring Master.xlsx</t>
+          <t>Data as of Thursday, 10 September 2026 - 15:56  |  Source: PSI AR Monitoring Master.xlsx</t>
         </is>
       </c>
     </row>
@@ -9243,10 +9243,10 @@
         <v>6114276610.20622</v>
       </c>
       <c r="BQ9" s="86" t="n">
-        <v>0</v>
+        <v>12748320195.01915</v>
       </c>
       <c r="BR9" s="36" t="n">
-        <v>6114276610.20622</v>
+        <v>-6634043584.81293</v>
       </c>
       <c r="BS9" s="85" t="n">
         <v>12771984527.48101</v>
@@ -9261,10 +9261,10 @@
         <v>120324890324.4144</v>
       </c>
       <c r="BW9" s="40" t="n">
-        <v>107576570129.3952</v>
+        <v>120324890324.4144</v>
       </c>
       <c r="BX9" s="40" t="n">
-        <v>12748320195.01917</v>
+        <v>1.52587890625e-05</v>
       </c>
     </row>
     <row r="10">
@@ -11509,10 +11509,10 @@
         <v>1929893.35</v>
       </c>
       <c r="BQ20" s="90" t="n">
-        <v>0</v>
+        <v>2848713.1</v>
       </c>
       <c r="BR20" s="91" t="n">
-        <v>1929893.35</v>
+        <v>-918819.7499999998</v>
       </c>
       <c r="BS20" s="89" t="n">
         <v>2888822.9</v>
@@ -11527,10 +11527,10 @@
         <v>35601356.752</v>
       </c>
       <c r="BW20" s="92" t="n">
-        <v>32752643.652</v>
+        <v>35601356.752</v>
       </c>
       <c r="BX20" s="92" t="n">
-        <v>2848713.099999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -16800,20 +16800,20 @@
         </is>
       </c>
       <c r="B16" s="36" t="n">
-        <v>33732241269.3454</v>
+        <v>46480561464.36454</v>
       </c>
       <c r="C16" s="36" t="n">
         <v>46435325979.07043</v>
       </c>
-      <c r="D16" s="100" t="n">
-        <v>-12703084709.72503</v>
+      <c r="D16" s="36" t="n">
+        <v>45235485.29411316</v>
       </c>
       <c r="E16" s="98" t="n">
-        <v>1.376585848781685</v>
+        <v>0.9990267870294812</v>
       </c>
       <c r="F16" s="99" t="inlineStr">
         <is>
-          <t>Catch-up: prior-month invoices issued</t>
+          <t>On track</t>
         </is>
       </c>
     </row>
@@ -86058,7 +86058,7 @@
         <v>46235</v>
       </c>
       <c r="L1094" s="104" t="n">
-        <v>38960</v>
+        <v>46265</v>
       </c>
       <c r="M1094" s="105" t="n">
         <v>19753.5</v>
@@ -86188,7 +86188,7 @@
         <v>46235</v>
       </c>
       <c r="L1096" s="104" t="n">
-        <v>38960</v>
+        <v>46265</v>
       </c>
       <c r="M1096" s="105" t="n">
         <v>1625945.55</v>
@@ -86253,7 +86253,7 @@
         <v>46235</v>
       </c>
       <c r="L1097" s="104" t="n">
-        <v>38960</v>
+        <v>46265</v>
       </c>
       <c r="M1097" s="105" t="n">
         <v>403173.25</v>
@@ -86318,7 +86318,7 @@
         <v>46235</v>
       </c>
       <c r="L1098" s="104" t="n">
-        <v>38960</v>
+        <v>46265</v>
       </c>
       <c r="M1098" s="105" t="n">
         <v>660572</v>
@@ -86383,7 +86383,7 @@
         <v>46235</v>
       </c>
       <c r="L1099" s="104" t="n">
-        <v>38960</v>
+        <v>46265</v>
       </c>
       <c r="M1099" s="105" t="n">
         <v>5756</v>
@@ -86448,7 +86448,7 @@
         <v>46235</v>
       </c>
       <c r="L1100" s="104" t="n">
-        <v>38960</v>
+        <v>46265</v>
       </c>
       <c r="M1100" s="105" t="n">
         <v>40223</v>
@@ -86513,7 +86513,7 @@
         <v>46235</v>
       </c>
       <c r="L1101" s="104" t="n">
-        <v>38960</v>
+        <v>46265</v>
       </c>
       <c r="M1101" s="105" t="n">
         <v>8166</v>
@@ -86578,7 +86578,7 @@
         <v>46235</v>
       </c>
       <c r="L1102" s="104" t="n">
-        <v>38960</v>
+        <v>46265</v>
       </c>
       <c r="M1102" s="105" t="n">
         <v>85023</v>
@@ -86643,7 +86643,7 @@
         <v>46235</v>
       </c>
       <c r="L1103" s="104" t="n">
-        <v>38960</v>
+        <v>46265</v>
       </c>
       <c r="M1103" s="105" t="n">
         <v>100.8</v>

</xml_diff>

<commit_message>
Auto-deploy AR dashboard 2026-09-11 17:01
</commit_message>
<xml_diff>
--- a/AR Movement Report.xlsx
+++ b/AR Movement Report.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$141</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daily Projection'!$A$4:$H$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Raw Data'!$A$1:$Q$1120</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1346,7 +1346,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data as of Friday, 11 September 2026 - 11:24  |  Source: PSI AR Monitoring Master.xlsx</t>
+          <t>Data as of Friday, 11 September 2026 - 17:00  |  Source: PSI AR Monitoring Master.xlsx</t>
         </is>
       </c>
     </row>
@@ -1383,13 +1383,13 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="9" t="n">
-        <v>130823792442.2642</v>
+        <v>125895200651.4888</v>
       </c>
       <c r="B7" s="10" t="n"/>
       <c r="C7" s="10" t="n"/>
       <c r="D7" s="11" t="n"/>
       <c r="E7" s="12" t="n">
-        <v>120701636512.7412</v>
+        <v>115773044721.9659</v>
       </c>
       <c r="F7" s="10" t="n"/>
       <c r="G7" s="11" t="n"/>
@@ -1440,14 +1440,14 @@
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="19" t="n">
-        <v>69090575311.29965</v>
+        <v>71428566763.53233</v>
       </c>
       <c r="B12" s="10" t="n"/>
       <c r="C12" s="10" t="n"/>
       <c r="D12" s="10" t="n"/>
       <c r="E12" s="11" t="n"/>
       <c r="F12" s="20" t="n">
-        <v>61733217130.96454</v>
+        <v>54466633887.95654</v>
       </c>
       <c r="G12" s="10" t="n"/>
       <c r="H12" s="10" t="n"/>
@@ -1507,15 +1507,15 @@
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="26" t="n">
-        <v>25157800975.93113</v>
+        <v>33521800123.54803</v>
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="27" t="n">
-        <v>3860725277.3516</v>
+        <v>9886732972.735821</v>
       </c>
       <c r="D17" s="11" t="n"/>
       <c r="E17" s="28" t="n">
-        <v>173958157025.0544</v>
+        <v>179984164720.4387</v>
       </c>
       <c r="F17" s="11" t="n"/>
       <c r="G17" s="29" t="n">
@@ -1667,7 +1667,7 @@
         <v>14599340397.24238</v>
       </c>
       <c r="C25" s="35" t="n">
-        <v>6619361474.967806</v>
+        <v>593353779.5835853</v>
       </c>
       <c r="D25" s="36" t="n">
         <v>0</v>
@@ -1824,10 +1824,10 @@
         </is>
       </c>
       <c r="B30" s="34" t="n">
-        <v>40393298882.67303</v>
+        <v>48757298030.28992</v>
       </c>
       <c r="C30" s="35" t="n">
-        <v>16137826356.519</v>
+        <v>8871243113.511</v>
       </c>
       <c r="D30" s="36" t="n">
         <v>0</v>
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="B41" s="49" t="n">
-        <v>62643302081.16026</v>
+        <v>64981293533.39294</v>
       </c>
       <c r="C41" s="49" t="n">
         <v>6447273230.139372</v>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B42" s="36" t="n">
-        <v>27426700719.026</v>
+        <v>20160117476.018</v>
       </c>
       <c r="C42" s="36" t="n">
         <v>3674882699.383585</v>
@@ -2166,7 +2166,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="57" t="n">
-        <v>16137826356.519</v>
+        <v>8871243113.511</v>
       </c>
       <c r="J49" s="57">
         <f>SUM(B49:I49)</f>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="51">
       <c r="A51" s="58" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="B51" s="36" t="n">
         <v>0</v>
@@ -2217,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="D51" s="36" t="n">
-        <v>6026007695.38422</v>
+        <v>0</v>
       </c>
       <c r="E51" s="36" t="n">
         <v>0</v>
@@ -2232,7 +2232,7 @@
         <v>0</v>
       </c>
       <c r="I51" s="36" t="n">
-        <v>0</v>
+        <v>326635952.80968</v>
       </c>
       <c r="J51" s="37">
         <f>SUM(B51:I51)</f>
@@ -2241,7 +2241,7 @@
     </row>
     <row r="52">
       <c r="A52" s="58" t="n">
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="B52" s="36" t="n">
         <v>0</v>
@@ -2265,7 +2265,7 @@
         <v>0</v>
       </c>
       <c r="I52" s="36" t="n">
-        <v>326635952.80968</v>
+        <v>570800977.7184</v>
       </c>
       <c r="J52" s="37">
         <f>SUM(B52:I52)</f>
@@ -2274,7 +2274,7 @@
     </row>
     <row r="53">
       <c r="A53" s="58" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="B53" s="36" t="n">
         <v>0</v>
@@ -2283,7 +2283,7 @@
         <v>0</v>
       </c>
       <c r="D53" s="36" t="n">
-        <v>0</v>
+        <v>88268914.82200001</v>
       </c>
       <c r="E53" s="36" t="n">
         <v>0</v>
@@ -2298,7 +2298,7 @@
         <v>0</v>
       </c>
       <c r="I53" s="36" t="n">
-        <v>570800977.7184</v>
+        <v>0</v>
       </c>
       <c r="J53" s="37">
         <f>SUM(B53:I53)</f>
@@ -2307,7 +2307,7 @@
     </row>
     <row r="54">
       <c r="A54" s="58" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="B54" s="36" t="n">
         <v>0</v>
@@ -2316,10 +2316,10 @@
         <v>0</v>
       </c>
       <c r="D54" s="36" t="n">
-        <v>88268914.82200001</v>
+        <v>0</v>
       </c>
       <c r="E54" s="36" t="n">
-        <v>0</v>
+        <v>841876812.3200001</v>
       </c>
       <c r="F54" s="36" t="n">
         <v>0</v>
@@ -2340,7 +2340,7 @@
     </row>
     <row r="55">
       <c r="A55" s="58" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B55" s="36" t="n">
         <v>0</v>
@@ -2352,7 +2352,7 @@
         <v>0</v>
       </c>
       <c r="E55" s="36" t="n">
-        <v>841876812.3200001</v>
+        <v>1613076622.9</v>
       </c>
       <c r="F55" s="36" t="n">
         <v>0</v>
@@ -2372,145 +2372,145 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="58" t="n">
-        <v>46293</v>
-      </c>
-      <c r="B56" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C56" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E56" s="36" t="n">
-        <v>1613076622.9</v>
-      </c>
-      <c r="F56" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" s="37">
-        <f>SUM(B56:I56)</f>
+      <c r="A56" s="59" t="inlineStr">
+        <is>
+          <t>Total upcoming in September</t>
+        </is>
+      </c>
+      <c r="B56" s="40">
+        <f>SUM(B50:B55)</f>
         <v/>
       </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="59" t="inlineStr">
-        <is>
-          <t>Total upcoming in September</t>
-        </is>
-      </c>
-      <c r="B57" s="40">
-        <f>SUM(B50:B56)</f>
+      <c r="C56" s="40">
+        <f>SUM(C50:C55)</f>
         <v/>
       </c>
-      <c r="C57" s="40">
-        <f>SUM(C50:C56)</f>
+      <c r="D56" s="40">
+        <f>SUM(D50:D55)</f>
         <v/>
       </c>
-      <c r="D57" s="40">
-        <f>SUM(D50:D56)</f>
+      <c r="E56" s="40">
+        <f>SUM(E50:E55)</f>
         <v/>
       </c>
-      <c r="E57" s="40">
-        <f>SUM(E50:E56)</f>
+      <c r="F56" s="40">
+        <f>SUM(F50:F55)</f>
         <v/>
       </c>
-      <c r="F57" s="40">
-        <f>SUM(F50:F56)</f>
+      <c r="G56" s="40">
+        <f>SUM(G50:G55)</f>
         <v/>
       </c>
-      <c r="G57" s="40">
-        <f>SUM(G50:G56)</f>
+      <c r="H56" s="40">
+        <f>SUM(H50:H55)</f>
         <v/>
       </c>
-      <c r="H57" s="40">
-        <f>SUM(H50:H56)</f>
+      <c r="I56" s="40">
+        <f>SUM(I50:I55)</f>
         <v/>
       </c>
-      <c r="I57" s="40">
-        <f>SUM(I50:I56)</f>
+      <c r="J56" s="40">
+        <f>SUM(J50:J55)</f>
         <v/>
       </c>
-      <c r="J57" s="40">
-        <f>SUM(J50:J56)</f>
+    </row>
+    <row r="58" ht="38" customHeight="1">
+      <c r="A58" s="55" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="B58" s="55" t="inlineStr">
+        <is>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C58" s="55" t="inlineStr">
+        <is>
+          <t>PT Alam Semesta Agro</t>
+        </is>
+      </c>
+      <c r="D58" s="55" t="inlineStr">
+        <is>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="E58" s="55" t="inlineStr">
+        <is>
+          <t>PT Bayer Indonesia</t>
+        </is>
+      </c>
+      <c r="F58" s="55" t="inlineStr">
+        <is>
+          <t>Nuziveedu</t>
+        </is>
+      </c>
+      <c r="G58" s="55" t="inlineStr">
+        <is>
+          <t>Bioseed</t>
+        </is>
+      </c>
+      <c r="H58" s="55" t="inlineStr">
+        <is>
+          <t>PT East West Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="I58" s="55" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="J58" s="55" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="58" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B59" s="36" t="n">
+        <v>3542176749.6</v>
+      </c>
+      <c r="C59" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="36" t="n">
+        <v>1175073592</v>
+      </c>
+      <c r="E59" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="37">
+        <f>SUM(B59:I59)</f>
         <v/>
-      </c>
-    </row>
-    <row r="59" ht="38" customHeight="1">
-      <c r="A59" s="55" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="B59" s="55" t="inlineStr">
-        <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C59" s="55" t="inlineStr">
-        <is>
-          <t>PT Alam Semesta Agro</t>
-        </is>
-      </c>
-      <c r="D59" s="55" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="E59" s="55" t="inlineStr">
-        <is>
-          <t>PT Bayer Indonesia</t>
-        </is>
-      </c>
-      <c r="F59" s="55" t="inlineStr">
-        <is>
-          <t>Nuziveedu</t>
-        </is>
-      </c>
-      <c r="G59" s="55" t="inlineStr">
-        <is>
-          <t>Bioseed</t>
-        </is>
-      </c>
-      <c r="H59" s="55" t="inlineStr">
-        <is>
-          <t>PT East West Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="I59" s="55" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="J59" s="55" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="58" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="B60" s="36" t="n">
-        <v>3542176749.6</v>
+        <v>0</v>
       </c>
       <c r="C60" s="36" t="n">
         <v>0</v>
       </c>
       <c r="D60" s="36" t="n">
-        <v>1175073592</v>
+        <v>0</v>
       </c>
       <c r="E60" s="36" t="n">
         <v>0</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="I60" s="36" t="n">
-        <v>0</v>
+        <v>18871809.6</v>
       </c>
       <c r="J60" s="37">
         <f>SUM(B60:I60)</f>
@@ -2534,7 +2534,7 @@
     </row>
     <row r="61">
       <c r="A61" s="58" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B61" s="36" t="n">
         <v>0</v>
@@ -2558,7 +2558,7 @@
         <v>0</v>
       </c>
       <c r="I61" s="36" t="n">
-        <v>18871809.6</v>
+        <v>4581266081.493601</v>
       </c>
       <c r="J61" s="37">
         <f>SUM(B61:I61)</f>
@@ -2567,7 +2567,7 @@
     </row>
     <row r="62">
       <c r="A62" s="58" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="B62" s="36" t="n">
         <v>0</v>
@@ -2576,7 +2576,7 @@
         <v>0</v>
       </c>
       <c r="D62" s="36" t="n">
-        <v>0</v>
+        <v>564013362.9393721</v>
       </c>
       <c r="E62" s="36" t="n">
         <v>0</v>
@@ -2591,7 +2591,7 @@
         <v>0</v>
       </c>
       <c r="I62" s="36" t="n">
-        <v>4581266081.493601</v>
+        <v>0</v>
       </c>
       <c r="J62" s="37">
         <f>SUM(B62:I62)</f>
@@ -2600,16 +2600,16 @@
     </row>
     <row r="63">
       <c r="A63" s="58" t="n">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="B63" s="36" t="n">
-        <v>0</v>
+        <v>1583364434.94</v>
       </c>
       <c r="C63" s="36" t="n">
         <v>0</v>
       </c>
       <c r="D63" s="36" t="n">
-        <v>564013362.9393721</v>
+        <v>0</v>
       </c>
       <c r="E63" s="36" t="n">
         <v>0</v>
@@ -2621,10 +2621,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="36" t="n">
-        <v>0</v>
+        <v>131959760</v>
       </c>
       <c r="I63" s="36" t="n">
-        <v>0</v>
+        <v>886307502.1920002</v>
       </c>
       <c r="J63" s="37">
         <f>SUM(B63:I63)</f>
@@ -2633,10 +2633,10 @@
     </row>
     <row r="64">
       <c r="A64" s="58" t="n">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B64" s="36" t="n">
-        <v>1583364434.94</v>
+        <v>0</v>
       </c>
       <c r="C64" s="36" t="n">
         <v>0</v>
@@ -2654,10 +2654,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="36" t="n">
-        <v>131959760</v>
+        <v>0</v>
       </c>
       <c r="I64" s="36" t="n">
-        <v>886307502.1920002</v>
+        <v>6240887631.5136</v>
       </c>
       <c r="J64" s="37">
         <f>SUM(B64:I64)</f>
@@ -2666,7 +2666,7 @@
     </row>
     <row r="65">
       <c r="A65" s="58" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="B65" s="36" t="n">
         <v>0</v>
@@ -2675,7 +2675,7 @@
         <v>0</v>
       </c>
       <c r="D65" s="36" t="n">
-        <v>0</v>
+        <v>12771984527.48101</v>
       </c>
       <c r="E65" s="36" t="n">
         <v>0</v>
@@ -2690,7 +2690,7 @@
         <v>0</v>
       </c>
       <c r="I65" s="36" t="n">
-        <v>6240887631.5136</v>
+        <v>0</v>
       </c>
       <c r="J65" s="37">
         <f>SUM(B65:I65)</f>
@@ -2699,7 +2699,7 @@
     </row>
     <row r="66">
       <c r="A66" s="58" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="B66" s="36" t="n">
         <v>0</v>
@@ -2708,7 +2708,7 @@
         <v>0</v>
       </c>
       <c r="D66" s="36" t="n">
-        <v>12771984527.48101</v>
+        <v>0</v>
       </c>
       <c r="E66" s="36" t="n">
         <v>0</v>
@@ -2723,7 +2723,7 @@
         <v>0</v>
       </c>
       <c r="I66" s="36" t="n">
-        <v>0</v>
+        <v>2718633281.2</v>
       </c>
       <c r="J66" s="37">
         <f>SUM(B66:I66)</f>
@@ -2732,7 +2732,7 @@
     </row>
     <row r="67">
       <c r="A67" s="58" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B67" s="36" t="n">
         <v>0</v>
@@ -2756,7 +2756,7 @@
         <v>0</v>
       </c>
       <c r="I67" s="36" t="n">
-        <v>2718633281.2</v>
+        <v>6961188446.9934</v>
       </c>
       <c r="J67" s="37">
         <f>SUM(B67:I67)</f>
@@ -2765,7 +2765,7 @@
     </row>
     <row r="68">
       <c r="A68" s="58" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="B68" s="36" t="n">
         <v>0</v>
@@ -2789,7 +2789,7 @@
         <v>0</v>
       </c>
       <c r="I68" s="36" t="n">
-        <v>6961188446.9934</v>
+        <v>11364602504.9616</v>
       </c>
       <c r="J68" s="37">
         <f>SUM(B68:I68)</f>
@@ -2797,136 +2797,136 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="58" t="n">
-        <v>46325</v>
-      </c>
-      <c r="B69" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C69" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F69" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="G69" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="H69" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="I69" s="36" t="n">
-        <v>11364602504.9616</v>
-      </c>
-      <c r="J69" s="37">
-        <f>SUM(B69:I69)</f>
+      <c r="A69" s="59" t="inlineStr">
+        <is>
+          <t>Total upcoming in October</t>
+        </is>
+      </c>
+      <c r="B69" s="40">
+        <f>SUM(B59:B68)</f>
         <v/>
       </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="59" t="inlineStr">
-        <is>
-          <t>Total upcoming in October</t>
-        </is>
-      </c>
-      <c r="B70" s="40">
-        <f>SUM(B60:B69)</f>
+      <c r="C69" s="40">
+        <f>SUM(C59:C68)</f>
         <v/>
       </c>
-      <c r="C70" s="40">
-        <f>SUM(C60:C69)</f>
+      <c r="D69" s="40">
+        <f>SUM(D59:D68)</f>
         <v/>
       </c>
-      <c r="D70" s="40">
-        <f>SUM(D60:D69)</f>
+      <c r="E69" s="40">
+        <f>SUM(E59:E68)</f>
         <v/>
       </c>
-      <c r="E70" s="40">
-        <f>SUM(E60:E69)</f>
+      <c r="F69" s="40">
+        <f>SUM(F59:F68)</f>
         <v/>
       </c>
-      <c r="F70" s="40">
-        <f>SUM(F60:F69)</f>
+      <c r="G69" s="40">
+        <f>SUM(G59:G68)</f>
         <v/>
       </c>
-      <c r="G70" s="40">
-        <f>SUM(G60:G69)</f>
+      <c r="H69" s="40">
+        <f>SUM(H59:H68)</f>
         <v/>
       </c>
-      <c r="H70" s="40">
-        <f>SUM(H60:H69)</f>
+      <c r="I69" s="40">
+        <f>SUM(I59:I68)</f>
         <v/>
       </c>
-      <c r="I70" s="40">
-        <f>SUM(I60:I69)</f>
+      <c r="J69" s="40">
+        <f>SUM(J59:J68)</f>
         <v/>
       </c>
-      <c r="J70" s="40">
-        <f>SUM(J60:J69)</f>
+    </row>
+    <row r="71" ht="38" customHeight="1">
+      <c r="A71" s="55" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="B71" s="55" t="inlineStr">
+        <is>
+          <t>PT Advanta Seeds Indonesia</t>
+        </is>
+      </c>
+      <c r="C71" s="55" t="inlineStr">
+        <is>
+          <t>PT Alam Semesta Agro</t>
+        </is>
+      </c>
+      <c r="D71" s="55" t="inlineStr">
+        <is>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="E71" s="55" t="inlineStr">
+        <is>
+          <t>PT Bayer Indonesia</t>
+        </is>
+      </c>
+      <c r="F71" s="55" t="inlineStr">
+        <is>
+          <t>Nuziveedu</t>
+        </is>
+      </c>
+      <c r="G71" s="55" t="inlineStr">
+        <is>
+          <t>Bioseed</t>
+        </is>
+      </c>
+      <c r="H71" s="55" t="inlineStr">
+        <is>
+          <t>PT East West Seed Indonesia</t>
+        </is>
+      </c>
+      <c r="I71" s="55" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="J71" s="55" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="58" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B72" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C72" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" s="36" t="n">
+        <v>4350483497.0188</v>
+      </c>
+      <c r="J72" s="37">
+        <f>SUM(B72:I72)</f>
         <v/>
-      </c>
-    </row>
-    <row r="72" ht="38" customHeight="1">
-      <c r="A72" s="55" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="B72" s="55" t="inlineStr">
-        <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C72" s="55" t="inlineStr">
-        <is>
-          <t>PT Alam Semesta Agro</t>
-        </is>
-      </c>
-      <c r="D72" s="55" t="inlineStr">
-        <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="E72" s="55" t="inlineStr">
-        <is>
-          <t>PT Bayer Indonesia</t>
-        </is>
-      </c>
-      <c r="F72" s="55" t="inlineStr">
-        <is>
-          <t>Nuziveedu</t>
-        </is>
-      </c>
-      <c r="G72" s="55" t="inlineStr">
-        <is>
-          <t>Bioseed</t>
-        </is>
-      </c>
-      <c r="H72" s="55" t="inlineStr">
-        <is>
-          <t>PT East West Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="I72" s="55" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="J72" s="55" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="58" t="n">
-        <v>46328</v>
+        <v>46335</v>
       </c>
       <c r="B73" s="36" t="n">
         <v>0</v>
@@ -2950,7 +2950,7 @@
         <v>0</v>
       </c>
       <c r="I73" s="36" t="n">
-        <v>4350483497.0188</v>
+        <v>2345778403.95195</v>
       </c>
       <c r="J73" s="37">
         <f>SUM(B73:I73)</f>
@@ -2959,7 +2959,7 @@
     </row>
     <row r="74">
       <c r="A74" s="58" t="n">
-        <v>46335</v>
+        <v>46336</v>
       </c>
       <c r="B74" s="36" t="n">
         <v>0</v>
@@ -2983,7 +2983,7 @@
         <v>0</v>
       </c>
       <c r="I74" s="36" t="n">
-        <v>2345778403.95195</v>
+        <v>8363999147.6169</v>
       </c>
       <c r="J74" s="37">
         <f>SUM(B74:I74)</f>
@@ -2997,39 +2997,39 @@
         </is>
       </c>
       <c r="B75" s="40">
-        <f>SUM(B73:B74)</f>
+        <f>SUM(B72:B74)</f>
         <v/>
       </c>
       <c r="C75" s="40">
-        <f>SUM(C73:C74)</f>
+        <f>SUM(C72:C74)</f>
         <v/>
       </c>
       <c r="D75" s="40">
-        <f>SUM(D73:D74)</f>
+        <f>SUM(D72:D74)</f>
         <v/>
       </c>
       <c r="E75" s="40">
-        <f>SUM(E73:E74)</f>
+        <f>SUM(E72:E74)</f>
         <v/>
       </c>
       <c r="F75" s="40">
-        <f>SUM(F73:F74)</f>
+        <f>SUM(F72:F74)</f>
         <v/>
       </c>
       <c r="G75" s="40">
-        <f>SUM(G73:G74)</f>
+        <f>SUM(G72:G74)</f>
         <v/>
       </c>
       <c r="H75" s="40">
-        <f>SUM(H73:H74)</f>
+        <f>SUM(H72:H74)</f>
         <v/>
       </c>
       <c r="I75" s="40">
-        <f>SUM(I73:I74)</f>
+        <f>SUM(I72:I74)</f>
         <v/>
       </c>
       <c r="J75" s="40">
-        <f>SUM(J73:J74)</f>
+        <f>SUM(J72:J74)</f>
         <v/>
       </c>
     </row>
@@ -3355,7 +3355,7 @@
         </is>
       </c>
       <c r="C12" s="36" t="n">
-        <v>6026007695.38422</v>
+        <v>0</v>
       </c>
       <c r="D12" s="36" t="n">
         <v>593353779.5835853</v>
@@ -3405,7 +3405,7 @@
         </is>
       </c>
       <c r="C14" s="36" t="n">
-        <v>37627950998.65303</v>
+        <v>45991950146.26993</v>
       </c>
       <c r="D14" s="36" t="n">
         <v>2765347884.02</v>
@@ -3430,7 +3430,7 @@
         </is>
       </c>
       <c r="C15" s="36" t="n">
-        <v>13056297436.719</v>
+        <v>5789714193.710999</v>
       </c>
       <c r="D15" s="36" t="n">
         <v>3081528919.8</v>
@@ -3478,7 +3478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H141"/>
+  <dimension ref="A1:H139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5037,11 +5037,11 @@
       <c r="C49" s="72" t="n"/>
       <c r="D49" s="72" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E49" s="73" t="n">
-        <v>7266583243.008001</v>
+        <v>552691555.2</v>
       </c>
       <c r="F49" s="71" t="n"/>
       <c r="G49" s="74" t="n">
@@ -5097,7 +5097,7 @@
         </is>
       </c>
       <c r="E51" s="73" t="n">
-        <v>552691555.2</v>
+        <v>71167361.40000001</v>
       </c>
       <c r="F51" s="71" t="n"/>
       <c r="G51" s="74" t="n">
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="E52" s="73" t="n">
-        <v>71167361.40000001</v>
+        <v>299652048</v>
       </c>
       <c r="F52" s="71" t="n"/>
       <c r="G52" s="74" t="n">
@@ -5149,11 +5149,11 @@
       <c r="C53" s="72" t="n"/>
       <c r="D53" s="72" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E53" s="73" t="n">
-        <v>299652048</v>
+        <v>5789714193.710999</v>
       </c>
       <c r="F53" s="71" t="n"/>
       <c r="G53" s="74" t="n">
@@ -5177,11 +5177,11 @@
       <c r="C54" s="72" t="n"/>
       <c r="D54" s="72" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E54" s="73" t="n">
-        <v>5789714193.710999</v>
+        <v>1605326400</v>
       </c>
       <c r="F54" s="71" t="n"/>
       <c r="G54" s="74" t="n">
@@ -5194,36 +5194,42 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="71" t="n">
-        <v>46276</v>
-      </c>
-      <c r="B55" s="72" t="inlineStr">
+      <c r="A55" s="75" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B55" s="76" t="inlineStr">
         <is>
           <t>PT Syngenta Indonesia</t>
         </is>
       </c>
-      <c r="C55" s="72" t="n"/>
-      <c r="D55" s="72" t="inlineStr">
+      <c r="C55" s="76" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/RENTAL/33/2026</t>
+        </is>
+      </c>
+      <c r="D55" s="76" t="inlineStr">
         <is>
           <t>Rental</t>
         </is>
       </c>
-      <c r="E55" s="73" t="n">
-        <v>1605326400</v>
-      </c>
-      <c r="F55" s="71" t="n"/>
-      <c r="G55" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="72" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+      <c r="E55" s="77" t="n">
+        <v>27842793.22</v>
+      </c>
+      <c r="F55" s="75" t="n">
+        <v>46278</v>
+      </c>
+      <c r="G55" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="H55" s="76" t="inlineStr">
+        <is>
+          <t>Future</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="75" t="n">
-        <v>46278</v>
+        <v>46284</v>
       </c>
       <c r="B56" s="76" t="inlineStr">
         <is>
@@ -5232,22 +5238,22 @@
       </c>
       <c r="C56" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/33/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
         </is>
       </c>
       <c r="D56" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E56" s="77" t="n">
-        <v>27842793.22</v>
+        <v>326395903.6008</v>
       </c>
       <c r="F56" s="75" t="n">
-        <v>46278</v>
+        <v>46284</v>
       </c>
       <c r="G56" s="78" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H56" s="76" t="inlineStr">
         <is>
@@ -5257,16 +5263,16 @@
     </row>
     <row r="57">
       <c r="A57" s="75" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="B57" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C57" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/49/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
         </is>
       </c>
       <c r="D57" s="76" t="inlineStr">
@@ -5275,13 +5281,13 @@
         </is>
       </c>
       <c r="E57" s="77" t="n">
-        <v>3981599123.659349</v>
+        <v>240049.20888</v>
       </c>
       <c r="F57" s="75" t="n">
-        <v>46276</v>
+        <v>46284</v>
       </c>
       <c r="G57" s="78" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H57" s="76" t="inlineStr">
         <is>
@@ -5291,16 +5297,16 @@
     </row>
     <row r="58">
       <c r="A58" s="75" t="n">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="B58" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C58" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/50/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
         </is>
       </c>
       <c r="D58" s="76" t="inlineStr">
@@ -5309,13 +5315,13 @@
         </is>
       </c>
       <c r="E58" s="77" t="n">
-        <v>1542175442.6694</v>
+        <v>570800977.7184</v>
       </c>
       <c r="F58" s="75" t="n">
-        <v>46276</v>
+        <v>46286</v>
       </c>
       <c r="G58" s="78" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H58" s="76" t="inlineStr">
         <is>
@@ -5325,7 +5331,7 @@
     </row>
     <row r="59">
       <c r="A59" s="75" t="n">
-        <v>46282</v>
+        <v>46289</v>
       </c>
       <c r="B59" s="76" t="inlineStr">
         <is>
@@ -5334,7 +5340,7 @@
       </c>
       <c r="C59" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/51/2026</t>
+          <t>PT.PSI/PT.CASI/REP/53/2026</t>
         </is>
       </c>
       <c r="D59" s="76" t="inlineStr">
@@ -5343,13 +5349,13 @@
         </is>
       </c>
       <c r="E59" s="77" t="n">
-        <v>487978078.30875</v>
+        <v>36849832.74</v>
       </c>
       <c r="F59" s="75" t="n">
-        <v>46276</v>
+        <v>46285</v>
       </c>
       <c r="G59" s="78" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="H59" s="76" t="inlineStr">
         <is>
@@ -5359,7 +5365,7 @@
     </row>
     <row r="60">
       <c r="A60" s="75" t="n">
-        <v>46282</v>
+        <v>46289</v>
       </c>
       <c r="B60" s="76" t="inlineStr">
         <is>
@@ -5368,7 +5374,7 @@
       </c>
       <c r="C60" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/52/2026</t>
+          <t>PT.PSI/PT.CASI/REP/54/2026</t>
         </is>
       </c>
       <c r="D60" s="76" t="inlineStr">
@@ -5377,13 +5383,13 @@
         </is>
       </c>
       <c r="E60" s="77" t="n">
-        <v>14255050.74672</v>
+        <v>31988016.36</v>
       </c>
       <c r="F60" s="75" t="n">
-        <v>46276</v>
+        <v>46285</v>
       </c>
       <c r="G60" s="78" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="H60" s="76" t="inlineStr">
         <is>
@@ -5393,16 +5399,16 @@
     </row>
     <row r="61">
       <c r="A61" s="75" t="n">
-        <v>46284</v>
+        <v>46289</v>
       </c>
       <c r="B61" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C61" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/32/2026</t>
+          <t>PT.PSI/PT.CASI/REP/55/2026</t>
         </is>
       </c>
       <c r="D61" s="76" t="inlineStr">
@@ -5411,13 +5417,13 @@
         </is>
       </c>
       <c r="E61" s="77" t="n">
-        <v>326395903.6008</v>
+        <v>19431065.722</v>
       </c>
       <c r="F61" s="75" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="G61" s="78" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H61" s="76" t="inlineStr">
         <is>
@@ -5427,16 +5433,16 @@
     </row>
     <row r="62">
       <c r="A62" s="75" t="n">
-        <v>46284</v>
+        <v>46292</v>
       </c>
       <c r="B62" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C62" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/33/2026</t>
+          <t>PT.PSI/PT.BI/FC/43/2026</t>
         </is>
       </c>
       <c r="D62" s="76" t="inlineStr">
@@ -5445,13 +5451,13 @@
         </is>
       </c>
       <c r="E62" s="77" t="n">
-        <v>240049.20888</v>
+        <v>103679056</v>
       </c>
       <c r="F62" s="75" t="n">
-        <v>46284</v>
+        <v>46292</v>
       </c>
       <c r="G62" s="78" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="H62" s="76" t="inlineStr">
         <is>
@@ -5461,16 +5467,16 @@
     </row>
     <row r="63">
       <c r="A63" s="75" t="n">
-        <v>46286</v>
+        <v>46292</v>
       </c>
       <c r="B63" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C63" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/34/2026</t>
+          <t>PT.PSI/PT.BI/FC/44/2026</t>
         </is>
       </c>
       <c r="D63" s="76" t="inlineStr">
@@ -5479,13 +5485,13 @@
         </is>
       </c>
       <c r="E63" s="77" t="n">
-        <v>570800977.7184</v>
+        <v>92863095</v>
       </c>
       <c r="F63" s="75" t="n">
-        <v>46286</v>
+        <v>46292</v>
       </c>
       <c r="G63" s="78" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="H63" s="76" t="inlineStr">
         <is>
@@ -5495,16 +5501,16 @@
     </row>
     <row r="64">
       <c r="A64" s="75" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="B64" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C64" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/53/2026</t>
+          <t>PT.PSI/PT.BI/FC/45/2026</t>
         </is>
       </c>
       <c r="D64" s="76" t="inlineStr">
@@ -5513,13 +5519,13 @@
         </is>
       </c>
       <c r="E64" s="77" t="n">
-        <v>36849832.74</v>
+        <v>17392258</v>
       </c>
       <c r="F64" s="75" t="n">
-        <v>46285</v>
+        <v>46292</v>
       </c>
       <c r="G64" s="78" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H64" s="76" t="inlineStr">
         <is>
@@ -5529,16 +5535,16 @@
     </row>
     <row r="65">
       <c r="A65" s="75" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="B65" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C65" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/54/2026</t>
+          <t>PT.PSI/PT.BI/FC/46/2026</t>
         </is>
       </c>
       <c r="D65" s="76" t="inlineStr">
@@ -5547,13 +5553,13 @@
         </is>
       </c>
       <c r="E65" s="77" t="n">
-        <v>31988016.36</v>
+        <v>197734556.5</v>
       </c>
       <c r="F65" s="75" t="n">
-        <v>46285</v>
+        <v>46292</v>
       </c>
       <c r="G65" s="78" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H65" s="76" t="inlineStr">
         <is>
@@ -5563,16 +5569,16 @@
     </row>
     <row r="66">
       <c r="A66" s="75" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="B66" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Bayer Indonesia</t>
         </is>
       </c>
       <c r="C66" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/55/2026</t>
+          <t>PT.PSI/PT.BI/FC/47/2026</t>
         </is>
       </c>
       <c r="D66" s="76" t="inlineStr">
@@ -5581,13 +5587,13 @@
         </is>
       </c>
       <c r="E66" s="77" t="n">
-        <v>19431065.722</v>
+        <v>254755628.4</v>
       </c>
       <c r="F66" s="75" t="n">
-        <v>46285</v>
+        <v>46292</v>
       </c>
       <c r="G66" s="78" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H66" s="76" t="inlineStr">
         <is>
@@ -5606,7 +5612,7 @@
       </c>
       <c r="C67" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/43/2026</t>
+          <t>PT.PSI/PT.BI/FC/48/2026</t>
         </is>
       </c>
       <c r="D67" s="76" t="inlineStr">
@@ -5615,7 +5621,7 @@
         </is>
       </c>
       <c r="E67" s="77" t="n">
-        <v>103679056</v>
+        <v>10599160</v>
       </c>
       <c r="F67" s="75" t="n">
         <v>46292</v>
@@ -5640,7 +5646,7 @@
       </c>
       <c r="C68" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/44/2026</t>
+          <t>PT.PSI/PT.BI/FC/49/2026</t>
         </is>
       </c>
       <c r="D68" s="76" t="inlineStr">
@@ -5649,7 +5655,7 @@
         </is>
       </c>
       <c r="E68" s="77" t="n">
-        <v>92863095</v>
+        <v>54405006.5</v>
       </c>
       <c r="F68" s="75" t="n">
         <v>46292</v>
@@ -5674,7 +5680,7 @@
       </c>
       <c r="C69" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/45/2026</t>
+          <t>PT.PSI/PT.BI/FC/50/2026</t>
         </is>
       </c>
       <c r="D69" s="76" t="inlineStr">
@@ -5683,7 +5689,7 @@
         </is>
       </c>
       <c r="E69" s="77" t="n">
-        <v>17392258</v>
+        <v>1075481.2</v>
       </c>
       <c r="F69" s="75" t="n">
         <v>46292</v>
@@ -5708,7 +5714,7 @@
       </c>
       <c r="C70" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/46/2026</t>
+          <t>PT.PSI/PT.BI/FC/51/2026</t>
         </is>
       </c>
       <c r="D70" s="76" t="inlineStr">
@@ -5717,7 +5723,7 @@
         </is>
       </c>
       <c r="E70" s="77" t="n">
-        <v>197734556.5</v>
+        <v>803447.72</v>
       </c>
       <c r="F70" s="75" t="n">
         <v>46292</v>
@@ -5742,7 +5748,7 @@
       </c>
       <c r="C71" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/47/2026</t>
+          <t>PT.PSI/PT.BI/FC/52/2026</t>
         </is>
       </c>
       <c r="D71" s="76" t="inlineStr">
@@ -5751,7 +5757,7 @@
         </is>
       </c>
       <c r="E71" s="77" t="n">
-        <v>254755628.4</v>
+        <v>7250789</v>
       </c>
       <c r="F71" s="75" t="n">
         <v>46292</v>
@@ -5776,7 +5782,7 @@
       </c>
       <c r="C72" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/48/2026</t>
+          <t>PT.PSI/PT.BI/FC/53/2026</t>
         </is>
       </c>
       <c r="D72" s="76" t="inlineStr">
@@ -5785,7 +5791,7 @@
         </is>
       </c>
       <c r="E72" s="77" t="n">
-        <v>10599160</v>
+        <v>101318334</v>
       </c>
       <c r="F72" s="75" t="n">
         <v>46292</v>
@@ -5801,7 +5807,7 @@
     </row>
     <row r="73">
       <c r="A73" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B73" s="76" t="inlineStr">
         <is>
@@ -5810,7 +5816,7 @@
       </c>
       <c r="C73" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/49/2026</t>
+          <t>PT.PSI/PT.BI/FC/54/2026</t>
         </is>
       </c>
       <c r="D73" s="76" t="inlineStr">
@@ -5819,13 +5825,13 @@
         </is>
       </c>
       <c r="E73" s="77" t="n">
-        <v>54405006.5</v>
+        <v>156400274.1</v>
       </c>
       <c r="F73" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G73" s="78" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H73" s="76" t="inlineStr">
         <is>
@@ -5835,7 +5841,7 @@
     </row>
     <row r="74">
       <c r="A74" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B74" s="76" t="inlineStr">
         <is>
@@ -5844,7 +5850,7 @@
       </c>
       <c r="C74" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/50/2026</t>
+          <t>PT.PSI/PT.BI/FC/55/2026</t>
         </is>
       </c>
       <c r="D74" s="76" t="inlineStr">
@@ -5853,13 +5859,13 @@
         </is>
       </c>
       <c r="E74" s="77" t="n">
-        <v>1075481.2</v>
+        <v>50838199.5</v>
       </c>
       <c r="F74" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G74" s="78" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H74" s="76" t="inlineStr">
         <is>
@@ -5869,7 +5875,7 @@
     </row>
     <row r="75">
       <c r="A75" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B75" s="76" t="inlineStr">
         <is>
@@ -5878,7 +5884,7 @@
       </c>
       <c r="C75" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/51/2026</t>
+          <t>PT.PSI/PT.BI/FC/56/2026</t>
         </is>
       </c>
       <c r="D75" s="76" t="inlineStr">
@@ -5887,13 +5893,13 @@
         </is>
       </c>
       <c r="E75" s="77" t="n">
-        <v>803447.72</v>
+        <v>376884765.6</v>
       </c>
       <c r="F75" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G75" s="78" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H75" s="76" t="inlineStr">
         <is>
@@ -5903,7 +5909,7 @@
     </row>
     <row r="76">
       <c r="A76" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B76" s="76" t="inlineStr">
         <is>
@@ -5912,7 +5918,7 @@
       </c>
       <c r="C76" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/52/2026</t>
+          <t>PT.PSI/PT.BI/FC/57/2026</t>
         </is>
       </c>
       <c r="D76" s="76" t="inlineStr">
@@ -5921,13 +5927,13 @@
         </is>
       </c>
       <c r="E76" s="77" t="n">
-        <v>7250789</v>
+        <v>100336789</v>
       </c>
       <c r="F76" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G76" s="78" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H76" s="76" t="inlineStr">
         <is>
@@ -5937,7 +5943,7 @@
     </row>
     <row r="77">
       <c r="A77" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="B77" s="76" t="inlineStr">
         <is>
@@ -5946,7 +5952,7 @@
       </c>
       <c r="C77" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/53/2026</t>
+          <t>PT.PSI/PT.BI/FC/58/2026</t>
         </is>
       </c>
       <c r="D77" s="76" t="inlineStr">
@@ -5955,13 +5961,13 @@
         </is>
       </c>
       <c r="E77" s="77" t="n">
-        <v>101318334</v>
+        <v>787756603.1999999</v>
       </c>
       <c r="F77" s="75" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="G77" s="78" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H77" s="76" t="inlineStr">
         <is>
@@ -5980,7 +5986,7 @@
       </c>
       <c r="C78" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/54/2026</t>
+          <t>PT.PSI/PT.BI/FC/59/2026</t>
         </is>
       </c>
       <c r="D78" s="76" t="inlineStr">
@@ -5989,7 +5995,7 @@
         </is>
       </c>
       <c r="E78" s="77" t="n">
-        <v>156400274.1</v>
+        <v>140859991.5</v>
       </c>
       <c r="F78" s="75" t="n">
         <v>46293</v>
@@ -6005,16 +6011,16 @@
     </row>
     <row r="79">
       <c r="A79" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="B79" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C79" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/55/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/66/2026 </t>
         </is>
       </c>
       <c r="D79" s="76" t="inlineStr">
@@ -6023,13 +6029,13 @@
         </is>
       </c>
       <c r="E79" s="77" t="n">
-        <v>50838199.5</v>
+        <v>3100200501.96</v>
       </c>
       <c r="F79" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="G79" s="78" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H79" s="76" t="inlineStr">
         <is>
@@ -6039,16 +6045,16 @@
     </row>
     <row r="80">
       <c r="A80" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="B80" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C80" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/56/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
         </is>
       </c>
       <c r="D80" s="76" t="inlineStr">
@@ -6057,13 +6063,13 @@
         </is>
       </c>
       <c r="E80" s="77" t="n">
-        <v>376884765.6</v>
+        <v>237729</v>
       </c>
       <c r="F80" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="G80" s="78" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H80" s="76" t="inlineStr">
         <is>
@@ -6073,16 +6079,16 @@
     </row>
     <row r="81">
       <c r="A81" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="B81" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C81" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/57/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
         </is>
       </c>
       <c r="D81" s="76" t="inlineStr">
@@ -6091,13 +6097,13 @@
         </is>
       </c>
       <c r="E81" s="77" t="n">
-        <v>100336789</v>
+        <v>142404425.58</v>
       </c>
       <c r="F81" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="G81" s="78" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H81" s="76" t="inlineStr">
         <is>
@@ -6107,16 +6113,16 @@
     </row>
     <row r="82">
       <c r="A82" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="B82" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C82" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/58/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
         </is>
       </c>
       <c r="D82" s="76" t="inlineStr">
@@ -6125,13 +6131,13 @@
         </is>
       </c>
       <c r="E82" s="77" t="n">
-        <v>787756603.1999999</v>
+        <v>270535602</v>
       </c>
       <c r="F82" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="G82" s="78" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H82" s="76" t="inlineStr">
         <is>
@@ -6141,16 +6147,16 @@
     </row>
     <row r="83">
       <c r="A83" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="B83" s="76" t="inlineStr">
         <is>
-          <t>PT Bayer Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C83" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.BI/FC/59/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.ASI/FC/68/2026 </t>
         </is>
       </c>
       <c r="D83" s="76" t="inlineStr">
@@ -6159,13 +6165,13 @@
         </is>
       </c>
       <c r="E83" s="77" t="n">
-        <v>140859991.5</v>
+        <v>28798491.06</v>
       </c>
       <c r="F83" s="75" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="G83" s="78" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H83" s="76" t="inlineStr">
         <is>
@@ -6179,24 +6185,24 @@
       </c>
       <c r="B84" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C84" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/66/2026 </t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/13/2026</t>
         </is>
       </c>
       <c r="D84" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E84" s="77" t="n">
-        <v>3100200501.96</v>
+        <v>872911811.2</v>
       </c>
       <c r="F84" s="75" t="n">
-        <v>46296</v>
+        <v>46295</v>
       </c>
       <c r="G84" s="78" t="n">
         <v>20</v>
@@ -6213,24 +6219,24 @@
       </c>
       <c r="B85" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C85" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
+          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/14/2026</t>
         </is>
       </c>
       <c r="D85" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E85" s="77" t="n">
-        <v>237729</v>
+        <v>302161780.8</v>
       </c>
       <c r="F85" s="75" t="n">
-        <v>46296</v>
+        <v>46295</v>
       </c>
       <c r="G85" s="78" t="n">
         <v>20</v>
@@ -6243,31 +6249,31 @@
     </row>
     <row r="86">
       <c r="A86" s="75" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="B86" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C86" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
+          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
         </is>
       </c>
       <c r="D86" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E86" s="77" t="n">
-        <v>142404425.58</v>
+        <v>18871809.6</v>
       </c>
       <c r="F86" s="75" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G86" s="78" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="H86" s="76" t="inlineStr">
         <is>
@@ -6277,16 +6283,16 @@
     </row>
     <row r="87">
       <c r="A87" s="75" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="B87" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C87" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/67/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
         </is>
       </c>
       <c r="D87" s="76" t="inlineStr">
@@ -6295,13 +6301,13 @@
         </is>
       </c>
       <c r="E87" s="77" t="n">
-        <v>270535602</v>
+        <v>226017285.066</v>
       </c>
       <c r="F87" s="75" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="G87" s="78" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H87" s="76" t="inlineStr">
         <is>
@@ -6311,16 +6317,16 @@
     </row>
     <row r="88">
       <c r="A88" s="75" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="B88" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C88" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.ASI/FC/68/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
         </is>
       </c>
       <c r="D88" s="76" t="inlineStr">
@@ -6329,13 +6335,13 @@
         </is>
       </c>
       <c r="E88" s="77" t="n">
-        <v>28798491.06</v>
+        <v>3356193038.598001</v>
       </c>
       <c r="F88" s="75" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="G88" s="78" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H88" s="76" t="inlineStr">
         <is>
@@ -6345,31 +6351,31 @@
     </row>
     <row r="89">
       <c r="A89" s="75" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="B89" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C89" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/13/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
         </is>
       </c>
       <c r="D89" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E89" s="77" t="n">
-        <v>872911811.2</v>
+        <v>767489805.3095999</v>
       </c>
       <c r="F89" s="75" t="n">
-        <v>46295</v>
+        <v>46301</v>
       </c>
       <c r="G89" s="78" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H89" s="76" t="inlineStr">
         <is>
@@ -6379,31 +6385,31 @@
     </row>
     <row r="90">
       <c r="A90" s="75" t="n">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="B90" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C90" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL WAREHOUSE/14/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
         </is>
       </c>
       <c r="D90" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E90" s="77" t="n">
-        <v>302161780.8</v>
+        <v>231565952.52</v>
       </c>
       <c r="F90" s="75" t="n">
-        <v>46295</v>
+        <v>46301</v>
       </c>
       <c r="G90" s="78" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H90" s="76" t="inlineStr">
         <is>
@@ -6413,16 +6419,16 @@
     </row>
     <row r="91">
       <c r="A91" s="75" t="n">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="B91" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C91" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL/34/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL COLD STORAGE_ PAS/15/2026</t>
         </is>
       </c>
       <c r="D91" s="76" t="inlineStr">
@@ -6431,13 +6437,13 @@
         </is>
       </c>
       <c r="E91" s="77" t="n">
-        <v>18871809.6</v>
+        <v>541504029.249372</v>
       </c>
       <c r="F91" s="75" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="G91" s="78" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="H91" s="76" t="inlineStr">
         <is>
@@ -6447,31 +6453,31 @@
     </row>
     <row r="92">
       <c r="A92" s="75" t="n">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="B92" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C92" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS/35/2026</t>
+          <t>PT.PSI/PT.CASI/RENTAL OFFICE/03/2026</t>
         </is>
       </c>
       <c r="D92" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E92" s="77" t="n">
-        <v>226017285.066</v>
+        <v>22509333.69</v>
       </c>
       <c r="F92" s="75" t="n">
-        <v>46301</v>
+        <v>46298</v>
       </c>
       <c r="G92" s="78" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H92" s="76" t="inlineStr">
         <is>
@@ -6481,31 +6487,31 @@
     </row>
     <row r="93">
       <c r="A93" s="75" t="n">
-        <v>46301</v>
+        <v>46305</v>
       </c>
       <c r="B93" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C93" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/36/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-25/IX/2026</t>
         </is>
       </c>
       <c r="D93" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E93" s="77" t="n">
-        <v>3356193038.598001</v>
+        <v>816231500</v>
       </c>
       <c r="F93" s="75" t="n">
-        <v>46301</v>
+        <v>46305</v>
       </c>
       <c r="G93" s="78" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H93" s="76" t="inlineStr">
         <is>
@@ -6515,31 +6521,31 @@
     </row>
     <row r="94">
       <c r="A94" s="75" t="n">
-        <v>46301</v>
+        <v>46305</v>
       </c>
       <c r="B94" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C94" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
+          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
         </is>
       </c>
       <c r="D94" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E94" s="77" t="n">
-        <v>767489805.3095999</v>
+        <v>11590259.94</v>
       </c>
       <c r="F94" s="75" t="n">
-        <v>46301</v>
+        <v>46305</v>
       </c>
       <c r="G94" s="78" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H94" s="76" t="inlineStr">
         <is>
@@ -6549,31 +6555,31 @@
     </row>
     <row r="95">
       <c r="A95" s="75" t="n">
-        <v>46301</v>
+        <v>46305</v>
       </c>
       <c r="B95" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C95" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/37/2026</t>
+          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
         </is>
       </c>
       <c r="D95" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E95" s="77" t="n">
-        <v>231565952.52</v>
+        <v>62675</v>
       </c>
       <c r="F95" s="75" t="n">
-        <v>46301</v>
+        <v>46305</v>
       </c>
       <c r="G95" s="78" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H95" s="76" t="inlineStr">
         <is>
@@ -6583,16 +6589,16 @@
     </row>
     <row r="96">
       <c r="A96" s="75" t="n">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="B96" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C96" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL COLD STORAGE_ PAS/15/2026</t>
+          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/27/IX/2026</t>
         </is>
       </c>
       <c r="D96" s="76" t="inlineStr">
@@ -6601,13 +6607,13 @@
         </is>
       </c>
       <c r="E96" s="77" t="n">
-        <v>541504029.249372</v>
+        <v>755480000</v>
       </c>
       <c r="F96" s="75" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="G96" s="78" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H96" s="76" t="inlineStr">
         <is>
@@ -6617,31 +6623,31 @@
     </row>
     <row r="97">
       <c r="A97" s="75" t="n">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="B97" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C97" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/RENTAL OFFICE/03/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/12/2026</t>
         </is>
       </c>
       <c r="D97" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E97" s="77" t="n">
-        <v>22509333.69</v>
+        <v>802240</v>
       </c>
       <c r="F97" s="75" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="G97" s="78" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H97" s="76" t="inlineStr">
         <is>
@@ -6655,21 +6661,21 @@
       </c>
       <c r="B98" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C98" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/RENTAL-CS-PAS2-25/IX/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/13/2026</t>
         </is>
       </c>
       <c r="D98" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E98" s="77" t="n">
-        <v>816231500</v>
+        <v>8632800</v>
       </c>
       <c r="F98" s="75" t="n">
         <v>46305</v>
@@ -6689,21 +6695,21 @@
       </c>
       <c r="B99" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C99" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/14/2026</t>
         </is>
       </c>
       <c r="D99" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E99" s="77" t="n">
-        <v>11590259.94</v>
+        <v>967920</v>
       </c>
       <c r="F99" s="75" t="n">
         <v>46305</v>
@@ -6723,21 +6729,21 @@
       </c>
       <c r="B100" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C100" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/HDL-CS-PAS2/26/IX/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/15/2026</t>
         </is>
       </c>
       <c r="D100" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E100" s="77" t="n">
-        <v>62675</v>
+        <v>20509440</v>
       </c>
       <c r="F100" s="75" t="n">
         <v>46305</v>
@@ -6757,21 +6763,21 @@
       </c>
       <c r="B101" s="76" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
+          <t>PT East West Seed Indonesia</t>
         </is>
       </c>
       <c r="C101" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.ASI/RENTAL-CS 3-PAS2/27/IX/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/16/2026</t>
         </is>
       </c>
       <c r="D101" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E101" s="77" t="n">
-        <v>755480000</v>
+        <v>2180000</v>
       </c>
       <c r="F101" s="75" t="n">
         <v>46305</v>
@@ -6796,7 +6802,7 @@
       </c>
       <c r="C102" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/12/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/17/2026</t>
         </is>
       </c>
       <c r="D102" s="76" t="inlineStr">
@@ -6805,7 +6811,7 @@
         </is>
       </c>
       <c r="E102" s="77" t="n">
-        <v>802240</v>
+        <v>540640</v>
       </c>
       <c r="F102" s="75" t="n">
         <v>46305</v>
@@ -6830,7 +6836,7 @@
       </c>
       <c r="C103" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/13/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/18/2026</t>
         </is>
       </c>
       <c r="D103" s="76" t="inlineStr">
@@ -6839,7 +6845,7 @@
         </is>
       </c>
       <c r="E103" s="77" t="n">
-        <v>8632800</v>
+        <v>47532720</v>
       </c>
       <c r="F103" s="75" t="n">
         <v>46305</v>
@@ -6864,7 +6870,7 @@
       </c>
       <c r="C104" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/14/2026</t>
+          <t>PT.PSI/PT.EWINDO_LMB/19/2026</t>
         </is>
       </c>
       <c r="D104" s="76" t="inlineStr">
@@ -6873,7 +6879,7 @@
         </is>
       </c>
       <c r="E104" s="77" t="n">
-        <v>967920</v>
+        <v>50794000</v>
       </c>
       <c r="F104" s="75" t="n">
         <v>46305</v>
@@ -6893,12 +6899,12 @@
       </c>
       <c r="B105" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C105" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/15/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
         </is>
       </c>
       <c r="D105" s="76" t="inlineStr">
@@ -6907,7 +6913,7 @@
         </is>
       </c>
       <c r="E105" s="77" t="n">
-        <v>20509440</v>
+        <v>886307502.1920002</v>
       </c>
       <c r="F105" s="75" t="n">
         <v>46305</v>
@@ -6923,16 +6929,16 @@
     </row>
     <row r="106">
       <c r="A106" s="75" t="n">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B106" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C106" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/16/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
         </is>
       </c>
       <c r="D106" s="76" t="inlineStr">
@@ -6941,13 +6947,13 @@
         </is>
       </c>
       <c r="E106" s="77" t="n">
-        <v>2180000</v>
+        <v>5676698527.872001</v>
       </c>
       <c r="F106" s="75" t="n">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="G106" s="78" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H106" s="76" t="inlineStr">
         <is>
@@ -6957,16 +6963,16 @@
     </row>
     <row r="107">
       <c r="A107" s="75" t="n">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B107" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C107" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/17/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
         </is>
       </c>
       <c r="D107" s="76" t="inlineStr">
@@ -6975,13 +6981,13 @@
         </is>
       </c>
       <c r="E107" s="77" t="n">
-        <v>540640</v>
+        <v>564189103.6416</v>
       </c>
       <c r="F107" s="75" t="n">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="G107" s="78" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H107" s="76" t="inlineStr">
         <is>
@@ -6991,16 +6997,16 @@
     </row>
     <row r="108">
       <c r="A108" s="75" t="n">
-        <v>46305</v>
+        <v>46310</v>
       </c>
       <c r="B108" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C108" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/18/2026</t>
+          <t>PT.PSI/PT.CASI/REP/56/2026</t>
         </is>
       </c>
       <c r="D108" s="76" t="inlineStr">
@@ -7009,13 +7015,13 @@
         </is>
       </c>
       <c r="E108" s="77" t="n">
-        <v>47532720</v>
+        <v>5535207.48</v>
       </c>
       <c r="F108" s="75" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="G108" s="78" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="H108" s="76" t="inlineStr">
         <is>
@@ -7025,16 +7031,16 @@
     </row>
     <row r="109">
       <c r="A109" s="75" t="n">
-        <v>46305</v>
+        <v>46310</v>
       </c>
       <c r="B109" s="76" t="inlineStr">
         <is>
-          <t>PT East West Seed Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C109" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.EWINDO_LMB/19/2026</t>
+          <t>PT.PSI/PT.CASI/REP/57/2026</t>
         </is>
       </c>
       <c r="D109" s="76" t="inlineStr">
@@ -7043,13 +7049,13 @@
         </is>
       </c>
       <c r="E109" s="77" t="n">
-        <v>50794000</v>
+        <v>4392388.26</v>
       </c>
       <c r="F109" s="75" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="G109" s="78" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="H109" s="76" t="inlineStr">
         <is>
@@ -7059,16 +7065,16 @@
     </row>
     <row r="110">
       <c r="A110" s="75" t="n">
-        <v>46305</v>
+        <v>46310</v>
       </c>
       <c r="B110" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C110" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/38/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/58/2026</t>
         </is>
       </c>
       <c r="D110" s="76" t="inlineStr">
@@ -7077,13 +7083,13 @@
         </is>
       </c>
       <c r="E110" s="77" t="n">
-        <v>886307502.1920002</v>
+        <v>18129124.98186</v>
       </c>
       <c r="F110" s="75" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="G110" s="78" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="H110" s="76" t="inlineStr">
         <is>
@@ -7093,16 +7099,16 @@
     </row>
     <row r="111">
       <c r="A111" s="75" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="B111" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C111" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/39/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/59/2026</t>
         </is>
       </c>
       <c r="D111" s="76" t="inlineStr">
@@ -7111,13 +7117,13 @@
         </is>
       </c>
       <c r="E111" s="77" t="n">
-        <v>5676698527.872001</v>
+        <v>9884824431.36027</v>
       </c>
       <c r="F111" s="75" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="G111" s="78" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H111" s="76" t="inlineStr">
         <is>
@@ -7127,16 +7133,16 @@
     </row>
     <row r="112">
       <c r="A112" s="75" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="B112" s="76" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C112" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/40/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/60/2026</t>
         </is>
       </c>
       <c r="D112" s="76" t="inlineStr">
@@ -7145,13 +7151,13 @@
         </is>
       </c>
       <c r="E112" s="77" t="n">
-        <v>564189103.6416</v>
+        <v>700304033.0543</v>
       </c>
       <c r="F112" s="75" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="G112" s="78" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H112" s="76" t="inlineStr">
         <is>
@@ -7170,7 +7176,7 @@
       </c>
       <c r="C113" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/56/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/61/2026</t>
         </is>
       </c>
       <c r="D113" s="76" t="inlineStr">
@@ -7179,7 +7185,7 @@
         </is>
       </c>
       <c r="E113" s="77" t="n">
-        <v>5535207.48</v>
+        <v>1147400616.7888</v>
       </c>
       <c r="F113" s="75" t="n">
         <v>46304</v>
@@ -7204,7 +7210,7 @@
       </c>
       <c r="C114" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/REP/57/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/62/2026</t>
         </is>
       </c>
       <c r="D114" s="76" t="inlineStr">
@@ -7213,7 +7219,7 @@
         </is>
       </c>
       <c r="E114" s="77" t="n">
-        <v>4392388.26</v>
+        <v>4999029.5912</v>
       </c>
       <c r="F114" s="75" t="n">
         <v>46304</v>
@@ -7238,7 +7244,7 @@
       </c>
       <c r="C115" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/58/2026</t>
+          <t>PT.PSI/PT.CASI/FC-C/63/2026</t>
         </is>
       </c>
       <c r="D115" s="76" t="inlineStr">
@@ -7247,7 +7253,7 @@
         </is>
       </c>
       <c r="E115" s="77" t="n">
-        <v>18129124.98186</v>
+        <v>34933281.3146</v>
       </c>
       <c r="F115" s="75" t="n">
         <v>46304</v>
@@ -7272,7 +7278,7 @@
       </c>
       <c r="C116" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/59/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/64/2026</t>
         </is>
       </c>
       <c r="D116" s="76" t="inlineStr">
@@ -7281,7 +7287,7 @@
         </is>
       </c>
       <c r="E116" s="77" t="n">
-        <v>9884824431.36027</v>
+        <v>85105002.66900001</v>
       </c>
       <c r="F116" s="75" t="n">
         <v>46304</v>
@@ -7306,7 +7312,7 @@
       </c>
       <c r="C117" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/60/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/65/2026</t>
         </is>
       </c>
       <c r="D117" s="76" t="inlineStr">
@@ -7315,7 +7321,7 @@
         </is>
       </c>
       <c r="E117" s="77" t="n">
-        <v>700304033.0543</v>
+        <v>886098780.5445001</v>
       </c>
       <c r="F117" s="75" t="n">
         <v>46304</v>
@@ -7340,7 +7346,7 @@
       </c>
       <c r="C118" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/61/2026</t>
+          <t>PT.PSI/PT.CASI/FC-PS/66/2026</t>
         </is>
       </c>
       <c r="D118" s="76" t="inlineStr">
@@ -7349,7 +7355,7 @@
         </is>
       </c>
       <c r="E118" s="77" t="n">
-        <v>1147400616.7888</v>
+        <v>262631.43648</v>
       </c>
       <c r="F118" s="75" t="n">
         <v>46304</v>
@@ -7365,31 +7371,31 @@
     </row>
     <row r="119">
       <c r="A119" s="75" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="B119" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C119" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/62/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
         </is>
       </c>
       <c r="D119" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E119" s="77" t="n">
-        <v>4999029.5912</v>
+        <v>1365520000</v>
       </c>
       <c r="F119" s="75" t="n">
-        <v>46304</v>
+        <v>46312</v>
       </c>
       <c r="G119" s="78" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H119" s="76" t="inlineStr">
         <is>
@@ -7399,31 +7405,31 @@
     </row>
     <row r="120">
       <c r="A120" s="75" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="B120" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C120" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-C/63/2026</t>
+          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
         </is>
       </c>
       <c r="D120" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E120" s="77" t="n">
-        <v>34933281.3146</v>
+        <v>9687031.199999999</v>
       </c>
       <c r="F120" s="75" t="n">
-        <v>46304</v>
+        <v>46312</v>
       </c>
       <c r="G120" s="78" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H120" s="76" t="inlineStr">
         <is>
@@ -7433,31 +7439,31 @@
     </row>
     <row r="121">
       <c r="A121" s="75" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="B121" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C121" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/64/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
         </is>
       </c>
       <c r="D121" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E121" s="77" t="n">
-        <v>85105002.66900001</v>
+        <v>1070726250</v>
       </c>
       <c r="F121" s="75" t="n">
-        <v>46304</v>
+        <v>46312</v>
       </c>
       <c r="G121" s="78" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H121" s="76" t="inlineStr">
         <is>
@@ -7467,31 +7473,31 @@
     </row>
     <row r="122">
       <c r="A122" s="75" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="B122" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C122" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/65/2026</t>
+          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
         </is>
       </c>
       <c r="D122" s="76" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="E122" s="77" t="n">
-        <v>886098780.5445001</v>
+        <v>272700000</v>
       </c>
       <c r="F122" s="75" t="n">
-        <v>46304</v>
+        <v>46312</v>
       </c>
       <c r="G122" s="78" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H122" s="76" t="inlineStr">
         <is>
@@ -7501,16 +7507,16 @@
     </row>
     <row r="123">
       <c r="A123" s="75" t="n">
-        <v>46310</v>
+        <v>46314</v>
       </c>
       <c r="B123" s="76" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
+          <t>PT Syngenta Indonesia</t>
         </is>
       </c>
       <c r="C123" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.CASI/FC-PS/66/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
         </is>
       </c>
       <c r="D123" s="76" t="inlineStr">
@@ -7519,13 +7525,13 @@
         </is>
       </c>
       <c r="E123" s="77" t="n">
-        <v>262631.43648</v>
+        <v>545818781.4912</v>
       </c>
       <c r="F123" s="75" t="n">
-        <v>46304</v>
+        <v>46314</v>
       </c>
       <c r="G123" s="78" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="H123" s="76" t="inlineStr">
         <is>
@@ -7535,7 +7541,7 @@
     </row>
     <row r="124">
       <c r="A124" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B124" s="76" t="inlineStr">
         <is>
@@ -7544,22 +7550,22 @@
       </c>
       <c r="C124" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-CS-PIER2/35/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
         </is>
       </c>
       <c r="D124" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E124" s="77" t="n">
-        <v>1365520000</v>
+        <v>767367847.5204</v>
       </c>
       <c r="F124" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="G124" s="78" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H124" s="76" t="inlineStr">
         <is>
@@ -7569,7 +7575,7 @@
     </row>
     <row r="125">
       <c r="A125" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B125" s="76" t="inlineStr">
         <is>
@@ -7578,22 +7584,22 @@
       </c>
       <c r="C125" s="76" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT.PSI/PT.SSI/RENTAL-H-PIER2/36/2026 </t>
+          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
         </is>
       </c>
       <c r="D125" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E125" s="77" t="n">
-        <v>9687031.199999999</v>
+        <v>4761468367.9458</v>
       </c>
       <c r="F125" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="G125" s="78" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H125" s="76" t="inlineStr">
         <is>
@@ -7603,7 +7609,7 @@
     </row>
     <row r="126">
       <c r="A126" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B126" s="76" t="inlineStr">
         <is>
@@ -7612,22 +7618,22 @@
       </c>
       <c r="C126" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-CS-MLG/37/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
         </is>
       </c>
       <c r="D126" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E126" s="77" t="n">
-        <v>1070726250</v>
+        <v>442076465.292</v>
       </c>
       <c r="F126" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="G126" s="78" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H126" s="76" t="inlineStr">
         <is>
@@ -7637,7 +7643,7 @@
     </row>
     <row r="127">
       <c r="A127" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B127" s="76" t="inlineStr">
         <is>
@@ -7646,22 +7652,22 @@
       </c>
       <c r="C127" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/RENTAL-WH-MLG/38/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
         </is>
       </c>
       <c r="D127" s="76" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="E127" s="77" t="n">
-        <v>272700000</v>
+        <v>444456984.744</v>
       </c>
       <c r="F127" s="75" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="G127" s="78" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H127" s="76" t="inlineStr">
         <is>
@@ -7671,7 +7677,7 @@
     </row>
     <row r="128">
       <c r="A128" s="75" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="B128" s="76" t="inlineStr">
         <is>
@@ -7680,7 +7686,7 @@
       </c>
       <c r="C128" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/41/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/45/2026</t>
         </is>
       </c>
       <c r="D128" s="76" t="inlineStr">
@@ -7689,13 +7695,13 @@
         </is>
       </c>
       <c r="E128" s="77" t="n">
-        <v>545818781.4912</v>
+        <v>337392787.2479999</v>
       </c>
       <c r="F128" s="75" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="G128" s="78" t="n">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="H128" s="76" t="inlineStr">
         <is>
@@ -7705,7 +7711,7 @@
     </row>
     <row r="129">
       <c r="A129" s="75" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="B129" s="76" t="inlineStr">
         <is>
@@ -7714,7 +7720,7 @@
       </c>
       <c r="C129" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/42/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/46/2026</t>
         </is>
       </c>
       <c r="D129" s="76" t="inlineStr">
@@ -7723,13 +7729,13 @@
         </is>
       </c>
       <c r="E129" s="77" t="n">
-        <v>767367847.5204</v>
+        <v>8211508178.4966</v>
       </c>
       <c r="F129" s="75" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="G129" s="78" t="n">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="H129" s="76" t="inlineStr">
         <is>
@@ -7739,7 +7745,7 @@
     </row>
     <row r="130">
       <c r="A130" s="75" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="B130" s="76" t="inlineStr">
         <is>
@@ -7748,7 +7754,7 @@
       </c>
       <c r="C130" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/43/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/47/2026</t>
         </is>
       </c>
       <c r="D130" s="76" t="inlineStr">
@@ -7757,13 +7763,13 @@
         </is>
       </c>
       <c r="E130" s="77" t="n">
-        <v>4761468367.9458</v>
+        <v>903022062.8508</v>
       </c>
       <c r="F130" s="75" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="G130" s="78" t="n">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="H130" s="76" t="inlineStr">
         <is>
@@ -7773,7 +7779,7 @@
     </row>
     <row r="131">
       <c r="A131" s="75" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="B131" s="76" t="inlineStr">
         <is>
@@ -7782,7 +7788,7 @@
       </c>
       <c r="C131" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/48/2026</t>
         </is>
       </c>
       <c r="D131" s="76" t="inlineStr">
@@ -7791,13 +7797,13 @@
         </is>
       </c>
       <c r="E131" s="77" t="n">
-        <v>442076465.292</v>
+        <v>1912679476.3662</v>
       </c>
       <c r="F131" s="75" t="n">
-        <v>46314</v>
+        <v>46325</v>
       </c>
       <c r="G131" s="78" t="n">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="H131" s="76" t="inlineStr">
         <is>
@@ -7807,7 +7813,7 @@
     </row>
     <row r="132">
       <c r="A132" s="75" t="n">
-        <v>46314</v>
+        <v>46328</v>
       </c>
       <c r="B132" s="76" t="inlineStr">
         <is>
@@ -7816,7 +7822,7 @@
       </c>
       <c r="C132" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/44/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/49/2026</t>
         </is>
       </c>
       <c r="D132" s="76" t="inlineStr">
@@ -7825,13 +7831,13 @@
         </is>
       </c>
       <c r="E132" s="77" t="n">
-        <v>444456984.744</v>
+        <v>479734948.6272</v>
       </c>
       <c r="F132" s="75" t="n">
-        <v>46314</v>
+        <v>46328</v>
       </c>
       <c r="G132" s="78" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="H132" s="76" t="inlineStr">
         <is>
@@ -7841,7 +7847,7 @@
     </row>
     <row r="133">
       <c r="A133" s="75" t="n">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="B133" s="76" t="inlineStr">
         <is>
@@ -7850,7 +7856,7 @@
       </c>
       <c r="C133" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/45/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/50/2026</t>
         </is>
       </c>
       <c r="D133" s="76" t="inlineStr">
@@ -7859,13 +7865,13 @@
         </is>
       </c>
       <c r="E133" s="77" t="n">
-        <v>337392787.2479999</v>
+        <v>3340238430.648</v>
       </c>
       <c r="F133" s="75" t="n">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="G133" s="78" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H133" s="76" t="inlineStr">
         <is>
@@ -7875,7 +7881,7 @@
     </row>
     <row r="134">
       <c r="A134" s="75" t="n">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="B134" s="76" t="inlineStr">
         <is>
@@ -7884,7 +7890,7 @@
       </c>
       <c r="C134" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/46/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/51/2026</t>
         </is>
       </c>
       <c r="D134" s="76" t="inlineStr">
@@ -7893,13 +7899,13 @@
         </is>
       </c>
       <c r="E134" s="77" t="n">
-        <v>8211508178.4966</v>
+        <v>530510117.7436</v>
       </c>
       <c r="F134" s="75" t="n">
-        <v>46325</v>
+        <v>46328</v>
       </c>
       <c r="G134" s="78" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H134" s="76" t="inlineStr">
         <is>
@@ -7909,7 +7915,7 @@
     </row>
     <row r="135">
       <c r="A135" s="75" t="n">
-        <v>46325</v>
+        <v>46335</v>
       </c>
       <c r="B135" s="76" t="inlineStr">
         <is>
@@ -7918,7 +7924,7 @@
       </c>
       <c r="C135" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/47/2026</t>
+          <t>PT.PSI/PT.SSI/SWC/01/2026</t>
         </is>
       </c>
       <c r="D135" s="76" t="inlineStr">
@@ -7927,13 +7933,13 @@
         </is>
       </c>
       <c r="E135" s="77" t="n">
-        <v>903022062.8508</v>
+        <v>2345778403.95195</v>
       </c>
       <c r="F135" s="75" t="n">
-        <v>46325</v>
+        <v>46335</v>
       </c>
       <c r="G135" s="78" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="H135" s="76" t="inlineStr">
         <is>
@@ -7943,7 +7949,7 @@
     </row>
     <row r="136">
       <c r="A136" s="75" t="n">
-        <v>46325</v>
+        <v>46336</v>
       </c>
       <c r="B136" s="76" t="inlineStr">
         <is>
@@ -7952,7 +7958,7 @@
       </c>
       <c r="C136" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/48/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/52/IX/2026</t>
         </is>
       </c>
       <c r="D136" s="76" t="inlineStr">
@@ -7961,13 +7967,13 @@
         </is>
       </c>
       <c r="E136" s="77" t="n">
-        <v>1912679476.3662</v>
+        <v>3872356057.5561</v>
       </c>
       <c r="F136" s="75" t="n">
-        <v>46325</v>
+        <v>46336</v>
       </c>
       <c r="G136" s="78" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="H136" s="76" t="inlineStr">
         <is>
@@ -7977,7 +7983,7 @@
     </row>
     <row r="137">
       <c r="A137" s="75" t="n">
-        <v>46328</v>
+        <v>46336</v>
       </c>
       <c r="B137" s="76" t="inlineStr">
         <is>
@@ -7986,7 +7992,7 @@
       </c>
       <c r="C137" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/49/2026</t>
+          <t>PT.PSI/PT.SSI/TC-MLG/52/IX/2026</t>
         </is>
       </c>
       <c r="D137" s="76" t="inlineStr">
@@ -7995,13 +8001,13 @@
         </is>
       </c>
       <c r="E137" s="77" t="n">
-        <v>479734948.6272</v>
+        <v>3951681440.2902</v>
       </c>
       <c r="F137" s="75" t="n">
-        <v>46328</v>
+        <v>46336</v>
       </c>
       <c r="G137" s="78" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="H137" s="76" t="inlineStr">
         <is>
@@ -8011,7 +8017,7 @@
     </row>
     <row r="138">
       <c r="A138" s="75" t="n">
-        <v>46328</v>
+        <v>46336</v>
       </c>
       <c r="B138" s="76" t="inlineStr">
         <is>
@@ -8020,7 +8026,7 @@
       </c>
       <c r="C138" s="76" t="inlineStr">
         <is>
-          <t>PT.PSI/PT.SSI/TC-MLG/50/2026</t>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/53/IX/2026</t>
         </is>
       </c>
       <c r="D138" s="76" t="inlineStr">
@@ -8029,13 +8035,13 @@
         </is>
       </c>
       <c r="E138" s="77" t="n">
-        <v>3340238430.648</v>
+        <v>539961649.7706</v>
       </c>
       <c r="F138" s="75" t="n">
-        <v>46328</v>
+        <v>46336</v>
       </c>
       <c r="G138" s="78" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="H138" s="76" t="inlineStr">
         <is>
@@ -8044,92 +8050,24 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="75" t="n">
-        <v>46328</v>
-      </c>
-      <c r="B139" s="76" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="C139" s="76" t="inlineStr">
-        <is>
-          <t>PT.PSI/PT.SSI/TC-PAS 2/51/2026</t>
-        </is>
-      </c>
-      <c r="D139" s="76" t="inlineStr">
-        <is>
-          <t>Tolling</t>
-        </is>
-      </c>
-      <c r="E139" s="77" t="n">
-        <v>530510117.7436</v>
-      </c>
-      <c r="F139" s="75" t="n">
-        <v>46328</v>
-      </c>
-      <c r="G139" s="78" t="n">
-        <v>52</v>
-      </c>
-      <c r="H139" s="76" t="inlineStr">
-        <is>
-          <t>Future</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="75" t="n">
-        <v>46335</v>
-      </c>
-      <c r="B140" s="76" t="inlineStr">
-        <is>
-          <t>PT Syngenta Indonesia</t>
-        </is>
-      </c>
-      <c r="C140" s="76" t="inlineStr">
-        <is>
-          <t>PT.PSI/PT.SSI/SWC/01/2026</t>
-        </is>
-      </c>
-      <c r="D140" s="76" t="inlineStr">
-        <is>
-          <t>Tolling</t>
-        </is>
-      </c>
-      <c r="E140" s="77" t="n">
-        <v>2345778403.95195</v>
-      </c>
-      <c r="F140" s="75" t="n">
-        <v>46335</v>
-      </c>
-      <c r="G140" s="78" t="n">
-        <v>59</v>
-      </c>
-      <c r="H140" s="76" t="inlineStr">
-        <is>
-          <t>Future</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="39" t="inlineStr">
+      <c r="A139" s="39" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B141" s="79" t="n"/>
-      <c r="C141" s="79" t="n"/>
-      <c r="D141" s="79" t="n"/>
-      <c r="E141" s="80">
-        <f>SUM(E5:E140)</f>
+      <c r="B139" s="79" t="n"/>
+      <c r="C139" s="79" t="n"/>
+      <c r="D139" s="79" t="n"/>
+      <c r="E139" s="80">
+        <f>SUM(E5:E138)</f>
         <v/>
       </c>
-      <c r="F141" s="79" t="n"/>
-      <c r="G141" s="79" t="n"/>
-      <c r="H141" s="79" t="n"/>
+      <c r="F139" s="79" t="n"/>
+      <c r="G139" s="79" t="n"/>
+      <c r="H139" s="79" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H141"/>
+  <autoFilter ref="A4:H139"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10171,28 +10109,28 @@
         <v>30034252167.1542</v>
       </c>
       <c r="BQ13" s="86" t="n">
-        <v>28706651567.7154</v>
+        <v>32579007625.2715</v>
       </c>
       <c r="BR13" s="36" t="n">
-        <v>1327600599.438805</v>
+        <v>-2544755458.117294</v>
       </c>
       <c r="BS13" s="85" t="n">
-        <v>6696261900.97075</v>
+        <v>15060261048.58765</v>
       </c>
       <c r="BT13" s="86" t="n">
-        <v>0</v>
+        <v>4491643090.0608</v>
       </c>
       <c r="BU13" s="36" t="n">
-        <v>6696261900.97075</v>
+        <v>10568617958.52685</v>
       </c>
       <c r="BV13" s="40" t="n">
-        <v>158803515500.6789</v>
+        <v>167167514648.2958</v>
       </c>
       <c r="BW13" s="40" t="n">
-        <v>158803515500.6789</v>
+        <v>167167514648.2958</v>
       </c>
       <c r="BX13" s="40" t="n">
-        <v>3.0517578125e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -12437,25 +12375,25 @@
         <v>7049979</v>
       </c>
       <c r="BQ24" s="90" t="n">
-        <v>6917350</v>
+        <v>7929259</v>
       </c>
       <c r="BR24" s="91" t="n">
-        <v>132629</v>
+        <v>-879280</v>
       </c>
       <c r="BS24" s="89" t="n">
-        <v>1073454.95</v>
+        <v>3157199.95</v>
       </c>
       <c r="BT24" s="90" t="n">
-        <v>0</v>
+        <v>1071836</v>
       </c>
       <c r="BU24" s="91" t="n">
-        <v>1073454.95</v>
+        <v>2085363.95</v>
       </c>
       <c r="BV24" s="92" t="n">
-        <v>40218526.96</v>
+        <v>42302271.96</v>
       </c>
       <c r="BW24" s="92" t="n">
-        <v>40218526.96</v>
+        <v>42302271.96</v>
       </c>
       <c r="BX24" s="92" t="n">
         <v>0</v>
@@ -16800,20 +16738,20 @@
         </is>
       </c>
       <c r="B16" s="36" t="n">
-        <v>46480561464.36454</v>
+        <v>50352917521.92064</v>
       </c>
       <c r="C16" s="36" t="n">
         <v>46435325979.07042</v>
       </c>
-      <c r="D16" s="36" t="n">
-        <v>45235485.29412079</v>
+      <c r="D16" s="97" t="n">
+        <v>3917591542.85022</v>
       </c>
       <c r="E16" s="98" t="n">
-        <v>0.9990267870294811</v>
+        <v>0.9221973276693504</v>
       </c>
       <c r="F16" s="99" t="inlineStr">
         <is>
-          <t>On track</t>
+          <t>Partially uninvoiced</t>
         </is>
       </c>
     </row>
@@ -16824,20 +16762,20 @@
         </is>
       </c>
       <c r="B17" s="36" t="n">
-        <v>0</v>
+        <v>4491643090.0608</v>
       </c>
       <c r="C17" s="36" t="n">
-        <v>25157800975.93113</v>
+        <v>33521800123.54803</v>
       </c>
       <c r="D17" s="100" t="n">
-        <v>-25157800975.93113</v>
+        <v>-29030157033.48723</v>
       </c>
       <c r="E17" s="98" t="n">
-        <v>0</v>
+        <v>7.463148663286662</v>
       </c>
       <c r="F17" s="99" t="inlineStr">
         <is>
-          <t>Billing only (prior-month catch-up)</t>
+          <t>Catch-up: prior-month invoices issued</t>
         </is>
       </c>
     </row>
@@ -16920,7 +16858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1118"/>
+  <dimension ref="A1:Q1120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -81436,10 +81374,12 @@
       <c r="E1021" s="104" t="n">
         <v>46276</v>
       </c>
-      <c r="F1021" s="103" t="n"/>
+      <c r="F1021" s="104" t="n">
+        <v>46276</v>
+      </c>
       <c r="G1021" s="103" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H1021" s="103" t="inlineStr">
@@ -81465,19 +81405,13 @@
       <c r="N1021" s="105" t="n">
         <v>3981599123.659349</v>
       </c>
-      <c r="O1021" s="103" t="n">
-        <v>0</v>
-      </c>
+      <c r="O1021" s="103" t="n"/>
       <c r="P1021" s="103" t="inlineStr">
         <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
-      <c r="Q1021" s="103" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="Q1021" s="103" t="n"/>
     </row>
     <row r="1022">
       <c r="A1022" s="103" t="inlineStr">
@@ -81501,10 +81435,12 @@
       <c r="E1022" s="104" t="n">
         <v>46276</v>
       </c>
-      <c r="F1022" s="103" t="n"/>
+      <c r="F1022" s="104" t="n">
+        <v>46276</v>
+      </c>
       <c r="G1022" s="103" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H1022" s="103" t="inlineStr">
@@ -81530,19 +81466,13 @@
       <c r="N1022" s="105" t="n">
         <v>1542175442.6694</v>
       </c>
-      <c r="O1022" s="103" t="n">
-        <v>0</v>
-      </c>
+      <c r="O1022" s="103" t="n"/>
       <c r="P1022" s="103" t="inlineStr">
         <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
-      <c r="Q1022" s="103" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="Q1022" s="103" t="n"/>
     </row>
     <row r="1023">
       <c r="A1023" s="103" t="inlineStr">
@@ -81566,10 +81496,12 @@
       <c r="E1023" s="104" t="n">
         <v>46276</v>
       </c>
-      <c r="F1023" s="103" t="n"/>
+      <c r="F1023" s="104" t="n">
+        <v>46276</v>
+      </c>
       <c r="G1023" s="103" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H1023" s="103" t="inlineStr">
@@ -81595,19 +81527,13 @@
       <c r="N1023" s="105" t="n">
         <v>487978078.30875</v>
       </c>
-      <c r="O1023" s="103" t="n">
-        <v>0</v>
-      </c>
+      <c r="O1023" s="103" t="n"/>
       <c r="P1023" s="103" t="inlineStr">
         <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
-      <c r="Q1023" s="103" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="Q1023" s="103" t="n"/>
     </row>
     <row r="1024">
       <c r="A1024" s="103" t="inlineStr">
@@ -81631,10 +81557,12 @@
       <c r="E1024" s="104" t="n">
         <v>46276</v>
       </c>
-      <c r="F1024" s="103" t="n"/>
+      <c r="F1024" s="104" t="n">
+        <v>46276</v>
+      </c>
       <c r="G1024" s="103" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="H1024" s="103" t="inlineStr">
@@ -81660,19 +81588,13 @@
       <c r="N1024" s="105" t="n">
         <v>14255050.74672</v>
       </c>
-      <c r="O1024" s="103" t="n">
-        <v>0</v>
-      </c>
+      <c r="O1024" s="103" t="n"/>
       <c r="P1024" s="103" t="inlineStr">
         <is>
-          <t>NOT YET DUE</t>
-        </is>
-      </c>
-      <c r="Q1024" s="103" t="inlineStr">
-        <is>
-          <t>0-30</t>
-        </is>
-      </c>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="Q1024" s="103" t="n"/>
     </row>
     <row r="1025">
       <c r="A1025" s="103" t="inlineStr">
@@ -87106,21 +87028,29 @@
       </c>
       <c r="B1109" s="103" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C1109" s="103" t="n"/>
-      <c r="D1109" s="103" t="n"/>
-      <c r="E1109" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1109" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/52/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1109" s="104" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E1109" s="104" t="n">
+        <v>46336</v>
+      </c>
       <c r="F1109" s="103" t="n"/>
       <c r="G1109" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1109" s="103" t="inlineStr">
         <is>
-          <t>FC</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1109" s="103" t="inlineStr">
@@ -87130,22 +87060,28 @@
       </c>
       <c r="J1109" s="103" t="n"/>
       <c r="K1109" s="104" t="n">
-        <v>46235</v>
+        <v>46261</v>
       </c>
       <c r="L1109" s="104" t="n">
         <v>46265</v>
       </c>
       <c r="M1109" s="105" t="n">
-        <v>3256990</v>
+        <v>1011909</v>
       </c>
       <c r="N1109" s="105" t="n">
-        <v>13247943944.279</v>
-      </c>
-      <c r="O1109" s="103" t="n"/>
-      <c r="P1109" s="103" t="n"/>
+        <v>3872356057.5561</v>
+      </c>
+      <c r="O1109" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1109" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1109" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -87157,21 +87093,29 @@
       </c>
       <c r="B1110" s="103" t="inlineStr">
         <is>
-          <t>PT Advanta Seeds Indonesia</t>
-        </is>
-      </c>
-      <c r="C1110" s="103" t="n"/>
-      <c r="D1110" s="103" t="n"/>
-      <c r="E1110" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1110" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-MLG/52/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1110" s="104" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E1110" s="104" t="n">
+        <v>46336</v>
+      </c>
       <c r="F1110" s="103" t="n"/>
       <c r="G1110" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1110" s="103" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1110" s="103" t="inlineStr">
@@ -87181,22 +87125,28 @@
       </c>
       <c r="J1110" s="103" t="n"/>
       <c r="K1110" s="104" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="L1110" s="104" t="n">
-        <v>46265</v>
+        <v>46271</v>
       </c>
       <c r="M1110" s="105" t="n">
-        <v>140026</v>
+        <v>1032638</v>
       </c>
       <c r="N1110" s="105" t="n">
-        <v>1122459338.028</v>
-      </c>
-      <c r="O1110" s="103" t="n"/>
-      <c r="P1110" s="103" t="n"/>
+        <v>3951681440.2902</v>
+      </c>
+      <c r="O1110" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1110" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1110" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -87208,46 +87158,60 @@
       </c>
       <c r="B1111" s="103" t="inlineStr">
         <is>
-          <t>PT Corteva Agriscience Seed Indonesia</t>
-        </is>
-      </c>
-      <c r="C1111" s="103" t="n"/>
-      <c r="D1111" s="103" t="n"/>
-      <c r="E1111" s="103" t="n"/>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1111" s="103" t="inlineStr">
+        <is>
+          <t>PT.PSI/PT.SSI/TC-PAS 2/53/IX/2026</t>
+        </is>
+      </c>
+      <c r="D1111" s="104" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E1111" s="104" t="n">
+        <v>46336</v>
+      </c>
       <c r="F1111" s="103" t="n"/>
       <c r="G1111" s="103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H1111" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="I1111" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1111" s="103" t="n"/>
       <c r="K1111" s="104" t="n">
-        <v>46235</v>
+        <v>46267</v>
       </c>
       <c r="L1111" s="104" t="n">
-        <v>46265</v>
+        <v>46269</v>
       </c>
       <c r="M1111" s="105" t="n">
-        <v>1654962.70767742</v>
+        <v>39198</v>
       </c>
       <c r="N1111" s="105" t="n">
-        <v>593353779.5835853</v>
-      </c>
-      <c r="O1111" s="103" t="n"/>
-      <c r="P1111" s="103" t="n"/>
+        <v>539961649.7706</v>
+      </c>
+      <c r="O1111" s="103" t="n">
+        <v>-60</v>
+      </c>
+      <c r="P1111" s="103" t="inlineStr">
+        <is>
+          <t>NOT YET DUE</t>
+        </is>
+      </c>
       <c r="Q1111" s="103" t="inlineStr">
         <is>
-          <t>0-30</t>
+          <t>NOT YET DUE</t>
         </is>
       </c>
     </row>
@@ -87259,7 +87223,7 @@
       </c>
       <c r="B1112" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1112" s="103" t="n"/>
@@ -87273,7 +87237,7 @@
       </c>
       <c r="H1112" s="103" t="inlineStr">
         <is>
-          <t>COMM</t>
+          <t>FC</t>
         </is>
       </c>
       <c r="I1112" s="103" t="inlineStr">
@@ -87289,10 +87253,10 @@
         <v>46265</v>
       </c>
       <c r="M1112" s="105" t="n">
-        <v>1878336</v>
+        <v>3256990</v>
       </c>
       <c r="N1112" s="105" t="n">
-        <v>7266583243.008001</v>
+        <v>13247943944.279</v>
       </c>
       <c r="O1112" s="103" t="n"/>
       <c r="P1112" s="103" t="n"/>
@@ -87310,7 +87274,7 @@
       </c>
       <c r="B1113" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Advanta Seeds Indonesia</t>
         </is>
       </c>
       <c r="C1113" s="103" t="n"/>
@@ -87324,12 +87288,12 @@
       </c>
       <c r="H1113" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="I1113" s="103" t="inlineStr">
         <is>
-          <t>Rental</t>
+          <t>Tolling</t>
         </is>
       </c>
       <c r="J1113" s="103" t="n"/>
@@ -87340,10 +87304,10 @@
         <v>46265</v>
       </c>
       <c r="M1113" s="105" t="n">
-        <v>1660000</v>
+        <v>140026</v>
       </c>
       <c r="N1113" s="105" t="n">
-        <v>552691555.2</v>
+        <v>1122459338.028</v>
       </c>
       <c r="O1113" s="103" t="n"/>
       <c r="P1113" s="103" t="n"/>
@@ -87361,7 +87325,7 @@
       </c>
       <c r="B1114" s="103" t="inlineStr">
         <is>
-          <t>PT Syngenta Indonesia</t>
+          <t>PT Corteva Agriscience Seed Indonesia</t>
         </is>
       </c>
       <c r="C1114" s="103" t="n"/>
@@ -87391,10 +87355,10 @@
         <v>46265</v>
       </c>
       <c r="M1114" s="105" t="n">
-        <v>1660000</v>
+        <v>1654962.70767742</v>
       </c>
       <c r="N1114" s="105" t="n">
-        <v>552691555.2</v>
+        <v>593353779.5835853</v>
       </c>
       <c r="O1114" s="103" t="n"/>
       <c r="P1114" s="103" t="n"/>
@@ -87426,7 +87390,7 @@
       </c>
       <c r="H1115" s="103" t="inlineStr">
         <is>
-          <t>RENTAL</t>
+          <t>RENTAL CS</t>
         </is>
       </c>
       <c r="I1115" s="103" t="inlineStr">
@@ -87442,10 +87406,10 @@
         <v>46265</v>
       </c>
       <c r="M1115" s="105" t="n">
-        <v>855000</v>
+        <v>1660000</v>
       </c>
       <c r="N1115" s="105" t="n">
-        <v>71167361.40000001</v>
+        <v>552691555.2</v>
       </c>
       <c r="O1115" s="103" t="n"/>
       <c r="P1115" s="103" t="n"/>
@@ -87477,7 +87441,7 @@
       </c>
       <c r="H1116" s="103" t="inlineStr">
         <is>
-          <t>RENTAL</t>
+          <t>RENTAL CS</t>
         </is>
       </c>
       <c r="I1116" s="103" t="inlineStr">
@@ -87493,10 +87457,10 @@
         <v>46265</v>
       </c>
       <c r="M1116" s="105" t="n">
-        <v>3600000</v>
+        <v>1660000</v>
       </c>
       <c r="N1116" s="105" t="n">
-        <v>299652048</v>
+        <v>552691555.2</v>
       </c>
       <c r="O1116" s="103" t="n"/>
       <c r="P1116" s="103" t="n"/>
@@ -87528,12 +87492,12 @@
       </c>
       <c r="H1117" s="103" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>RENTAL</t>
         </is>
       </c>
       <c r="I1117" s="103" t="inlineStr">
         <is>
-          <t>Tolling</t>
+          <t>Rental</t>
         </is>
       </c>
       <c r="J1117" s="103" t="n"/>
@@ -87544,10 +87508,10 @@
         <v>46265</v>
       </c>
       <c r="M1117" s="105" t="n">
-        <v>855189</v>
+        <v>855000</v>
       </c>
       <c r="N1117" s="105" t="n">
-        <v>5789714193.710999</v>
+        <v>71167361.40000001</v>
       </c>
       <c r="O1117" s="103" t="n"/>
       <c r="P1117" s="103" t="n"/>
@@ -87579,7 +87543,7 @@
       </c>
       <c r="H1118" s="103" t="inlineStr">
         <is>
-          <t>RENTAL CS</t>
+          <t>RENTAL</t>
         </is>
       </c>
       <c r="I1118" s="103" t="inlineStr">
@@ -87595,10 +87559,10 @@
         <v>46265</v>
       </c>
       <c r="M1118" s="105" t="n">
-        <v>4000000</v>
+        <v>3600000</v>
       </c>
       <c r="N1118" s="105" t="n">
-        <v>1605326400</v>
+        <v>299652048</v>
       </c>
       <c r="O1118" s="103" t="n"/>
       <c r="P1118" s="103" t="n"/>
@@ -87608,8 +87572,110 @@
         </is>
       </c>
     </row>
+    <row r="1119">
+      <c r="A1119" s="103" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B1119" s="103" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1119" s="103" t="n"/>
+      <c r="D1119" s="103" t="n"/>
+      <c r="E1119" s="103" t="n"/>
+      <c r="F1119" s="103" t="n"/>
+      <c r="G1119" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1119" s="103" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="I1119" s="103" t="inlineStr">
+        <is>
+          <t>Tolling</t>
+        </is>
+      </c>
+      <c r="J1119" s="103" t="n"/>
+      <c r="K1119" s="104" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1119" s="104" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1119" s="105" t="n">
+        <v>855189</v>
+      </c>
+      <c r="N1119" s="105" t="n">
+        <v>5789714193.710999</v>
+      </c>
+      <c r="O1119" s="103" t="n"/>
+      <c r="P1119" s="103" t="n"/>
+      <c r="Q1119" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="103" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B1120" s="103" t="inlineStr">
+        <is>
+          <t>PT Syngenta Indonesia</t>
+        </is>
+      </c>
+      <c r="C1120" s="103" t="n"/>
+      <c r="D1120" s="103" t="n"/>
+      <c r="E1120" s="103" t="n"/>
+      <c r="F1120" s="103" t="n"/>
+      <c r="G1120" s="103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H1120" s="103" t="inlineStr">
+        <is>
+          <t>RENTAL CS</t>
+        </is>
+      </c>
+      <c r="I1120" s="103" t="inlineStr">
+        <is>
+          <t>Rental</t>
+        </is>
+      </c>
+      <c r="J1120" s="103" t="n"/>
+      <c r="K1120" s="104" t="n">
+        <v>46235</v>
+      </c>
+      <c r="L1120" s="104" t="n">
+        <v>46265</v>
+      </c>
+      <c r="M1120" s="105" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="N1120" s="105" t="n">
+        <v>1605326400</v>
+      </c>
+      <c r="O1120" s="103" t="n"/>
+      <c r="P1120" s="103" t="n"/>
+      <c r="Q1120" s="103" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q1118"/>
+  <autoFilter ref="A1:Q1120"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>